<commit_message>
Fase 4: cierre de resultados 2026-09-15
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1111"/>
+  <dimension ref="A1:L1142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47329,8 +47329,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1020" t="inlineStr"/>
-      <c r="F1020" t="inlineStr"/>
       <c r="G1020" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -47377,8 +47375,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1021" t="inlineStr"/>
-      <c r="F1021" t="inlineStr"/>
       <c r="G1021" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -47425,8 +47421,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1022" t="inlineStr"/>
-      <c r="F1022" t="inlineStr"/>
       <c r="G1022" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -47473,8 +47467,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1023" t="inlineStr"/>
-      <c r="F1023" t="inlineStr"/>
       <c r="G1023" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -47521,8 +47513,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1024" t="inlineStr"/>
-      <c r="F1024" t="inlineStr"/>
       <c r="G1024" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -47569,8 +47559,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1025" t="inlineStr"/>
-      <c r="F1025" t="inlineStr"/>
       <c r="G1025" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -47617,8 +47605,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1026" t="inlineStr"/>
-      <c r="F1026" t="inlineStr"/>
       <c r="G1026" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -47665,8 +47651,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1027" t="inlineStr"/>
-      <c r="F1027" t="inlineStr"/>
       <c r="G1027" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -47713,8 +47697,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1028" t="inlineStr"/>
-      <c r="F1028" t="inlineStr"/>
       <c r="G1028" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -47761,8 +47743,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1029" t="inlineStr"/>
-      <c r="F1029" t="inlineStr"/>
       <c r="G1029" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -47809,8 +47789,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1030" t="inlineStr"/>
-      <c r="F1030" t="inlineStr"/>
       <c r="G1030" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -47857,8 +47835,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1031" t="inlineStr"/>
-      <c r="F1031" t="inlineStr"/>
       <c r="G1031" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -47905,8 +47881,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1032" t="inlineStr"/>
-      <c r="F1032" t="inlineStr"/>
       <c r="G1032" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -47953,8 +47927,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1033" t="inlineStr"/>
-      <c r="F1033" t="inlineStr"/>
       <c r="G1033" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -48001,8 +47973,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1034" t="inlineStr"/>
-      <c r="F1034" t="inlineStr"/>
       <c r="G1034" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -48049,8 +48019,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1035" t="inlineStr"/>
-      <c r="F1035" t="inlineStr"/>
       <c r="G1035" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -48097,8 +48065,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1036" t="inlineStr"/>
-      <c r="F1036" t="inlineStr"/>
       <c r="G1036" t="inlineStr">
         <is>
           <t>8-1</t>
@@ -48145,8 +48111,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1037" t="inlineStr"/>
-      <c r="F1037" t="inlineStr"/>
       <c r="G1037" t="inlineStr">
         <is>
           <t>0-5</t>
@@ -48193,8 +48157,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1038" t="inlineStr"/>
-      <c r="F1038" t="inlineStr"/>
       <c r="G1038" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -48241,8 +48203,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1039" t="inlineStr"/>
-      <c r="F1039" t="inlineStr"/>
       <c r="G1039" t="inlineStr">
         <is>
           <t>5-1</t>
@@ -48289,8 +48249,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1040" t="inlineStr"/>
-      <c r="F1040" t="inlineStr"/>
       <c r="G1040" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -48337,8 +48295,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1041" t="inlineStr"/>
-      <c r="F1041" t="inlineStr"/>
       <c r="G1041" t="inlineStr">
         <is>
           <t>5-0</t>
@@ -48385,8 +48341,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1042" t="inlineStr"/>
-      <c r="F1042" t="inlineStr"/>
       <c r="G1042" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -48433,8 +48387,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1043" t="inlineStr"/>
-      <c r="F1043" t="inlineStr"/>
       <c r="G1043" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -48481,8 +48433,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1044" t="inlineStr"/>
-      <c r="F1044" t="inlineStr"/>
       <c r="G1044" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -48529,8 +48479,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1045" t="inlineStr"/>
-      <c r="F1045" t="inlineStr"/>
       <c r="G1045" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -48577,8 +48525,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1046" t="inlineStr"/>
-      <c r="F1046" t="inlineStr"/>
       <c r="G1046" t="inlineStr">
         <is>
           <t>2-4</t>
@@ -48625,8 +48571,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1047" t="inlineStr"/>
-      <c r="F1047" t="inlineStr"/>
       <c r="G1047" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -48673,8 +48617,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1048" t="inlineStr"/>
-      <c r="F1048" t="inlineStr"/>
       <c r="G1048" t="inlineStr">
         <is>
           <t>0-7</t>
@@ -48721,8 +48663,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1049" t="inlineStr"/>
-      <c r="F1049" t="inlineStr"/>
       <c r="G1049" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -48769,8 +48709,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1050" t="inlineStr"/>
-      <c r="F1050" t="inlineStr"/>
       <c r="G1050" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -48817,8 +48755,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1051" t="inlineStr"/>
-      <c r="F1051" t="inlineStr"/>
       <c r="G1051" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -48865,8 +48801,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1052" t="inlineStr"/>
-      <c r="F1052" t="inlineStr"/>
       <c r="G1052" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -48913,8 +48847,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1053" t="inlineStr"/>
-      <c r="F1053" t="inlineStr"/>
       <c r="G1053" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -48961,8 +48893,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1054" t="inlineStr"/>
-      <c r="F1054" t="inlineStr"/>
       <c r="G1054" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -49009,8 +48939,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1055" t="inlineStr"/>
-      <c r="F1055" t="inlineStr"/>
       <c r="G1055" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -49057,8 +48985,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1056" t="inlineStr"/>
-      <c r="F1056" t="inlineStr"/>
       <c r="G1056" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -49105,8 +49031,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1057" t="inlineStr"/>
-      <c r="F1057" t="inlineStr"/>
       <c r="G1057" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -49153,8 +49077,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1058" t="inlineStr"/>
-      <c r="F1058" t="inlineStr"/>
       <c r="G1058" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -49201,8 +49123,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1059" t="inlineStr"/>
-      <c r="F1059" t="inlineStr"/>
       <c r="G1059" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -49249,8 +49169,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1060" t="inlineStr"/>
-      <c r="F1060" t="inlineStr"/>
       <c r="G1060" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -49297,8 +49215,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1061" t="inlineStr"/>
-      <c r="F1061" t="inlineStr"/>
       <c r="G1061" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -49345,8 +49261,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1062" t="inlineStr"/>
-      <c r="F1062" t="inlineStr"/>
       <c r="G1062" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -49393,8 +49307,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1063" t="inlineStr"/>
-      <c r="F1063" t="inlineStr"/>
       <c r="G1063" t="inlineStr">
         <is>
           <t>4-2</t>
@@ -49441,8 +49353,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1064" t="inlineStr"/>
-      <c r="F1064" t="inlineStr"/>
       <c r="G1064" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -49489,8 +49399,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1065" t="inlineStr"/>
-      <c r="F1065" t="inlineStr"/>
       <c r="G1065" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -49537,8 +49445,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1066" t="inlineStr"/>
-      <c r="F1066" t="inlineStr"/>
       <c r="G1066" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -49585,8 +49491,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1067" t="inlineStr"/>
-      <c r="F1067" t="inlineStr"/>
       <c r="G1067" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -49633,8 +49537,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1068" t="inlineStr"/>
-      <c r="F1068" t="inlineStr"/>
       <c r="G1068" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -49681,8 +49583,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1069" t="inlineStr"/>
-      <c r="F1069" t="inlineStr"/>
       <c r="G1069" t="inlineStr">
         <is>
           <t>5-0</t>
@@ -49729,8 +49629,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1070" t="inlineStr"/>
-      <c r="F1070" t="inlineStr"/>
       <c r="G1070" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -49777,8 +49675,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1071" t="inlineStr"/>
-      <c r="F1071" t="inlineStr"/>
       <c r="G1071" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -49825,8 +49721,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1072" t="inlineStr"/>
-      <c r="F1072" t="inlineStr"/>
       <c r="G1072" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -49873,8 +49767,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1073" t="inlineStr"/>
-      <c r="F1073" t="inlineStr"/>
       <c r="G1073" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -49921,8 +49813,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1074" t="inlineStr"/>
-      <c r="F1074" t="inlineStr"/>
       <c r="G1074" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -49969,8 +49859,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1075" t="inlineStr"/>
-      <c r="F1075" t="inlineStr"/>
       <c r="G1075" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -50017,8 +49905,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1076" t="inlineStr"/>
-      <c r="F1076" t="inlineStr"/>
       <c r="G1076" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -50065,8 +49951,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1077" t="inlineStr"/>
-      <c r="F1077" t="inlineStr"/>
       <c r="G1077" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -50113,8 +49997,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1078" t="inlineStr"/>
-      <c r="F1078" t="inlineStr"/>
       <c r="G1078" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -50161,8 +50043,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1079" t="inlineStr"/>
-      <c r="F1079" t="inlineStr"/>
       <c r="G1079" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -50209,8 +50089,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1080" t="inlineStr"/>
-      <c r="F1080" t="inlineStr"/>
       <c r="G1080" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -50257,8 +50135,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1081" t="inlineStr"/>
-      <c r="F1081" t="inlineStr"/>
       <c r="G1081" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -50305,8 +50181,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1082" t="inlineStr"/>
-      <c r="F1082" t="inlineStr"/>
       <c r="G1082" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -50353,8 +50227,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1083" t="inlineStr"/>
-      <c r="F1083" t="inlineStr"/>
       <c r="G1083" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -50401,8 +50273,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1084" t="inlineStr"/>
-      <c r="F1084" t="inlineStr"/>
       <c r="G1084" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -50449,8 +50319,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1085" t="inlineStr"/>
-      <c r="F1085" t="inlineStr"/>
       <c r="G1085" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -50497,8 +50365,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1086" t="inlineStr"/>
-      <c r="F1086" t="inlineStr"/>
       <c r="G1086" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -50545,8 +50411,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1087" t="inlineStr"/>
-      <c r="F1087" t="inlineStr"/>
       <c r="G1087" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -50593,8 +50457,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1088" t="inlineStr"/>
-      <c r="F1088" t="inlineStr"/>
       <c r="G1088" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -50641,8 +50503,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1089" t="inlineStr"/>
-      <c r="F1089" t="inlineStr"/>
       <c r="G1089" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -50689,8 +50549,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1090" t="inlineStr"/>
-      <c r="F1090" t="inlineStr"/>
       <c r="G1090" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -50737,8 +50595,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1091" t="inlineStr"/>
-      <c r="F1091" t="inlineStr"/>
       <c r="G1091" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -50785,8 +50641,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1092" t="inlineStr"/>
-      <c r="F1092" t="inlineStr"/>
       <c r="G1092" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -50833,8 +50687,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1093" t="inlineStr"/>
-      <c r="F1093" t="inlineStr"/>
       <c r="G1093" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -50881,8 +50733,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1094" t="inlineStr"/>
-      <c r="F1094" t="inlineStr"/>
       <c r="G1094" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -50929,8 +50779,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1095" t="inlineStr"/>
-      <c r="F1095" t="inlineStr"/>
       <c r="G1095" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -50977,8 +50825,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1096" t="inlineStr"/>
-      <c r="F1096" t="inlineStr"/>
       <c r="G1096" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -51025,8 +50871,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1097" t="inlineStr"/>
-      <c r="F1097" t="inlineStr"/>
       <c r="G1097" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -51073,8 +50917,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1098" t="inlineStr"/>
-      <c r="F1098" t="inlineStr"/>
       <c r="G1098" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -51121,8 +50963,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1099" t="inlineStr"/>
-      <c r="F1099" t="inlineStr"/>
       <c r="G1099" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -51169,8 +51009,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1100" t="inlineStr"/>
-      <c r="F1100" t="inlineStr"/>
       <c r="G1100" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -51217,8 +51055,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1101" t="inlineStr"/>
-      <c r="F1101" t="inlineStr"/>
       <c r="G1101" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -51265,8 +51101,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1102" t="inlineStr"/>
-      <c r="F1102" t="inlineStr"/>
       <c r="G1102" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -51313,8 +51147,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1103" t="inlineStr"/>
-      <c r="F1103" t="inlineStr"/>
       <c r="G1103" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -51361,8 +51193,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1104" t="inlineStr"/>
-      <c r="F1104" t="inlineStr"/>
       <c r="G1104" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -51409,8 +51239,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1105" t="inlineStr"/>
-      <c r="F1105" t="inlineStr"/>
       <c r="G1105" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -51457,8 +51285,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1106" t="inlineStr"/>
-      <c r="F1106" t="inlineStr"/>
       <c r="G1106" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -51505,8 +51331,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1107" t="inlineStr"/>
-      <c r="F1107" t="inlineStr"/>
       <c r="G1107" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -51553,8 +51377,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1108" t="inlineStr"/>
-      <c r="F1108" t="inlineStr"/>
       <c r="G1108" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -51601,8 +51423,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1109" t="inlineStr"/>
-      <c r="F1109" t="inlineStr"/>
       <c r="G1109" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -51649,8 +51469,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1110" t="inlineStr"/>
-      <c r="F1110" t="inlineStr"/>
       <c r="G1110" t="inlineStr">
         <is>
           <t>0-5</t>
@@ -51697,8 +51515,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1111" t="inlineStr"/>
-      <c r="F1111" t="inlineStr"/>
       <c r="G1111" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -51719,6 +51535,1494 @@
         <v>0</v>
       </c>
       <c r="L1111" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>Neftchi Fergana vs Air Force Club</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>Neftchi Fergana</t>
+        </is>
+      </c>
+      <c r="D1112" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1112" t="inlineStr"/>
+      <c r="F1112" t="inlineStr"/>
+      <c r="G1112" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1112" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1112" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1112" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1112" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1112" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>Shabab Al-Ahli vs Traktor Sazi FC</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>Shabab Al-Ahli</t>
+        </is>
+      </c>
+      <c r="D1113" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1113" t="inlineStr"/>
+      <c r="F1113" t="inlineStr"/>
+      <c r="G1113" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1113" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1113" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1113" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1113" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1113" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>Como vs Parma</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="D1114" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1114" t="inlineStr"/>
+      <c r="F1114" t="inlineStr"/>
+      <c r="G1114" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1114" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1114" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1114" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1114" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1114" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>Torino vs AS Roma</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>AS Roma</t>
+        </is>
+      </c>
+      <c r="D1115" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1115" t="inlineStr"/>
+      <c r="F1115" t="inlineStr"/>
+      <c r="G1115" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1115" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1115" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1115" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1115" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1115" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>FC Midtjylland vs Brøndby IF</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>FC Midtjylland</t>
+        </is>
+      </c>
+      <c r="D1116" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1116" t="inlineStr"/>
+      <c r="F1116" t="inlineStr"/>
+      <c r="G1116" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H1116" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1116" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1116" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1116" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1116" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>Bodo/Glimt vs Sandefjord</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>Bodo/Glimt</t>
+        </is>
+      </c>
+      <c r="D1117" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1117" t="inlineStr"/>
+      <c r="F1117" t="inlineStr"/>
+      <c r="G1117" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1117" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1117" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1117" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1117" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1117" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>Djurgården vs GAIS</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>Djurgården</t>
+        </is>
+      </c>
+      <c r="D1118" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1118" t="inlineStr"/>
+      <c r="F1118" t="inlineStr"/>
+      <c r="G1118" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1118" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1118" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1118" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1118" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1118" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>Gaziantep FK vs Fenerbahce</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>Fenerbahce</t>
+        </is>
+      </c>
+      <c r="D1119" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1119" t="inlineStr"/>
+      <c r="F1119" t="inlineStr"/>
+      <c r="G1119" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1119" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1119" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1119" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1119" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1119" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>IK Sirius vs Degerfors IF</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>IK Sirius</t>
+        </is>
+      </c>
+      <c r="D1120" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1120" t="inlineStr"/>
+      <c r="F1120" t="inlineStr"/>
+      <c r="G1120" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1120" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1120" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1120" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1120" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1120" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>Jong PSV vs Jong AZ</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>Jong AZ</t>
+        </is>
+      </c>
+      <c r="D1121" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1121" t="inlineStr"/>
+      <c r="F1121" t="inlineStr"/>
+      <c r="G1121" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1121" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1121" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1121" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1121" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1121" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>Jong FC Utrecht vs Jong Ajax</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>Jong FC Utrecht</t>
+        </is>
+      </c>
+      <c r="D1122" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1122" t="inlineStr"/>
+      <c r="F1122" t="inlineStr"/>
+      <c r="G1122" t="inlineStr">
+        <is>
+          <t>6-1</t>
+        </is>
+      </c>
+      <c r="H1122" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1122" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1122" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1122" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1122" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>Esteghlal vs Al Sadd</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>Al Sadd</t>
+        </is>
+      </c>
+      <c r="D1123" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1123" t="inlineStr"/>
+      <c r="F1123" t="inlineStr"/>
+      <c r="G1123" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1123" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1123" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1123" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1123" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1123" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>Al Ahli vs Pakhtakor Tashkent</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>Al Ahli</t>
+        </is>
+      </c>
+      <c r="D1124" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1124" t="inlineStr"/>
+      <c r="F1124" t="inlineStr"/>
+      <c r="G1124" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1124" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1124" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1124" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1124" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1124" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>Al Qadsiah vs Al Wasl</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>Al Qadsiah</t>
+        </is>
+      </c>
+      <c r="D1125" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1125" t="inlineStr"/>
+      <c r="F1125" t="inlineStr"/>
+      <c r="G1125" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1125" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1125" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1125" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1125" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1125" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>Defensores de Belgrano vs Deportivo Madryn</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>Defensores de Belgrano</t>
+        </is>
+      </c>
+      <c r="D1126" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1126" t="inlineStr"/>
+      <c r="F1126" t="inlineStr"/>
+      <c r="G1126" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1126" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1126" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1126" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1126" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1126" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>Internazionale vs Udinese</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>Internazionale</t>
+        </is>
+      </c>
+      <c r="D1127" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1127" t="inlineStr"/>
+      <c r="F1127" t="inlineStr"/>
+      <c r="G1127" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H1127" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1127" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1127" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1127" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1127" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>Red Star FC 93 vs Metz</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>Red Star FC 93</t>
+        </is>
+      </c>
+      <c r="D1128" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1128" t="inlineStr"/>
+      <c r="F1128" t="inlineStr"/>
+      <c r="G1128" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1128" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1128" t="n">
+        <v>6</v>
+      </c>
+      <c r="J1128" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1128" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1128" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>Leeds United vs Newcastle United</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>Leeds United</t>
+        </is>
+      </c>
+      <c r="D1129" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1129" t="inlineStr"/>
+      <c r="F1129" t="inlineStr"/>
+      <c r="G1129" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H1129" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1129" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1129" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1129" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1129" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>Villarreal vs Real Betis</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1130" t="inlineStr"/>
+      <c r="F1130" t="inlineStr"/>
+      <c r="G1130" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1130" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1130" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1130" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1130" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1130" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>Moreirense vs Maritimo</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>Moreirense</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1131" t="inlineStr"/>
+      <c r="F1131" t="inlineStr"/>
+      <c r="G1131" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1131" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1131" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1131" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1131" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1131" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>Braga vs Estoril</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="D1132" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1132" t="inlineStr"/>
+      <c r="F1132" t="inlineStr"/>
+      <c r="G1132" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1132" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1132" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1132" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1132" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1132" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>Banfield vs Barracas Central</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>Banfield</t>
+        </is>
+      </c>
+      <c r="D1133" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1133" t="inlineStr"/>
+      <c r="F1133" t="inlineStr"/>
+      <c r="G1133" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1133" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1133" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1133" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1133" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1133" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>América Mineiro vs São Bernardo</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>América Mineiro</t>
+        </is>
+      </c>
+      <c r="D1134" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1134" t="inlineStr"/>
+      <c r="F1134" t="inlineStr"/>
+      <c r="G1134" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1134" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1134" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1134" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1134" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1134" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>Botafogo-SP vs Goiás</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>Botafogo-SP</t>
+        </is>
+      </c>
+      <c r="D1135" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1135" t="inlineStr"/>
+      <c r="F1135" t="inlineStr"/>
+      <c r="G1135" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H1135" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1135" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1135" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1135" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1135" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>Bahia vs Remo</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>Bahia</t>
+        </is>
+      </c>
+      <c r="D1136" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1136" t="inlineStr"/>
+      <c r="F1136" t="inlineStr"/>
+      <c r="G1136" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1136" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1136" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1136" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1136" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1136" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>Unión La Calera vs Deportes Limache</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>Unión La Calera</t>
+        </is>
+      </c>
+      <c r="D1137" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1137" t="inlineStr"/>
+      <c r="F1137" t="inlineStr"/>
+      <c r="G1137" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1137" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1137" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1137" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1137" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1137" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>Universidad Católica (Quito) vs Orense</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>Universidad Católica (Quito)</t>
+        </is>
+      </c>
+      <c r="D1138" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1138" t="inlineStr"/>
+      <c r="F1138" t="inlineStr"/>
+      <c r="G1138" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1138" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1138" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1138" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1138" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1138" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>Instituto (Córdoba) vs Estudiantes de Río Cuarto</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>Instituto (Córdoba)</t>
+        </is>
+      </c>
+      <c r="D1139" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1139" t="inlineStr"/>
+      <c r="F1139" t="inlineStr"/>
+      <c r="G1139" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1139" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1139" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1139" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1139" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1139" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>León vs Atlético de San Luis</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>León</t>
+        </is>
+      </c>
+      <c r="D1140" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1140" t="inlineStr"/>
+      <c r="F1140" t="inlineStr"/>
+      <c r="G1140" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1140" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1140" t="n">
+        <v>7</v>
+      </c>
+      <c r="J1140" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1140" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1140" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>América de Cali vs Deportivo Pasto</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>América de Cali</t>
+        </is>
+      </c>
+      <c r="D1141" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1141" t="inlineStr"/>
+      <c r="F1141" t="inlineStr"/>
+      <c r="G1141" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1141" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1141" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1141" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1141" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1141" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>Antigua GFC vs Suchitepequez</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>Antigua GFC</t>
+        </is>
+      </c>
+      <c r="D1142" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1142" t="inlineStr"/>
+      <c r="F1142" t="inlineStr"/>
+      <c r="G1142" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1142" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1142" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1142" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1142" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1142" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -51735,7 +53039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52049,6 +53353,25 @@
       </c>
       <c r="E17" t="n">
         <v>92</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>31</v>
+      </c>
+      <c r="C18" t="n">
+        <v>24</v>
+      </c>
+      <c r="D18" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="E18" t="n">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -52062,7 +53385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53289,6 +54612,258 @@
         <v>0</v>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>11</v>
+      </c>
+      <c r="D59" t="n">
+        <v>2</v>
+      </c>
+      <c r="E59" t="n">
+        <v>18.2</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>17</v>
+      </c>
+      <c r="D60" t="n">
+        <v>5</v>
+      </c>
+      <c r="E60" t="n">
+        <v>29.4</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>18</v>
+      </c>
+      <c r="D61" t="n">
+        <v>4</v>
+      </c>
+      <c r="E61" t="n">
+        <v>22.2</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>fav_domina_no_gana</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>5</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>4</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>value_alert</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>12</v>
+      </c>
+      <c r="D65" t="n">
+        <v>2</v>
+      </c>
+      <c r="E65" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>no_fav_domina</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>9</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>siguen_empatados_22</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>4</v>
+      </c>
+      <c r="D69" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>siguen_empatados_70</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-16
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1142"/>
+  <dimension ref="A1:L1189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51561,8 +51561,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1112" t="inlineStr"/>
-      <c r="F1112" t="inlineStr"/>
       <c r="G1112" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -51609,8 +51607,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1113" t="inlineStr"/>
-      <c r="F1113" t="inlineStr"/>
       <c r="G1113" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -51657,8 +51653,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1114" t="inlineStr"/>
-      <c r="F1114" t="inlineStr"/>
       <c r="G1114" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -51705,8 +51699,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1115" t="inlineStr"/>
-      <c r="F1115" t="inlineStr"/>
       <c r="G1115" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -51753,8 +51745,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1116" t="inlineStr"/>
-      <c r="F1116" t="inlineStr"/>
       <c r="G1116" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -51801,8 +51791,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1117" t="inlineStr"/>
-      <c r="F1117" t="inlineStr"/>
       <c r="G1117" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -51849,8 +51837,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1118" t="inlineStr"/>
-      <c r="F1118" t="inlineStr"/>
       <c r="G1118" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -51897,8 +51883,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1119" t="inlineStr"/>
-      <c r="F1119" t="inlineStr"/>
       <c r="G1119" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -51945,8 +51929,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1120" t="inlineStr"/>
-      <c r="F1120" t="inlineStr"/>
       <c r="G1120" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -51993,8 +51975,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1121" t="inlineStr"/>
-      <c r="F1121" t="inlineStr"/>
       <c r="G1121" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -52041,8 +52021,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1122" t="inlineStr"/>
-      <c r="F1122" t="inlineStr"/>
       <c r="G1122" t="inlineStr">
         <is>
           <t>6-1</t>
@@ -52089,8 +52067,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1123" t="inlineStr"/>
-      <c r="F1123" t="inlineStr"/>
       <c r="G1123" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -52137,8 +52113,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1124" t="inlineStr"/>
-      <c r="F1124" t="inlineStr"/>
       <c r="G1124" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -52185,8 +52159,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1125" t="inlineStr"/>
-      <c r="F1125" t="inlineStr"/>
       <c r="G1125" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -52233,8 +52205,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1126" t="inlineStr"/>
-      <c r="F1126" t="inlineStr"/>
       <c r="G1126" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -52281,8 +52251,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1127" t="inlineStr"/>
-      <c r="F1127" t="inlineStr"/>
       <c r="G1127" t="inlineStr">
         <is>
           <t>5-3</t>
@@ -52329,8 +52297,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1128" t="inlineStr"/>
-      <c r="F1128" t="inlineStr"/>
       <c r="G1128" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -52377,8 +52343,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1129" t="inlineStr"/>
-      <c r="F1129" t="inlineStr"/>
       <c r="G1129" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -52425,8 +52389,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1130" t="inlineStr"/>
-      <c r="F1130" t="inlineStr"/>
       <c r="G1130" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -52473,8 +52435,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1131" t="inlineStr"/>
-      <c r="F1131" t="inlineStr"/>
       <c r="G1131" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -52521,8 +52481,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1132" t="inlineStr"/>
-      <c r="F1132" t="inlineStr"/>
       <c r="G1132" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -52569,8 +52527,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1133" t="inlineStr"/>
-      <c r="F1133" t="inlineStr"/>
       <c r="G1133" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -52617,8 +52573,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1134" t="inlineStr"/>
-      <c r="F1134" t="inlineStr"/>
       <c r="G1134" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -52665,8 +52619,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1135" t="inlineStr"/>
-      <c r="F1135" t="inlineStr"/>
       <c r="G1135" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -52713,8 +52665,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1136" t="inlineStr"/>
-      <c r="F1136" t="inlineStr"/>
       <c r="G1136" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -52761,8 +52711,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1137" t="inlineStr"/>
-      <c r="F1137" t="inlineStr"/>
       <c r="G1137" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -52809,8 +52757,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1138" t="inlineStr"/>
-      <c r="F1138" t="inlineStr"/>
       <c r="G1138" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -52857,8 +52803,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1139" t="inlineStr"/>
-      <c r="F1139" t="inlineStr"/>
       <c r="G1139" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -52905,8 +52849,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1140" t="inlineStr"/>
-      <c r="F1140" t="inlineStr"/>
       <c r="G1140" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -52953,8 +52895,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1141" t="inlineStr"/>
-      <c r="F1141" t="inlineStr"/>
       <c r="G1141" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -53001,8 +52941,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1142" t="inlineStr"/>
-      <c r="F1142" t="inlineStr"/>
       <c r="G1142" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -53023,6 +52961,2262 @@
         <v>0</v>
       </c>
       <c r="L1142" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>Daejeon Hana Citizen vs Kyoto Sanga</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>Daejeon Hana Citizen</t>
+        </is>
+      </c>
+      <c r="D1143" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1143" t="inlineStr"/>
+      <c r="F1143" t="inlineStr"/>
+      <c r="G1143" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1143" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1143" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1143" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1143" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1143" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>Kashima Antlers vs Newcastle Jets</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>Kashima Antlers</t>
+        </is>
+      </c>
+      <c r="D1144" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1144" t="inlineStr"/>
+      <c r="F1144" t="inlineStr"/>
+      <c r="G1144" t="inlineStr">
+        <is>
+          <t>7-1</t>
+        </is>
+      </c>
+      <c r="H1144" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1144" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1144" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1144" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1144" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>Beijing Guoan vs Pohang Steelers</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>Beijing Guoan</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1145" t="inlineStr"/>
+      <c r="F1145" t="inlineStr"/>
+      <c r="G1145" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1145" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1145" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1145" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1145" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1145" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>Johor Darul Ta'zim vs Buriram United</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>Johor Darul Ta'zim</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1146" t="inlineStr"/>
+      <c r="F1146" t="inlineStr"/>
+      <c r="G1146" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1146" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1146" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1146" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1146" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1146" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>Al Ain vs Al Nassr</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>Al Nassr</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1147" t="inlineStr"/>
+      <c r="F1147" t="inlineStr"/>
+      <c r="G1147" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H1147" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1147" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1147" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1147" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1147" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>Genoa vs Sudtirol</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>Genoa</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1148" t="inlineStr"/>
+      <c r="F1148" t="inlineStr"/>
+      <c r="G1148" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1148" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1148" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1148" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1148" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1148" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>Rayo Vallecano vs Espanyol</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1149" t="inlineStr"/>
+      <c r="F1149" t="inlineStr"/>
+      <c r="G1149" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1149" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1149" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1149" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1149" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1149" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>Alavés vs Valencia</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>Alavés</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1150" t="inlineStr"/>
+      <c r="F1150" t="inlineStr"/>
+      <c r="G1150" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1150" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1150" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1150" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1150" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1150" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>Ajax Amsterdam vs Willem II</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>Ajax Amsterdam</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1151" t="inlineStr"/>
+      <c r="F1151" t="inlineStr"/>
+      <c r="G1151" t="inlineStr">
+        <is>
+          <t>5-1</t>
+        </is>
+      </c>
+      <c r="H1151" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1151" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1151" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1151" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1151" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>York City vs Newcastle United U21</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>York City</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1152" t="inlineStr"/>
+      <c r="F1152" t="inlineStr"/>
+      <c r="G1152" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H1152" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1152" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1152" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1152" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1152" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>Chesterfield vs Manchester City U21</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>Chesterfield</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1153" t="inlineStr"/>
+      <c r="F1153" t="inlineStr"/>
+      <c r="G1153" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H1153" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1153" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1153" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1153" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1153" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>Wycombe Wanderers vs Chelsea U21</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>Wycombe Wanderers</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1154" t="inlineStr"/>
+      <c r="F1154" t="inlineStr"/>
+      <c r="G1154" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1154" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1154" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1154" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1154" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1154" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>Swindon Town vs Crystal Palace U21</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>Swindon Town</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1155" t="inlineStr"/>
+      <c r="F1155" t="inlineStr"/>
+      <c r="G1155" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1155" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1155" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1155" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1155" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1155" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>Leyton Orient vs Arsenal U21</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>Leyton Orient</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1156" t="inlineStr"/>
+      <c r="F1156" t="inlineStr"/>
+      <c r="G1156" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1156" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1156" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1156" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1156" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1156" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>Peterborough United vs Barnsley</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>Peterborough United</t>
+        </is>
+      </c>
+      <c r="D1157" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1157" t="inlineStr"/>
+      <c r="F1157" t="inlineStr"/>
+      <c r="G1157" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H1157" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1157" t="n">
+        <v>6</v>
+      </c>
+      <c r="J1157" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1157" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1157" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>Bristol City vs Lincoln City</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>Bristol City</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1158" t="inlineStr"/>
+      <c r="F1158" t="inlineStr"/>
+      <c r="G1158" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1158" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1158" t="n">
+        <v>7</v>
+      </c>
+      <c r="J1158" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1158" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1158" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>Middlesbrough vs Millwall</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>Middlesbrough</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1159" t="inlineStr"/>
+      <c r="F1159" t="inlineStr"/>
+      <c r="G1159" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H1159" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1159" t="n">
+        <v>7</v>
+      </c>
+      <c r="J1159" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1159" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1159" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>Stenhousemuir vs Partick Thistle</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>Partick Thistle</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1160" t="inlineStr"/>
+      <c r="F1160" t="inlineStr"/>
+      <c r="G1160" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1160" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1160" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1160" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1160" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1160" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>Falkirk vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1161" t="inlineStr"/>
+      <c r="F1161" t="inlineStr"/>
+      <c r="G1161" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1161" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1161" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1161" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1161" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1161" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>Hibernian vs Kilmarnock</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>Hibernian</t>
+        </is>
+      </c>
+      <c r="D1162" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1162" t="inlineStr"/>
+      <c r="F1162" t="inlineStr"/>
+      <c r="G1162" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1162" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1162" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1162" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1162" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1162" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>Motherwell vs Aberdeen</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>Motherwell</t>
+        </is>
+      </c>
+      <c r="D1163" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1163" t="inlineStr"/>
+      <c r="F1163" t="inlineStr"/>
+      <c r="G1163" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H1163" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1163" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1163" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1163" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1163" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>West Ham United vs Fulham</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>Fulham</t>
+        </is>
+      </c>
+      <c r="D1164" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1164" t="inlineStr"/>
+      <c r="F1164" t="inlineStr"/>
+      <c r="G1164" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H1164" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1164" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1164" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1164" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1164" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>Aldershot Town vs Yeovil Town</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>Aldershot Town</t>
+        </is>
+      </c>
+      <c r="D1165" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1165" t="inlineStr"/>
+      <c r="F1165" t="inlineStr"/>
+      <c r="G1165" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1165" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1165" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1165" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1165" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1165" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>Boston United vs Woking</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>Boston United</t>
+        </is>
+      </c>
+      <c r="D1166" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1166" t="inlineStr"/>
+      <c r="F1166" t="inlineStr"/>
+      <c r="G1166" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1166" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1166" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1166" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1166" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1166" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>Carlisle United vs Forest Green Rovers</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>Carlisle United</t>
+        </is>
+      </c>
+      <c r="D1167" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1167" t="inlineStr"/>
+      <c r="F1167" t="inlineStr"/>
+      <c r="G1167" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1167" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1167" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1167" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1167" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1167" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>Harrogate Town vs AFC Fylde</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>Harrogate Town</t>
+        </is>
+      </c>
+      <c r="D1168" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1168" t="inlineStr"/>
+      <c r="F1168" t="inlineStr"/>
+      <c r="G1168" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1168" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1168" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1168" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1168" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1168" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>Solihull Moors vs Barrow</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>Barrow</t>
+        </is>
+      </c>
+      <c r="D1169" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1169" t="inlineStr"/>
+      <c r="F1169" t="inlineStr"/>
+      <c r="G1169" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1169" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1169" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1169" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1169" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1169" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>Southend United vs Tamworth</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>Southend United</t>
+        </is>
+      </c>
+      <c r="D1170" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1170" t="inlineStr"/>
+      <c r="F1170" t="inlineStr"/>
+      <c r="G1170" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1170" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1170" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1170" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1170" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>Sutton United vs Eastleigh</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>Sutton United</t>
+        </is>
+      </c>
+      <c r="D1171" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1171" t="inlineStr"/>
+      <c r="F1171" t="inlineStr"/>
+      <c r="G1171" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1171" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1171" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1171" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1171" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1171" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>Wealdstone vs FC Halifax Town</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>Wealdstone</t>
+        </is>
+      </c>
+      <c r="D1172" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1172" t="inlineStr"/>
+      <c r="F1172" t="inlineStr"/>
+      <c r="G1172" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1172" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1172" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1172" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1172" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1172" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>Worthing vs AFC Hornchurch</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>Worthing</t>
+        </is>
+      </c>
+      <c r="D1173" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1173" t="inlineStr"/>
+      <c r="F1173" t="inlineStr"/>
+      <c r="G1173" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1173" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1173" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1173" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1173" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1173" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>Ipswich Town vs Arsenal</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="D1174" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1174" t="inlineStr"/>
+      <c r="F1174" t="inlineStr"/>
+      <c r="G1174" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H1174" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1174" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1174" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1174" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1174" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>Liverpool vs Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>Liverpool</t>
+        </is>
+      </c>
+      <c r="D1175" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1175" t="inlineStr"/>
+      <c r="F1175" t="inlineStr"/>
+      <c r="G1175" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1175" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1175" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1175" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1175" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1175" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>Reading vs Brentford</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>Brentford</t>
+        </is>
+      </c>
+      <c r="D1176" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1176" t="inlineStr"/>
+      <c r="F1176" t="inlineStr"/>
+      <c r="G1176" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1176" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1176" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1176" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1176" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1176" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>Fiorentina vs Pisa</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="D1177" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1177" t="inlineStr"/>
+      <c r="F1177" t="inlineStr"/>
+      <c r="G1177" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1177" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1177" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1177" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1177" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1177" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>Real Oruro vs Real Potosí</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>Real Potosí</t>
+        </is>
+      </c>
+      <c r="D1178" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1178" t="inlineStr"/>
+      <c r="F1178" t="inlineStr"/>
+      <c r="G1178" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1178" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1178" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1178" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1178" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1178" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>Elche vs Real Madrid</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="D1179" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1179" t="inlineStr"/>
+      <c r="F1179" t="inlineStr"/>
+      <c r="G1179" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H1179" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1179" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1179" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1179" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1179" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>ABB vs The Strongest</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>The Strongest</t>
+        </is>
+      </c>
+      <c r="D1180" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1180" t="inlineStr"/>
+      <c r="F1180" t="inlineStr"/>
+      <c r="G1180" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1180" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1180" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1180" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1180" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1180" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>Vasco da Gama vs Independiente Santa Fe</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>Vasco da Gama</t>
+        </is>
+      </c>
+      <c r="D1181" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1181" t="inlineStr"/>
+      <c r="F1181" t="inlineStr"/>
+      <c r="G1181" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1181" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1181" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1181" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1181" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1181" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>Londrina vs Ponte Preta</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="D1182" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1182" t="inlineStr"/>
+      <c r="F1182" t="inlineStr"/>
+      <c r="G1182" t="inlineStr">
+        <is>
+          <t>6-0</t>
+        </is>
+      </c>
+      <c r="H1182" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1182" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1182" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1182" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>Náutico vs Operário PR</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>Náutico</t>
+        </is>
+      </c>
+      <c r="D1183" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1183" t="inlineStr"/>
+      <c r="F1183" t="inlineStr"/>
+      <c r="G1183" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H1183" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1183" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1183" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1183" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1183" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>Indy Eleven vs Brooklyn FC</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>Indy Eleven</t>
+        </is>
+      </c>
+      <c r="D1184" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1184" t="inlineStr"/>
+      <c r="F1184" t="inlineStr"/>
+      <c r="G1184" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H1184" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1184" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1184" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1184" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1184" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>CRB vs Sport</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="D1185" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1185" t="inlineStr"/>
+      <c r="F1185" t="inlineStr"/>
+      <c r="G1185" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1185" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1185" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1185" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1185" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1185" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>São Paulo vs Boca Juniors</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="D1186" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1186" t="inlineStr"/>
+      <c r="F1186" t="inlineStr"/>
+      <c r="G1186" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1186" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1186" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1186" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1186" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1186" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>Boyacá Chicó FC vs Alianza FC</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>Boyacá Chicó FC</t>
+        </is>
+      </c>
+      <c r="D1187" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1187" t="inlineStr"/>
+      <c r="F1187" t="inlineStr"/>
+      <c r="G1187" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1187" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1187" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1187" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1187" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1187" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>Puebla vs Toluca</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>Toluca</t>
+        </is>
+      </c>
+      <c r="D1188" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1188" t="inlineStr"/>
+      <c r="F1188" t="inlineStr"/>
+      <c r="G1188" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1188" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1188" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1188" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1188" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1188" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>Dorados de Sinaloa vs Cancún FC</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>Dorados de Sinaloa</t>
+        </is>
+      </c>
+      <c r="D1189" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1189" t="inlineStr"/>
+      <c r="F1189" t="inlineStr"/>
+      <c r="G1189" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1189" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1189" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1189" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1189" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1189" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -53039,7 +55233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53372,6 +55566,25 @@
       </c>
       <c r="E18" t="n">
         <v>31</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>47</v>
+      </c>
+      <c r="C19" t="n">
+        <v>32</v>
+      </c>
+      <c r="D19" t="n">
+        <v>68.09999999999999</v>
+      </c>
+      <c r="E19" t="n">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -53385,7 +55598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54864,6 +57077,258 @@
         <v>0</v>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>value_alert</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>4</v>
+      </c>
+      <c r="D71" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>12</v>
+      </c>
+      <c r="D72" t="n">
+        <v>2</v>
+      </c>
+      <c r="E72" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>no_fav_domina</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>11</v>
+      </c>
+      <c r="D73" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>15</v>
+      </c>
+      <c r="D74" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" t="n">
+        <v>6.7</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>5</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>fav_domina_no_gana</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>8</v>
+      </c>
+      <c r="D76" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>8</v>
+      </c>
+      <c r="D77" t="n">
+        <v>3</v>
+      </c>
+      <c r="E77" t="n">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>12</v>
+      </c>
+      <c r="D78" t="n">
+        <v>2</v>
+      </c>
+      <c r="E78" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>siguen_empatados_22</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>4</v>
+      </c>
+      <c r="D79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>6</v>
+      </c>
+      <c r="D80" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>siguen_empatados_70</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>2</v>
+      </c>
+      <c r="D81" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>3</v>
+      </c>
+      <c r="D82" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-17
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1189"/>
+  <dimension ref="A1:L1246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52987,8 +52987,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1143" t="inlineStr"/>
-      <c r="F1143" t="inlineStr"/>
       <c r="G1143" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -53035,8 +53033,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1144" t="inlineStr"/>
-      <c r="F1144" t="inlineStr"/>
       <c r="G1144" t="inlineStr">
         <is>
           <t>7-1</t>
@@ -53083,8 +53079,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1145" t="inlineStr"/>
-      <c r="F1145" t="inlineStr"/>
       <c r="G1145" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -53131,8 +53125,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1146" t="inlineStr"/>
-      <c r="F1146" t="inlineStr"/>
       <c r="G1146" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -53179,8 +53171,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1147" t="inlineStr"/>
-      <c r="F1147" t="inlineStr"/>
       <c r="G1147" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -53227,8 +53217,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1148" t="inlineStr"/>
-      <c r="F1148" t="inlineStr"/>
       <c r="G1148" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -53275,8 +53263,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1149" t="inlineStr"/>
-      <c r="F1149" t="inlineStr"/>
       <c r="G1149" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -53323,8 +53309,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1150" t="inlineStr"/>
-      <c r="F1150" t="inlineStr"/>
       <c r="G1150" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -53371,8 +53355,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1151" t="inlineStr"/>
-      <c r="F1151" t="inlineStr"/>
       <c r="G1151" t="inlineStr">
         <is>
           <t>5-1</t>
@@ -53419,8 +53401,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1152" t="inlineStr"/>
-      <c r="F1152" t="inlineStr"/>
       <c r="G1152" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -53467,8 +53447,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1153" t="inlineStr"/>
-      <c r="F1153" t="inlineStr"/>
       <c r="G1153" t="inlineStr">
         <is>
           <t>5-3</t>
@@ -53515,8 +53493,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1154" t="inlineStr"/>
-      <c r="F1154" t="inlineStr"/>
       <c r="G1154" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -53563,8 +53539,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1155" t="inlineStr"/>
-      <c r="F1155" t="inlineStr"/>
       <c r="G1155" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -53611,8 +53585,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1156" t="inlineStr"/>
-      <c r="F1156" t="inlineStr"/>
       <c r="G1156" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -53659,8 +53631,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1157" t="inlineStr"/>
-      <c r="F1157" t="inlineStr"/>
       <c r="G1157" t="inlineStr">
         <is>
           <t>3-3</t>
@@ -53707,8 +53677,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1158" t="inlineStr"/>
-      <c r="F1158" t="inlineStr"/>
       <c r="G1158" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -53755,8 +53723,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1159" t="inlineStr"/>
-      <c r="F1159" t="inlineStr"/>
       <c r="G1159" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -53803,8 +53769,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1160" t="inlineStr"/>
-      <c r="F1160" t="inlineStr"/>
       <c r="G1160" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -53851,8 +53815,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1161" t="inlineStr"/>
-      <c r="F1161" t="inlineStr"/>
       <c r="G1161" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -53899,8 +53861,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1162" t="inlineStr"/>
-      <c r="F1162" t="inlineStr"/>
       <c r="G1162" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -53947,8 +53907,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1163" t="inlineStr"/>
-      <c r="F1163" t="inlineStr"/>
       <c r="G1163" t="inlineStr">
         <is>
           <t>0-4</t>
@@ -53995,8 +53953,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1164" t="inlineStr"/>
-      <c r="F1164" t="inlineStr"/>
       <c r="G1164" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -54043,8 +53999,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1165" t="inlineStr"/>
-      <c r="F1165" t="inlineStr"/>
       <c r="G1165" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -54091,8 +54045,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1166" t="inlineStr"/>
-      <c r="F1166" t="inlineStr"/>
       <c r="G1166" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -54139,8 +54091,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1167" t="inlineStr"/>
-      <c r="F1167" t="inlineStr"/>
       <c r="G1167" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -54187,8 +54137,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1168" t="inlineStr"/>
-      <c r="F1168" t="inlineStr"/>
       <c r="G1168" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -54235,8 +54183,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1169" t="inlineStr"/>
-      <c r="F1169" t="inlineStr"/>
       <c r="G1169" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -54283,8 +54229,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1170" t="inlineStr"/>
-      <c r="F1170" t="inlineStr"/>
       <c r="G1170" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -54331,8 +54275,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1171" t="inlineStr"/>
-      <c r="F1171" t="inlineStr"/>
       <c r="G1171" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -54379,8 +54321,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1172" t="inlineStr"/>
-      <c r="F1172" t="inlineStr"/>
       <c r="G1172" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -54427,8 +54367,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1173" t="inlineStr"/>
-      <c r="F1173" t="inlineStr"/>
       <c r="G1173" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -54475,8 +54413,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1174" t="inlineStr"/>
-      <c r="F1174" t="inlineStr"/>
       <c r="G1174" t="inlineStr">
         <is>
           <t>2-4</t>
@@ -54523,8 +54459,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1175" t="inlineStr"/>
-      <c r="F1175" t="inlineStr"/>
       <c r="G1175" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -54571,8 +54505,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1176" t="inlineStr"/>
-      <c r="F1176" t="inlineStr"/>
       <c r="G1176" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -54619,8 +54551,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1177" t="inlineStr"/>
-      <c r="F1177" t="inlineStr"/>
       <c r="G1177" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -54667,8 +54597,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1178" t="inlineStr"/>
-      <c r="F1178" t="inlineStr"/>
       <c r="G1178" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -54715,8 +54643,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1179" t="inlineStr"/>
-      <c r="F1179" t="inlineStr"/>
       <c r="G1179" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -54763,8 +54689,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1180" t="inlineStr"/>
-      <c r="F1180" t="inlineStr"/>
       <c r="G1180" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -54811,8 +54735,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1181" t="inlineStr"/>
-      <c r="F1181" t="inlineStr"/>
       <c r="G1181" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -54859,8 +54781,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1182" t="inlineStr"/>
-      <c r="F1182" t="inlineStr"/>
       <c r="G1182" t="inlineStr">
         <is>
           <t>6-0</t>
@@ -54907,8 +54827,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1183" t="inlineStr"/>
-      <c r="F1183" t="inlineStr"/>
       <c r="G1183" t="inlineStr">
         <is>
           <t>3-3</t>
@@ -54955,8 +54873,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1184" t="inlineStr"/>
-      <c r="F1184" t="inlineStr"/>
       <c r="G1184" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -55003,8 +54919,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1185" t="inlineStr"/>
-      <c r="F1185" t="inlineStr"/>
       <c r="G1185" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -55051,8 +54965,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1186" t="inlineStr"/>
-      <c r="F1186" t="inlineStr"/>
       <c r="G1186" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -55099,8 +55011,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1187" t="inlineStr"/>
-      <c r="F1187" t="inlineStr"/>
       <c r="G1187" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -55147,8 +55057,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1188" t="inlineStr"/>
-      <c r="F1188" t="inlineStr"/>
       <c r="G1188" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -55195,8 +55103,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1189" t="inlineStr"/>
-      <c r="F1189" t="inlineStr"/>
       <c r="G1189" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -55217,6 +55123,2742 @@
         <v>0</v>
       </c>
       <c r="L1189" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>Jeonbuk Motors vs Kashiwa Reysol</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>Kashiwa Reysol</t>
+        </is>
+      </c>
+      <c r="D1190" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1190" t="inlineStr"/>
+      <c r="F1190" t="inlineStr"/>
+      <c r="G1190" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1190" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1190" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1190" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1190" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1190" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>FC Seoul vs Persib</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>FC Seoul</t>
+        </is>
+      </c>
+      <c r="D1191" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1191" t="inlineStr"/>
+      <c r="F1191" t="inlineStr"/>
+      <c r="G1191" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1191" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1191" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1191" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1191" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1191" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>Port FC vs Vissel Kobe</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>Vissel Kobe</t>
+        </is>
+      </c>
+      <c r="D1192" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1192" t="inlineStr"/>
+      <c r="F1192" t="inlineStr"/>
+      <c r="G1192" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1192" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1192" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1192" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1192" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1192" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>Viettel vs Melbourne Victory</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>Melbourne Victory</t>
+        </is>
+      </c>
+      <c r="D1193" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1193" t="inlineStr"/>
+      <c r="F1193" t="inlineStr"/>
+      <c r="G1193" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1193" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1193" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1193" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1193" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1193" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>Greenville Triumph vs Corpus Christi FC</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>Greenville Triumph</t>
+        </is>
+      </c>
+      <c r="D1194" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1194" t="inlineStr"/>
+      <c r="F1194" t="inlineStr"/>
+      <c r="G1194" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1194" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1194" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1194" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1194" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1194" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>Spartak Moscow vs Fakel Voronezh</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>Spartak Moscow</t>
+        </is>
+      </c>
+      <c r="D1195" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1195" t="inlineStr"/>
+      <c r="F1195" t="inlineStr"/>
+      <c r="G1195" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1195" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1195" t="n">
+        <v>11</v>
+      </c>
+      <c r="J1195" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1195" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1195" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>Al Hussein vs SC East Bengal</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>Al Hussein</t>
+        </is>
+      </c>
+      <c r="D1196" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1196" t="inlineStr"/>
+      <c r="F1196" t="inlineStr"/>
+      <c r="G1196" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H1196" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1196" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1196" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1196" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1196" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>Khaldiya vs Nasaf Qarshi</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>Khaldiya</t>
+        </is>
+      </c>
+      <c r="D1197" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1197" t="inlineStr"/>
+      <c r="F1197" t="inlineStr"/>
+      <c r="G1197" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1197" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1197" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1197" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1197" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1197" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>Al-Nahda Muscat Club vs Al Taawoun</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>Al Taawoun</t>
+        </is>
+      </c>
+      <c r="D1198" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1198" t="inlineStr"/>
+      <c r="F1198" t="inlineStr"/>
+      <c r="G1198" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1198" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1198" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1198" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1198" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1198" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>Omonia Nicosia vs Celta Vigo</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>Celta Vigo</t>
+        </is>
+      </c>
+      <c r="D1199" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1199" t="inlineStr"/>
+      <c r="F1199" t="inlineStr"/>
+      <c r="G1199" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1199" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1199" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1199" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1199" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1199" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>Atlético Madrid vs Osasuna</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>Atlético Madrid</t>
+        </is>
+      </c>
+      <c r="D1200" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1200" t="inlineStr"/>
+      <c r="F1200" t="inlineStr"/>
+      <c r="G1200" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H1200" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1200" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1200" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1200" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1200" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>Deportivo vs Sevilla</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>Deportivo</t>
+        </is>
+      </c>
+      <c r="D1201" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1201" t="inlineStr"/>
+      <c r="F1201" t="inlineStr"/>
+      <c r="G1201" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1201" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1201" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1201" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1201" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1201" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>AIK vs Mjällby AIF</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>AIK</t>
+        </is>
+      </c>
+      <c r="D1202" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1202" t="inlineStr"/>
+      <c r="F1202" t="inlineStr"/>
+      <c r="G1202" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1202" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1202" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1202" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1202" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1202" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>Union Omaha vs Spokane Velocity FC</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>Union Omaha</t>
+        </is>
+      </c>
+      <c r="D1203" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1203" t="inlineStr"/>
+      <c r="F1203" t="inlineStr"/>
+      <c r="G1203" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1203" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1203" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1203" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1203" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1203" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>FC Baltika Kaliningrad vs Zenit St Petersburg</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>Zenit St Petersburg</t>
+        </is>
+      </c>
+      <c r="D1204" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1204" t="inlineStr"/>
+      <c r="F1204" t="inlineStr"/>
+      <c r="G1204" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H1204" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1204" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1204" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1204" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1204" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>Lokomotiv Moscow vs Krylia Sovetov</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>Lokomotiv Moscow</t>
+        </is>
+      </c>
+      <c r="D1205" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1205" t="inlineStr"/>
+      <c r="F1205" t="inlineStr"/>
+      <c r="G1205" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1205" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1205" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1205" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1205" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1205" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>San Martín (San Juan) vs Tristán Suárez</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>San Martín (San Juan)</t>
+        </is>
+      </c>
+      <c r="D1206" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1206" t="inlineStr"/>
+      <c r="F1206" t="inlineStr"/>
+      <c r="G1206" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1206" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1206" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1206" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1206" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1206" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>Al Rayyan vs Al-Faisaly</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>Al Rayyan</t>
+        </is>
+      </c>
+      <c r="D1207" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1207" t="inlineStr"/>
+      <c r="F1207" t="inlineStr"/>
+      <c r="G1207" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H1207" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1207" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1207" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1207" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1207" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>Everton vs Wolverhampton Wanderers</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>Everton</t>
+        </is>
+      </c>
+      <c r="D1208" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1208" t="inlineStr"/>
+      <c r="F1208" t="inlineStr"/>
+      <c r="G1208" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1208" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1208" t="n">
+        <v>7</v>
+      </c>
+      <c r="J1208" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1208" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1208" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>Fleetwood Town vs Sheffield United</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>Sheffield United</t>
+        </is>
+      </c>
+      <c r="D1209" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1209" t="inlineStr"/>
+      <c r="F1209" t="inlineStr"/>
+      <c r="G1209" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1209" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1209" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1209" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1209" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1209" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>Altrincham vs Hartlepool United</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>Altrincham</t>
+        </is>
+      </c>
+      <c r="D1210" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1210" t="inlineStr"/>
+      <c r="F1210" t="inlineStr"/>
+      <c r="G1210" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1210" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1210" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1210" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1210" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1210" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>Kidderminster Harriers vs Gateshead</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>Kidderminster Harriers</t>
+        </is>
+      </c>
+      <c r="D1211" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1211" t="inlineStr"/>
+      <c r="F1211" t="inlineStr"/>
+      <c r="G1211" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1211" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1211" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1211" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1211" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1211" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>Scunthorpe United vs Boreham Wood</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>Boreham Wood</t>
+        </is>
+      </c>
+      <c r="D1212" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1212" t="inlineStr"/>
+      <c r="F1212" t="inlineStr"/>
+      <c r="G1212" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1212" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1212" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1212" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1212" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1212" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>AC Milan vs Benfica</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>AC Milan</t>
+        </is>
+      </c>
+      <c r="D1213" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1213" t="inlineStr"/>
+      <c r="F1213" t="inlineStr"/>
+      <c r="G1213" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1213" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1213" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1213" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1213" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1213" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>Anderlecht vs Lyon</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="D1214" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1214" t="inlineStr"/>
+      <c r="F1214" t="inlineStr"/>
+      <c r="G1214" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1214" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1214" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1214" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1214" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1214" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>Bayer Leverkusen vs NK Celje</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="D1215" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1215" t="inlineStr"/>
+      <c r="F1215" t="inlineStr"/>
+      <c r="G1215" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1215" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1215" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1215" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1215" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1215" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>Hapoel Be'er vs Dinamo Zagreb</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>Dinamo Zagreb</t>
+        </is>
+      </c>
+      <c r="D1216" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1216" t="inlineStr"/>
+      <c r="F1216" t="inlineStr"/>
+      <c r="G1216" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1216" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1216" t="n">
+        <v>6</v>
+      </c>
+      <c r="J1216" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1216" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1216" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>Olympiacos vs Jagiellonia Bialystok</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>Olympiacos</t>
+        </is>
+      </c>
+      <c r="D1217" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1217" t="inlineStr"/>
+      <c r="F1217" t="inlineStr"/>
+      <c r="G1217" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1217" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1217" t="n">
+        <v>9</v>
+      </c>
+      <c r="J1217" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1217" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1217" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>SK Sturm Graz vs Stade Rennais</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>Stade Rennais</t>
+        </is>
+      </c>
+      <c r="D1218" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1218" t="inlineStr"/>
+      <c r="F1218" t="inlineStr"/>
+      <c r="G1218" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1218" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1218" t="n">
+        <v>7</v>
+      </c>
+      <c r="J1218" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1218" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1218" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>Sunderland vs AZ Alkmaar</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>Sunderland</t>
+        </is>
+      </c>
+      <c r="D1219" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1219" t="inlineStr"/>
+      <c r="F1219" t="inlineStr"/>
+      <c r="G1219" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1219" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1219" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1219" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1219" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1219" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>Guabirá vs Aurora</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>Guabirá</t>
+        </is>
+      </c>
+      <c r="D1220" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1220" t="inlineStr"/>
+      <c r="F1220" t="inlineStr"/>
+      <c r="G1220" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1220" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1220" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1220" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1220" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1220" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>Coventry City vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="D1221" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1221" t="inlineStr"/>
+      <c r="F1221" t="inlineStr"/>
+      <c r="G1221" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H1221" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1221" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1221" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1221" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1221" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>Manchester United vs Brighton &amp; Hove Albion</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>Manchester United</t>
+        </is>
+      </c>
+      <c r="D1222" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1222" t="inlineStr"/>
+      <c r="F1222" t="inlineStr"/>
+      <c r="G1222" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H1222" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1222" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1222" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1222" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1222" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>Barcelona vs Racing Santander</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D1223" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1223" t="inlineStr"/>
+      <c r="F1223" t="inlineStr"/>
+      <c r="G1223" t="inlineStr">
+        <is>
+          <t>7-2</t>
+        </is>
+      </c>
+      <c r="H1223" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1223" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1223" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1223" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1223" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>Levante vs Athletic Club</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="D1224" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1224" t="inlineStr"/>
+      <c r="F1224" t="inlineStr"/>
+      <c r="G1224" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1224" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1224" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1224" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1224" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1224" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>Portuguesa vs Estudiantes de Mérida</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>Portuguesa</t>
+        </is>
+      </c>
+      <c r="D1225" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1225" t="inlineStr"/>
+      <c r="F1225" t="inlineStr"/>
+      <c r="G1225" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1225" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1225" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1225" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1225" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1225" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>Atlético-MG vs Santos</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>Atlético-MG</t>
+        </is>
+      </c>
+      <c r="D1226" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1226" t="inlineStr"/>
+      <c r="F1226" t="inlineStr"/>
+      <c r="G1226" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H1226" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1226" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1226" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1226" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1226" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia vs Atlético Tucumán</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="D1227" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1227" t="inlineStr"/>
+      <c r="F1227" t="inlineStr"/>
+      <c r="G1227" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1227" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1227" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1227" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1227" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1227" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>Nacional Potosí vs Always Ready</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>Always Ready</t>
+        </is>
+      </c>
+      <c r="D1228" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1228" t="inlineStr"/>
+      <c r="F1228" t="inlineStr"/>
+      <c r="G1228" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H1228" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1228" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1228" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1228" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1228" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>Hartford Athletic vs Sporting JAX</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>Hartford Athletic</t>
+        </is>
+      </c>
+      <c r="D1229" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1229" t="inlineStr"/>
+      <c r="F1229" t="inlineStr"/>
+      <c r="G1229" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1229" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1229" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1229" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1229" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1229" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>Monagas SC vs Zamora FC</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>Monagas SC</t>
+        </is>
+      </c>
+      <c r="D1230" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1230" t="inlineStr"/>
+      <c r="F1230" t="inlineStr"/>
+      <c r="G1230" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1230" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1230" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1230" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1230" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1230" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>Botafogo vs Grêmio</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>Botafogo</t>
+        </is>
+      </c>
+      <c r="D1231" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1231" t="inlineStr"/>
+      <c r="F1231" t="inlineStr"/>
+      <c r="G1231" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1231" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1231" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1231" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1231" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1231" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>Columbus Crew vs Orlando City SC</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>Columbus Crew</t>
+        </is>
+      </c>
+      <c r="D1232" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1232" t="inlineStr"/>
+      <c r="F1232" t="inlineStr"/>
+      <c r="G1232" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1232" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1232" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1232" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1232" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1232" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>Trujillanos vs Rayo Zuliano</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>Trujillanos</t>
+        </is>
+      </c>
+      <c r="D1233" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1233" t="inlineStr"/>
+      <c r="F1233" t="inlineStr"/>
+      <c r="G1233" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H1233" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1233" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1233" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1233" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1233" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>Westchester SC vs Richmond Kickers</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>Westchester SC</t>
+        </is>
+      </c>
+      <c r="D1234" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1234" t="inlineStr"/>
+      <c r="F1234" t="inlineStr"/>
+      <c r="G1234" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H1234" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1234" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1234" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1234" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1234" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>Once Caldas vs Deportes Tolima</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>Once Caldas</t>
+        </is>
+      </c>
+      <c r="D1235" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1235" t="inlineStr"/>
+      <c r="F1235" t="inlineStr"/>
+      <c r="G1235" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1235" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1235" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1235" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1235" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1235" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>Metropolitanos vs Caracas FC</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>Metropolitanos</t>
+        </is>
+      </c>
+      <c r="D1236" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1236" t="inlineStr"/>
+      <c r="F1236" t="inlineStr"/>
+      <c r="G1236" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1236" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1236" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1236" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1236" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1236" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>Fort Wayne vs One Knoxville</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>Fort Wayne</t>
+        </is>
+      </c>
+      <c r="D1237" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1237" t="inlineStr"/>
+      <c r="F1237" t="inlineStr"/>
+      <c r="G1237" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H1237" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1237" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1237" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1237" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1237" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>Corinthians vs Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>Corinthians</t>
+        </is>
+      </c>
+      <c r="D1238" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1238" t="inlineStr"/>
+      <c r="F1238" t="inlineStr"/>
+      <c r="G1238" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1238" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1238" t="n">
+        <v>7</v>
+      </c>
+      <c r="J1238" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1238" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1238" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>Blooming vs Universitario de Vinto</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>Blooming</t>
+        </is>
+      </c>
+      <c r="D1239" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1239" t="inlineStr"/>
+      <c r="F1239" t="inlineStr"/>
+      <c r="G1239" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1239" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1239" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1239" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1239" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1239" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>Birmingham Legion FC vs New Mexico United</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>Birmingham Legion FC</t>
+        </is>
+      </c>
+      <c r="D1240" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1240" t="inlineStr"/>
+      <c r="F1240" t="inlineStr"/>
+      <c r="G1240" t="inlineStr">
+        <is>
+          <t>4-4</t>
+        </is>
+      </c>
+      <c r="H1240" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1240" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1240" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1240" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1240" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>Cartaginés vs Saprissa</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>Cartaginés</t>
+        </is>
+      </c>
+      <c r="D1241" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1241" t="inlineStr"/>
+      <c r="F1241" t="inlineStr"/>
+      <c r="G1241" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1241" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1241" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1241" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1241" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1241" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>Internacional Santa Tecla vs CD FAS</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>CD FAS</t>
+        </is>
+      </c>
+      <c r="D1242" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1242" t="inlineStr"/>
+      <c r="F1242" t="inlineStr"/>
+      <c r="G1242" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H1242" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1242" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1242" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1242" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1242" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>Athletic Club Boise vs Charlotte Independence</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>Athletic Club Boise</t>
+        </is>
+      </c>
+      <c r="D1243" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1243" t="inlineStr"/>
+      <c r="F1243" t="inlineStr"/>
+      <c r="G1243" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1243" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1243" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1243" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1243" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1243" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>Internacional de Bogotá vs Atlético Nacional</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>Atlético Nacional</t>
+        </is>
+      </c>
+      <c r="D1244" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1244" t="inlineStr"/>
+      <c r="F1244" t="inlineStr"/>
+      <c r="G1244" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H1244" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1244" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1244" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1244" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1244" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>Colorado Rapids vs St. Louis CITY SC</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>Colorado Rapids</t>
+        </is>
+      </c>
+      <c r="D1245" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1245" t="inlineStr"/>
+      <c r="F1245" t="inlineStr"/>
+      <c r="G1245" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H1245" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1245" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1245" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1245" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1245" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>Alianza FC vs FC Motagua</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>FC Motagua</t>
+        </is>
+      </c>
+      <c r="D1246" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1246" t="inlineStr"/>
+      <c r="F1246" t="inlineStr"/>
+      <c r="G1246" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1246" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1246" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1246" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1246" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1246" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -55233,7 +57875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55585,6 +58227,25 @@
       </c>
       <c r="E19" t="n">
         <v>47</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>57</v>
+      </c>
+      <c r="C20" t="n">
+        <v>43</v>
+      </c>
+      <c r="D20" t="n">
+        <v>75.40000000000001</v>
+      </c>
+      <c r="E20" t="n">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -55598,7 +58259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57329,6 +59990,237 @@
         <v>0</v>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>9</v>
+      </c>
+      <c r="D83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>24</v>
+      </c>
+      <c r="D84" t="n">
+        <v>3</v>
+      </c>
+      <c r="E84" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>fav_domina_no_gana</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>10</v>
+      </c>
+      <c r="D85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>4</v>
+      </c>
+      <c r="D86" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>7</v>
+      </c>
+      <c r="D87" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" t="n">
+        <v>14.3</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>4</v>
+      </c>
+      <c r="D88" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>9</v>
+      </c>
+      <c r="D89" t="n">
+        <v>4</v>
+      </c>
+      <c r="E89" t="n">
+        <v>44.4</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>no_fav_domina</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>7</v>
+      </c>
+      <c r="D90" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>11</v>
+      </c>
+      <c r="D91" t="n">
+        <v>1</v>
+      </c>
+      <c r="E91" t="n">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>value_alert</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>4</v>
+      </c>
+      <c r="D92" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>siguen_empatados_22</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>1</v>
+      </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-18
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1246"/>
+  <dimension ref="A1:L1268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55149,8 +55149,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1190" t="inlineStr"/>
-      <c r="F1190" t="inlineStr"/>
       <c r="G1190" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -55197,8 +55195,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1191" t="inlineStr"/>
-      <c r="F1191" t="inlineStr"/>
       <c r="G1191" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -55245,8 +55241,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1192" t="inlineStr"/>
-      <c r="F1192" t="inlineStr"/>
       <c r="G1192" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -55293,8 +55287,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1193" t="inlineStr"/>
-      <c r="F1193" t="inlineStr"/>
       <c r="G1193" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -55341,8 +55333,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1194" t="inlineStr"/>
-      <c r="F1194" t="inlineStr"/>
       <c r="G1194" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -55389,8 +55379,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1195" t="inlineStr"/>
-      <c r="F1195" t="inlineStr"/>
       <c r="G1195" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -55437,8 +55425,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1196" t="inlineStr"/>
-      <c r="F1196" t="inlineStr"/>
       <c r="G1196" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -55485,8 +55471,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1197" t="inlineStr"/>
-      <c r="F1197" t="inlineStr"/>
       <c r="G1197" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -55533,8 +55517,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1198" t="inlineStr"/>
-      <c r="F1198" t="inlineStr"/>
       <c r="G1198" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -55581,8 +55563,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1199" t="inlineStr"/>
-      <c r="F1199" t="inlineStr"/>
       <c r="G1199" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -55629,8 +55609,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1200" t="inlineStr"/>
-      <c r="F1200" t="inlineStr"/>
       <c r="G1200" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -55677,8 +55655,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1201" t="inlineStr"/>
-      <c r="F1201" t="inlineStr"/>
       <c r="G1201" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -55725,8 +55701,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1202" t="inlineStr"/>
-      <c r="F1202" t="inlineStr"/>
       <c r="G1202" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -55773,8 +55747,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1203" t="inlineStr"/>
-      <c r="F1203" t="inlineStr"/>
       <c r="G1203" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -55821,8 +55793,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1204" t="inlineStr"/>
-      <c r="F1204" t="inlineStr"/>
       <c r="G1204" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -55869,8 +55839,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1205" t="inlineStr"/>
-      <c r="F1205" t="inlineStr"/>
       <c r="G1205" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -55917,8 +55885,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1206" t="inlineStr"/>
-      <c r="F1206" t="inlineStr"/>
       <c r="G1206" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -55965,8 +55931,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1207" t="inlineStr"/>
-      <c r="F1207" t="inlineStr"/>
       <c r="G1207" t="inlineStr">
         <is>
           <t>4-3</t>
@@ -56013,8 +55977,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1208" t="inlineStr"/>
-      <c r="F1208" t="inlineStr"/>
       <c r="G1208" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -56061,8 +56023,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1209" t="inlineStr"/>
-      <c r="F1209" t="inlineStr"/>
       <c r="G1209" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -56109,8 +56069,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1210" t="inlineStr"/>
-      <c r="F1210" t="inlineStr"/>
       <c r="G1210" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -56157,8 +56115,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1211" t="inlineStr"/>
-      <c r="F1211" t="inlineStr"/>
       <c r="G1211" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -56205,8 +56161,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1212" t="inlineStr"/>
-      <c r="F1212" t="inlineStr"/>
       <c r="G1212" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -56253,8 +56207,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1213" t="inlineStr"/>
-      <c r="F1213" t="inlineStr"/>
       <c r="G1213" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -56301,8 +56253,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1214" t="inlineStr"/>
-      <c r="F1214" t="inlineStr"/>
       <c r="G1214" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -56349,8 +56299,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1215" t="inlineStr"/>
-      <c r="F1215" t="inlineStr"/>
       <c r="G1215" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -56397,8 +56345,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1216" t="inlineStr"/>
-      <c r="F1216" t="inlineStr"/>
       <c r="G1216" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -56445,8 +56391,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1217" t="inlineStr"/>
-      <c r="F1217" t="inlineStr"/>
       <c r="G1217" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -56493,8 +56437,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1218" t="inlineStr"/>
-      <c r="F1218" t="inlineStr"/>
       <c r="G1218" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -56541,8 +56483,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1219" t="inlineStr"/>
-      <c r="F1219" t="inlineStr"/>
       <c r="G1219" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -56589,8 +56529,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1220" t="inlineStr"/>
-      <c r="F1220" t="inlineStr"/>
       <c r="G1220" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -56637,8 +56575,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1221" t="inlineStr"/>
-      <c r="F1221" t="inlineStr"/>
       <c r="G1221" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -56685,8 +56621,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1222" t="inlineStr"/>
-      <c r="F1222" t="inlineStr"/>
       <c r="G1222" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -56733,8 +56667,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1223" t="inlineStr"/>
-      <c r="F1223" t="inlineStr"/>
       <c r="G1223" t="inlineStr">
         <is>
           <t>7-2</t>
@@ -56781,8 +56713,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1224" t="inlineStr"/>
-      <c r="F1224" t="inlineStr"/>
       <c r="G1224" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -56829,8 +56759,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1225" t="inlineStr"/>
-      <c r="F1225" t="inlineStr"/>
       <c r="G1225" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -56877,8 +56805,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1226" t="inlineStr"/>
-      <c r="F1226" t="inlineStr"/>
       <c r="G1226" t="inlineStr">
         <is>
           <t>4-2</t>
@@ -56925,8 +56851,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1227" t="inlineStr"/>
-      <c r="F1227" t="inlineStr"/>
       <c r="G1227" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -56973,8 +56897,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1228" t="inlineStr"/>
-      <c r="F1228" t="inlineStr"/>
       <c r="G1228" t="inlineStr">
         <is>
           <t>0-4</t>
@@ -57021,8 +56943,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1229" t="inlineStr"/>
-      <c r="F1229" t="inlineStr"/>
       <c r="G1229" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -57069,8 +56989,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1230" t="inlineStr"/>
-      <c r="F1230" t="inlineStr"/>
       <c r="G1230" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -57117,8 +57035,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1231" t="inlineStr"/>
-      <c r="F1231" t="inlineStr"/>
       <c r="G1231" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -57165,8 +57081,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1232" t="inlineStr"/>
-      <c r="F1232" t="inlineStr"/>
       <c r="G1232" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -57213,8 +57127,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1233" t="inlineStr"/>
-      <c r="F1233" t="inlineStr"/>
       <c r="G1233" t="inlineStr">
         <is>
           <t>2-4</t>
@@ -57261,8 +57173,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1234" t="inlineStr"/>
-      <c r="F1234" t="inlineStr"/>
       <c r="G1234" t="inlineStr">
         <is>
           <t>5-2</t>
@@ -57309,8 +57219,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1235" t="inlineStr"/>
-      <c r="F1235" t="inlineStr"/>
       <c r="G1235" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -57357,8 +57265,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1236" t="inlineStr"/>
-      <c r="F1236" t="inlineStr"/>
       <c r="G1236" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -57405,8 +57311,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1237" t="inlineStr"/>
-      <c r="F1237" t="inlineStr"/>
       <c r="G1237" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -57453,8 +57357,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1238" t="inlineStr"/>
-      <c r="F1238" t="inlineStr"/>
       <c r="G1238" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -57501,8 +57403,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1239" t="inlineStr"/>
-      <c r="F1239" t="inlineStr"/>
       <c r="G1239" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -57549,8 +57449,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1240" t="inlineStr"/>
-      <c r="F1240" t="inlineStr"/>
       <c r="G1240" t="inlineStr">
         <is>
           <t>4-4</t>
@@ -57597,8 +57495,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1241" t="inlineStr"/>
-      <c r="F1241" t="inlineStr"/>
       <c r="G1241" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -57645,8 +57541,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1242" t="inlineStr"/>
-      <c r="F1242" t="inlineStr"/>
       <c r="G1242" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -57693,8 +57587,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1243" t="inlineStr"/>
-      <c r="F1243" t="inlineStr"/>
       <c r="G1243" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -57741,8 +57633,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1244" t="inlineStr"/>
-      <c r="F1244" t="inlineStr"/>
       <c r="G1244" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -57789,8 +57679,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1245" t="inlineStr"/>
-      <c r="F1245" t="inlineStr"/>
       <c r="G1245" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -57837,8 +57725,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1246" t="inlineStr"/>
-      <c r="F1246" t="inlineStr"/>
       <c r="G1246" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -57859,6 +57745,1062 @@
         <v>0</v>
       </c>
       <c r="L1246" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>Machida Zelvia vs Preah Khan Reach Svay Rieng FC</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>Machida Zelvia</t>
+        </is>
+      </c>
+      <c r="D1247" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1247" t="inlineStr"/>
+      <c r="F1247" t="inlineStr"/>
+      <c r="G1247" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1247" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1247" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1247" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1247" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1247" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>Adelaide United vs Tai Po FC</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>Adelaide United</t>
+        </is>
+      </c>
+      <c r="D1248" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1248" t="inlineStr"/>
+      <c r="F1248" t="inlineStr"/>
+      <c r="G1248" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1248" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1248" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1248" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1248" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1248" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>Kitchee vs Gangwon FC</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>Kitchee</t>
+        </is>
+      </c>
+      <c r="D1249" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1249" t="inlineStr"/>
+      <c r="F1249" t="inlineStr"/>
+      <c r="G1249" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1249" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1249" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1249" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1249" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1249" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>Shanghai Shenhua vs BG Tampines Rovers FC</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>Shanghai Shenhua</t>
+        </is>
+      </c>
+      <c r="D1250" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1250" t="inlineStr"/>
+      <c r="F1250" t="inlineStr"/>
+      <c r="G1250" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1250" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1250" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1250" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1250" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1250" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>Gazovik Orenburg vs Krasnodar</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>Krasnodar</t>
+        </is>
+      </c>
+      <c r="D1251" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1251" t="inlineStr"/>
+      <c r="F1251" t="inlineStr"/>
+      <c r="G1251" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1251" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1251" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1251" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1251" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1251" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>Akron Tolyatti vs Akhmat Grozny</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>Akhmat Grozny</t>
+        </is>
+      </c>
+      <c r="D1252" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1252" t="inlineStr"/>
+      <c r="F1252" t="inlineStr"/>
+      <c r="G1252" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1252" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1252" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1252" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1252" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1252" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>OFI Crete vs TSG Hoffenheim</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>TSG Hoffenheim</t>
+        </is>
+      </c>
+      <c r="D1253" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1253" t="inlineStr"/>
+      <c r="F1253" t="inlineStr"/>
+      <c r="G1253" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1253" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1253" t="n">
+        <v>6</v>
+      </c>
+      <c r="J1253" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1253" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1253" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>Real Betis vs Getafe</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>Real Betis</t>
+        </is>
+      </c>
+      <c r="D1254" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1254" t="inlineStr"/>
+      <c r="F1254" t="inlineStr"/>
+      <c r="G1254" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1254" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1254" t="n">
+        <v>6</v>
+      </c>
+      <c r="J1254" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1254" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1254" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>Orlando Pirates vs Durban City</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>Orlando Pirates</t>
+        </is>
+      </c>
+      <c r="D1255" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1255" t="inlineStr"/>
+      <c r="F1255" t="inlineStr"/>
+      <c r="G1255" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1255" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1255" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1255" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1255" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1255" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>Dynamo Makhachkala vs CSKA Moscow</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>CSKA Moscow</t>
+        </is>
+      </c>
+      <c r="D1256" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1256" t="inlineStr"/>
+      <c r="F1256" t="inlineStr"/>
+      <c r="G1256" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H1256" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1256" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1256" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1256" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1256" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>Manchester City vs Norwich City</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="D1257" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1257" t="inlineStr"/>
+      <c r="F1257" t="inlineStr"/>
+      <c r="G1257" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H1257" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1257" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1257" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1257" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1257" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>Besiktas vs Marseille</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="D1258" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1258" t="inlineStr"/>
+      <c r="F1258" t="inlineStr"/>
+      <c r="G1258" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H1258" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1258" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1258" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1258" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1258" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>Celtic vs Ferencvaros</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>Celtic</t>
+        </is>
+      </c>
+      <c r="D1259" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1259" t="inlineStr"/>
+      <c r="F1259" t="inlineStr"/>
+      <c r="G1259" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H1259" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1259" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1259" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1259" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1259" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>Crystal Palace vs Lech Poznan</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>Crystal Palace</t>
+        </is>
+      </c>
+      <c r="D1260" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1260" t="inlineStr"/>
+      <c r="F1260" t="inlineStr"/>
+      <c r="G1260" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H1260" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1260" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1260" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1260" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1260" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>Juventus vs NEC Nijmegen</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>Juventus</t>
+        </is>
+      </c>
+      <c r="D1261" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1261" t="inlineStr"/>
+      <c r="F1261" t="inlineStr"/>
+      <c r="G1261" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H1261" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1261" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1261" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1261" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1261" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>Lillestrom vs Torreense</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>Lillestrom</t>
+        </is>
+      </c>
+      <c r="D1262" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1262" t="inlineStr"/>
+      <c r="F1262" t="inlineStr"/>
+      <c r="G1262" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1262" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1262" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1262" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1262" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1262" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>Real Sociedad vs AFC Bournemouth</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>AFC Bournemouth</t>
+        </is>
+      </c>
+      <c r="D1263" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1263" t="inlineStr"/>
+      <c r="F1263" t="inlineStr"/>
+      <c r="G1263" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1263" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1263" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1263" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1263" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1263" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>AFC Wimbledon vs Milton Keynes Dons</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>Milton Keynes Dons</t>
+        </is>
+      </c>
+      <c r="D1264" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1264" t="inlineStr"/>
+      <c r="F1264" t="inlineStr"/>
+      <c r="G1264" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1264" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1264" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1264" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1264" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1264" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>Málaga vs Villarreal</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="D1265" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1265" t="inlineStr"/>
+      <c r="F1265" t="inlineStr"/>
+      <c r="G1265" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H1265" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1265" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1265" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1265" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1265" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Oriente Petrolero</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="D1266" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1266" t="inlineStr"/>
+      <c r="F1266" t="inlineStr"/>
+      <c r="G1266" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1266" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1266" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1266" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1266" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1266" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>Atlético Bucaramanga vs Independiente Medellín</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>Atlético Bucaramanga</t>
+        </is>
+      </c>
+      <c r="D1267" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1267" t="inlineStr"/>
+      <c r="F1267" t="inlineStr"/>
+      <c r="G1267" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H1267" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1267" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1267" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1267" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1267" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>Flamengo vs Independiente del Valle</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="D1268" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1268" t="inlineStr"/>
+      <c r="F1268" t="inlineStr"/>
+      <c r="G1268" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1268" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1268" t="n">
+        <v>7</v>
+      </c>
+      <c r="J1268" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1268" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1268" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -57875,7 +58817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58246,6 +59188,25 @@
       </c>
       <c r="E20" t="n">
         <v>57</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>22</v>
+      </c>
+      <c r="C21" t="n">
+        <v>16</v>
+      </c>
+      <c r="D21" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="E21" t="n">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -58259,7 +59220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E93"/>
+  <dimension ref="A1:E104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -60221,6 +61182,237 @@
         <v>0</v>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>6</v>
+      </c>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>8</v>
+      </c>
+      <c r="D95" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>no_fav_domina</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>6</v>
+      </c>
+      <c r="D96" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>siguen_empatados_22</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>2</v>
+      </c>
+      <c r="D97" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>8</v>
+      </c>
+      <c r="D98" t="n">
+        <v>2</v>
+      </c>
+      <c r="E98" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>fav_domina_no_gana</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>6</v>
+      </c>
+      <c r="D99" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>1</v>
+      </c>
+      <c r="D100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>5</v>
+      </c>
+      <c r="D101" t="n">
+        <v>1</v>
+      </c>
+      <c r="E101" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>6</v>
+      </c>
+      <c r="D102" t="n">
+        <v>4</v>
+      </c>
+      <c r="E102" t="n">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>4</v>
+      </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
+      <c r="E103" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>value_alert</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>1</v>
+      </c>
+      <c r="D104" t="n">
+        <v>0</v>
+      </c>
+      <c r="E104" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-19
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1268"/>
+  <dimension ref="A1:L1318"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57771,8 +57771,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1247" t="inlineStr"/>
-      <c r="F1247" t="inlineStr"/>
       <c r="G1247" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -57819,8 +57817,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1248" t="inlineStr"/>
-      <c r="F1248" t="inlineStr"/>
       <c r="G1248" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -57867,8 +57863,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1249" t="inlineStr"/>
-      <c r="F1249" t="inlineStr"/>
       <c r="G1249" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -57915,8 +57909,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1250" t="inlineStr"/>
-      <c r="F1250" t="inlineStr"/>
       <c r="G1250" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -57963,8 +57955,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1251" t="inlineStr"/>
-      <c r="F1251" t="inlineStr"/>
       <c r="G1251" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -58011,8 +58001,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1252" t="inlineStr"/>
-      <c r="F1252" t="inlineStr"/>
       <c r="G1252" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -58059,8 +58047,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1253" t="inlineStr"/>
-      <c r="F1253" t="inlineStr"/>
       <c r="G1253" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -58107,8 +58093,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1254" t="inlineStr"/>
-      <c r="F1254" t="inlineStr"/>
       <c r="G1254" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -58155,8 +58139,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1255" t="inlineStr"/>
-      <c r="F1255" t="inlineStr"/>
       <c r="G1255" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -58203,8 +58185,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1256" t="inlineStr"/>
-      <c r="F1256" t="inlineStr"/>
       <c r="G1256" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -58251,8 +58231,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1257" t="inlineStr"/>
-      <c r="F1257" t="inlineStr"/>
       <c r="G1257" t="inlineStr">
         <is>
           <t>5-0</t>
@@ -58299,8 +58277,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1258" t="inlineStr"/>
-      <c r="F1258" t="inlineStr"/>
       <c r="G1258" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -58347,8 +58323,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1259" t="inlineStr"/>
-      <c r="F1259" t="inlineStr"/>
       <c r="G1259" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -58395,8 +58369,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1260" t="inlineStr"/>
-      <c r="F1260" t="inlineStr"/>
       <c r="G1260" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -58443,8 +58415,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1261" t="inlineStr"/>
-      <c r="F1261" t="inlineStr"/>
       <c r="G1261" t="inlineStr">
         <is>
           <t>5-0</t>
@@ -58491,8 +58461,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1262" t="inlineStr"/>
-      <c r="F1262" t="inlineStr"/>
       <c r="G1262" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -58539,8 +58507,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1263" t="inlineStr"/>
-      <c r="F1263" t="inlineStr"/>
       <c r="G1263" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -58587,8 +58553,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1264" t="inlineStr"/>
-      <c r="F1264" t="inlineStr"/>
       <c r="G1264" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -58635,8 +58599,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1265" t="inlineStr"/>
-      <c r="F1265" t="inlineStr"/>
       <c r="G1265" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -58683,8 +58645,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1266" t="inlineStr"/>
-      <c r="F1266" t="inlineStr"/>
       <c r="G1266" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -58731,8 +58691,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1267" t="inlineStr"/>
-      <c r="F1267" t="inlineStr"/>
       <c r="G1267" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -58779,8 +58737,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1268" t="inlineStr"/>
-      <c r="F1268" t="inlineStr"/>
       <c r="G1268" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -58801,6 +58757,2406 @@
         <v>0</v>
       </c>
       <c r="L1268" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>SpVgg Greuther Fürth vs 1. FC Magdeburg</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>1. FC Magdeburg</t>
+        </is>
+      </c>
+      <c r="D1269" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1269" t="inlineStr"/>
+      <c r="F1269" t="inlineStr"/>
+      <c r="G1269" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1269" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1269" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1269" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1269" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1269" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>VfL Wolfsburg vs SV Darmstadt 98</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>VfL Wolfsburg</t>
+        </is>
+      </c>
+      <c r="D1270" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1270" t="inlineStr"/>
+      <c r="F1270" t="inlineStr"/>
+      <c r="G1270" t="inlineStr">
+        <is>
+          <t>5-1</t>
+        </is>
+      </c>
+      <c r="H1270" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1270" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1270" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1270" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1270" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>Lyngby Boldklub vs Silkeborg IF</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>Lyngby Boldklub</t>
+        </is>
+      </c>
+      <c r="D1271" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1271" t="inlineStr"/>
+      <c r="F1271" t="inlineStr"/>
+      <c r="G1271" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H1271" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1271" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1271" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1271" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1271" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>Sarpsborg FK vs KFUM Oslo</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>Sarpsborg FK</t>
+        </is>
+      </c>
+      <c r="D1272" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1272" t="inlineStr"/>
+      <c r="F1272" t="inlineStr"/>
+      <c r="G1272" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H1272" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1272" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1272" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1272" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1272" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>Kasimpasa vs Konyaspor</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>Kasimpasa</t>
+        </is>
+      </c>
+      <c r="D1273" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1273" t="inlineStr"/>
+      <c r="F1273" t="inlineStr"/>
+      <c r="G1273" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1273" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1273" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1273" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1273" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1273" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>Rapid Vienna vs WSG Swarovski Tirol</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>Rapid Vienna</t>
+        </is>
+      </c>
+      <c r="D1274" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1274" t="inlineStr"/>
+      <c r="F1274" t="inlineStr"/>
+      <c r="G1274" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1274" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1274" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1274" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1274" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1274" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>FC Groningen vs PEC Zwolle</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>FC Groningen</t>
+        </is>
+      </c>
+      <c r="D1275" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1275" t="inlineStr"/>
+      <c r="F1275" t="inlineStr"/>
+      <c r="G1275" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1275" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1275" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1275" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1275" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1275" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>Comunicaciones vs Defensores Unidos</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>Comunicaciones</t>
+        </is>
+      </c>
+      <c r="D1276" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1276" t="inlineStr"/>
+      <c r="F1276" t="inlineStr"/>
+      <c r="G1276" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1276" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1276" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1276" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1276" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1276" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>Annecy vs Dijon FCO</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>Annecy</t>
+        </is>
+      </c>
+      <c r="D1277" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1277" t="inlineStr"/>
+      <c r="F1277" t="inlineStr"/>
+      <c r="G1277" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1277" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1277" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1277" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1277" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1277" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>Grenoble vs Clermont Foot</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>Grenoble</t>
+        </is>
+      </c>
+      <c r="D1278" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1278" t="inlineStr"/>
+      <c r="F1278" t="inlineStr"/>
+      <c r="G1278" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1278" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1278" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1278" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1278" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1278" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>Stade Laval vs Sochaux</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>Stade Laval</t>
+        </is>
+      </c>
+      <c r="D1279" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1279" t="inlineStr"/>
+      <c r="F1279" t="inlineStr"/>
+      <c r="G1279" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1279" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1279" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1279" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1279" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1279" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>Pau vs Dunkerque</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>Pau</t>
+        </is>
+      </c>
+      <c r="D1280" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1280" t="inlineStr"/>
+      <c r="F1280" t="inlineStr"/>
+      <c r="G1280" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1280" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1280" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1280" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1280" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1280" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>Stade de Reims vs Montpellier</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>Stade de Reims</t>
+        </is>
+      </c>
+      <c r="D1281" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1281" t="inlineStr"/>
+      <c r="F1281" t="inlineStr"/>
+      <c r="G1281" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1281" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1281" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1281" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1281" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1281" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>Rodez Aveyron vs AS Nancy Lorraine</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>Rodez Aveyron</t>
+        </is>
+      </c>
+      <c r="D1282" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1282" t="inlineStr"/>
+      <c r="F1282" t="inlineStr"/>
+      <c r="G1282" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H1282" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1282" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1282" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1282" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1282" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>Almere City vs Heracles Almelo</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>Heracles Almelo</t>
+        </is>
+      </c>
+      <c r="D1283" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1283" t="inlineStr"/>
+      <c r="F1283" t="inlineStr"/>
+      <c r="G1283" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1283" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1283" t="n">
+        <v>6</v>
+      </c>
+      <c r="J1283" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1283" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1283" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>FC Den Bosch vs Helmond Sport</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>FC Den Bosch</t>
+        </is>
+      </c>
+      <c r="D1284" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1284" t="inlineStr"/>
+      <c r="F1284" t="inlineStr"/>
+      <c r="G1284" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1284" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1284" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1284" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1284" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1284" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>FC Eindhoven vs FC Emmen</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>FC Emmen</t>
+        </is>
+      </c>
+      <c r="D1285" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1285" t="inlineStr"/>
+      <c r="F1285" t="inlineStr"/>
+      <c r="G1285" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1285" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1285" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1285" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1285" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1285" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>Jong Ajax vs Roda JC Kerkrade</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>Roda JC Kerkrade</t>
+        </is>
+      </c>
+      <c r="D1286" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1286" t="inlineStr"/>
+      <c r="F1286" t="inlineStr"/>
+      <c r="G1286" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1286" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1286" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1286" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1286" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1286" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>Jong AZ vs FC Volendam</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>FC Volendam</t>
+        </is>
+      </c>
+      <c r="D1287" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1287" t="inlineStr"/>
+      <c r="F1287" t="inlineStr"/>
+      <c r="G1287" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H1287" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1287" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1287" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1287" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1287" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>Jong FC Utrecht vs VVV-Venlo</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>Jong FC Utrecht</t>
+        </is>
+      </c>
+      <c r="D1288" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1288" t="inlineStr"/>
+      <c r="F1288" t="inlineStr"/>
+      <c r="G1288" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H1288" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1288" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1288" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1288" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1288" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>RKC Waalwijk vs MVV Maastricht</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>RKC Waalwijk</t>
+        </is>
+      </c>
+      <c r="D1289" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1289" t="inlineStr"/>
+      <c r="F1289" t="inlineStr"/>
+      <c r="G1289" t="inlineStr">
+        <is>
+          <t>6-1</t>
+        </is>
+      </c>
+      <c r="H1289" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1289" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1289" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1289" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1289" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>Bayern Munich vs 1. FC Union Berlin</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="D1290" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1290" t="inlineStr"/>
+      <c r="F1290" t="inlineStr"/>
+      <c r="G1290" t="inlineStr">
+        <is>
+          <t>7-0</t>
+        </is>
+      </c>
+      <c r="H1290" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1290" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1290" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1290" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1290" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>Queen's Park vs Ayr United</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>Ayr United</t>
+        </is>
+      </c>
+      <c r="D1291" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1291" t="inlineStr"/>
+      <c r="F1291" t="inlineStr"/>
+      <c r="G1291" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1291" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1291" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1291" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1291" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1291" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>Juve Stabia vs Cesena</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>Juve Stabia</t>
+        </is>
+      </c>
+      <c r="D1292" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1292" t="inlineStr"/>
+      <c r="F1292" t="inlineStr"/>
+      <c r="G1292" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1292" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1292" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1292" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1292" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1292" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>Albacete vs Córdoba</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>Albacete</t>
+        </is>
+      </c>
+      <c r="D1293" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1293" t="inlineStr"/>
+      <c r="F1293" t="inlineStr"/>
+      <c r="G1293" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1293" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1293" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1293" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1293" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1293" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>AS Monaco vs Lens</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>AS Monaco</t>
+        </is>
+      </c>
+      <c r="D1294" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1294" t="inlineStr"/>
+      <c r="F1294" t="inlineStr"/>
+      <c r="G1294" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1294" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1294" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1294" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1294" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1294" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>Monza vs Sassuolo</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>Sassuolo</t>
+        </is>
+      </c>
+      <c r="D1295" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1295" t="inlineStr"/>
+      <c r="F1295" t="inlineStr"/>
+      <c r="G1295" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1295" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1295" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1295" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1295" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1295" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>KAA Gent vs Standard Liege</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>KAA Gent</t>
+        </is>
+      </c>
+      <c r="D1296" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1296" t="inlineStr"/>
+      <c r="F1296" t="inlineStr"/>
+      <c r="G1296" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1296" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1296" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1296" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1296" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1296" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>Yeovil Town vs Solihull Moors</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>Yeovil Town</t>
+        </is>
+      </c>
+      <c r="D1297" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1297" t="inlineStr"/>
+      <c r="F1297" t="inlineStr"/>
+      <c r="G1297" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H1297" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1297" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1297" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1297" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1297" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>Worcester City vs Stratford Town</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>Worcester City</t>
+        </is>
+      </c>
+      <c r="D1298" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1298" t="inlineStr"/>
+      <c r="F1298" t="inlineStr"/>
+      <c r="G1298" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1298" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1298" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1298" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1298" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1298" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>Yate Town vs Chippenham Town</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>Yate Town</t>
+        </is>
+      </c>
+      <c r="D1299" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1299" t="inlineStr"/>
+      <c r="F1299" t="inlineStr"/>
+      <c r="G1299" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1299" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1299" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1299" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1299" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1299" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>Brentford vs Chelsea</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>Chelsea</t>
+        </is>
+      </c>
+      <c r="D1300" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1300" t="inlineStr"/>
+      <c r="F1300" t="inlineStr"/>
+      <c r="G1300" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1300" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1300" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1300" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1300" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1300" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>Espanyol vs Elche</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>Espanyol</t>
+        </is>
+      </c>
+      <c r="D1301" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1301" t="inlineStr"/>
+      <c r="F1301" t="inlineStr"/>
+      <c r="G1301" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H1301" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1301" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1301" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1301" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1301" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>Bristol City vs Watford</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>Bristol City</t>
+        </is>
+      </c>
+      <c r="D1302" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1302" t="inlineStr"/>
+      <c r="F1302" t="inlineStr"/>
+      <c r="G1302" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1302" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1302" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1302" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1302" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1302" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>Sportivo Trinidense vs Guaraní</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>Sportivo Trinidense</t>
+        </is>
+      </c>
+      <c r="D1303" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1303" t="inlineStr"/>
+      <c r="F1303" t="inlineStr"/>
+      <c r="G1303" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1303" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1303" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1303" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1303" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1303" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>Alianza Atlético vs Comerciantes Unidos</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>Alianza Atlético</t>
+        </is>
+      </c>
+      <c r="D1304" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1304" t="inlineStr"/>
+      <c r="F1304" t="inlineStr"/>
+      <c r="G1304" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1304" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1304" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1304" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1304" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1304" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>Águilas Doradas vs Deportivo Pereira</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>Águilas Doradas</t>
+        </is>
+      </c>
+      <c r="D1305" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1305" t="inlineStr"/>
+      <c r="F1305" t="inlineStr"/>
+      <c r="G1305" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H1305" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1305" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1305" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1305" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1305" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>Platense vs UPNFM</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>Platense</t>
+        </is>
+      </c>
+      <c r="D1306" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1306" t="inlineStr"/>
+      <c r="F1306" t="inlineStr"/>
+      <c r="G1306" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1306" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1306" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1306" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1306" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1306" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>Nacional Asunción vs 2 de Mayo</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>Nacional Asunción</t>
+        </is>
+      </c>
+      <c r="D1307" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1307" t="inlineStr"/>
+      <c r="F1307" t="inlineStr"/>
+      <c r="G1307" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1307" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1307" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1307" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1307" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1307" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>Vila Nova vs América Mineiro</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="D1308" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1308" t="inlineStr"/>
+      <c r="F1308" t="inlineStr"/>
+      <c r="G1308" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1308" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1308" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1308" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1308" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1308" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>Independiente Petrolero vs San Antonio Bulo Bulo</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>Independiente Petrolero</t>
+        </is>
+      </c>
+      <c r="D1309" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1309" t="inlineStr"/>
+      <c r="F1309" t="inlineStr"/>
+      <c r="G1309" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H1309" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1309" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1309" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1309" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1309" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>Ceará vs Novorizontino</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>Novorizontino</t>
+        </is>
+      </c>
+      <c r="D1310" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1310" t="inlineStr"/>
+      <c r="F1310" t="inlineStr"/>
+      <c r="G1310" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1310" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1310" t="n">
+        <v>9</v>
+      </c>
+      <c r="J1310" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1310" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1310" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>São Bernardo vs Atlético Goianiense</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>São Bernardo</t>
+        </is>
+      </c>
+      <c r="D1311" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1311" t="inlineStr"/>
+      <c r="F1311" t="inlineStr"/>
+      <c r="G1311" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1311" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1311" t="n">
+        <v>4</v>
+      </c>
+      <c r="J1311" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1311" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1311" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>Racing Club vs Sarmiento (Junín)</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>Racing Club</t>
+        </is>
+      </c>
+      <c r="D1312" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1312" t="inlineStr"/>
+      <c r="F1312" t="inlineStr"/>
+      <c r="G1312" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1312" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1312" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1312" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1312" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1312" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>Puebla vs Atlante</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="D1313" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1313" t="inlineStr"/>
+      <c r="F1313" t="inlineStr"/>
+      <c r="G1313" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1313" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1313" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1313" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1313" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1313" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>Tepatitlán FC vs Mineros de Zacatecas</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>Mineros de Zacatecas</t>
+        </is>
+      </c>
+      <c r="D1314" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1314" t="inlineStr"/>
+      <c r="F1314" t="inlineStr"/>
+      <c r="G1314" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1314" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1314" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1314" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1314" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1314" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>Piratas vs Venados FC</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>Piratas</t>
+        </is>
+      </c>
+      <c r="D1315" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1315" t="inlineStr"/>
+      <c r="F1315" t="inlineStr"/>
+      <c r="G1315" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1315" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1315" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1315" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1315" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1315" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>Alianza Lima vs ADT</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>Alianza Lima</t>
+        </is>
+      </c>
+      <c r="D1316" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1316" t="inlineStr"/>
+      <c r="F1316" t="inlineStr"/>
+      <c r="G1316" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1316" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1316" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1316" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1316" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1316" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>Pérez Zeledón vs Sporting San José</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>Sporting San José</t>
+        </is>
+      </c>
+      <c r="D1317" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1317" t="inlineStr"/>
+      <c r="F1317" t="inlineStr"/>
+      <c r="G1317" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1317" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1317" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1317" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1317" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1317" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>FC Juarez vs Tigres UANL</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>FC Juarez</t>
+        </is>
+      </c>
+      <c r="D1318" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1318" t="inlineStr"/>
+      <c r="F1318" t="inlineStr"/>
+      <c r="G1318" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1318" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1318" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1318" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1318" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1318" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -58817,7 +61173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -59207,6 +61563,25 @@
       </c>
       <c r="E21" t="n">
         <v>22</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>50</v>
+      </c>
+      <c r="C22" t="n">
+        <v>32</v>
+      </c>
+      <c r="D22" t="n">
+        <v>64</v>
+      </c>
+      <c r="E22" t="n">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -59220,7 +61595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E104"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61413,6 +63788,237 @@
         <v>0</v>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>10</v>
+      </c>
+      <c r="D105" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>no_fav_domina</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>12</v>
+      </c>
+      <c r="D106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>18</v>
+      </c>
+      <c r="D107" t="n">
+        <v>3</v>
+      </c>
+      <c r="E107" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>23</v>
+      </c>
+      <c r="D108" t="n">
+        <v>6</v>
+      </c>
+      <c r="E108" t="n">
+        <v>26.1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>fav_domina_no_gana</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>8</v>
+      </c>
+      <c r="D109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>9</v>
+      </c>
+      <c r="D110" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>7</v>
+      </c>
+      <c r="D111" t="n">
+        <v>2</v>
+      </c>
+      <c r="E111" t="n">
+        <v>28.6</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>24</v>
+      </c>
+      <c r="D112" t="n">
+        <v>6</v>
+      </c>
+      <c r="E112" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>value_alert</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>1</v>
+      </c>
+      <c r="D113" t="n">
+        <v>0</v>
+      </c>
+      <c r="E113" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>7</v>
+      </c>
+      <c r="D114" t="n">
+        <v>1</v>
+      </c>
+      <c r="E114" t="n">
+        <v>14.3</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>siguen_empatados_22</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>1</v>
+      </c>
+      <c r="D115" t="n">
+        <v>0</v>
+      </c>
+      <c r="E115" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-22
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1588"/>
+  <dimension ref="A1:L1596"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -68673,8 +68673,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1484" t="inlineStr"/>
-      <c r="F1484" t="inlineStr"/>
       <c r="G1484" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -68721,8 +68719,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1485" t="inlineStr"/>
-      <c r="F1485" t="inlineStr"/>
       <c r="G1485" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -68769,8 +68765,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1486" t="inlineStr"/>
-      <c r="F1486" t="inlineStr"/>
       <c r="G1486" t="inlineStr">
         <is>
           <t>5-0</t>
@@ -68817,8 +68811,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1487" t="inlineStr"/>
-      <c r="F1487" t="inlineStr"/>
       <c r="G1487" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -68865,8 +68857,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1488" t="inlineStr"/>
-      <c r="F1488" t="inlineStr"/>
       <c r="G1488" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -68913,8 +68903,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1489" t="inlineStr"/>
-      <c r="F1489" t="inlineStr"/>
       <c r="G1489" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -68961,8 +68949,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1490" t="inlineStr"/>
-      <c r="F1490" t="inlineStr"/>
       <c r="G1490" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -69009,8 +68995,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1491" t="inlineStr"/>
-      <c r="F1491" t="inlineStr"/>
       <c r="G1491" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -69057,8 +69041,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1492" t="inlineStr"/>
-      <c r="F1492" t="inlineStr"/>
       <c r="G1492" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -69105,8 +69087,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1493" t="inlineStr"/>
-      <c r="F1493" t="inlineStr"/>
       <c r="G1493" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -69153,8 +69133,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1494" t="inlineStr"/>
-      <c r="F1494" t="inlineStr"/>
       <c r="G1494" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -69201,8 +69179,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1495" t="inlineStr"/>
-      <c r="F1495" t="inlineStr"/>
       <c r="G1495" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -69249,8 +69225,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1496" t="inlineStr"/>
-      <c r="F1496" t="inlineStr"/>
       <c r="G1496" t="inlineStr">
         <is>
           <t>4-2</t>
@@ -69297,8 +69271,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1497" t="inlineStr"/>
-      <c r="F1497" t="inlineStr"/>
       <c r="G1497" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -69345,8 +69317,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1498" t="inlineStr"/>
-      <c r="F1498" t="inlineStr"/>
       <c r="G1498" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -69393,8 +69363,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1499" t="inlineStr"/>
-      <c r="F1499" t="inlineStr"/>
       <c r="G1499" t="inlineStr">
         <is>
           <t>0-5</t>
@@ -69441,8 +69409,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1500" t="inlineStr"/>
-      <c r="F1500" t="inlineStr"/>
       <c r="G1500" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -69489,8 +69455,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1501" t="inlineStr"/>
-      <c r="F1501" t="inlineStr"/>
       <c r="G1501" t="inlineStr">
         <is>
           <t>3-4</t>
@@ -69537,8 +69501,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1502" t="inlineStr"/>
-      <c r="F1502" t="inlineStr"/>
       <c r="G1502" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -69585,8 +69547,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1503" t="inlineStr"/>
-      <c r="F1503" t="inlineStr"/>
       <c r="G1503" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -69633,8 +69593,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1504" t="inlineStr"/>
-      <c r="F1504" t="inlineStr"/>
       <c r="G1504" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -69681,8 +69639,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1505" t="inlineStr"/>
-      <c r="F1505" t="inlineStr"/>
       <c r="G1505" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -69729,8 +69685,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1506" t="inlineStr"/>
-      <c r="F1506" t="inlineStr"/>
       <c r="G1506" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -69777,8 +69731,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1507" t="inlineStr"/>
-      <c r="F1507" t="inlineStr"/>
       <c r="G1507" t="inlineStr">
         <is>
           <t>5-3</t>
@@ -69825,8 +69777,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1508" t="inlineStr"/>
-      <c r="F1508" t="inlineStr"/>
       <c r="G1508" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -69873,8 +69823,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1509" t="inlineStr"/>
-      <c r="F1509" t="inlineStr"/>
       <c r="G1509" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -69921,8 +69869,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1510" t="inlineStr"/>
-      <c r="F1510" t="inlineStr"/>
       <c r="G1510" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -69969,8 +69915,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1511" t="inlineStr"/>
-      <c r="F1511" t="inlineStr"/>
       <c r="G1511" t="inlineStr">
         <is>
           <t>1-4</t>
@@ -70017,8 +69961,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1512" t="inlineStr"/>
-      <c r="F1512" t="inlineStr"/>
       <c r="G1512" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -70065,8 +70007,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1513" t="inlineStr"/>
-      <c r="F1513" t="inlineStr"/>
       <c r="G1513" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -70113,8 +70053,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1514" t="inlineStr"/>
-      <c r="F1514" t="inlineStr"/>
       <c r="G1514" t="inlineStr">
         <is>
           <t>0-4</t>
@@ -70161,8 +70099,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1515" t="inlineStr"/>
-      <c r="F1515" t="inlineStr"/>
       <c r="G1515" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -70209,8 +70145,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1516" t="inlineStr"/>
-      <c r="F1516" t="inlineStr"/>
       <c r="G1516" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -70257,8 +70191,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1517" t="inlineStr"/>
-      <c r="F1517" t="inlineStr"/>
       <c r="G1517" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -70305,8 +70237,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1518" t="inlineStr"/>
-      <c r="F1518" t="inlineStr"/>
       <c r="G1518" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -70353,8 +70283,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1519" t="inlineStr"/>
-      <c r="F1519" t="inlineStr"/>
       <c r="G1519" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -70401,8 +70329,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1520" t="inlineStr"/>
-      <c r="F1520" t="inlineStr"/>
       <c r="G1520" t="inlineStr">
         <is>
           <t>8-0</t>
@@ -70449,8 +70375,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1521" t="inlineStr"/>
-      <c r="F1521" t="inlineStr"/>
       <c r="G1521" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -70497,8 +70421,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1522" t="inlineStr"/>
-      <c r="F1522" t="inlineStr"/>
       <c r="G1522" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -70545,8 +70467,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1523" t="inlineStr"/>
-      <c r="F1523" t="inlineStr"/>
       <c r="G1523" t="inlineStr">
         <is>
           <t>6-1</t>
@@ -70593,8 +70513,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1524" t="inlineStr"/>
-      <c r="F1524" t="inlineStr"/>
       <c r="G1524" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -70641,8 +70559,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1525" t="inlineStr"/>
-      <c r="F1525" t="inlineStr"/>
       <c r="G1525" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -70689,8 +70605,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1526" t="inlineStr"/>
-      <c r="F1526" t="inlineStr"/>
       <c r="G1526" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -70737,8 +70651,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1527" t="inlineStr"/>
-      <c r="F1527" t="inlineStr"/>
       <c r="G1527" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -70785,8 +70697,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1528" t="inlineStr"/>
-      <c r="F1528" t="inlineStr"/>
       <c r="G1528" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -70833,8 +70743,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1529" t="inlineStr"/>
-      <c r="F1529" t="inlineStr"/>
       <c r="G1529" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -70881,8 +70789,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1530" t="inlineStr"/>
-      <c r="F1530" t="inlineStr"/>
       <c r="G1530" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -70929,8 +70835,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1531" t="inlineStr"/>
-      <c r="F1531" t="inlineStr"/>
       <c r="G1531" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -70977,8 +70881,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1532" t="inlineStr"/>
-      <c r="F1532" t="inlineStr"/>
       <c r="G1532" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -71025,8 +70927,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1533" t="inlineStr"/>
-      <c r="F1533" t="inlineStr"/>
       <c r="G1533" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -71073,8 +70973,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1534" t="inlineStr"/>
-      <c r="F1534" t="inlineStr"/>
       <c r="G1534" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -71121,8 +71019,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1535" t="inlineStr"/>
-      <c r="F1535" t="inlineStr"/>
       <c r="G1535" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -71169,8 +71065,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1536" t="inlineStr"/>
-      <c r="F1536" t="inlineStr"/>
       <c r="G1536" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -71217,8 +71111,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1537" t="inlineStr"/>
-      <c r="F1537" t="inlineStr"/>
       <c r="G1537" t="inlineStr">
         <is>
           <t>5-1</t>
@@ -71265,8 +71157,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1538" t="inlineStr"/>
-      <c r="F1538" t="inlineStr"/>
       <c r="G1538" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -71313,8 +71203,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1539" t="inlineStr"/>
-      <c r="F1539" t="inlineStr"/>
       <c r="G1539" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -71361,8 +71249,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1540" t="inlineStr"/>
-      <c r="F1540" t="inlineStr"/>
       <c r="G1540" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -71409,8 +71295,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1541" t="inlineStr"/>
-      <c r="F1541" t="inlineStr"/>
       <c r="G1541" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -71457,8 +71341,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1542" t="inlineStr"/>
-      <c r="F1542" t="inlineStr"/>
       <c r="G1542" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -71505,8 +71387,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1543" t="inlineStr"/>
-      <c r="F1543" t="inlineStr"/>
       <c r="G1543" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -71553,8 +71433,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1544" t="inlineStr"/>
-      <c r="F1544" t="inlineStr"/>
       <c r="G1544" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -71601,8 +71479,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1545" t="inlineStr"/>
-      <c r="F1545" t="inlineStr"/>
       <c r="G1545" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -71649,8 +71525,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1546" t="inlineStr"/>
-      <c r="F1546" t="inlineStr"/>
       <c r="G1546" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -71697,8 +71571,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1547" t="inlineStr"/>
-      <c r="F1547" t="inlineStr"/>
       <c r="G1547" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -71745,8 +71617,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1548" t="inlineStr"/>
-      <c r="F1548" t="inlineStr"/>
       <c r="G1548" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -71793,8 +71663,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1549" t="inlineStr"/>
-      <c r="F1549" t="inlineStr"/>
       <c r="G1549" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -71841,8 +71709,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1550" t="inlineStr"/>
-      <c r="F1550" t="inlineStr"/>
       <c r="G1550" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -71889,8 +71755,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1551" t="inlineStr"/>
-      <c r="F1551" t="inlineStr"/>
       <c r="G1551" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -71937,8 +71801,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1552" t="inlineStr"/>
-      <c r="F1552" t="inlineStr"/>
       <c r="G1552" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -71985,8 +71847,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1553" t="inlineStr"/>
-      <c r="F1553" t="inlineStr"/>
       <c r="G1553" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -72033,8 +71893,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1554" t="inlineStr"/>
-      <c r="F1554" t="inlineStr"/>
       <c r="G1554" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -72081,8 +71939,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1555" t="inlineStr"/>
-      <c r="F1555" t="inlineStr"/>
       <c r="G1555" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -72129,8 +71985,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1556" t="inlineStr"/>
-      <c r="F1556" t="inlineStr"/>
       <c r="G1556" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -72177,8 +72031,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1557" t="inlineStr"/>
-      <c r="F1557" t="inlineStr"/>
       <c r="G1557" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -72225,8 +72077,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1558" t="inlineStr"/>
-      <c r="F1558" t="inlineStr"/>
       <c r="G1558" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -72273,8 +72123,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1559" t="inlineStr"/>
-      <c r="F1559" t="inlineStr"/>
       <c r="G1559" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -72321,8 +72169,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1560" t="inlineStr"/>
-      <c r="F1560" t="inlineStr"/>
       <c r="G1560" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -72369,8 +72215,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1561" t="inlineStr"/>
-      <c r="F1561" t="inlineStr"/>
       <c r="G1561" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -72417,8 +72261,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1562" t="inlineStr"/>
-      <c r="F1562" t="inlineStr"/>
       <c r="G1562" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -72465,8 +72307,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1563" t="inlineStr"/>
-      <c r="F1563" t="inlineStr"/>
       <c r="G1563" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -72513,8 +72353,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1564" t="inlineStr"/>
-      <c r="F1564" t="inlineStr"/>
       <c r="G1564" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -72561,8 +72399,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1565" t="inlineStr"/>
-      <c r="F1565" t="inlineStr"/>
       <c r="G1565" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -72609,8 +72445,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1566" t="inlineStr"/>
-      <c r="F1566" t="inlineStr"/>
       <c r="G1566" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -72657,8 +72491,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1567" t="inlineStr"/>
-      <c r="F1567" t="inlineStr"/>
       <c r="G1567" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -72705,8 +72537,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1568" t="inlineStr"/>
-      <c r="F1568" t="inlineStr"/>
       <c r="G1568" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -72753,8 +72583,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1569" t="inlineStr"/>
-      <c r="F1569" t="inlineStr"/>
       <c r="G1569" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -72801,8 +72629,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1570" t="inlineStr"/>
-      <c r="F1570" t="inlineStr"/>
       <c r="G1570" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -72849,8 +72675,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1571" t="inlineStr"/>
-      <c r="F1571" t="inlineStr"/>
       <c r="G1571" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -72897,8 +72721,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1572" t="inlineStr"/>
-      <c r="F1572" t="inlineStr"/>
       <c r="G1572" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -72945,8 +72767,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1573" t="inlineStr"/>
-      <c r="F1573" t="inlineStr"/>
       <c r="G1573" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -72993,8 +72813,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1574" t="inlineStr"/>
-      <c r="F1574" t="inlineStr"/>
       <c r="G1574" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -73041,8 +72859,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1575" t="inlineStr"/>
-      <c r="F1575" t="inlineStr"/>
       <c r="G1575" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -73089,8 +72905,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1576" t="inlineStr"/>
-      <c r="F1576" t="inlineStr"/>
       <c r="G1576" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -73137,8 +72951,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1577" t="inlineStr"/>
-      <c r="F1577" t="inlineStr"/>
       <c r="G1577" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -73185,8 +72997,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1578" t="inlineStr"/>
-      <c r="F1578" t="inlineStr"/>
       <c r="G1578" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -73233,8 +73043,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1579" t="inlineStr"/>
-      <c r="F1579" t="inlineStr"/>
       <c r="G1579" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -73281,8 +73089,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1580" t="inlineStr"/>
-      <c r="F1580" t="inlineStr"/>
       <c r="G1580" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -73329,8 +73135,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1581" t="inlineStr"/>
-      <c r="F1581" t="inlineStr"/>
       <c r="G1581" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -73377,8 +73181,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1582" t="inlineStr"/>
-      <c r="F1582" t="inlineStr"/>
       <c r="G1582" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -73425,8 +73227,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1583" t="inlineStr"/>
-      <c r="F1583" t="inlineStr"/>
       <c r="G1583" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -73473,8 +73273,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1584" t="inlineStr"/>
-      <c r="F1584" t="inlineStr"/>
       <c r="G1584" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -73521,8 +73319,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1585" t="inlineStr"/>
-      <c r="F1585" t="inlineStr"/>
       <c r="G1585" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -73569,8 +73365,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1586" t="inlineStr"/>
-      <c r="F1586" t="inlineStr"/>
       <c r="G1586" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -73617,8 +73411,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1587" t="inlineStr"/>
-      <c r="F1587" t="inlineStr"/>
       <c r="G1587" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -73665,8 +73457,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1588" t="inlineStr"/>
-      <c r="F1588" t="inlineStr"/>
       <c r="G1588" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -73687,6 +73477,390 @@
         <v>0</v>
       </c>
       <c r="L1588" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1589">
+      <c r="A1589" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B1589" t="inlineStr">
+        <is>
+          <t>New Caledonia vs Solomon Islands</t>
+        </is>
+      </c>
+      <c r="C1589" t="inlineStr">
+        <is>
+          <t>New Caledonia</t>
+        </is>
+      </c>
+      <c r="D1589" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1589" t="inlineStr"/>
+      <c r="F1589" t="inlineStr"/>
+      <c r="G1589" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1589" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1589" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1589" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1589" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1589" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1590">
+      <c r="A1590" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B1590" t="inlineStr">
+        <is>
+          <t>Fiji vs Vanuatu</t>
+        </is>
+      </c>
+      <c r="C1590" t="inlineStr">
+        <is>
+          <t>Fiji</t>
+        </is>
+      </c>
+      <c r="D1590" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1590" t="inlineStr"/>
+      <c r="F1590" t="inlineStr"/>
+      <c r="G1590" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1590" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1590" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1590" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1590" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1590" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1591">
+      <c r="A1591" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B1591" t="inlineStr">
+        <is>
+          <t>Tristán Suárez vs Atlanta</t>
+        </is>
+      </c>
+      <c r="C1591" t="inlineStr">
+        <is>
+          <t>Tristán Suárez</t>
+        </is>
+      </c>
+      <c r="D1591" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1591" t="inlineStr"/>
+      <c r="F1591" t="inlineStr"/>
+      <c r="G1591" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1591" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1591" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1591" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1591" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1591" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1592">
+      <c r="A1592" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B1592" t="inlineStr">
+        <is>
+          <t>Barracas Central vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="C1592" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="D1592" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1592" t="inlineStr"/>
+      <c r="F1592" t="inlineStr"/>
+      <c r="G1592" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1592" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1592" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1592" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1592" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1592" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1593">
+      <c r="A1593" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B1593" t="inlineStr">
+        <is>
+          <t>Nueva Chicago vs Patronato</t>
+        </is>
+      </c>
+      <c r="C1593" t="inlineStr">
+        <is>
+          <t>Nueva Chicago</t>
+        </is>
+      </c>
+      <c r="D1593" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1593" t="inlineStr"/>
+      <c r="F1593" t="inlineStr"/>
+      <c r="G1593" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1593" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1593" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1593" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1593" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1593" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1594">
+      <c r="A1594" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B1594" t="inlineStr">
+        <is>
+          <t>Guabirá vs San Antonio Bulo Bulo</t>
+        </is>
+      </c>
+      <c r="C1594" t="inlineStr">
+        <is>
+          <t>Guabirá</t>
+        </is>
+      </c>
+      <c r="D1594" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1594" t="inlineStr"/>
+      <c r="F1594" t="inlineStr"/>
+      <c r="G1594" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1594" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1594" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1594" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1594" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1594" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1595">
+      <c r="A1595" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B1595" t="inlineStr">
+        <is>
+          <t>Lanús vs Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="C1595" t="inlineStr">
+        <is>
+          <t>Lanús</t>
+        </is>
+      </c>
+      <c r="D1595" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1595" t="inlineStr"/>
+      <c r="F1595" t="inlineStr"/>
+      <c r="G1595" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1595" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1595" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1595" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1595" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1595" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1596">
+      <c r="A1596" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B1596" t="inlineStr">
+        <is>
+          <t>Cuiabá vs Náutico</t>
+        </is>
+      </c>
+      <c r="C1596" t="inlineStr">
+        <is>
+          <t>Cuiabá</t>
+        </is>
+      </c>
+      <c r="D1596" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1596" t="inlineStr"/>
+      <c r="F1596" t="inlineStr"/>
+      <c r="G1596" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1596" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1596" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1596" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1596" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1596" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -73703,7 +73877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74150,6 +74324,25 @@
       </c>
       <c r="E24" t="n">
         <v>106</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C25" t="n">
+        <v>6</v>
+      </c>
+      <c r="D25" t="n">
+        <v>75</v>
+      </c>
+      <c r="E25" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -74163,7 +74356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G138"/>
+  <dimension ref="A1:G140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77202,6 +77395,60 @@
         <v>0</v>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>1</v>
+      </c>
+      <c r="D139" t="n">
+        <v>0</v>
+      </c>
+      <c r="E139" t="n">
+        <v>0</v>
+      </c>
+      <c r="F139" t="n">
+        <v>1</v>
+      </c>
+      <c r="G139" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>no_fav_domina</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>1</v>
+      </c>
+      <c r="D140" t="n">
+        <v>0</v>
+      </c>
+      <c r="E140" t="n">
+        <v>0</v>
+      </c>
+      <c r="F140" t="n">
+        <v>1</v>
+      </c>
+      <c r="G140" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-23
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1596"/>
+  <dimension ref="A1:L1637"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -73503,8 +73503,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1589" t="inlineStr"/>
-      <c r="F1589" t="inlineStr"/>
       <c r="G1589" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -73551,8 +73549,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1590" t="inlineStr"/>
-      <c r="F1590" t="inlineStr"/>
       <c r="G1590" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -73599,8 +73595,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1591" t="inlineStr"/>
-      <c r="F1591" t="inlineStr"/>
       <c r="G1591" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -73647,8 +73641,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1592" t="inlineStr"/>
-      <c r="F1592" t="inlineStr"/>
       <c r="G1592" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -73695,8 +73687,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1593" t="inlineStr"/>
-      <c r="F1593" t="inlineStr"/>
       <c r="G1593" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -73743,8 +73733,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1594" t="inlineStr"/>
-      <c r="F1594" t="inlineStr"/>
       <c r="G1594" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -73791,8 +73779,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1595" t="inlineStr"/>
-      <c r="F1595" t="inlineStr"/>
       <c r="G1595" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -73839,8 +73825,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1596" t="inlineStr"/>
-      <c r="F1596" t="inlineStr"/>
       <c r="G1596" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -73861,6 +73845,1974 @@
         <v>0</v>
       </c>
       <c r="L1596" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1597">
+      <c r="A1597" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1597" t="inlineStr">
+        <is>
+          <t>Salford City vs Sheffield Wednesday</t>
+        </is>
+      </c>
+      <c r="C1597" t="inlineStr">
+        <is>
+          <t>Sheffield Wednesday</t>
+        </is>
+      </c>
+      <c r="D1597" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1597" t="inlineStr"/>
+      <c r="F1597" t="inlineStr"/>
+      <c r="G1597" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1597" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1597" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1597" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1597" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1597" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1598">
+      <c r="A1598" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1598" t="inlineStr">
+        <is>
+          <t>Accrington Stanley vs Sunderland U21</t>
+        </is>
+      </c>
+      <c r="C1598" t="inlineStr">
+        <is>
+          <t>Accrington Stanley</t>
+        </is>
+      </c>
+      <c r="D1598" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1598" t="inlineStr"/>
+      <c r="F1598" t="inlineStr"/>
+      <c r="G1598" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H1598" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1598" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1598" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1598" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1598" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1599">
+      <c r="A1599" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1599" t="inlineStr">
+        <is>
+          <t>Wigan Athletic vs Blackpool</t>
+        </is>
+      </c>
+      <c r="C1599" t="inlineStr">
+        <is>
+          <t>Wigan Athletic</t>
+        </is>
+      </c>
+      <c r="D1599" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1599" t="inlineStr"/>
+      <c r="F1599" t="inlineStr"/>
+      <c r="G1599" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1599" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1599" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1599" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1599" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1599" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1600">
+      <c r="A1600" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1600" t="inlineStr">
+        <is>
+          <t>Crewe Alexandra vs Aston Villa U21</t>
+        </is>
+      </c>
+      <c r="C1600" t="inlineStr">
+        <is>
+          <t>Crewe Alexandra</t>
+        </is>
+      </c>
+      <c r="D1600" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1600" t="inlineStr"/>
+      <c r="F1600" t="inlineStr"/>
+      <c r="G1600" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H1600" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1600" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1600" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1600" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1600" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1601">
+      <c r="A1601" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1601" t="inlineStr">
+        <is>
+          <t>York City vs Rotherham United</t>
+        </is>
+      </c>
+      <c r="C1601" t="inlineStr">
+        <is>
+          <t>York City</t>
+        </is>
+      </c>
+      <c r="D1601" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1601" t="inlineStr"/>
+      <c r="F1601" t="inlineStr"/>
+      <c r="G1601" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1601" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1601" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1601" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1601" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1601" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1602">
+      <c r="A1602" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1602" t="inlineStr">
+        <is>
+          <t>Chesterfield vs Port Vale</t>
+        </is>
+      </c>
+      <c r="C1602" t="inlineStr">
+        <is>
+          <t>Chesterfield</t>
+        </is>
+      </c>
+      <c r="D1602" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1602" t="inlineStr"/>
+      <c r="F1602" t="inlineStr"/>
+      <c r="G1602" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1602" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1602" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1602" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1602" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1602" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1603">
+      <c r="A1603" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1603" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Shrewsbury Town</t>
+        </is>
+      </c>
+      <c r="C1603" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="D1603" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1603" t="inlineStr"/>
+      <c r="F1603" t="inlineStr"/>
+      <c r="G1603" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1603" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1603" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1603" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1603" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1603" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1604">
+      <c r="A1604" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1604" t="inlineStr">
+        <is>
+          <t>Burton Albion vs Nottingham Forest U21</t>
+        </is>
+      </c>
+      <c r="C1604" t="inlineStr">
+        <is>
+          <t>Burton Albion</t>
+        </is>
+      </c>
+      <c r="D1604" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1604" t="inlineStr"/>
+      <c r="F1604" t="inlineStr"/>
+      <c r="G1604" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1604" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1604" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1604" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1604" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1604" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1605">
+      <c r="A1605" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1605" t="inlineStr">
+        <is>
+          <t>Notts County vs Grimsby Town</t>
+        </is>
+      </c>
+      <c r="C1605" t="inlineStr">
+        <is>
+          <t>Notts County</t>
+        </is>
+      </c>
+      <c r="D1605" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1605" t="inlineStr"/>
+      <c r="F1605" t="inlineStr"/>
+      <c r="G1605" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1605" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1605" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1605" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1605" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1605" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1606">
+      <c r="A1606" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1606" t="inlineStr">
+        <is>
+          <t>Barnsley vs Leeds United U21</t>
+        </is>
+      </c>
+      <c r="C1606" t="inlineStr">
+        <is>
+          <t>Barnsley</t>
+        </is>
+      </c>
+      <c r="D1606" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1606" t="inlineStr"/>
+      <c r="F1606" t="inlineStr"/>
+      <c r="G1606" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H1606" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1606" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1606" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1606" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1606" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1607">
+      <c r="A1607" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1607" t="inlineStr">
+        <is>
+          <t>ACV vs Hoogeveen</t>
+        </is>
+      </c>
+      <c r="C1607" t="inlineStr">
+        <is>
+          <t>ACV</t>
+        </is>
+      </c>
+      <c r="D1607" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1607" t="inlineStr"/>
+      <c r="F1607" t="inlineStr"/>
+      <c r="G1607" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1607" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1607" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1607" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1607" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1607" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1608">
+      <c r="A1608" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1608" t="inlineStr">
+        <is>
+          <t>Eemdijk vs RBC Roosendaal</t>
+        </is>
+      </c>
+      <c r="C1608" t="inlineStr">
+        <is>
+          <t>RBC Roosendaal</t>
+        </is>
+      </c>
+      <c r="D1608" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1608" t="inlineStr"/>
+      <c r="F1608" t="inlineStr"/>
+      <c r="G1608" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1608" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1608" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1608" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1608" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1608" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1609">
+      <c r="A1609" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1609" t="inlineStr">
+        <is>
+          <t>EVV Echt vs RKSV Halsteren</t>
+        </is>
+      </c>
+      <c r="C1609" t="inlineStr">
+        <is>
+          <t>EVV Echt</t>
+        </is>
+      </c>
+      <c r="D1609" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1609" t="inlineStr"/>
+      <c r="F1609" t="inlineStr"/>
+      <c r="G1609" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1609" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1609" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1609" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1609" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1609" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1610">
+      <c r="A1610" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1610" t="inlineStr">
+        <is>
+          <t>GVVV vs DVS '33 Ermelo</t>
+        </is>
+      </c>
+      <c r="C1610" t="inlineStr">
+        <is>
+          <t>GVVV</t>
+        </is>
+      </c>
+      <c r="D1610" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1610" t="inlineStr"/>
+      <c r="F1610" t="inlineStr"/>
+      <c r="G1610" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H1610" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1610" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1610" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1610" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1610" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1611">
+      <c r="A1611" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1611" t="inlineStr">
+        <is>
+          <t>HHC Hardenberg vs BVV Barendrecht</t>
+        </is>
+      </c>
+      <c r="C1611" t="inlineStr">
+        <is>
+          <t>HHC Hardenberg</t>
+        </is>
+      </c>
+      <c r="D1611" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1611" t="inlineStr"/>
+      <c r="F1611" t="inlineStr"/>
+      <c r="G1611" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1611" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1611" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1611" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1611" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1611" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1612">
+      <c r="A1612" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1612" t="inlineStr">
+        <is>
+          <t>Koninklijke HFC vs DOVO</t>
+        </is>
+      </c>
+      <c r="C1612" t="inlineStr">
+        <is>
+          <t>Koninklijke HFC</t>
+        </is>
+      </c>
+      <c r="D1612" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1612" t="inlineStr"/>
+      <c r="F1612" t="inlineStr"/>
+      <c r="G1612" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1612" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1612" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1612" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1612" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1612" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1613">
+      <c r="A1613" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1613" t="inlineStr">
+        <is>
+          <t>FC Rijnvogels vs VVSB</t>
+        </is>
+      </c>
+      <c r="C1613" t="inlineStr">
+        <is>
+          <t>FC Rijnvogels</t>
+        </is>
+      </c>
+      <c r="D1613" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1613" t="inlineStr"/>
+      <c r="F1613" t="inlineStr"/>
+      <c r="G1613" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1613" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1613" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1613" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1613" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1613" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1614">
+      <c r="A1614" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1614" t="inlineStr">
+        <is>
+          <t>RKAV Volendam vs Spakenburg</t>
+        </is>
+      </c>
+      <c r="C1614" t="inlineStr">
+        <is>
+          <t>Spakenburg</t>
+        </is>
+      </c>
+      <c r="D1614" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1614" t="inlineStr"/>
+      <c r="F1614" t="inlineStr"/>
+      <c r="G1614" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H1614" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1614" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1614" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1614" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1614" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1615">
+      <c r="A1615" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1615" t="inlineStr">
+        <is>
+          <t>Sportlust '46 vs Excelsior Maassluis</t>
+        </is>
+      </c>
+      <c r="C1615" t="inlineStr">
+        <is>
+          <t>Excelsior Maassluis</t>
+        </is>
+      </c>
+      <c r="D1615" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1615" t="inlineStr"/>
+      <c r="F1615" t="inlineStr"/>
+      <c r="G1615" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1615" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1615" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1615" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1615" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1615" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1616">
+      <c r="A1616" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1616" t="inlineStr">
+        <is>
+          <t>Bradford City vs Newcastle United U21</t>
+        </is>
+      </c>
+      <c r="C1616" t="inlineStr">
+        <is>
+          <t>Bradford City</t>
+        </is>
+      </c>
+      <c r="D1616" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1616" t="inlineStr"/>
+      <c r="F1616" t="inlineStr"/>
+      <c r="G1616" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1616" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1616" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1616" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1616" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1616" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1617">
+      <c r="A1617" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1617" t="inlineStr">
+        <is>
+          <t>Clachnacuddin vs Ross County</t>
+        </is>
+      </c>
+      <c r="C1617" t="inlineStr">
+        <is>
+          <t>Ross County</t>
+        </is>
+      </c>
+      <c r="D1617" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1617" t="inlineStr"/>
+      <c r="F1617" t="inlineStr"/>
+      <c r="G1617" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
+      <c r="H1617" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1617" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1617" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1617" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1617" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1618">
+      <c r="A1618" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1618" t="inlineStr">
+        <is>
+          <t>East Kilbride vs Celtic B</t>
+        </is>
+      </c>
+      <c r="C1618" t="inlineStr">
+        <is>
+          <t>East Kilbride</t>
+        </is>
+      </c>
+      <c r="D1618" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1618" t="inlineStr"/>
+      <c r="F1618" t="inlineStr"/>
+      <c r="G1618" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H1618" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1618" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1618" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1618" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1618" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1619">
+      <c r="A1619" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1619" t="inlineStr">
+        <is>
+          <t>Edinburgh City vs Dundee United B</t>
+        </is>
+      </c>
+      <c r="C1619" t="inlineStr">
+        <is>
+          <t>Edinburgh City</t>
+        </is>
+      </c>
+      <c r="D1619" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1619" t="inlineStr"/>
+      <c r="F1619" t="inlineStr"/>
+      <c r="G1619" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1619" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1619" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1619" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1619" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1619" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1620">
+      <c r="A1620" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1620" t="inlineStr">
+        <is>
+          <t>Elgin City vs Dundee B</t>
+        </is>
+      </c>
+      <c r="C1620" t="inlineStr">
+        <is>
+          <t>Elgin City</t>
+        </is>
+      </c>
+      <c r="D1620" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1620" t="inlineStr"/>
+      <c r="F1620" t="inlineStr"/>
+      <c r="G1620" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1620" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1620" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1620" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1620" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1620" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1621">
+      <c r="A1621" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1621" t="inlineStr">
+        <is>
+          <t>Forfar Athletic vs Peterhead</t>
+        </is>
+      </c>
+      <c r="C1621" t="inlineStr">
+        <is>
+          <t>Peterhead</t>
+        </is>
+      </c>
+      <c r="D1621" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1621" t="inlineStr"/>
+      <c r="F1621" t="inlineStr"/>
+      <c r="G1621" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1621" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1621" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1621" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1621" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1621" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1622">
+      <c r="A1622" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1622" t="inlineStr">
+        <is>
+          <t>Formartine United vs Montrose</t>
+        </is>
+      </c>
+      <c r="C1622" t="inlineStr">
+        <is>
+          <t>Montrose</t>
+        </is>
+      </c>
+      <c r="D1622" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1622" t="inlineStr"/>
+      <c r="F1622" t="inlineStr"/>
+      <c r="G1622" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1622" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1622" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1622" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1622" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1622" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1623">
+      <c r="A1623" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1623" t="inlineStr">
+        <is>
+          <t>Fraserburgh vs Cove Rangers</t>
+        </is>
+      </c>
+      <c r="C1623" t="inlineStr">
+        <is>
+          <t>Cove Rangers</t>
+        </is>
+      </c>
+      <c r="D1623" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1623" t="inlineStr"/>
+      <c r="F1623" t="inlineStr"/>
+      <c r="G1623" t="inlineStr">
+        <is>
+          <t>0-5</t>
+        </is>
+      </c>
+      <c r="H1623" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1623" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1623" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1623" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1623" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1624">
+      <c r="A1624" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1624" t="inlineStr">
+        <is>
+          <t>Gala Fairydean vs Spartans FC</t>
+        </is>
+      </c>
+      <c r="C1624" t="inlineStr">
+        <is>
+          <t>Spartans FC</t>
+        </is>
+      </c>
+      <c r="D1624" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1624" t="inlineStr"/>
+      <c r="F1624" t="inlineStr"/>
+      <c r="G1624" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1624" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1624" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1624" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1624" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1624" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1625">
+      <c r="A1625" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1625" t="inlineStr">
+        <is>
+          <t>Dagenham &amp; Redbridge vs Waltham Abbey</t>
+        </is>
+      </c>
+      <c r="C1625" t="inlineStr">
+        <is>
+          <t>Dagenham &amp; Redbridge</t>
+        </is>
+      </c>
+      <c r="D1625" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1625" t="inlineStr"/>
+      <c r="F1625" t="inlineStr"/>
+      <c r="G1625" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1625" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1625" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1625" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1625" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1625" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1626">
+      <c r="A1626" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1626" t="inlineStr">
+        <is>
+          <t>Gainsborough Trinity vs Leamington</t>
+        </is>
+      </c>
+      <c r="C1626" t="inlineStr">
+        <is>
+          <t>Gainsborough Trinity</t>
+        </is>
+      </c>
+      <c r="D1626" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1626" t="inlineStr"/>
+      <c r="F1626" t="inlineStr"/>
+      <c r="G1626" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1626" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1626" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1626" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1626" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1626" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1627">
+      <c r="A1627" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1627" t="inlineStr">
+        <is>
+          <t>Truro City vs Merthyr Town</t>
+        </is>
+      </c>
+      <c r="C1627" t="inlineStr">
+        <is>
+          <t>Truro City</t>
+        </is>
+      </c>
+      <c r="D1627" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1627" t="inlineStr"/>
+      <c r="F1627" t="inlineStr"/>
+      <c r="G1627" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1627" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1627" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1627" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1627" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1627" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1628">
+      <c r="A1628" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1628" t="inlineStr">
+        <is>
+          <t>Worksop Town vs AFC Telford United</t>
+        </is>
+      </c>
+      <c r="C1628" t="inlineStr">
+        <is>
+          <t>Worksop Town</t>
+        </is>
+      </c>
+      <c r="D1628" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1628" t="inlineStr"/>
+      <c r="F1628" t="inlineStr"/>
+      <c r="G1628" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H1628" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1628" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1628" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1628" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1628" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1629">
+      <c r="A1629" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1629" t="inlineStr">
+        <is>
+          <t>Alloa Athletic vs Hibernian B</t>
+        </is>
+      </c>
+      <c r="C1629" t="inlineStr">
+        <is>
+          <t>Alloa Athletic</t>
+        </is>
+      </c>
+      <c r="D1629" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1629" t="inlineStr"/>
+      <c r="F1629" t="inlineStr"/>
+      <c r="G1629" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H1629" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1629" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1629" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1629" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1629" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1630">
+      <c r="A1630" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1630" t="inlineStr">
+        <is>
+          <t>Berwick Rangers vs Stranraer</t>
+        </is>
+      </c>
+      <c r="C1630" t="inlineStr">
+        <is>
+          <t>Stranraer</t>
+        </is>
+      </c>
+      <c r="D1630" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1630" t="inlineStr"/>
+      <c r="F1630" t="inlineStr"/>
+      <c r="G1630" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1630" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1630" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1630" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1630" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1630" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1631">
+      <c r="A1631" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1631" t="inlineStr">
+        <is>
+          <t>Dumbarton vs Kilmarnock B</t>
+        </is>
+      </c>
+      <c r="C1631" t="inlineStr">
+        <is>
+          <t>Dumbarton</t>
+        </is>
+      </c>
+      <c r="D1631" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1631" t="inlineStr"/>
+      <c r="F1631" t="inlineStr"/>
+      <c r="G1631" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1631" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1631" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1631" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1631" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1631" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1632">
+      <c r="A1632" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1632" t="inlineStr">
+        <is>
+          <t>Puerto Montt vs Ñublense</t>
+        </is>
+      </c>
+      <c r="C1632" t="inlineStr">
+        <is>
+          <t>Ñublense</t>
+        </is>
+      </c>
+      <c r="D1632" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1632" t="inlineStr"/>
+      <c r="F1632" t="inlineStr"/>
+      <c r="G1632" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1632" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1632" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1632" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1632" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1632" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1633">
+      <c r="A1633" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1633" t="inlineStr">
+        <is>
+          <t>Independiente Medellín vs Jaguares de Córdoba</t>
+        </is>
+      </c>
+      <c r="C1633" t="inlineStr">
+        <is>
+          <t>Independiente Medellín</t>
+        </is>
+      </c>
+      <c r="D1633" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1633" t="inlineStr"/>
+      <c r="F1633" t="inlineStr"/>
+      <c r="G1633" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1633" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1633" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1633" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1633" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1633" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1634">
+      <c r="A1634" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1634" t="inlineStr">
+        <is>
+          <t>Nacional Potosí vs Real Potosí</t>
+        </is>
+      </c>
+      <c r="C1634" t="inlineStr">
+        <is>
+          <t>Nacional Potosí</t>
+        </is>
+      </c>
+      <c r="D1634" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1634" t="inlineStr"/>
+      <c r="F1634" t="inlineStr"/>
+      <c r="G1634" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1634" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1634" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1634" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1634" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1634" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1635">
+      <c r="A1635" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1635" t="inlineStr">
+        <is>
+          <t>Audax Italiano vs Colo Colo</t>
+        </is>
+      </c>
+      <c r="C1635" t="inlineStr">
+        <is>
+          <t>Colo Colo</t>
+        </is>
+      </c>
+      <c r="D1635" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1635" t="inlineStr"/>
+      <c r="F1635" t="inlineStr"/>
+      <c r="G1635" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1635" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1635" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1635" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1635" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1635" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1636">
+      <c r="A1636" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1636" t="inlineStr">
+        <is>
+          <t>Cobreloa vs Coquimbo Unido</t>
+        </is>
+      </c>
+      <c r="C1636" t="inlineStr">
+        <is>
+          <t>Coquimbo Unido</t>
+        </is>
+      </c>
+      <c r="D1636" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1636" t="inlineStr"/>
+      <c r="F1636" t="inlineStr"/>
+      <c r="G1636" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1636" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1636" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1636" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1636" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1636" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1637">
+      <c r="A1637" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B1637" t="inlineStr">
+        <is>
+          <t>Independiente Santa Fe vs Deportivo Cali</t>
+        </is>
+      </c>
+      <c r="C1637" t="inlineStr">
+        <is>
+          <t>Independiente Santa Fe</t>
+        </is>
+      </c>
+      <c r="D1637" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1637" t="inlineStr"/>
+      <c r="F1637" t="inlineStr"/>
+      <c r="G1637" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1637" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1637" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1637" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1637" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1637" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -73877,7 +75829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74343,6 +76295,25 @@
       </c>
       <c r="E25" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>41</v>
+      </c>
+      <c r="C26" t="n">
+        <v>28</v>
+      </c>
+      <c r="D26" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="E26" t="n">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -74356,7 +76327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77449,6 +79420,273 @@
         <v>0</v>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>3</v>
+      </c>
+      <c r="D141" t="n">
+        <v>0</v>
+      </c>
+      <c r="E141" t="n">
+        <v>0</v>
+      </c>
+      <c r="F141" t="n">
+        <v>3</v>
+      </c>
+      <c r="G141" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>no_fav_domina</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>3</v>
+      </c>
+      <c r="D142" t="n">
+        <v>2</v>
+      </c>
+      <c r="E142" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F142" t="n">
+        <v>1</v>
+      </c>
+      <c r="G142" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>siguen_empatados_22</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>1</v>
+      </c>
+      <c r="D143" t="n">
+        <v>0</v>
+      </c>
+      <c r="E143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G143" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>siguen_empatados_70</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>1</v>
+      </c>
+      <c r="D144" t="n">
+        <v>0</v>
+      </c>
+      <c r="E144" t="n">
+        <v>0</v>
+      </c>
+      <c r="F144" t="n">
+        <v>1</v>
+      </c>
+      <c r="G144" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>4</v>
+      </c>
+      <c r="D145" t="n">
+        <v>2</v>
+      </c>
+      <c r="E145" t="n">
+        <v>50</v>
+      </c>
+      <c r="F145" t="n">
+        <v>2</v>
+      </c>
+      <c r="G145" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>4</v>
+      </c>
+      <c r="D146" t="n">
+        <v>1</v>
+      </c>
+      <c r="E146" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="F146" t="n">
+        <v>2</v>
+      </c>
+      <c r="G146" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>fav_domina_no_gana</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>2</v>
+      </c>
+      <c r="D147" t="n">
+        <v>1</v>
+      </c>
+      <c r="E147" t="n">
+        <v>50</v>
+      </c>
+      <c r="F147" t="n">
+        <v>1</v>
+      </c>
+      <c r="G147" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>2</v>
+      </c>
+      <c r="D148" t="n">
+        <v>0</v>
+      </c>
+      <c r="F148" t="n">
+        <v>0</v>
+      </c>
+      <c r="G148" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>1</v>
+      </c>
+      <c r="D149" t="n">
+        <v>0</v>
+      </c>
+      <c r="E149" t="n">
+        <v>0</v>
+      </c>
+      <c r="F149" t="n">
+        <v>1</v>
+      </c>
+      <c r="G149" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>1</v>
+      </c>
+      <c r="D150" t="n">
+        <v>0</v>
+      </c>
+      <c r="E150" t="n">
+        <v>0</v>
+      </c>
+      <c r="F150" t="n">
+        <v>1</v>
+      </c>
+      <c r="G150" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-24
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1637"/>
+  <dimension ref="A1:L1655"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -73871,8 +73871,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1597" t="inlineStr"/>
-      <c r="F1597" t="inlineStr"/>
       <c r="G1597" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -73919,8 +73917,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1598" t="inlineStr"/>
-      <c r="F1598" t="inlineStr"/>
       <c r="G1598" t="inlineStr">
         <is>
           <t>3-3</t>
@@ -73967,8 +73963,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1599" t="inlineStr"/>
-      <c r="F1599" t="inlineStr"/>
       <c r="G1599" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -74015,8 +74009,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1600" t="inlineStr"/>
-      <c r="F1600" t="inlineStr"/>
       <c r="G1600" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -74063,8 +74055,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1601" t="inlineStr"/>
-      <c r="F1601" t="inlineStr"/>
       <c r="G1601" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -74111,8 +74101,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1602" t="inlineStr"/>
-      <c r="F1602" t="inlineStr"/>
       <c r="G1602" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -74159,8 +74147,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1603" t="inlineStr"/>
-      <c r="F1603" t="inlineStr"/>
       <c r="G1603" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -74207,8 +74193,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1604" t="inlineStr"/>
-      <c r="F1604" t="inlineStr"/>
       <c r="G1604" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -74255,8 +74239,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1605" t="inlineStr"/>
-      <c r="F1605" t="inlineStr"/>
       <c r="G1605" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -74303,8 +74285,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1606" t="inlineStr"/>
-      <c r="F1606" t="inlineStr"/>
       <c r="G1606" t="inlineStr">
         <is>
           <t>3-4</t>
@@ -74351,8 +74331,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1607" t="inlineStr"/>
-      <c r="F1607" t="inlineStr"/>
       <c r="G1607" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -74399,8 +74377,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1608" t="inlineStr"/>
-      <c r="F1608" t="inlineStr"/>
       <c r="G1608" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -74447,8 +74423,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1609" t="inlineStr"/>
-      <c r="F1609" t="inlineStr"/>
       <c r="G1609" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -74495,8 +74469,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1610" t="inlineStr"/>
-      <c r="F1610" t="inlineStr"/>
       <c r="G1610" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -74543,8 +74515,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1611" t="inlineStr"/>
-      <c r="F1611" t="inlineStr"/>
       <c r="G1611" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -74591,8 +74561,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1612" t="inlineStr"/>
-      <c r="F1612" t="inlineStr"/>
       <c r="G1612" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -74639,8 +74607,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1613" t="inlineStr"/>
-      <c r="F1613" t="inlineStr"/>
       <c r="G1613" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -74687,8 +74653,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1614" t="inlineStr"/>
-      <c r="F1614" t="inlineStr"/>
       <c r="G1614" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -74735,8 +74699,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1615" t="inlineStr"/>
-      <c r="F1615" t="inlineStr"/>
       <c r="G1615" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -74783,8 +74745,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1616" t="inlineStr"/>
-      <c r="F1616" t="inlineStr"/>
       <c r="G1616" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -74831,8 +74791,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1617" t="inlineStr"/>
-      <c r="F1617" t="inlineStr"/>
       <c r="G1617" t="inlineStr">
         <is>
           <t>1-5</t>
@@ -74879,8 +74837,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1618" t="inlineStr"/>
-      <c r="F1618" t="inlineStr"/>
       <c r="G1618" t="inlineStr">
         <is>
           <t>3-3</t>
@@ -74927,8 +74883,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1619" t="inlineStr"/>
-      <c r="F1619" t="inlineStr"/>
       <c r="G1619" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -74975,8 +74929,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1620" t="inlineStr"/>
-      <c r="F1620" t="inlineStr"/>
       <c r="G1620" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -75023,8 +74975,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1621" t="inlineStr"/>
-      <c r="F1621" t="inlineStr"/>
       <c r="G1621" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -75071,8 +75021,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1622" t="inlineStr"/>
-      <c r="F1622" t="inlineStr"/>
       <c r="G1622" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -75119,8 +75067,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1623" t="inlineStr"/>
-      <c r="F1623" t="inlineStr"/>
       <c r="G1623" t="inlineStr">
         <is>
           <t>0-5</t>
@@ -75167,8 +75113,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1624" t="inlineStr"/>
-      <c r="F1624" t="inlineStr"/>
       <c r="G1624" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -75215,8 +75159,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1625" t="inlineStr"/>
-      <c r="F1625" t="inlineStr"/>
       <c r="G1625" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -75263,8 +75205,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1626" t="inlineStr"/>
-      <c r="F1626" t="inlineStr"/>
       <c r="G1626" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -75311,8 +75251,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1627" t="inlineStr"/>
-      <c r="F1627" t="inlineStr"/>
       <c r="G1627" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -75359,8 +75297,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1628" t="inlineStr"/>
-      <c r="F1628" t="inlineStr"/>
       <c r="G1628" t="inlineStr">
         <is>
           <t>5-2</t>
@@ -75407,8 +75343,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1629" t="inlineStr"/>
-      <c r="F1629" t="inlineStr"/>
       <c r="G1629" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -75455,8 +75389,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1630" t="inlineStr"/>
-      <c r="F1630" t="inlineStr"/>
       <c r="G1630" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -75503,8 +75435,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1631" t="inlineStr"/>
-      <c r="F1631" t="inlineStr"/>
       <c r="G1631" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -75551,8 +75481,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1632" t="inlineStr"/>
-      <c r="F1632" t="inlineStr"/>
       <c r="G1632" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -75599,8 +75527,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1633" t="inlineStr"/>
-      <c r="F1633" t="inlineStr"/>
       <c r="G1633" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -75647,8 +75573,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1634" t="inlineStr"/>
-      <c r="F1634" t="inlineStr"/>
       <c r="G1634" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -75695,8 +75619,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1635" t="inlineStr"/>
-      <c r="F1635" t="inlineStr"/>
       <c r="G1635" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -75743,8 +75665,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1636" t="inlineStr"/>
-      <c r="F1636" t="inlineStr"/>
       <c r="G1636" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -75791,8 +75711,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1637" t="inlineStr"/>
-      <c r="F1637" t="inlineStr"/>
       <c r="G1637" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -75813,6 +75731,870 @@
         <v>0</v>
       </c>
       <c r="L1637" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1638">
+      <c r="A1638" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1638" t="inlineStr">
+        <is>
+          <t>Iraq vs Oman</t>
+        </is>
+      </c>
+      <c r="C1638" t="inlineStr">
+        <is>
+          <t>Iraq</t>
+        </is>
+      </c>
+      <c r="D1638" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1638" t="inlineStr"/>
+      <c r="F1638" t="inlineStr"/>
+      <c r="G1638" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1638" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1638" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1638" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1638" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1638" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1639">
+      <c r="A1639" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1639" t="inlineStr">
+        <is>
+          <t>Birmingham Legion FC vs Brooklyn FC</t>
+        </is>
+      </c>
+      <c r="C1639" t="inlineStr">
+        <is>
+          <t>Birmingham Legion FC</t>
+        </is>
+      </c>
+      <c r="D1639" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1639" t="inlineStr"/>
+      <c r="F1639" t="inlineStr"/>
+      <c r="G1639" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H1639" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1639" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1639" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1639" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1639" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1640">
+      <c r="A1640" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1640" t="inlineStr">
+        <is>
+          <t>Azerbaijan vs Tajikistan</t>
+        </is>
+      </c>
+      <c r="C1640" t="inlineStr">
+        <is>
+          <t>Azerbaijan</t>
+        </is>
+      </c>
+      <c r="D1640" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1640" t="inlineStr"/>
+      <c r="F1640" t="inlineStr"/>
+      <c r="G1640" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1640" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1640" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1640" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1640" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1640" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1641">
+      <c r="A1641" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1641" t="inlineStr">
+        <is>
+          <t>Gibraltar vs Sao Tome and Principe</t>
+        </is>
+      </c>
+      <c r="C1641" t="inlineStr">
+        <is>
+          <t>Gibraltar</t>
+        </is>
+      </c>
+      <c r="D1641" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1641" t="inlineStr"/>
+      <c r="F1641" t="inlineStr"/>
+      <c r="G1641" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1641" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1641" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1641" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1641" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1641" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1642">
+      <c r="A1642" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1642" t="inlineStr">
+        <is>
+          <t>IJsselmeervogels vs Gemert</t>
+        </is>
+      </c>
+      <c r="C1642" t="inlineStr">
+        <is>
+          <t>IJsselmeervogels</t>
+        </is>
+      </c>
+      <c r="D1642" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1642" t="inlineStr"/>
+      <c r="F1642" t="inlineStr"/>
+      <c r="G1642" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H1642" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1642" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1642" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1642" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1642" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1643">
+      <c r="A1643" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1643" t="inlineStr">
+        <is>
+          <t>Zwaluwen '30 vs Purmersteijn</t>
+        </is>
+      </c>
+      <c r="C1643" t="inlineStr">
+        <is>
+          <t>Zwaluwen '30</t>
+        </is>
+      </c>
+      <c r="D1643" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1643" t="inlineStr"/>
+      <c r="F1643" t="inlineStr"/>
+      <c r="G1643" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1643" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1643" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1643" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1643" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1643" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1644">
+      <c r="A1644" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1644" t="inlineStr">
+        <is>
+          <t>Saudi Arabia vs Kuwait</t>
+        </is>
+      </c>
+      <c r="C1644" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="D1644" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1644" t="inlineStr"/>
+      <c r="F1644" t="inlineStr"/>
+      <c r="G1644" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1644" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1644" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1644" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1644" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1644" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1645">
+      <c r="A1645" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1645" t="inlineStr">
+        <is>
+          <t>Hamilton Academical vs Cowdenbeath</t>
+        </is>
+      </c>
+      <c r="C1645" t="inlineStr">
+        <is>
+          <t>Hamilton Academical</t>
+        </is>
+      </c>
+      <c r="D1645" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1645" t="inlineStr"/>
+      <c r="F1645" t="inlineStr"/>
+      <c r="G1645" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1645" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1645" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1645" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1645" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1645" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1646">
+      <c r="A1646" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1646" t="inlineStr">
+        <is>
+          <t>Turks and Caicos Islands vs Montserrat</t>
+        </is>
+      </c>
+      <c r="C1646" t="inlineStr">
+        <is>
+          <t>Montserrat</t>
+        </is>
+      </c>
+      <c r="D1646" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1646" t="inlineStr"/>
+      <c r="F1646" t="inlineStr"/>
+      <c r="G1646" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1646" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1646" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1646" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1646" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1646" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1647">
+      <c r="A1647" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1647" t="inlineStr">
+        <is>
+          <t>ADT vs Cienciano del Cusco</t>
+        </is>
+      </c>
+      <c r="C1647" t="inlineStr">
+        <is>
+          <t>Cienciano del Cusco</t>
+        </is>
+      </c>
+      <c r="D1647" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1647" t="inlineStr"/>
+      <c r="F1647" t="inlineStr"/>
+      <c r="G1647" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1647" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1647" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1647" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1647" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1647" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1648">
+      <c r="A1648" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1648" t="inlineStr">
+        <is>
+          <t>Bahamas vs St. Martin</t>
+        </is>
+      </c>
+      <c r="C1648" t="inlineStr">
+        <is>
+          <t>St. Martin</t>
+        </is>
+      </c>
+      <c r="D1648" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1648" t="inlineStr"/>
+      <c r="F1648" t="inlineStr"/>
+      <c r="G1648" t="inlineStr">
+        <is>
+          <t>0-8</t>
+        </is>
+      </c>
+      <c r="H1648" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1648" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1648" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1648" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1648" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1649" t="inlineStr">
+        <is>
+          <t>Curicó Unido vs Deportes Concepcion</t>
+        </is>
+      </c>
+      <c r="C1649" t="inlineStr">
+        <is>
+          <t>Deportes Concepcion</t>
+        </is>
+      </c>
+      <c r="D1649" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1649" t="inlineStr"/>
+      <c r="F1649" t="inlineStr"/>
+      <c r="G1649" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H1649" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1649" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1649" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1649" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1649" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1650" t="inlineStr">
+        <is>
+          <t>Aruba vs Antigua and Barbuda</t>
+        </is>
+      </c>
+      <c r="C1650" t="inlineStr">
+        <is>
+          <t>Antigua and Barbuda</t>
+        </is>
+      </c>
+      <c r="D1650" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1650" t="inlineStr"/>
+      <c r="F1650" t="inlineStr"/>
+      <c r="G1650" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1650" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1650" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1650" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1650" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1650" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1651">
+      <c r="A1651" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1651" t="inlineStr">
+        <is>
+          <t>América de Cali vs Águilas Doradas</t>
+        </is>
+      </c>
+      <c r="C1651" t="inlineStr">
+        <is>
+          <t>América de Cali</t>
+        </is>
+      </c>
+      <c r="D1651" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1651" t="inlineStr"/>
+      <c r="F1651" t="inlineStr"/>
+      <c r="G1651" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1651" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1651" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1651" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1651" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1651" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1652">
+      <c r="A1652" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1652" t="inlineStr">
+        <is>
+          <t>Luis Ángel Firpo vs Cacahuatique</t>
+        </is>
+      </c>
+      <c r="C1652" t="inlineStr">
+        <is>
+          <t>Luis Ángel Firpo</t>
+        </is>
+      </c>
+      <c r="D1652" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1652" t="inlineStr"/>
+      <c r="F1652" t="inlineStr"/>
+      <c r="G1652" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1652" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1652" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1652" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1652" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1652" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1653">
+      <c r="A1653" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1653" t="inlineStr">
+        <is>
+          <t>Alianza FC vs Fuerte San Francisco</t>
+        </is>
+      </c>
+      <c r="C1653" t="inlineStr">
+        <is>
+          <t>Alianza FC</t>
+        </is>
+      </c>
+      <c r="D1653" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1653" t="inlineStr"/>
+      <c r="F1653" t="inlineStr"/>
+      <c r="G1653" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H1653" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1653" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1653" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1653" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1653" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1654" t="inlineStr">
+        <is>
+          <t>Seattle Sounders FC vs Real Salt Lake</t>
+        </is>
+      </c>
+      <c r="C1654" t="inlineStr">
+        <is>
+          <t>Seattle Sounders FC</t>
+        </is>
+      </c>
+      <c r="D1654" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1654" t="inlineStr"/>
+      <c r="F1654" t="inlineStr"/>
+      <c r="G1654" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1654" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1654" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1654" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1654" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1654" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B1655" t="inlineStr">
+        <is>
+          <t>Xelajú MC vs Antigua GFC</t>
+        </is>
+      </c>
+      <c r="C1655" t="inlineStr">
+        <is>
+          <t>Xelajú MC</t>
+        </is>
+      </c>
+      <c r="D1655" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1655" t="inlineStr"/>
+      <c r="F1655" t="inlineStr"/>
+      <c r="G1655" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H1655" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1655" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1655" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1655" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1655" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -75829,7 +76611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -76314,6 +77096,25 @@
       </c>
       <c r="E26" t="n">
         <v>41</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>18</v>
+      </c>
+      <c r="C27" t="n">
+        <v>11</v>
+      </c>
+      <c r="D27" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -76327,7 +77128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G150"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -79687,6 +80488,114 @@
         <v>0</v>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>1</v>
+      </c>
+      <c r="D151" t="n">
+        <v>1</v>
+      </c>
+      <c r="E151" t="n">
+        <v>100</v>
+      </c>
+      <c r="F151" t="n">
+        <v>0</v>
+      </c>
+      <c r="G151" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>1</v>
+      </c>
+      <c r="D152" t="n">
+        <v>1</v>
+      </c>
+      <c r="E152" t="n">
+        <v>100</v>
+      </c>
+      <c r="F152" t="n">
+        <v>0</v>
+      </c>
+      <c r="G152" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>fav_domina_no_gana</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>2</v>
+      </c>
+      <c r="D153" t="n">
+        <v>2</v>
+      </c>
+      <c r="E153" t="n">
+        <v>100</v>
+      </c>
+      <c r="F153" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>1</v>
+      </c>
+      <c r="D154" t="n">
+        <v>0</v>
+      </c>
+      <c r="E154" t="n">
+        <v>0</v>
+      </c>
+      <c r="F154" t="n">
+        <v>1</v>
+      </c>
+      <c r="G154" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-25
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1655"/>
+  <dimension ref="A1:L1689"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75757,8 +75757,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1638" t="inlineStr"/>
-      <c r="F1638" t="inlineStr"/>
       <c r="G1638" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -75805,8 +75803,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1639" t="inlineStr"/>
-      <c r="F1639" t="inlineStr"/>
       <c r="G1639" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -75853,8 +75849,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1640" t="inlineStr"/>
-      <c r="F1640" t="inlineStr"/>
       <c r="G1640" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -75901,8 +75895,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1641" t="inlineStr"/>
-      <c r="F1641" t="inlineStr"/>
       <c r="G1641" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -75949,8 +75941,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1642" t="inlineStr"/>
-      <c r="F1642" t="inlineStr"/>
       <c r="G1642" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -75997,8 +75987,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1643" t="inlineStr"/>
-      <c r="F1643" t="inlineStr"/>
       <c r="G1643" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -76045,8 +76033,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1644" t="inlineStr"/>
-      <c r="F1644" t="inlineStr"/>
       <c r="G1644" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -76093,8 +76079,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1645" t="inlineStr"/>
-      <c r="F1645" t="inlineStr"/>
       <c r="G1645" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -76141,8 +76125,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1646" t="inlineStr"/>
-      <c r="F1646" t="inlineStr"/>
       <c r="G1646" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -76189,8 +76171,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1647" t="inlineStr"/>
-      <c r="F1647" t="inlineStr"/>
       <c r="G1647" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -76237,8 +76217,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1648" t="inlineStr"/>
-      <c r="F1648" t="inlineStr"/>
       <c r="G1648" t="inlineStr">
         <is>
           <t>0-8</t>
@@ -76285,8 +76263,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1649" t="inlineStr"/>
-      <c r="F1649" t="inlineStr"/>
       <c r="G1649" t="inlineStr">
         <is>
           <t>0-4</t>
@@ -76333,8 +76309,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1650" t="inlineStr"/>
-      <c r="F1650" t="inlineStr"/>
       <c r="G1650" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -76381,8 +76355,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1651" t="inlineStr"/>
-      <c r="F1651" t="inlineStr"/>
       <c r="G1651" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -76429,8 +76401,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1652" t="inlineStr"/>
-      <c r="F1652" t="inlineStr"/>
       <c r="G1652" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -76477,8 +76447,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1653" t="inlineStr"/>
-      <c r="F1653" t="inlineStr"/>
       <c r="G1653" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -76525,8 +76493,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1654" t="inlineStr"/>
-      <c r="F1654" t="inlineStr"/>
       <c r="G1654" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -76573,8 +76539,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1655" t="inlineStr"/>
-      <c r="F1655" t="inlineStr"/>
       <c r="G1655" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -76595,6 +76559,1638 @@
         <v>0</v>
       </c>
       <c r="L1655" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1656">
+      <c r="A1656" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1656" t="inlineStr">
+        <is>
+          <t>Solomon Islands vs Vanuatu</t>
+        </is>
+      </c>
+      <c r="C1656" t="inlineStr">
+        <is>
+          <t>Solomon Islands</t>
+        </is>
+      </c>
+      <c r="D1656" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1656" t="inlineStr"/>
+      <c r="F1656" t="inlineStr"/>
+      <c r="G1656" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H1656" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1656" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1656" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1656" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1656" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1657">
+      <c r="A1657" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1657" t="inlineStr">
+        <is>
+          <t>Papua New Guinea vs New Caledonia</t>
+        </is>
+      </c>
+      <c r="C1657" t="inlineStr">
+        <is>
+          <t>Papua New Guinea</t>
+        </is>
+      </c>
+      <c r="D1657" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1657" t="inlineStr"/>
+      <c r="F1657" t="inlineStr"/>
+      <c r="G1657" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1657" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1657" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1657" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1657" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1657" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1658">
+      <c r="A1658" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1658" t="inlineStr">
+        <is>
+          <t>Palestine vs New Zealand</t>
+        </is>
+      </c>
+      <c r="C1658" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="D1658" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1658" t="inlineStr"/>
+      <c r="F1658" t="inlineStr"/>
+      <c r="G1658" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H1658" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1658" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1658" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1658" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1658" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1659">
+      <c r="A1659" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1659" t="inlineStr">
+        <is>
+          <t>Japan vs Uruguay</t>
+        </is>
+      </c>
+      <c r="C1659" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D1659" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1659" t="inlineStr"/>
+      <c r="F1659" t="inlineStr"/>
+      <c r="G1659" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1659" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1659" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1659" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1659" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1659" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1660">
+      <c r="A1660" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1660" t="inlineStr">
+        <is>
+          <t>South Korea vs Ecuador</t>
+        </is>
+      </c>
+      <c r="C1660" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="D1660" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1660" t="inlineStr"/>
+      <c r="F1660" t="inlineStr"/>
+      <c r="G1660" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1660" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1660" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1660" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1660" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1660" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1661">
+      <c r="A1661" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1661" t="inlineStr">
+        <is>
+          <t>China vs Maldives</t>
+        </is>
+      </c>
+      <c r="C1661" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="D1661" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1661" t="inlineStr"/>
+      <c r="F1661" t="inlineStr"/>
+      <c r="G1661" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1661" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1661" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1661" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1661" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1661" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1662">
+      <c r="A1662" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1662" t="inlineStr">
+        <is>
+          <t>Namibia vs Congo</t>
+        </is>
+      </c>
+      <c r="C1662" t="inlineStr">
+        <is>
+          <t>Namibia</t>
+        </is>
+      </c>
+      <c r="D1662" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1662" t="inlineStr"/>
+      <c r="F1662" t="inlineStr"/>
+      <c r="G1662" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1662" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1662" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1662" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1662" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1662" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1663" t="inlineStr">
+        <is>
+          <t>United Arab Emirates vs Yemen</t>
+        </is>
+      </c>
+      <c r="C1663" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="D1663" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1663" t="inlineStr"/>
+      <c r="F1663" t="inlineStr"/>
+      <c r="G1663" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H1663" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1663" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1663" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1663" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1663" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1664">
+      <c r="A1664" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1664" t="inlineStr">
+        <is>
+          <t>Andorra vs Malta</t>
+        </is>
+      </c>
+      <c r="C1664" t="inlineStr">
+        <is>
+          <t>Malta</t>
+        </is>
+      </c>
+      <c r="D1664" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1664" t="inlineStr"/>
+      <c r="F1664" t="inlineStr"/>
+      <c r="G1664" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1664" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1664" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1664" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1664" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1664" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1665">
+      <c r="A1665" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1665" t="inlineStr">
+        <is>
+          <t>Congo DR vs Equatorial Guinea</t>
+        </is>
+      </c>
+      <c r="C1665" t="inlineStr">
+        <is>
+          <t>Congo DR</t>
+        </is>
+      </c>
+      <c r="D1665" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1665" t="inlineStr"/>
+      <c r="F1665" t="inlineStr"/>
+      <c r="G1665" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1665" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1665" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1665" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1665" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1665" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1666">
+      <c r="A1666" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1666" t="inlineStr">
+        <is>
+          <t>Libya vs Botswana</t>
+        </is>
+      </c>
+      <c r="C1666" t="inlineStr">
+        <is>
+          <t>Libya</t>
+        </is>
+      </c>
+      <c r="D1666" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1666" t="inlineStr"/>
+      <c r="F1666" t="inlineStr"/>
+      <c r="G1666" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H1666" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1666" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1666" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1666" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1666" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1667">
+      <c r="A1667" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1667" t="inlineStr">
+        <is>
+          <t>Mauritania vs Central African Republic</t>
+        </is>
+      </c>
+      <c r="C1667" t="inlineStr">
+        <is>
+          <t>Mauritania</t>
+        </is>
+      </c>
+      <c r="D1667" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1667" t="inlineStr"/>
+      <c r="F1667" t="inlineStr"/>
+      <c r="G1667" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1667" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1667" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1667" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1667" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1667" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1668">
+      <c r="A1668" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1668" t="inlineStr">
+        <is>
+          <t>Belgium U21 vs Belarus U21</t>
+        </is>
+      </c>
+      <c r="C1668" t="inlineStr">
+        <is>
+          <t>Belgium U21</t>
+        </is>
+      </c>
+      <c r="D1668" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1668" t="inlineStr"/>
+      <c r="F1668" t="inlineStr"/>
+      <c r="G1668" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1668" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1668" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1668" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1668" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1668" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1669">
+      <c r="A1669" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1669" t="inlineStr">
+        <is>
+          <t>Qatar vs Bahrain</t>
+        </is>
+      </c>
+      <c r="C1669" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="D1669" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1669" t="inlineStr"/>
+      <c r="F1669" t="inlineStr"/>
+      <c r="G1669" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1669" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1669" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1669" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1669" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1669" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1670">
+      <c r="A1670" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1670" t="inlineStr">
+        <is>
+          <t>San Marino U21 vs Kosovo U21</t>
+        </is>
+      </c>
+      <c r="C1670" t="inlineStr">
+        <is>
+          <t>Kosovo U21</t>
+        </is>
+      </c>
+      <c r="D1670" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1670" t="inlineStr"/>
+      <c r="F1670" t="inlineStr"/>
+      <c r="G1670" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H1670" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1670" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1670" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1670" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1670" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1671">
+      <c r="A1671" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1671" t="inlineStr">
+        <is>
+          <t>Austria vs Israel</t>
+        </is>
+      </c>
+      <c r="C1671" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="D1671" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1671" t="inlineStr"/>
+      <c r="F1671" t="inlineStr"/>
+      <c r="G1671" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1671" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1671" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1671" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1671" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1671" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1672">
+      <c r="A1672" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1672" t="inlineStr">
+        <is>
+          <t>Netherlands vs Germany</t>
+        </is>
+      </c>
+      <c r="C1672" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="D1672" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1672" t="inlineStr"/>
+      <c r="F1672" t="inlineStr"/>
+      <c r="G1672" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1672" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1672" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1672" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1672" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1672" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1673">
+      <c r="A1673" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1673" t="inlineStr">
+        <is>
+          <t>Portugal vs Wales</t>
+        </is>
+      </c>
+      <c r="C1673" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D1673" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1673" t="inlineStr"/>
+      <c r="F1673" t="inlineStr"/>
+      <c r="G1673" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1673" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1673" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1673" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1673" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1673" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1674">
+      <c r="A1674" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1674" t="inlineStr">
+        <is>
+          <t>Norway vs Denmark</t>
+        </is>
+      </c>
+      <c r="C1674" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="D1674" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1674" t="inlineStr"/>
+      <c r="F1674" t="inlineStr"/>
+      <c r="G1674" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1674" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1674" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1674" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1674" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1674" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1675">
+      <c r="A1675" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1675" t="inlineStr">
+        <is>
+          <t>Kosovo vs Republic of Ireland</t>
+        </is>
+      </c>
+      <c r="C1675" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+      <c r="D1675" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1675" t="inlineStr"/>
+      <c r="F1675" t="inlineStr"/>
+      <c r="G1675" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1675" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1675" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1675" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1675" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1675" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1676">
+      <c r="A1676" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1676" t="inlineStr">
+        <is>
+          <t>Liechtenstein vs Lithuania</t>
+        </is>
+      </c>
+      <c r="C1676" t="inlineStr">
+        <is>
+          <t>Lithuania</t>
+        </is>
+      </c>
+      <c r="D1676" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1676" t="inlineStr"/>
+      <c r="F1676" t="inlineStr"/>
+      <c r="G1676" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1676" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1676" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1676" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1676" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1676" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1677">
+      <c r="A1677" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1677" t="inlineStr">
+        <is>
+          <t>Tunisia vs Uganda</t>
+        </is>
+      </c>
+      <c r="C1677" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="D1677" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1677" t="inlineStr"/>
+      <c r="F1677" t="inlineStr"/>
+      <c r="G1677" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1677" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1677" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1677" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1677" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1677" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1678">
+      <c r="A1678" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1678" t="inlineStr">
+        <is>
+          <t>Sierra Leone vs Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C1678" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="D1678" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1678" t="inlineStr"/>
+      <c r="F1678" t="inlineStr"/>
+      <c r="G1678" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H1678" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1678" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1678" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1678" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1678" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1679">
+      <c r="A1679" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1679" t="inlineStr">
+        <is>
+          <t>Cameroon vs Comoros</t>
+        </is>
+      </c>
+      <c r="C1679" t="inlineStr">
+        <is>
+          <t>Cameroon</t>
+        </is>
+      </c>
+      <c r="D1679" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1679" t="inlineStr"/>
+      <c r="F1679" t="inlineStr"/>
+      <c r="G1679" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1679" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1679" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1679" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1679" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1679" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1680">
+      <c r="A1680" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1680" t="inlineStr">
+        <is>
+          <t>Ivory Coast vs Ghana</t>
+        </is>
+      </c>
+      <c r="C1680" t="inlineStr">
+        <is>
+          <t>Ivory Coast</t>
+        </is>
+      </c>
+      <c r="D1680" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1680" t="inlineStr"/>
+      <c r="F1680" t="inlineStr"/>
+      <c r="G1680" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1680" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1680" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1680" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1680" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1680" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1681">
+      <c r="A1681" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1681" t="inlineStr">
+        <is>
+          <t>Puerto Rico vs Guyana</t>
+        </is>
+      </c>
+      <c r="C1681" t="inlineStr">
+        <is>
+          <t>Guyana</t>
+        </is>
+      </c>
+      <c r="D1681" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1681" t="inlineStr"/>
+      <c r="F1681" t="inlineStr"/>
+      <c r="G1681" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1681" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1681" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1681" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1681" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1681" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1682">
+      <c r="A1682" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1682" t="inlineStr">
+        <is>
+          <t>O'Higgins vs Deportes Santa Cruz</t>
+        </is>
+      </c>
+      <c r="C1682" t="inlineStr">
+        <is>
+          <t>O'Higgins</t>
+        </is>
+      </c>
+      <c r="D1682" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1682" t="inlineStr"/>
+      <c r="F1682" t="inlineStr"/>
+      <c r="G1682" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1682" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1682" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1682" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1682" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1682" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1683">
+      <c r="A1683" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1683" t="inlineStr">
+        <is>
+          <t>Dominican Republic vs Nicaragua</t>
+        </is>
+      </c>
+      <c r="C1683" t="inlineStr">
+        <is>
+          <t>Dominican Republic</t>
+        </is>
+      </c>
+      <c r="D1683" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1683" t="inlineStr"/>
+      <c r="F1683" t="inlineStr"/>
+      <c r="G1683" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1683" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1683" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1683" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1683" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1683" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1684">
+      <c r="A1684" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1684" t="inlineStr">
+        <is>
+          <t>Cayman Islands vs Dominica</t>
+        </is>
+      </c>
+      <c r="C1684" t="inlineStr">
+        <is>
+          <t>Dominica</t>
+        </is>
+      </c>
+      <c r="D1684" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1684" t="inlineStr"/>
+      <c r="F1684" t="inlineStr"/>
+      <c r="G1684" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1684" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1684" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1684" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1684" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1684" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1685">
+      <c r="A1685" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1685" t="inlineStr">
+        <is>
+          <t>Haiti vs Trinidad and Tobago</t>
+        </is>
+      </c>
+      <c r="C1685" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+      <c r="D1685" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1685" t="inlineStr"/>
+      <c r="F1685" t="inlineStr"/>
+      <c r="G1685" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1685" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1685" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1685" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1685" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1685" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1686">
+      <c r="A1686" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1686" t="inlineStr">
+        <is>
+          <t>Atlético Nacional vs Millonarios</t>
+        </is>
+      </c>
+      <c r="C1686" t="inlineStr">
+        <is>
+          <t>Atlético Nacional</t>
+        </is>
+      </c>
+      <c r="D1686" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1686" t="inlineStr"/>
+      <c r="F1686" t="inlineStr"/>
+      <c r="G1686" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1686" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1686" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1686" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1686" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1686" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1687">
+      <c r="A1687" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1687" t="inlineStr">
+        <is>
+          <t>Mineros de Zacatecas vs Piratas</t>
+        </is>
+      </c>
+      <c r="C1687" t="inlineStr">
+        <is>
+          <t>Piratas</t>
+        </is>
+      </c>
+      <c r="D1687" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1687" t="inlineStr"/>
+      <c r="F1687" t="inlineStr"/>
+      <c r="G1687" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1687" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1687" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1687" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1687" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1687" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1688">
+      <c r="A1688" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1688" t="inlineStr">
+        <is>
+          <t>Municipal vs Suchitepequez</t>
+        </is>
+      </c>
+      <c r="C1688" t="inlineStr">
+        <is>
+          <t>Municipal</t>
+        </is>
+      </c>
+      <c r="D1688" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1688" t="inlineStr"/>
+      <c r="F1688" t="inlineStr"/>
+      <c r="G1688" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1688" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1688" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1688" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1688" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1688" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1689">
+      <c r="A1689" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1689" t="inlineStr">
+        <is>
+          <t>Costa Rica vs Curaçao</t>
+        </is>
+      </c>
+      <c r="C1689" t="inlineStr">
+        <is>
+          <t>Costa Rica</t>
+        </is>
+      </c>
+      <c r="D1689" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1689" t="inlineStr"/>
+      <c r="F1689" t="inlineStr"/>
+      <c r="G1689" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H1689" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1689" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1689" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1689" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1689" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -76611,7 +78207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77115,6 +78711,25 @@
       </c>
       <c r="E27" t="n">
         <v>18</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>34</v>
+      </c>
+      <c r="C28" t="n">
+        <v>28</v>
+      </c>
+      <c r="D28" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="E28" t="n">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -77128,7 +78743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G154"/>
+  <dimension ref="A1:G155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -80596,6 +82211,33 @@
         <v>0</v>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>fav_domina_no_gana</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>1</v>
+      </c>
+      <c r="D155" t="n">
+        <v>0</v>
+      </c>
+      <c r="E155" t="n">
+        <v>0</v>
+      </c>
+      <c r="F155" t="n">
+        <v>1</v>
+      </c>
+      <c r="G155" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-26
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1689"/>
+  <dimension ref="A1:L1750"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -76585,8 +76585,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1656" t="inlineStr"/>
-      <c r="F1656" t="inlineStr"/>
       <c r="G1656" t="inlineStr">
         <is>
           <t>3-3</t>
@@ -76633,8 +76631,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1657" t="inlineStr"/>
-      <c r="F1657" t="inlineStr"/>
       <c r="G1657" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -76681,8 +76677,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1658" t="inlineStr"/>
-      <c r="F1658" t="inlineStr"/>
       <c r="G1658" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -76729,8 +76723,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1659" t="inlineStr"/>
-      <c r="F1659" t="inlineStr"/>
       <c r="G1659" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -76777,8 +76769,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1660" t="inlineStr"/>
-      <c r="F1660" t="inlineStr"/>
       <c r="G1660" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -76825,8 +76815,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1661" t="inlineStr"/>
-      <c r="F1661" t="inlineStr"/>
       <c r="G1661" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -76873,8 +76861,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1662" t="inlineStr"/>
-      <c r="F1662" t="inlineStr"/>
       <c r="G1662" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -76921,8 +76907,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1663" t="inlineStr"/>
-      <c r="F1663" t="inlineStr"/>
       <c r="G1663" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -76969,8 +76953,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1664" t="inlineStr"/>
-      <c r="F1664" t="inlineStr"/>
       <c r="G1664" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -77017,8 +76999,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1665" t="inlineStr"/>
-      <c r="F1665" t="inlineStr"/>
       <c r="G1665" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -77065,8 +77045,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1666" t="inlineStr"/>
-      <c r="F1666" t="inlineStr"/>
       <c r="G1666" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -77113,8 +77091,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1667" t="inlineStr"/>
-      <c r="F1667" t="inlineStr"/>
       <c r="G1667" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -77161,8 +77137,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1668" t="inlineStr"/>
-      <c r="F1668" t="inlineStr"/>
       <c r="G1668" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -77209,8 +77183,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1669" t="inlineStr"/>
-      <c r="F1669" t="inlineStr"/>
       <c r="G1669" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -77257,8 +77229,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1670" t="inlineStr"/>
-      <c r="F1670" t="inlineStr"/>
       <c r="G1670" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -77305,8 +77275,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1671" t="inlineStr"/>
-      <c r="F1671" t="inlineStr"/>
       <c r="G1671" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -77353,8 +77321,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1672" t="inlineStr"/>
-      <c r="F1672" t="inlineStr"/>
       <c r="G1672" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -77401,8 +77367,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1673" t="inlineStr"/>
-      <c r="F1673" t="inlineStr"/>
       <c r="G1673" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -77449,8 +77413,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1674" t="inlineStr"/>
-      <c r="F1674" t="inlineStr"/>
       <c r="G1674" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -77497,8 +77459,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1675" t="inlineStr"/>
-      <c r="F1675" t="inlineStr"/>
       <c r="G1675" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -77545,8 +77505,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1676" t="inlineStr"/>
-      <c r="F1676" t="inlineStr"/>
       <c r="G1676" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -77593,8 +77551,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1677" t="inlineStr"/>
-      <c r="F1677" t="inlineStr"/>
       <c r="G1677" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -77641,8 +77597,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1678" t="inlineStr"/>
-      <c r="F1678" t="inlineStr"/>
       <c r="G1678" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -77689,8 +77643,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1679" t="inlineStr"/>
-      <c r="F1679" t="inlineStr"/>
       <c r="G1679" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -77737,8 +77689,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1680" t="inlineStr"/>
-      <c r="F1680" t="inlineStr"/>
       <c r="G1680" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -77785,8 +77735,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1681" t="inlineStr"/>
-      <c r="F1681" t="inlineStr"/>
       <c r="G1681" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -77833,8 +77781,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1682" t="inlineStr"/>
-      <c r="F1682" t="inlineStr"/>
       <c r="G1682" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -77881,8 +77827,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1683" t="inlineStr"/>
-      <c r="F1683" t="inlineStr"/>
       <c r="G1683" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -77929,8 +77873,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1684" t="inlineStr"/>
-      <c r="F1684" t="inlineStr"/>
       <c r="G1684" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -77977,8 +77919,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1685" t="inlineStr"/>
-      <c r="F1685" t="inlineStr"/>
       <c r="G1685" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -78025,8 +77965,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1686" t="inlineStr"/>
-      <c r="F1686" t="inlineStr"/>
       <c r="G1686" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -78073,8 +78011,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1687" t="inlineStr"/>
-      <c r="F1687" t="inlineStr"/>
       <c r="G1687" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -78121,8 +78057,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1688" t="inlineStr"/>
-      <c r="F1688" t="inlineStr"/>
       <c r="G1688" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -78169,8 +78103,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1689" t="inlineStr"/>
-      <c r="F1689" t="inlineStr"/>
       <c r="G1689" t="inlineStr">
         <is>
           <t>3-4</t>
@@ -78191,6 +78123,2934 @@
         <v>0</v>
       </c>
       <c r="L1689" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1690">
+      <c r="A1690" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1690" t="inlineStr">
+        <is>
+          <t>Australia vs Brazil</t>
+        </is>
+      </c>
+      <c r="C1690" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="D1690" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1690" t="inlineStr"/>
+      <c r="F1690" t="inlineStr"/>
+      <c r="G1690" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1690" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1690" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1690" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1690" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1690" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1691">
+      <c r="A1691" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1691" t="inlineStr">
+        <is>
+          <t>Sudan vs Ethiopia</t>
+        </is>
+      </c>
+      <c r="C1691" t="inlineStr">
+        <is>
+          <t>Sudan</t>
+        </is>
+      </c>
+      <c r="D1691" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1691" t="inlineStr"/>
+      <c r="F1691" t="inlineStr"/>
+      <c r="G1691" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1691" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1691" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1691" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1691" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1691" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1692">
+      <c r="A1692" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1692" t="inlineStr">
+        <is>
+          <t>India vs Panama</t>
+        </is>
+      </c>
+      <c r="C1692" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="D1692" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1692" t="inlineStr"/>
+      <c r="F1692" t="inlineStr"/>
+      <c r="G1692" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1692" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1692" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1692" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1692" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1692" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1693" t="inlineStr">
+        <is>
+          <t>VfB Stuttgart vs 1. FC Heidenheim 1846</t>
+        </is>
+      </c>
+      <c r="C1693" t="inlineStr">
+        <is>
+          <t>VfB Stuttgart</t>
+        </is>
+      </c>
+      <c r="D1693" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1693" t="inlineStr"/>
+      <c r="F1693" t="inlineStr"/>
+      <c r="G1693" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1693" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1693" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1693" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1693" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1693" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1694" t="inlineStr">
+        <is>
+          <t>Niger vs Lesotho</t>
+        </is>
+      </c>
+      <c r="C1694" t="inlineStr">
+        <is>
+          <t>Niger</t>
+        </is>
+      </c>
+      <c r="D1694" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1694" t="inlineStr"/>
+      <c r="F1694" t="inlineStr"/>
+      <c r="G1694" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1694" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1694" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1694" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1694" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1694" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1695" t="inlineStr">
+        <is>
+          <t>Iceland U21 vs France U21</t>
+        </is>
+      </c>
+      <c r="C1695" t="inlineStr">
+        <is>
+          <t>France U21</t>
+        </is>
+      </c>
+      <c r="D1695" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1695" t="inlineStr"/>
+      <c r="F1695" t="inlineStr"/>
+      <c r="G1695" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1695" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1695" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1695" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1695" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1695" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1696">
+      <c r="A1696" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1696" t="inlineStr">
+        <is>
+          <t>Finland U21 vs Spain U21</t>
+        </is>
+      </c>
+      <c r="C1696" t="inlineStr">
+        <is>
+          <t>Spain U21</t>
+        </is>
+      </c>
+      <c r="D1696" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1696" t="inlineStr"/>
+      <c r="F1696" t="inlineStr"/>
+      <c r="G1696" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1696" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1696" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1696" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1696" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1696" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1697" t="inlineStr">
+        <is>
+          <t>Bulgaria U21 vs Portugal U21</t>
+        </is>
+      </c>
+      <c r="C1697" t="inlineStr">
+        <is>
+          <t>Portugal U21</t>
+        </is>
+      </c>
+      <c r="D1697" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1697" t="inlineStr"/>
+      <c r="F1697" t="inlineStr"/>
+      <c r="G1697" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1697" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1697" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1697" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1697" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1697" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1698" t="inlineStr">
+        <is>
+          <t>Georgia vs Northern Ireland</t>
+        </is>
+      </c>
+      <c r="C1698" t="inlineStr">
+        <is>
+          <t>Georgia</t>
+        </is>
+      </c>
+      <c r="D1698" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1698" t="inlineStr"/>
+      <c r="F1698" t="inlineStr"/>
+      <c r="G1698" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1698" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1698" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1698" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1698" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1698" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1699" t="inlineStr">
+        <is>
+          <t>Armenia vs Latvia</t>
+        </is>
+      </c>
+      <c r="C1699" t="inlineStr">
+        <is>
+          <t>Armenia</t>
+        </is>
+      </c>
+      <c r="D1699" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1699" t="inlineStr"/>
+      <c r="F1699" t="inlineStr"/>
+      <c r="G1699" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1699" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1699" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1699" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1699" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1699" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1700" t="inlineStr">
+        <is>
+          <t>Gambia vs Somalia</t>
+        </is>
+      </c>
+      <c r="C1700" t="inlineStr">
+        <is>
+          <t>Gambia</t>
+        </is>
+      </c>
+      <c r="D1700" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1700" t="inlineStr"/>
+      <c r="F1700" t="inlineStr"/>
+      <c r="G1700" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1700" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1700" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1700" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1700" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1700" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1701" t="inlineStr">
+        <is>
+          <t>Malawi vs South Sudan</t>
+        </is>
+      </c>
+      <c r="C1701" t="inlineStr">
+        <is>
+          <t>Malawi</t>
+        </is>
+      </c>
+      <c r="D1701" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1701" t="inlineStr"/>
+      <c r="F1701" t="inlineStr"/>
+      <c r="G1701" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1701" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1701" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1701" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1701" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1701" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1702">
+      <c r="A1702" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1702" t="inlineStr">
+        <is>
+          <t>Nigeria vs Madagascar</t>
+        </is>
+      </c>
+      <c r="C1702" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="D1702" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1702" t="inlineStr"/>
+      <c r="F1702" t="inlineStr"/>
+      <c r="G1702" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1702" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1702" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1702" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1702" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1702" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1703">
+      <c r="A1703" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1703" t="inlineStr">
+        <is>
+          <t>Rwanda vs Liberia</t>
+        </is>
+      </c>
+      <c r="C1703" t="inlineStr">
+        <is>
+          <t>Rwanda</t>
+        </is>
+      </c>
+      <c r="D1703" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1703" t="inlineStr"/>
+      <c r="F1703" t="inlineStr"/>
+      <c r="G1703" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1703" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1703" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1703" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1703" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1703" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1704">
+      <c r="A1704" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1704" t="inlineStr">
+        <is>
+          <t>Estonia U21 vs Faroe Islands U21</t>
+        </is>
+      </c>
+      <c r="C1704" t="inlineStr">
+        <is>
+          <t>Estonia U21</t>
+        </is>
+      </c>
+      <c r="D1704" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1704" t="inlineStr"/>
+      <c r="F1704" t="inlineStr"/>
+      <c r="G1704" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1704" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1704" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1704" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1704" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1704" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1705">
+      <c r="A1705" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1705" t="inlineStr">
+        <is>
+          <t>Cyprus U21 vs Romania U21</t>
+        </is>
+      </c>
+      <c r="C1705" t="inlineStr">
+        <is>
+          <t>Romania U21</t>
+        </is>
+      </c>
+      <c r="D1705" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1705" t="inlineStr"/>
+      <c r="F1705" t="inlineStr"/>
+      <c r="G1705" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H1705" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1705" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1705" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1705" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1705" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1706">
+      <c r="A1706" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1706" t="inlineStr">
+        <is>
+          <t>Slovakia U21 vs Republic of Ireland U21</t>
+        </is>
+      </c>
+      <c r="C1706" t="inlineStr">
+        <is>
+          <t>Slovakia U21</t>
+        </is>
+      </c>
+      <c r="D1706" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1706" t="inlineStr"/>
+      <c r="F1706" t="inlineStr"/>
+      <c r="G1706" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1706" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1706" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1706" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1706" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1706" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1707">
+      <c r="A1707" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1707" t="inlineStr">
+        <is>
+          <t>Netherlands U21 vs Norway U21</t>
+        </is>
+      </c>
+      <c r="C1707" t="inlineStr">
+        <is>
+          <t>Netherlands U21</t>
+        </is>
+      </c>
+      <c r="D1707" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1707" t="inlineStr"/>
+      <c r="F1707" t="inlineStr"/>
+      <c r="G1707" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1707" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1707" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1707" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1707" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1707" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1708" t="inlineStr">
+        <is>
+          <t>Switzerland U21 vs Luxembourg U21</t>
+        </is>
+      </c>
+      <c r="C1708" t="inlineStr">
+        <is>
+          <t>Switzerland U21</t>
+        </is>
+      </c>
+      <c r="D1708" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1708" t="inlineStr"/>
+      <c r="F1708" t="inlineStr"/>
+      <c r="G1708" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H1708" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1708" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1708" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1708" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1708" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1709">
+      <c r="A1709" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1709" t="inlineStr">
+        <is>
+          <t>Girona vs Albacete</t>
+        </is>
+      </c>
+      <c r="C1709" t="inlineStr">
+        <is>
+          <t>Girona</t>
+        </is>
+      </c>
+      <c r="D1709" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1709" t="inlineStr"/>
+      <c r="F1709" t="inlineStr"/>
+      <c r="G1709" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1709" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1709" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1709" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1709" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1709" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1710">
+      <c r="A1710" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1710" t="inlineStr">
+        <is>
+          <t>England U21 vs Kazakhstan U21</t>
+        </is>
+      </c>
+      <c r="C1710" t="inlineStr">
+        <is>
+          <t>England U21</t>
+        </is>
+      </c>
+      <c r="D1710" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1710" t="inlineStr"/>
+      <c r="F1710" t="inlineStr"/>
+      <c r="G1710" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H1710" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1710" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1710" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1710" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1710" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1711">
+      <c r="A1711" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1711" t="inlineStr">
+        <is>
+          <t>Arbroath vs Queen's Park</t>
+        </is>
+      </c>
+      <c r="C1711" t="inlineStr">
+        <is>
+          <t>Arbroath</t>
+        </is>
+      </c>
+      <c r="D1711" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1711" t="inlineStr"/>
+      <c r="F1711" t="inlineStr"/>
+      <c r="G1711" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1711" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1711" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1711" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1711" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1711" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1712">
+      <c r="A1712" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1712" t="inlineStr">
+        <is>
+          <t>Ayr United vs Stenhousemuir</t>
+        </is>
+      </c>
+      <c r="C1712" t="inlineStr">
+        <is>
+          <t>Ayr United</t>
+        </is>
+      </c>
+      <c r="D1712" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1712" t="inlineStr"/>
+      <c r="F1712" t="inlineStr"/>
+      <c r="G1712" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1712" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1712" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1712" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1712" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1712" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1713">
+      <c r="A1713" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1713" t="inlineStr">
+        <is>
+          <t>Inverness Caledonian Thistle vs Greenock Morton</t>
+        </is>
+      </c>
+      <c r="C1713" t="inlineStr">
+        <is>
+          <t>Inverness Caledonian Thistle</t>
+        </is>
+      </c>
+      <c r="D1713" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1713" t="inlineStr"/>
+      <c r="F1713" t="inlineStr"/>
+      <c r="G1713" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1713" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1713" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1713" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1713" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1713" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1714">
+      <c r="A1714" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1714" t="inlineStr">
+        <is>
+          <t>Raith Rovers vs Livingston</t>
+        </is>
+      </c>
+      <c r="C1714" t="inlineStr">
+        <is>
+          <t>Raith Rovers</t>
+        </is>
+      </c>
+      <c r="D1714" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1714" t="inlineStr"/>
+      <c r="F1714" t="inlineStr"/>
+      <c r="G1714" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1714" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1714" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1714" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1714" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1714" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1715">
+      <c r="A1715" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1715" t="inlineStr">
+        <is>
+          <t>Türkiye vs France</t>
+        </is>
+      </c>
+      <c r="C1715" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D1715" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1715" t="inlineStr"/>
+      <c r="F1715" t="inlineStr"/>
+      <c r="G1715" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1715" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1715" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1715" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1715" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1715" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1716">
+      <c r="A1716" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1716" t="inlineStr">
+        <is>
+          <t>Italy vs Belgium</t>
+        </is>
+      </c>
+      <c r="C1716" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="D1716" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1716" t="inlineStr"/>
+      <c r="F1716" t="inlineStr"/>
+      <c r="G1716" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1716" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1716" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1716" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1716" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1716" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1717">
+      <c r="A1717" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1717" t="inlineStr">
+        <is>
+          <t>Hungary vs Ukraine</t>
+        </is>
+      </c>
+      <c r="C1717" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="D1717" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1717" t="inlineStr"/>
+      <c r="F1717" t="inlineStr"/>
+      <c r="G1717" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1717" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1717" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1717" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1717" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1717" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1718">
+      <c r="A1718" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1718" t="inlineStr">
+        <is>
+          <t>Poland vs Bosnia-Herzegovina</t>
+        </is>
+      </c>
+      <c r="C1718" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="D1718" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1718" t="inlineStr"/>
+      <c r="F1718" t="inlineStr"/>
+      <c r="G1718" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1718" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1718" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1718" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1718" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1718" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1719">
+      <c r="A1719" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1719" t="inlineStr">
+        <is>
+          <t>Sweden vs Romania</t>
+        </is>
+      </c>
+      <c r="C1719" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="D1719" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1719" t="inlineStr"/>
+      <c r="F1719" t="inlineStr"/>
+      <c r="G1719" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1719" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1719" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1719" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1719" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1719" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1720" t="inlineStr">
+        <is>
+          <t>Montenegro vs Cyprus</t>
+        </is>
+      </c>
+      <c r="C1720" t="inlineStr">
+        <is>
+          <t>Montenegro</t>
+        </is>
+      </c>
+      <c r="D1720" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1720" t="inlineStr"/>
+      <c r="F1720" t="inlineStr"/>
+      <c r="G1720" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1720" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1720" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1720" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1720" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1720" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1721" t="inlineStr">
+        <is>
+          <t>Spartans FC vs Dundee B</t>
+        </is>
+      </c>
+      <c r="C1721" t="inlineStr">
+        <is>
+          <t>Spartans FC</t>
+        </is>
+      </c>
+      <c r="D1721" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1721" t="inlineStr"/>
+      <c r="F1721" t="inlineStr"/>
+      <c r="G1721" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1721" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1721" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1721" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1721" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1721" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1722" t="inlineStr">
+        <is>
+          <t>FC Dordrecht vs Almere City</t>
+        </is>
+      </c>
+      <c r="C1722" t="inlineStr">
+        <is>
+          <t>Almere City</t>
+        </is>
+      </c>
+      <c r="D1722" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1722" t="inlineStr"/>
+      <c r="F1722" t="inlineStr"/>
+      <c r="G1722" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1722" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1722" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1722" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1722" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1722" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1723" t="inlineStr">
+        <is>
+          <t>Algeria vs Zambia</t>
+        </is>
+      </c>
+      <c r="C1723" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="D1723" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1723" t="inlineStr"/>
+      <c r="F1723" t="inlineStr"/>
+      <c r="G1723" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1723" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1723" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1723" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1723" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1723" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1724" t="inlineStr">
+        <is>
+          <t>Burkina Faso vs Benin</t>
+        </is>
+      </c>
+      <c r="C1724" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="D1724" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1724" t="inlineStr"/>
+      <c r="F1724" t="inlineStr"/>
+      <c r="G1724" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1724" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1724" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1724" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1724" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1724" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1725" t="inlineStr">
+        <is>
+          <t>Egypt vs Angola</t>
+        </is>
+      </c>
+      <c r="C1725" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="D1725" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1725" t="inlineStr"/>
+      <c r="F1725" t="inlineStr"/>
+      <c r="G1725" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1725" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1725" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1725" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1725" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1725" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1726" t="inlineStr">
+        <is>
+          <t>Morocco vs Gabon</t>
+        </is>
+      </c>
+      <c r="C1726" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="D1726" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1726" t="inlineStr"/>
+      <c r="F1726" t="inlineStr"/>
+      <c r="G1726" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1726" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1726" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1726" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1726" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1726" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1727">
+      <c r="A1727" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1727" t="inlineStr">
+        <is>
+          <t>Bermuda vs Guadeloupe</t>
+        </is>
+      </c>
+      <c r="C1727" t="inlineStr">
+        <is>
+          <t>Guadeloupe</t>
+        </is>
+      </c>
+      <c r="D1727" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1727" t="inlineStr"/>
+      <c r="F1727" t="inlineStr"/>
+      <c r="G1727" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1727" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1727" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1727" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1727" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1727" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1728">
+      <c r="A1728" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1728" t="inlineStr">
+        <is>
+          <t>San Antonio Bulo Bulo vs Real Potosí</t>
+        </is>
+      </c>
+      <c r="C1728" t="inlineStr">
+        <is>
+          <t>San Antonio Bulo Bulo</t>
+        </is>
+      </c>
+      <c r="D1728" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1728" t="inlineStr"/>
+      <c r="F1728" t="inlineStr"/>
+      <c r="G1728" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1728" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1728" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1728" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1728" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1728" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1729">
+      <c r="A1729" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1729" t="inlineStr">
+        <is>
+          <t>Mali vs Cape Verde</t>
+        </is>
+      </c>
+      <c r="C1729" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="D1729" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1729" t="inlineStr"/>
+      <c r="F1729" t="inlineStr"/>
+      <c r="G1729" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1729" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1729" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1729" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1729" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1729" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1730">
+      <c r="A1730" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1730" t="inlineStr">
+        <is>
+          <t>Sportivo Luqueño vs Guaraní</t>
+        </is>
+      </c>
+      <c r="C1730" t="inlineStr">
+        <is>
+          <t>Guaraní</t>
+        </is>
+      </c>
+      <c r="D1730" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1730" t="inlineStr"/>
+      <c r="F1730" t="inlineStr"/>
+      <c r="G1730" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1730" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1730" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1730" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1730" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1730" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1731">
+      <c r="A1731" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1731" t="inlineStr">
+        <is>
+          <t>Grenada vs Cuba</t>
+        </is>
+      </c>
+      <c r="C1731" t="inlineStr">
+        <is>
+          <t>Cuba</t>
+        </is>
+      </c>
+      <c r="D1731" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1731" t="inlineStr"/>
+      <c r="F1731" t="inlineStr"/>
+      <c r="G1731" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H1731" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1731" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1731" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1731" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1731" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1732">
+      <c r="A1732" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1732" t="inlineStr">
+        <is>
+          <t>ABB vs Aurora</t>
+        </is>
+      </c>
+      <c r="C1732" t="inlineStr">
+        <is>
+          <t>Aurora</t>
+        </is>
+      </c>
+      <c r="D1732" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1732" t="inlineStr"/>
+      <c r="F1732" t="inlineStr"/>
+      <c r="G1732" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1732" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1732" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1732" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1732" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1732" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1733">
+      <c r="A1733" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1733" t="inlineStr">
+        <is>
+          <t>Ituzaingó vs Defensores Unidos</t>
+        </is>
+      </c>
+      <c r="C1733" t="inlineStr">
+        <is>
+          <t>Defensores Unidos</t>
+        </is>
+      </c>
+      <c r="D1733" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1733" t="inlineStr"/>
+      <c r="F1733" t="inlineStr"/>
+      <c r="G1733" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1733" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1733" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1733" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1733" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1733" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1734">
+      <c r="A1734" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1734" t="inlineStr">
+        <is>
+          <t>Nacional Asunción vs Sportivo Ameliano</t>
+        </is>
+      </c>
+      <c r="C1734" t="inlineStr">
+        <is>
+          <t>Nacional Asunción</t>
+        </is>
+      </c>
+      <c r="D1734" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1734" t="inlineStr"/>
+      <c r="F1734" t="inlineStr"/>
+      <c r="G1734" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1734" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1734" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1734" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1734" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1734" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1735">
+      <c r="A1735" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1735" t="inlineStr">
+        <is>
+          <t>Novorizontino vs São Bernardo</t>
+        </is>
+      </c>
+      <c r="C1735" t="inlineStr">
+        <is>
+          <t>Novorizontino</t>
+        </is>
+      </c>
+      <c r="D1735" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1735" t="inlineStr"/>
+      <c r="F1735" t="inlineStr"/>
+      <c r="G1735" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1735" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1735" t="n">
+        <v>6</v>
+      </c>
+      <c r="J1735" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1735" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1735" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1736">
+      <c r="A1736" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1736" t="inlineStr">
+        <is>
+          <t>Excursionistas vs Real Pilar</t>
+        </is>
+      </c>
+      <c r="C1736" t="inlineStr">
+        <is>
+          <t>Excursionistas</t>
+        </is>
+      </c>
+      <c r="D1736" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1736" t="inlineStr"/>
+      <c r="F1736" t="inlineStr"/>
+      <c r="G1736" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1736" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1736" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1736" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1736" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1736" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1737">
+      <c r="A1737" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1737" t="inlineStr">
+        <is>
+          <t>Colo Colo vs Audax Italiano</t>
+        </is>
+      </c>
+      <c r="C1737" t="inlineStr">
+        <is>
+          <t>Colo Colo</t>
+        </is>
+      </c>
+      <c r="D1737" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1737" t="inlineStr"/>
+      <c r="F1737" t="inlineStr"/>
+      <c r="G1737" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1737" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1737" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1737" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1737" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1737" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1738">
+      <c r="A1738" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1738" t="inlineStr">
+        <is>
+          <t>Unión Magdalena vs Independiente Santa Fe</t>
+        </is>
+      </c>
+      <c r="C1738" t="inlineStr">
+        <is>
+          <t>Independiente Santa Fe</t>
+        </is>
+      </c>
+      <c r="D1738" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1738" t="inlineStr"/>
+      <c r="F1738" t="inlineStr"/>
+      <c r="G1738" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1738" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1738" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1738" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1738" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1738" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1739">
+      <c r="A1739" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1739" t="inlineStr">
+        <is>
+          <t>Hartford Athletic vs Louisville City FC</t>
+        </is>
+      </c>
+      <c r="C1739" t="inlineStr">
+        <is>
+          <t>Louisville City FC</t>
+        </is>
+      </c>
+      <c r="D1739" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1739" t="inlineStr"/>
+      <c r="F1739" t="inlineStr"/>
+      <c r="G1739" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H1739" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1739" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1739" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1739" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1739" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1740">
+      <c r="A1740" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1740" t="inlineStr">
+        <is>
+          <t>Vila Nova vs Londrina</t>
+        </is>
+      </c>
+      <c r="C1740" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="D1740" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1740" t="inlineStr"/>
+      <c r="F1740" t="inlineStr"/>
+      <c r="G1740" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1740" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1740" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1740" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1740" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1740" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1741">
+      <c r="A1741" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1741" t="inlineStr">
+        <is>
+          <t>Sporting JAX vs Loudoun United FC</t>
+        </is>
+      </c>
+      <c r="C1741" t="inlineStr">
+        <is>
+          <t>Loudoun United FC</t>
+        </is>
+      </c>
+      <c r="D1741" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1741" t="inlineStr"/>
+      <c r="F1741" t="inlineStr"/>
+      <c r="G1741" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H1741" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1741" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1741" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1741" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1741" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1742">
+      <c r="A1742" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1742" t="inlineStr">
+        <is>
+          <t>Nacional Potosí vs Always Ready</t>
+        </is>
+      </c>
+      <c r="C1742" t="inlineStr">
+        <is>
+          <t>Nacional Potosí</t>
+        </is>
+      </c>
+      <c r="D1742" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1742" t="inlineStr"/>
+      <c r="F1742" t="inlineStr"/>
+      <c r="G1742" t="inlineStr">
+        <is>
+          <t>9-0</t>
+        </is>
+      </c>
+      <c r="H1742" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1742" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1742" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1742" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1742" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1743">
+      <c r="A1743" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1743" t="inlineStr">
+        <is>
+          <t>Barbados vs St. Lucia</t>
+        </is>
+      </c>
+      <c r="C1743" t="inlineStr">
+        <is>
+          <t>St. Lucia</t>
+        </is>
+      </c>
+      <c r="D1743" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1743" t="inlineStr"/>
+      <c r="F1743" t="inlineStr"/>
+      <c r="G1743" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1743" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1743" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1743" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1743" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1743" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1744">
+      <c r="A1744" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1744" t="inlineStr">
+        <is>
+          <t>Jamaica vs Guatemala</t>
+        </is>
+      </c>
+      <c r="C1744" t="inlineStr">
+        <is>
+          <t>Jamaica</t>
+        </is>
+      </c>
+      <c r="D1744" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1744" t="inlineStr"/>
+      <c r="F1744" t="inlineStr"/>
+      <c r="G1744" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1744" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1744" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1744" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1744" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1744" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1745">
+      <c r="A1745" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1745" t="inlineStr">
+        <is>
+          <t>Atlante vs Monterrey</t>
+        </is>
+      </c>
+      <c r="C1745" t="inlineStr">
+        <is>
+          <t>Monterrey</t>
+        </is>
+      </c>
+      <c r="D1745" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1745" t="inlineStr"/>
+      <c r="F1745" t="inlineStr"/>
+      <c r="G1745" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H1745" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1745" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1745" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1745" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1745" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1746">
+      <c r="A1746" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1746" t="inlineStr">
+        <is>
+          <t>El Paso Locomotive FC vs FC Tulsa</t>
+        </is>
+      </c>
+      <c r="C1746" t="inlineStr">
+        <is>
+          <t>El Paso Locomotive FC</t>
+        </is>
+      </c>
+      <c r="D1746" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1746" t="inlineStr"/>
+      <c r="F1746" t="inlineStr"/>
+      <c r="G1746" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1746" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1746" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1746" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1746" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1746" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1747">
+      <c r="A1747" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1747" t="inlineStr">
+        <is>
+          <t>Honduras vs Suriname</t>
+        </is>
+      </c>
+      <c r="C1747" t="inlineStr">
+        <is>
+          <t>Honduras</t>
+        </is>
+      </c>
+      <c r="D1747" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1747" t="inlineStr"/>
+      <c r="F1747" t="inlineStr"/>
+      <c r="G1747" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H1747" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1747" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1747" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1747" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1747" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1748">
+      <c r="A1748" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1748" t="inlineStr">
+        <is>
+          <t>Once Caldas vs Atlético Bucaramanga</t>
+        </is>
+      </c>
+      <c r="C1748" t="inlineStr">
+        <is>
+          <t>Once Caldas</t>
+        </is>
+      </c>
+      <c r="D1748" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1748" t="inlineStr"/>
+      <c r="F1748" t="inlineStr"/>
+      <c r="G1748" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H1748" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1748" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1748" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1748" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1748" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1749">
+      <c r="A1749" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1749" t="inlineStr">
+        <is>
+          <t>Tijuana vs Atlas</t>
+        </is>
+      </c>
+      <c r="C1749" t="inlineStr">
+        <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
+      <c r="D1749" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1749" t="inlineStr"/>
+      <c r="F1749" t="inlineStr"/>
+      <c r="G1749" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H1749" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1749" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1749" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1749" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1749" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1750">
+      <c r="A1750" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B1750" t="inlineStr">
+        <is>
+          <t>El Salvador vs Martinique</t>
+        </is>
+      </c>
+      <c r="C1750" t="inlineStr">
+        <is>
+          <t>El Salvador</t>
+        </is>
+      </c>
+      <c r="D1750" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1750" t="inlineStr"/>
+      <c r="F1750" t="inlineStr"/>
+      <c r="G1750" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1750" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1750" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1750" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1750" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1750" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -78207,7 +81067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -78730,6 +81590,25 @@
       </c>
       <c r="E28" t="n">
         <v>34</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>61</v>
+      </c>
+      <c r="C29" t="n">
+        <v>39</v>
+      </c>
+      <c r="D29" t="n">
+        <v>63.9</v>
+      </c>
+      <c r="E29" t="n">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -78743,7 +81622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G155"/>
+  <dimension ref="A1:G161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82238,6 +85117,168 @@
         <v>0</v>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>1</v>
+      </c>
+      <c r="D156" t="n">
+        <v>0</v>
+      </c>
+      <c r="E156" t="n">
+        <v>0</v>
+      </c>
+      <c r="F156" t="n">
+        <v>1</v>
+      </c>
+      <c r="G156" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>3</v>
+      </c>
+      <c r="D157" t="n">
+        <v>1</v>
+      </c>
+      <c r="E157" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="F157" t="n">
+        <v>2</v>
+      </c>
+      <c r="G157" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>fav_domina_no_gana</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>3</v>
+      </c>
+      <c r="D158" t="n">
+        <v>1</v>
+      </c>
+      <c r="E158" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="F158" t="n">
+        <v>2</v>
+      </c>
+      <c r="G158" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>1</v>
+      </c>
+      <c r="D159" t="n">
+        <v>0</v>
+      </c>
+      <c r="E159" t="n">
+        <v>0</v>
+      </c>
+      <c r="F159" t="n">
+        <v>1</v>
+      </c>
+      <c r="G159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>siguen_empatados_22</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>1</v>
+      </c>
+      <c r="D160" t="n">
+        <v>0</v>
+      </c>
+      <c r="E160" t="n">
+        <v>0</v>
+      </c>
+      <c r="F160" t="n">
+        <v>1</v>
+      </c>
+      <c r="G160" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>siguen_empatados_70</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>1</v>
+      </c>
+      <c r="D161" t="n">
+        <v>0</v>
+      </c>
+      <c r="E161" t="n">
+        <v>0</v>
+      </c>
+      <c r="F161" t="n">
+        <v>1</v>
+      </c>
+      <c r="G161" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-28
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1842"/>
+  <dimension ref="A1:L1894"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -80955,8 +80955,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1751" t="inlineStr"/>
-      <c r="F1751" t="inlineStr"/>
       <c r="G1751" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -81003,8 +81001,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1752" t="inlineStr"/>
-      <c r="F1752" t="inlineStr"/>
       <c r="G1752" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -81051,8 +81047,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1753" t="inlineStr"/>
-      <c r="F1753" t="inlineStr"/>
       <c r="G1753" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -81099,8 +81093,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1754" t="inlineStr"/>
-      <c r="F1754" t="inlineStr"/>
       <c r="G1754" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -81147,8 +81139,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1755" t="inlineStr"/>
-      <c r="F1755" t="inlineStr"/>
       <c r="G1755" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -81195,8 +81185,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1756" t="inlineStr"/>
-      <c r="F1756" t="inlineStr"/>
       <c r="G1756" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -81243,8 +81231,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1757" t="inlineStr"/>
-      <c r="F1757" t="inlineStr"/>
       <c r="G1757" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -81291,8 +81277,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1758" t="inlineStr"/>
-      <c r="F1758" t="inlineStr"/>
       <c r="G1758" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -81339,8 +81323,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1759" t="inlineStr"/>
-      <c r="F1759" t="inlineStr"/>
       <c r="G1759" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -81387,8 +81369,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1760" t="inlineStr"/>
-      <c r="F1760" t="inlineStr"/>
       <c r="G1760" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -81435,8 +81415,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1761" t="inlineStr"/>
-      <c r="F1761" t="inlineStr"/>
       <c r="G1761" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -81483,8 +81461,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1762" t="inlineStr"/>
-      <c r="F1762" t="inlineStr"/>
       <c r="G1762" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -81531,8 +81507,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1763" t="inlineStr"/>
-      <c r="F1763" t="inlineStr"/>
       <c r="G1763" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -81579,8 +81553,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1764" t="inlineStr"/>
-      <c r="F1764" t="inlineStr"/>
       <c r="G1764" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -81627,8 +81599,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1765" t="inlineStr"/>
-      <c r="F1765" t="inlineStr"/>
       <c r="G1765" t="inlineStr">
         <is>
           <t>5-1</t>
@@ -81675,8 +81645,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1766" t="inlineStr"/>
-      <c r="F1766" t="inlineStr"/>
       <c r="G1766" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -81723,8 +81691,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1767" t="inlineStr"/>
-      <c r="F1767" t="inlineStr"/>
       <c r="G1767" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -81771,8 +81737,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1768" t="inlineStr"/>
-      <c r="F1768" t="inlineStr"/>
       <c r="G1768" t="inlineStr">
         <is>
           <t>2-5</t>
@@ -81819,8 +81783,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1769" t="inlineStr"/>
-      <c r="F1769" t="inlineStr"/>
       <c r="G1769" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -81867,8 +81829,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1770" t="inlineStr"/>
-      <c r="F1770" t="inlineStr"/>
       <c r="G1770" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -81915,8 +81875,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1771" t="inlineStr"/>
-      <c r="F1771" t="inlineStr"/>
       <c r="G1771" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -81963,8 +81921,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1772" t="inlineStr"/>
-      <c r="F1772" t="inlineStr"/>
       <c r="G1772" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -82011,8 +81967,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1773" t="inlineStr"/>
-      <c r="F1773" t="inlineStr"/>
       <c r="G1773" t="inlineStr">
         <is>
           <t>2-4</t>
@@ -82059,8 +82013,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1774" t="inlineStr"/>
-      <c r="F1774" t="inlineStr"/>
       <c r="G1774" t="inlineStr">
         <is>
           <t>3-3</t>
@@ -82107,8 +82059,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1775" t="inlineStr"/>
-      <c r="F1775" t="inlineStr"/>
       <c r="G1775" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -82155,8 +82105,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1776" t="inlineStr"/>
-      <c r="F1776" t="inlineStr"/>
       <c r="G1776" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -82203,8 +82151,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1777" t="inlineStr"/>
-      <c r="F1777" t="inlineStr"/>
       <c r="G1777" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -82251,8 +82197,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1778" t="inlineStr"/>
-      <c r="F1778" t="inlineStr"/>
       <c r="G1778" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -82299,8 +82243,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1779" t="inlineStr"/>
-      <c r="F1779" t="inlineStr"/>
       <c r="G1779" t="inlineStr">
         <is>
           <t>3-3</t>
@@ -82347,8 +82289,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1780" t="inlineStr"/>
-      <c r="F1780" t="inlineStr"/>
       <c r="G1780" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -82395,8 +82335,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1781" t="inlineStr"/>
-      <c r="F1781" t="inlineStr"/>
       <c r="G1781" t="inlineStr">
         <is>
           <t>2-4</t>
@@ -82443,8 +82381,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1782" t="inlineStr"/>
-      <c r="F1782" t="inlineStr"/>
       <c r="G1782" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -82491,8 +82427,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1783" t="inlineStr"/>
-      <c r="F1783" t="inlineStr"/>
       <c r="G1783" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -82539,8 +82473,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1784" t="inlineStr"/>
-      <c r="F1784" t="inlineStr"/>
       <c r="G1784" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -82587,8 +82519,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1785" t="inlineStr"/>
-      <c r="F1785" t="inlineStr"/>
       <c r="G1785" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -82635,8 +82565,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1786" t="inlineStr"/>
-      <c r="F1786" t="inlineStr"/>
       <c r="G1786" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -82683,8 +82611,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1787" t="inlineStr"/>
-      <c r="F1787" t="inlineStr"/>
       <c r="G1787" t="inlineStr">
         <is>
           <t>0-7</t>
@@ -82731,8 +82657,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1788" t="inlineStr"/>
-      <c r="F1788" t="inlineStr"/>
       <c r="G1788" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -82779,8 +82703,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1789" t="inlineStr"/>
-      <c r="F1789" t="inlineStr"/>
       <c r="G1789" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -82827,8 +82749,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1790" t="inlineStr"/>
-      <c r="F1790" t="inlineStr"/>
       <c r="G1790" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -82875,8 +82795,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1791" t="inlineStr"/>
-      <c r="F1791" t="inlineStr"/>
       <c r="G1791" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -82923,8 +82841,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1792" t="inlineStr"/>
-      <c r="F1792" t="inlineStr"/>
       <c r="G1792" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -82971,8 +82887,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1793" t="inlineStr"/>
-      <c r="F1793" t="inlineStr"/>
       <c r="G1793" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -83019,8 +82933,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1794" t="inlineStr"/>
-      <c r="F1794" t="inlineStr"/>
       <c r="G1794" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -83067,8 +82979,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1795" t="inlineStr"/>
-      <c r="F1795" t="inlineStr"/>
       <c r="G1795" t="inlineStr">
         <is>
           <t>4-2</t>
@@ -83115,8 +83025,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1796" t="inlineStr"/>
-      <c r="F1796" t="inlineStr"/>
       <c r="G1796" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -83163,8 +83071,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1797" t="inlineStr"/>
-      <c r="F1797" t="inlineStr"/>
       <c r="G1797" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -83211,8 +83117,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1798" t="inlineStr"/>
-      <c r="F1798" t="inlineStr"/>
       <c r="G1798" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -83259,8 +83163,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1799" t="inlineStr"/>
-      <c r="F1799" t="inlineStr"/>
       <c r="G1799" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -83307,8 +83209,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1800" t="inlineStr"/>
-      <c r="F1800" t="inlineStr"/>
       <c r="G1800" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -83355,8 +83255,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1801" t="inlineStr"/>
-      <c r="F1801" t="inlineStr"/>
       <c r="G1801" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -83403,8 +83301,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1802" t="inlineStr"/>
-      <c r="F1802" t="inlineStr"/>
       <c r="G1802" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -83451,8 +83347,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1803" t="inlineStr"/>
-      <c r="F1803" t="inlineStr"/>
       <c r="G1803" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -83499,8 +83393,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1804" t="inlineStr"/>
-      <c r="F1804" t="inlineStr"/>
       <c r="G1804" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -83547,8 +83439,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1805" t="inlineStr"/>
-      <c r="F1805" t="inlineStr"/>
       <c r="G1805" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -83595,8 +83485,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1806" t="inlineStr"/>
-      <c r="F1806" t="inlineStr"/>
       <c r="G1806" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -83643,8 +83531,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1807" t="inlineStr"/>
-      <c r="F1807" t="inlineStr"/>
       <c r="G1807" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -83691,8 +83577,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1808" t="inlineStr"/>
-      <c r="F1808" t="inlineStr"/>
       <c r="G1808" t="inlineStr">
         <is>
           <t>1-4</t>
@@ -83739,8 +83623,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1809" t="inlineStr"/>
-      <c r="F1809" t="inlineStr"/>
       <c r="G1809" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -83787,8 +83669,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1810" t="inlineStr"/>
-      <c r="F1810" t="inlineStr"/>
       <c r="G1810" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -83835,8 +83715,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1811" t="inlineStr"/>
-      <c r="F1811" t="inlineStr"/>
       <c r="G1811" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -83883,8 +83761,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1812" t="inlineStr"/>
-      <c r="F1812" t="inlineStr"/>
       <c r="G1812" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -83931,8 +83807,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1813" t="inlineStr"/>
-      <c r="F1813" t="inlineStr"/>
       <c r="G1813" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -83979,8 +83853,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1814" t="inlineStr"/>
-      <c r="F1814" t="inlineStr"/>
       <c r="G1814" t="inlineStr">
         <is>
           <t>3-3</t>
@@ -84027,8 +83899,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1815" t="inlineStr"/>
-      <c r="F1815" t="inlineStr"/>
       <c r="G1815" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -84075,8 +83945,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1816" t="inlineStr"/>
-      <c r="F1816" t="inlineStr"/>
       <c r="G1816" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -84123,8 +83991,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1817" t="inlineStr"/>
-      <c r="F1817" t="inlineStr"/>
       <c r="G1817" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -84171,8 +84037,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1818" t="inlineStr"/>
-      <c r="F1818" t="inlineStr"/>
       <c r="G1818" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -84219,8 +84083,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1819" t="inlineStr"/>
-      <c r="F1819" t="inlineStr"/>
       <c r="G1819" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -84267,8 +84129,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1820" t="inlineStr"/>
-      <c r="F1820" t="inlineStr"/>
       <c r="G1820" t="inlineStr">
         <is>
           <t>5-0</t>
@@ -84315,8 +84175,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1821" t="inlineStr"/>
-      <c r="F1821" t="inlineStr"/>
       <c r="G1821" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -84363,8 +84221,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1822" t="inlineStr"/>
-      <c r="F1822" t="inlineStr"/>
       <c r="G1822" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -84411,8 +84267,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1823" t="inlineStr"/>
-      <c r="F1823" t="inlineStr"/>
       <c r="G1823" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -84459,8 +84313,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1824" t="inlineStr"/>
-      <c r="F1824" t="inlineStr"/>
       <c r="G1824" t="inlineStr">
         <is>
           <t>4-2</t>
@@ -84507,8 +84359,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1825" t="inlineStr"/>
-      <c r="F1825" t="inlineStr"/>
       <c r="G1825" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -84555,8 +84405,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1826" t="inlineStr"/>
-      <c r="F1826" t="inlineStr"/>
       <c r="G1826" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -84603,8 +84451,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1827" t="inlineStr"/>
-      <c r="F1827" t="inlineStr"/>
       <c r="G1827" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -84651,8 +84497,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1828" t="inlineStr"/>
-      <c r="F1828" t="inlineStr"/>
       <c r="G1828" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -84699,8 +84543,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1829" t="inlineStr"/>
-      <c r="F1829" t="inlineStr"/>
       <c r="G1829" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -84747,8 +84589,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1830" t="inlineStr"/>
-      <c r="F1830" t="inlineStr"/>
       <c r="G1830" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -84795,8 +84635,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1831" t="inlineStr"/>
-      <c r="F1831" t="inlineStr"/>
       <c r="G1831" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -84843,8 +84681,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1832" t="inlineStr"/>
-      <c r="F1832" t="inlineStr"/>
       <c r="G1832" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -84891,8 +84727,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1833" t="inlineStr"/>
-      <c r="F1833" t="inlineStr"/>
       <c r="G1833" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -84939,8 +84773,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1834" t="inlineStr"/>
-      <c r="F1834" t="inlineStr"/>
       <c r="G1834" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -84987,8 +84819,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1835" t="inlineStr"/>
-      <c r="F1835" t="inlineStr"/>
       <c r="G1835" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -85035,8 +84865,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1836" t="inlineStr"/>
-      <c r="F1836" t="inlineStr"/>
       <c r="G1836" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -85083,8 +84911,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1837" t="inlineStr"/>
-      <c r="F1837" t="inlineStr"/>
       <c r="G1837" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -85131,8 +84957,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1838" t="inlineStr"/>
-      <c r="F1838" t="inlineStr"/>
       <c r="G1838" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -85179,8 +85003,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1839" t="inlineStr"/>
-      <c r="F1839" t="inlineStr"/>
       <c r="G1839" t="inlineStr">
         <is>
           <t>3-3</t>
@@ -85227,8 +85049,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1840" t="inlineStr"/>
-      <c r="F1840" t="inlineStr"/>
       <c r="G1840" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -85275,8 +85095,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1841" t="inlineStr"/>
-      <c r="F1841" t="inlineStr"/>
       <c r="G1841" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -85323,8 +85141,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1842" t="inlineStr"/>
-      <c r="F1842" t="inlineStr"/>
       <c r="G1842" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -85345,6 +85161,2502 @@
         <v>0</v>
       </c>
       <c r="L1842" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1843">
+      <c r="A1843" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1843" t="inlineStr">
+        <is>
+          <t>Vanuatu vs New Caledonia</t>
+        </is>
+      </c>
+      <c r="C1843" t="inlineStr">
+        <is>
+          <t>New Caledonia</t>
+        </is>
+      </c>
+      <c r="D1843" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1843" t="inlineStr"/>
+      <c r="F1843" t="inlineStr"/>
+      <c r="G1843" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H1843" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1843" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1843" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1843" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1843" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1844">
+      <c r="A1844" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1844" t="inlineStr">
+        <is>
+          <t>Fiji vs Papua New Guinea</t>
+        </is>
+      </c>
+      <c r="C1844" t="inlineStr">
+        <is>
+          <t>Fiji</t>
+        </is>
+      </c>
+      <c r="D1844" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1844" t="inlineStr"/>
+      <c r="F1844" t="inlineStr"/>
+      <c r="G1844" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1844" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1844" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1844" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1844" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1844" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1845">
+      <c r="A1845" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1845" t="inlineStr">
+        <is>
+          <t>China vs New Zealand</t>
+        </is>
+      </c>
+      <c r="C1845" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="D1845" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1845" t="inlineStr"/>
+      <c r="F1845" t="inlineStr"/>
+      <c r="G1845" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H1845" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1845" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1845" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1845" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1845" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1846">
+      <c r="A1846" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1846" t="inlineStr">
+        <is>
+          <t>Real Valladolid vs Córdoba</t>
+        </is>
+      </c>
+      <c r="C1846" t="inlineStr">
+        <is>
+          <t>Real Valladolid</t>
+        </is>
+      </c>
+      <c r="D1846" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1846" t="inlineStr"/>
+      <c r="F1846" t="inlineStr"/>
+      <c r="G1846" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1846" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1846" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1846" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1846" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1846" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1847">
+      <c r="A1847" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1847" t="inlineStr">
+        <is>
+          <t>Shanghai Shenhua vs Zenit St Petersburg</t>
+        </is>
+      </c>
+      <c r="C1847" t="inlineStr">
+        <is>
+          <t>Zenit St Petersburg</t>
+        </is>
+      </c>
+      <c r="D1847" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1847" t="inlineStr"/>
+      <c r="F1847" t="inlineStr"/>
+      <c r="G1847" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1847" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1847" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1847" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1847" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1847" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1848">
+      <c r="A1848" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1848" t="inlineStr">
+        <is>
+          <t>De Graafschap vs FC Den Bosch</t>
+        </is>
+      </c>
+      <c r="C1848" t="inlineStr">
+        <is>
+          <t>De Graafschap</t>
+        </is>
+      </c>
+      <c r="D1848" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1848" t="inlineStr"/>
+      <c r="F1848" t="inlineStr"/>
+      <c r="G1848" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1848" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1848" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1848" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1848" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1848" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1849">
+      <c r="A1849" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1849" t="inlineStr">
+        <is>
+          <t>Lithuania vs Azerbaijan</t>
+        </is>
+      </c>
+      <c r="C1849" t="inlineStr">
+        <is>
+          <t>Lithuania</t>
+        </is>
+      </c>
+      <c r="D1849" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1849" t="inlineStr"/>
+      <c r="F1849" t="inlineStr"/>
+      <c r="G1849" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1849" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1849" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1849" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1849" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1849" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1850">
+      <c r="A1850" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1850" t="inlineStr">
+        <is>
+          <t>Central Español Fútbol Club vs Liverpool</t>
+        </is>
+      </c>
+      <c r="C1850" t="inlineStr">
+        <is>
+          <t>Liverpool</t>
+        </is>
+      </c>
+      <c r="D1850" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1850" t="inlineStr"/>
+      <c r="F1850" t="inlineStr"/>
+      <c r="G1850" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1850" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1850" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1850" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1850" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1850" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1851">
+      <c r="A1851" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1851" t="inlineStr">
+        <is>
+          <t>Criciúma vs Avaí</t>
+        </is>
+      </c>
+      <c r="C1851" t="inlineStr">
+        <is>
+          <t>Criciúma</t>
+        </is>
+      </c>
+      <c r="D1851" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1851" t="inlineStr"/>
+      <c r="F1851" t="inlineStr"/>
+      <c r="G1851" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1851" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1851" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1851" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1851" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1851" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1852">
+      <c r="A1852" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1852" t="inlineStr">
+        <is>
+          <t>Camacha vs Florgrade</t>
+        </is>
+      </c>
+      <c r="C1852" t="inlineStr">
+        <is>
+          <t>Camacha</t>
+        </is>
+      </c>
+      <c r="D1852" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1852" t="inlineStr"/>
+      <c r="F1852" t="inlineStr"/>
+      <c r="G1852" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1852" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1852" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1852" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1852" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1852" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1853">
+      <c r="A1853" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1853" t="inlineStr">
+        <is>
+          <t>Mallorca vs Almería</t>
+        </is>
+      </c>
+      <c r="C1853" t="inlineStr">
+        <is>
+          <t>Mallorca</t>
+        </is>
+      </c>
+      <c r="D1853" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1853" t="inlineStr"/>
+      <c r="F1853" t="inlineStr"/>
+      <c r="G1853" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1853" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1853" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1853" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1853" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1853" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1854">
+      <c r="A1854" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1854" t="inlineStr">
+        <is>
+          <t>Antofagasta vs Deportes Iquique</t>
+        </is>
+      </c>
+      <c r="C1854" t="inlineStr">
+        <is>
+          <t>Antofagasta</t>
+        </is>
+      </c>
+      <c r="D1854" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1854" t="inlineStr"/>
+      <c r="F1854" t="inlineStr"/>
+      <c r="G1854" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H1854" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1854" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1854" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1854" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1854" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1855">
+      <c r="A1855" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1855" t="inlineStr">
+        <is>
+          <t>Serbia vs Netherlands</t>
+        </is>
+      </c>
+      <c r="C1855" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="D1855" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1855" t="inlineStr"/>
+      <c r="F1855" t="inlineStr"/>
+      <c r="G1855" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1855" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1855" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1855" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1855" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1855" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1856">
+      <c r="A1856" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1856" t="inlineStr">
+        <is>
+          <t>Denmark vs Wales</t>
+        </is>
+      </c>
+      <c r="C1856" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="D1856" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1856" t="inlineStr"/>
+      <c r="F1856" t="inlineStr"/>
+      <c r="G1856" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1856" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1856" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1856" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1856" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1856" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1857">
+      <c r="A1857" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1857" t="inlineStr">
+        <is>
+          <t>Austria vs Kosovo</t>
+        </is>
+      </c>
+      <c r="C1857" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="D1857" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1857" t="inlineStr"/>
+      <c r="F1857" t="inlineStr"/>
+      <c r="G1857" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1857" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1857" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1857" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1857" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1857" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1858">
+      <c r="A1858" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1858" t="inlineStr">
+        <is>
+          <t>Gibraltar vs Andorra</t>
+        </is>
+      </c>
+      <c r="C1858" t="inlineStr">
+        <is>
+          <t>Andorra</t>
+        </is>
+      </c>
+      <c r="D1858" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1858" t="inlineStr"/>
+      <c r="F1858" t="inlineStr"/>
+      <c r="G1858" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1858" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1858" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1858" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1858" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1858" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1859">
+      <c r="A1859" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1859" t="inlineStr">
+        <is>
+          <t>Burgos vs Eldense</t>
+        </is>
+      </c>
+      <c r="C1859" t="inlineStr">
+        <is>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="D1859" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1859" t="inlineStr"/>
+      <c r="F1859" t="inlineStr"/>
+      <c r="G1859" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1859" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1859" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1859" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1859" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1859" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1860">
+      <c r="A1860" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1860" t="inlineStr">
+        <is>
+          <t>Eibar vs Las Palmas</t>
+        </is>
+      </c>
+      <c r="C1860" t="inlineStr">
+        <is>
+          <t>Eibar</t>
+        </is>
+      </c>
+      <c r="D1860" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1860" t="inlineStr"/>
+      <c r="F1860" t="inlineStr"/>
+      <c r="G1860" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1860" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1860" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1860" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1860" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1860" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1861">
+      <c r="A1861" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1861" t="inlineStr">
+        <is>
+          <t>Malta vs Liechtenstein</t>
+        </is>
+      </c>
+      <c r="C1861" t="inlineStr">
+        <is>
+          <t>Malta</t>
+        </is>
+      </c>
+      <c r="D1861" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1861" t="inlineStr"/>
+      <c r="F1861" t="inlineStr"/>
+      <c r="G1861" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1861" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1861" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1861" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1861" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1861" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1862">
+      <c r="A1862" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1862" t="inlineStr">
+        <is>
+          <t>Jordan vs Syria</t>
+        </is>
+      </c>
+      <c r="C1862" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="D1862" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1862" t="inlineStr"/>
+      <c r="F1862" t="inlineStr"/>
+      <c r="G1862" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1862" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1862" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1862" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1862" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1862" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1863">
+      <c r="A1863" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1863" t="inlineStr">
+        <is>
+          <t>Pumas UNAM vs Atlético de San Luis</t>
+        </is>
+      </c>
+      <c r="C1863" t="inlineStr">
+        <is>
+          <t>Pumas UNAM</t>
+        </is>
+      </c>
+      <c r="D1863" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1863" t="inlineStr"/>
+      <c r="F1863" t="inlineStr"/>
+      <c r="G1863" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H1863" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1863" t="n">
+        <v>3</v>
+      </c>
+      <c r="J1863" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1863" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1863" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1864">
+      <c r="A1864" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1864" t="inlineStr">
+        <is>
+          <t>Juventud vs Cerro</t>
+        </is>
+      </c>
+      <c r="C1864" t="inlineStr">
+        <is>
+          <t>Juventud</t>
+        </is>
+      </c>
+      <c r="D1864" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1864" t="inlineStr"/>
+      <c r="F1864" t="inlineStr"/>
+      <c r="G1864" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1864" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1864" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1864" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1864" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1864" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1865">
+      <c r="A1865" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1865" t="inlineStr">
+        <is>
+          <t>Argentino de Quilmes vs Comunicaciones</t>
+        </is>
+      </c>
+      <c r="C1865" t="inlineStr">
+        <is>
+          <t>Comunicaciones</t>
+        </is>
+      </c>
+      <c r="D1865" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1865" t="inlineStr"/>
+      <c r="F1865" t="inlineStr"/>
+      <c r="G1865" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1865" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1865" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1865" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1865" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1865" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1866">
+      <c r="A1866" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1866" t="inlineStr">
+        <is>
+          <t>Villa Dálmine vs UAI Urquiza</t>
+        </is>
+      </c>
+      <c r="C1866" t="inlineStr">
+        <is>
+          <t>Villa Dálmine</t>
+        </is>
+      </c>
+      <c r="D1866" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1866" t="inlineStr"/>
+      <c r="F1866" t="inlineStr"/>
+      <c r="G1866" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1866" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1866" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1866" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1866" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1866" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1867">
+      <c r="A1867" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1867" t="inlineStr">
+        <is>
+          <t>Deportes Concepcion vs Curicó Unido</t>
+        </is>
+      </c>
+      <c r="C1867" t="inlineStr">
+        <is>
+          <t>Deportes Concepcion</t>
+        </is>
+      </c>
+      <c r="D1867" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1867" t="inlineStr"/>
+      <c r="F1867" t="inlineStr"/>
+      <c r="G1867" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1867" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1867" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1867" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1867" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1867" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1868">
+      <c r="A1868" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1868" t="inlineStr">
+        <is>
+          <t>Almagro vs Nueva Chicago</t>
+        </is>
+      </c>
+      <c r="C1868" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="D1868" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1868" t="inlineStr"/>
+      <c r="F1868" t="inlineStr"/>
+      <c r="G1868" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1868" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1868" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1868" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1868" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1868" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1869">
+      <c r="A1869" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1869" t="inlineStr">
+        <is>
+          <t>Atlanta vs Agropecuario</t>
+        </is>
+      </c>
+      <c r="C1869" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="D1869" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1869" t="inlineStr"/>
+      <c r="F1869" t="inlineStr"/>
+      <c r="G1869" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1869" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1869" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1869" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1869" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1869" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1870">
+      <c r="A1870" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1870" t="inlineStr">
+        <is>
+          <t>Germany vs Greece</t>
+        </is>
+      </c>
+      <c r="C1870" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D1870" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1870" t="inlineStr"/>
+      <c r="F1870" t="inlineStr"/>
+      <c r="G1870" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1870" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1870" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1870" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1870" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1870" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1871">
+      <c r="A1871" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1871" t="inlineStr">
+        <is>
+          <t>Israel vs Republic of Ireland</t>
+        </is>
+      </c>
+      <c r="C1871" t="inlineStr">
+        <is>
+          <t>Republic of Ireland</t>
+        </is>
+      </c>
+      <c r="D1871" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1871" t="inlineStr"/>
+      <c r="F1871" t="inlineStr"/>
+      <c r="G1871" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H1871" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1871" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1871" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1871" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1871" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1872">
+      <c r="A1872" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1872" t="inlineStr">
+        <is>
+          <t>Mitre (Santiago del Estero) vs San Telmo</t>
+        </is>
+      </c>
+      <c r="C1872" t="inlineStr">
+        <is>
+          <t>Mitre (Santiago del Estero)</t>
+        </is>
+      </c>
+      <c r="D1872" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1872" t="inlineStr"/>
+      <c r="F1872" t="inlineStr"/>
+      <c r="G1872" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1872" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1872" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1872" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1872" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1872" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1873">
+      <c r="A1873" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1873" t="inlineStr">
+        <is>
+          <t>CRB vs Cuiabá</t>
+        </is>
+      </c>
+      <c r="C1873" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="D1873" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1873" t="inlineStr"/>
+      <c r="F1873" t="inlineStr"/>
+      <c r="G1873" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1873" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1873" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1873" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1873" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1873" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1874">
+      <c r="A1874" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1874" t="inlineStr">
+        <is>
+          <t>Cobán Imperial vs Aurora FC</t>
+        </is>
+      </c>
+      <c r="C1874" t="inlineStr">
+        <is>
+          <t>Cobán Imperial</t>
+        </is>
+      </c>
+      <c r="D1874" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1874" t="inlineStr"/>
+      <c r="F1874" t="inlineStr"/>
+      <c r="G1874" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1874" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1874" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1874" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1874" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1874" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1875">
+      <c r="A1875" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1875" t="inlineStr">
+        <is>
+          <t>Real Oviedo vs Sporting Gijón</t>
+        </is>
+      </c>
+      <c r="C1875" t="inlineStr">
+        <is>
+          <t>Real Oviedo</t>
+        </is>
+      </c>
+      <c r="D1875" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1875" t="inlineStr"/>
+      <c r="F1875" t="inlineStr"/>
+      <c r="G1875" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1875" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1875" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1875" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1875" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1875" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1876">
+      <c r="A1876" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1876" t="inlineStr">
+        <is>
+          <t>Guyana vs Cayman Islands</t>
+        </is>
+      </c>
+      <c r="C1876" t="inlineStr">
+        <is>
+          <t>Guyana</t>
+        </is>
+      </c>
+      <c r="D1876" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1876" t="inlineStr"/>
+      <c r="F1876" t="inlineStr"/>
+      <c r="G1876" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1876" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1876" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1876" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1876" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1876" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1877">
+      <c r="A1877" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1877" t="inlineStr">
+        <is>
+          <t>Deportivo Maipú vs Temperley</t>
+        </is>
+      </c>
+      <c r="C1877" t="inlineStr">
+        <is>
+          <t>Deportivo Maipú</t>
+        </is>
+      </c>
+      <c r="D1877" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1877" t="inlineStr"/>
+      <c r="F1877" t="inlineStr"/>
+      <c r="G1877" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1877" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1877" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1877" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1877" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1877" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1878">
+      <c r="A1878" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1878" t="inlineStr">
+        <is>
+          <t>Midland vs Tristán Suárez</t>
+        </is>
+      </c>
+      <c r="C1878" t="inlineStr">
+        <is>
+          <t>Midland</t>
+        </is>
+      </c>
+      <c r="D1878" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1878" t="inlineStr"/>
+      <c r="F1878" t="inlineStr"/>
+      <c r="G1878" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1878" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1878" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1878" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1878" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1878" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1879">
+      <c r="A1879" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1879" t="inlineStr">
+        <is>
+          <t>Racing Club vs Boca Juniors</t>
+        </is>
+      </c>
+      <c r="C1879" t="inlineStr">
+        <is>
+          <t>Boca Juniors</t>
+        </is>
+      </c>
+      <c r="D1879" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1879" t="inlineStr"/>
+      <c r="F1879" t="inlineStr"/>
+      <c r="G1879" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H1879" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1879" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1879" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1879" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1879" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1880">
+      <c r="A1880" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1880" t="inlineStr">
+        <is>
+          <t>Bolivia vs Paraguay</t>
+        </is>
+      </c>
+      <c r="C1880" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D1880" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1880" t="inlineStr"/>
+      <c r="F1880" t="inlineStr"/>
+      <c r="G1880" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1880" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1880" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1880" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1880" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1880" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1881">
+      <c r="A1881" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1881" t="inlineStr">
+        <is>
+          <t>Defensor Sporting vs Danubio</t>
+        </is>
+      </c>
+      <c r="C1881" t="inlineStr">
+        <is>
+          <t>Defensor Sporting</t>
+        </is>
+      </c>
+      <c r="D1881" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1881" t="inlineStr"/>
+      <c r="F1881" t="inlineStr"/>
+      <c r="G1881" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1881" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1881" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1881" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1881" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1881" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1882">
+      <c r="A1882" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1882" t="inlineStr">
+        <is>
+          <t>Gimnasia y Tiro (Salta) vs Atletico Rafaela</t>
+        </is>
+      </c>
+      <c r="C1882" t="inlineStr">
+        <is>
+          <t>Gimnasia y Tiro (Salta)</t>
+        </is>
+      </c>
+      <c r="D1882" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1882" t="inlineStr"/>
+      <c r="F1882" t="inlineStr"/>
+      <c r="G1882" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1882" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1882" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1882" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1882" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1882" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1883">
+      <c r="A1883" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1883" t="inlineStr">
+        <is>
+          <t>Jaguares de Córdoba vs Alianza FC</t>
+        </is>
+      </c>
+      <c r="C1883" t="inlineStr">
+        <is>
+          <t>Jaguares de Córdoba</t>
+        </is>
+      </c>
+      <c r="D1883" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1883" t="inlineStr"/>
+      <c r="F1883" t="inlineStr"/>
+      <c r="G1883" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1883" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1883" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1883" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1883" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1883" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1884">
+      <c r="A1884" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1884" t="inlineStr">
+        <is>
+          <t>Deportivo Mixco vs Antigua GFC</t>
+        </is>
+      </c>
+      <c r="C1884" t="inlineStr">
+        <is>
+          <t>Deportivo Mixco</t>
+        </is>
+      </c>
+      <c r="D1884" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1884" t="inlineStr"/>
+      <c r="F1884" t="inlineStr"/>
+      <c r="G1884" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1884" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1884" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1884" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1884" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1884" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1885">
+      <c r="A1885" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1885" t="inlineStr">
+        <is>
+          <t>Bolívar vs Blooming</t>
+        </is>
+      </c>
+      <c r="C1885" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="D1885" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1885" t="inlineStr"/>
+      <c r="F1885" t="inlineStr"/>
+      <c r="G1885" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1885" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1885" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1885" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1885" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1885" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1886">
+      <c r="A1886" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1886" t="inlineStr">
+        <is>
+          <t>Fortaleza vs Athletic</t>
+        </is>
+      </c>
+      <c r="C1886" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="D1886" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1886" t="inlineStr"/>
+      <c r="F1886" t="inlineStr"/>
+      <c r="G1886" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H1886" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1886" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1886" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1886" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1886" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1887">
+      <c r="A1887" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1887" t="inlineStr">
+        <is>
+          <t>Columbus Crew vs Inter Miami CF</t>
+        </is>
+      </c>
+      <c r="C1887" t="inlineStr">
+        <is>
+          <t>Inter Miami CF</t>
+        </is>
+      </c>
+      <c r="D1887" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1887" t="inlineStr"/>
+      <c r="F1887" t="inlineStr"/>
+      <c r="G1887" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1887" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1887" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1887" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1887" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1887" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1888">
+      <c r="A1888" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1888" t="inlineStr">
+        <is>
+          <t>One Knoxville vs Westchester SC</t>
+        </is>
+      </c>
+      <c r="C1888" t="inlineStr">
+        <is>
+          <t>One Knoxville</t>
+        </is>
+      </c>
+      <c r="D1888" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1888" t="inlineStr"/>
+      <c r="F1888" t="inlineStr"/>
+      <c r="G1888" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1888" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1888" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1888" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1888" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1888" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1889">
+      <c r="A1889" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1889" t="inlineStr">
+        <is>
+          <t>Deportes Santa Cruz vs O'Higgins</t>
+        </is>
+      </c>
+      <c r="C1889" t="inlineStr">
+        <is>
+          <t>O'Higgins</t>
+        </is>
+      </c>
+      <c r="D1889" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1889" t="inlineStr"/>
+      <c r="F1889" t="inlineStr"/>
+      <c r="G1889" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H1889" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1889" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1889" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1889" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1889" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1890">
+      <c r="A1890" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1890" t="inlineStr">
+        <is>
+          <t>Haiti vs Costa Rica</t>
+        </is>
+      </c>
+      <c r="C1890" t="inlineStr">
+        <is>
+          <t>Costa Rica</t>
+        </is>
+      </c>
+      <c r="D1890" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1890" t="inlineStr"/>
+      <c r="F1890" t="inlineStr"/>
+      <c r="G1890" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1890" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1890" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1890" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1890" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1890" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1891">
+      <c r="A1891" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1891" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Real Oruro</t>
+        </is>
+      </c>
+      <c r="C1891" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="D1891" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1891" t="inlineStr"/>
+      <c r="F1891" t="inlineStr"/>
+      <c r="G1891" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1891" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1891" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1891" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1891" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1891" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1892">
+      <c r="A1892" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1892" t="inlineStr">
+        <is>
+          <t>León vs FC Juarez</t>
+        </is>
+      </c>
+      <c r="C1892" t="inlineStr">
+        <is>
+          <t>León</t>
+        </is>
+      </c>
+      <c r="D1892" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1892" t="inlineStr"/>
+      <c r="F1892" t="inlineStr"/>
+      <c r="G1892" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1892" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1892" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1892" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1892" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1892" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1893">
+      <c r="A1893" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1893" t="inlineStr">
+        <is>
+          <t>Deportivo Cali vs Águilas Doradas</t>
+        </is>
+      </c>
+      <c r="C1893" t="inlineStr">
+        <is>
+          <t>Deportivo Cali</t>
+        </is>
+      </c>
+      <c r="D1893" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1893" t="inlineStr"/>
+      <c r="F1893" t="inlineStr"/>
+      <c r="G1893" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1893" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1893" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1893" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1893" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1893" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1894">
+      <c r="A1894" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B1894" t="inlineStr">
+        <is>
+          <t>Necaxa vs América</t>
+        </is>
+      </c>
+      <c r="C1894" t="inlineStr">
+        <is>
+          <t>América</t>
+        </is>
+      </c>
+      <c r="D1894" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1894" t="inlineStr"/>
+      <c r="F1894" t="inlineStr"/>
+      <c r="G1894" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H1894" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1894" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1894" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1894" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1894" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -85361,7 +87673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85922,6 +88234,25 @@
       </c>
       <c r="E30" t="n">
         <v>92</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>52</v>
+      </c>
+      <c r="C31" t="n">
+        <v>37</v>
+      </c>
+      <c r="D31" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -85935,7 +88266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G170"/>
+  <dimension ref="A1:G174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -89835,6 +92166,114 @@
         <v>0</v>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D171" t="n">
+        <v>1</v>
+      </c>
+      <c r="E171" t="n">
+        <v>100</v>
+      </c>
+      <c r="F171" t="n">
+        <v>0</v>
+      </c>
+      <c r="G171" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>fav_domina_no_gana</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>3</v>
+      </c>
+      <c r="D172" t="n">
+        <v>1</v>
+      </c>
+      <c r="E172" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="F172" t="n">
+        <v>2</v>
+      </c>
+      <c r="G172" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>1</v>
+      </c>
+      <c r="D173" t="n">
+        <v>0</v>
+      </c>
+      <c r="E173" t="n">
+        <v>0</v>
+      </c>
+      <c r="F173" t="n">
+        <v>1</v>
+      </c>
+      <c r="G173" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>1</v>
+      </c>
+      <c r="D174" t="n">
+        <v>1</v>
+      </c>
+      <c r="E174" t="n">
+        <v>100</v>
+      </c>
+      <c r="F174" t="n">
+        <v>0</v>
+      </c>
+      <c r="G174" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-29
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1894"/>
+  <dimension ref="A1:L1921"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85187,8 +85187,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1843" t="inlineStr"/>
-      <c r="F1843" t="inlineStr"/>
       <c r="G1843" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -85235,8 +85233,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1844" t="inlineStr"/>
-      <c r="F1844" t="inlineStr"/>
       <c r="G1844" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -85283,8 +85279,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1845" t="inlineStr"/>
-      <c r="F1845" t="inlineStr"/>
       <c r="G1845" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -85331,8 +85325,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1846" t="inlineStr"/>
-      <c r="F1846" t="inlineStr"/>
       <c r="G1846" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -85379,8 +85371,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1847" t="inlineStr"/>
-      <c r="F1847" t="inlineStr"/>
       <c r="G1847" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -85427,8 +85417,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1848" t="inlineStr"/>
-      <c r="F1848" t="inlineStr"/>
       <c r="G1848" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -85475,8 +85463,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1849" t="inlineStr"/>
-      <c r="F1849" t="inlineStr"/>
       <c r="G1849" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -85523,8 +85509,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1850" t="inlineStr"/>
-      <c r="F1850" t="inlineStr"/>
       <c r="G1850" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -85571,8 +85555,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1851" t="inlineStr"/>
-      <c r="F1851" t="inlineStr"/>
       <c r="G1851" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -85619,8 +85601,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1852" t="inlineStr"/>
-      <c r="F1852" t="inlineStr"/>
       <c r="G1852" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -85667,8 +85647,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1853" t="inlineStr"/>
-      <c r="F1853" t="inlineStr"/>
       <c r="G1853" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -85715,8 +85693,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1854" t="inlineStr"/>
-      <c r="F1854" t="inlineStr"/>
       <c r="G1854" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -85763,8 +85739,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1855" t="inlineStr"/>
-      <c r="F1855" t="inlineStr"/>
       <c r="G1855" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -85811,8 +85785,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1856" t="inlineStr"/>
-      <c r="F1856" t="inlineStr"/>
       <c r="G1856" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -85859,8 +85831,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1857" t="inlineStr"/>
-      <c r="F1857" t="inlineStr"/>
       <c r="G1857" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -85907,8 +85877,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1858" t="inlineStr"/>
-      <c r="F1858" t="inlineStr"/>
       <c r="G1858" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -85955,8 +85923,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1859" t="inlineStr"/>
-      <c r="F1859" t="inlineStr"/>
       <c r="G1859" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -86003,8 +85969,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1860" t="inlineStr"/>
-      <c r="F1860" t="inlineStr"/>
       <c r="G1860" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -86051,8 +86015,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1861" t="inlineStr"/>
-      <c r="F1861" t="inlineStr"/>
       <c r="G1861" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -86099,8 +86061,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1862" t="inlineStr"/>
-      <c r="F1862" t="inlineStr"/>
       <c r="G1862" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -86147,8 +86107,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1863" t="inlineStr"/>
-      <c r="F1863" t="inlineStr"/>
       <c r="G1863" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -86195,8 +86153,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1864" t="inlineStr"/>
-      <c r="F1864" t="inlineStr"/>
       <c r="G1864" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -86243,8 +86199,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1865" t="inlineStr"/>
-      <c r="F1865" t="inlineStr"/>
       <c r="G1865" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -86291,8 +86245,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1866" t="inlineStr"/>
-      <c r="F1866" t="inlineStr"/>
       <c r="G1866" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -86339,8 +86291,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1867" t="inlineStr"/>
-      <c r="F1867" t="inlineStr"/>
       <c r="G1867" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -86387,8 +86337,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1868" t="inlineStr"/>
-      <c r="F1868" t="inlineStr"/>
       <c r="G1868" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -86435,8 +86383,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1869" t="inlineStr"/>
-      <c r="F1869" t="inlineStr"/>
       <c r="G1869" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -86483,8 +86429,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1870" t="inlineStr"/>
-      <c r="F1870" t="inlineStr"/>
       <c r="G1870" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -86531,8 +86475,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1871" t="inlineStr"/>
-      <c r="F1871" t="inlineStr"/>
       <c r="G1871" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -86579,8 +86521,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1872" t="inlineStr"/>
-      <c r="F1872" t="inlineStr"/>
       <c r="G1872" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -86627,8 +86567,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1873" t="inlineStr"/>
-      <c r="F1873" t="inlineStr"/>
       <c r="G1873" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -86675,8 +86613,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1874" t="inlineStr"/>
-      <c r="F1874" t="inlineStr"/>
       <c r="G1874" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -86723,8 +86659,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1875" t="inlineStr"/>
-      <c r="F1875" t="inlineStr"/>
       <c r="G1875" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -86771,8 +86705,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1876" t="inlineStr"/>
-      <c r="F1876" t="inlineStr"/>
       <c r="G1876" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -86819,8 +86751,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1877" t="inlineStr"/>
-      <c r="F1877" t="inlineStr"/>
       <c r="G1877" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -86867,8 +86797,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1878" t="inlineStr"/>
-      <c r="F1878" t="inlineStr"/>
       <c r="G1878" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -86915,8 +86843,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1879" t="inlineStr"/>
-      <c r="F1879" t="inlineStr"/>
       <c r="G1879" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -86963,8 +86889,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1880" t="inlineStr"/>
-      <c r="F1880" t="inlineStr"/>
       <c r="G1880" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -87011,8 +86935,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1881" t="inlineStr"/>
-      <c r="F1881" t="inlineStr"/>
       <c r="G1881" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -87059,8 +86981,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1882" t="inlineStr"/>
-      <c r="F1882" t="inlineStr"/>
       <c r="G1882" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -87107,8 +87027,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1883" t="inlineStr"/>
-      <c r="F1883" t="inlineStr"/>
       <c r="G1883" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -87155,8 +87073,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1884" t="inlineStr"/>
-      <c r="F1884" t="inlineStr"/>
       <c r="G1884" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -87203,8 +87119,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1885" t="inlineStr"/>
-      <c r="F1885" t="inlineStr"/>
       <c r="G1885" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -87251,8 +87165,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1886" t="inlineStr"/>
-      <c r="F1886" t="inlineStr"/>
       <c r="G1886" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -87299,8 +87211,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1887" t="inlineStr"/>
-      <c r="F1887" t="inlineStr"/>
       <c r="G1887" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -87347,8 +87257,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1888" t="inlineStr"/>
-      <c r="F1888" t="inlineStr"/>
       <c r="G1888" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -87395,8 +87303,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1889" t="inlineStr"/>
-      <c r="F1889" t="inlineStr"/>
       <c r="G1889" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -87443,8 +87349,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1890" t="inlineStr"/>
-      <c r="F1890" t="inlineStr"/>
       <c r="G1890" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -87491,8 +87395,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1891" t="inlineStr"/>
-      <c r="F1891" t="inlineStr"/>
       <c r="G1891" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -87539,8 +87441,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1892" t="inlineStr"/>
-      <c r="F1892" t="inlineStr"/>
       <c r="G1892" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -87587,8 +87487,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1893" t="inlineStr"/>
-      <c r="F1893" t="inlineStr"/>
       <c r="G1893" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -87635,8 +87533,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1894" t="inlineStr"/>
-      <c r="F1894" t="inlineStr"/>
       <c r="G1894" t="inlineStr">
         <is>
           <t>2-4</t>
@@ -87657,6 +87553,1302 @@
         <v>0</v>
       </c>
       <c r="L1894" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1895">
+      <c r="A1895" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1895" t="inlineStr">
+        <is>
+          <t>Australia vs Brazil</t>
+        </is>
+      </c>
+      <c r="C1895" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="D1895" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1895" t="inlineStr"/>
+      <c r="F1895" t="inlineStr"/>
+      <c r="G1895" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1895" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1895" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1895" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1895" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1895" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1896">
+      <c r="A1896" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1896" t="inlineStr">
+        <is>
+          <t>Ethiopia vs Senegal</t>
+        </is>
+      </c>
+      <c r="C1896" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="D1896" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1896" t="inlineStr"/>
+      <c r="F1896" t="inlineStr"/>
+      <c r="G1896" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1896" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1896" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1896" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1896" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1896" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1897">
+      <c r="A1897" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1897" t="inlineStr">
+        <is>
+          <t>Lesotho vs Morocco</t>
+        </is>
+      </c>
+      <c r="C1897" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="D1897" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1897" t="inlineStr"/>
+      <c r="F1897" t="inlineStr"/>
+      <c r="G1897" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1897" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1897" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1897" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1897" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1897" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1898">
+      <c r="A1898" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1898" t="inlineStr">
+        <is>
+          <t>South Sudan vs Egypt</t>
+        </is>
+      </c>
+      <c r="C1898" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="D1898" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1898" t="inlineStr"/>
+      <c r="F1898" t="inlineStr"/>
+      <c r="G1898" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1898" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1898" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1898" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1898" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1898" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1899">
+      <c r="A1899" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1899" t="inlineStr">
+        <is>
+          <t>Finland vs Belarus</t>
+        </is>
+      </c>
+      <c r="C1899" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D1899" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1899" t="inlineStr"/>
+      <c r="F1899" t="inlineStr"/>
+      <c r="G1899" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1899" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1899" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1899" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1899" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1899" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1900">
+      <c r="A1900" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1900" t="inlineStr">
+        <is>
+          <t>Cape Verde vs Rwanda</t>
+        </is>
+      </c>
+      <c r="C1900" t="inlineStr">
+        <is>
+          <t>Cape Verde</t>
+        </is>
+      </c>
+      <c r="D1900" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1900" t="inlineStr"/>
+      <c r="F1900" t="inlineStr"/>
+      <c r="G1900" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1900" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1900" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1900" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1900" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1900" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1901">
+      <c r="A1901" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1901" t="inlineStr">
+        <is>
+          <t>Boreham Wood vs Kidderminster Harriers</t>
+        </is>
+      </c>
+      <c r="C1901" t="inlineStr">
+        <is>
+          <t>Boreham Wood</t>
+        </is>
+      </c>
+      <c r="D1901" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1901" t="inlineStr"/>
+      <c r="F1901" t="inlineStr"/>
+      <c r="G1901" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1901" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1901" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1901" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1901" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1901" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1902">
+      <c r="A1902" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1902" t="inlineStr">
+        <is>
+          <t>Spain vs Croatia</t>
+        </is>
+      </c>
+      <c r="C1902" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D1902" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1902" t="inlineStr"/>
+      <c r="F1902" t="inlineStr"/>
+      <c r="G1902" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1902" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1902" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1902" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1902" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1902" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1903">
+      <c r="A1903" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1903" t="inlineStr">
+        <is>
+          <t>Czechia vs England</t>
+        </is>
+      </c>
+      <c r="C1903" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D1903" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1903" t="inlineStr"/>
+      <c r="F1903" t="inlineStr"/>
+      <c r="G1903" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1903" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1903" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1903" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1903" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1903" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1904">
+      <c r="A1904" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1904" t="inlineStr">
+        <is>
+          <t>San Marino vs Albania</t>
+        </is>
+      </c>
+      <c r="C1904" t="inlineStr">
+        <is>
+          <t>Albania</t>
+        </is>
+      </c>
+      <c r="D1904" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1904" t="inlineStr"/>
+      <c r="F1904" t="inlineStr"/>
+      <c r="G1904" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1904" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1904" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1904" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1904" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1904" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1905">
+      <c r="A1905" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1905" t="inlineStr">
+        <is>
+          <t>Slovakia vs Kazakhstan</t>
+        </is>
+      </c>
+      <c r="C1905" t="inlineStr">
+        <is>
+          <t>Slovakia</t>
+        </is>
+      </c>
+      <c r="D1905" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1905" t="inlineStr"/>
+      <c r="F1905" t="inlineStr"/>
+      <c r="G1905" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1905" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1905" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1905" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1905" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1905" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1906">
+      <c r="A1906" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1906" t="inlineStr">
+        <is>
+          <t>Bulgaria vs Estonia</t>
+        </is>
+      </c>
+      <c r="C1906" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="D1906" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1906" t="inlineStr"/>
+      <c r="F1906" t="inlineStr"/>
+      <c r="G1906" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1906" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1906" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1906" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1906" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1906" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1907">
+      <c r="A1907" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1907" t="inlineStr">
+        <is>
+          <t>Luxembourg vs Iceland</t>
+        </is>
+      </c>
+      <c r="C1907" t="inlineStr">
+        <is>
+          <t>Iceland</t>
+        </is>
+      </c>
+      <c r="D1907" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1907" t="inlineStr"/>
+      <c r="F1907" t="inlineStr"/>
+      <c r="G1907" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1907" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1907" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1907" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1907" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1907" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1908">
+      <c r="A1908" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1908" t="inlineStr">
+        <is>
+          <t>Scotland vs Switzerland</t>
+        </is>
+      </c>
+      <c r="C1908" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D1908" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1908" t="inlineStr"/>
+      <c r="F1908" t="inlineStr"/>
+      <c r="G1908" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1908" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1908" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1908" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1908" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1908" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1909">
+      <c r="A1909" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1909" t="inlineStr">
+        <is>
+          <t>Slovenia vs North Macedonia</t>
+        </is>
+      </c>
+      <c r="C1909" t="inlineStr">
+        <is>
+          <t>Slovenia</t>
+        </is>
+      </c>
+      <c r="D1909" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1909" t="inlineStr"/>
+      <c r="F1909" t="inlineStr"/>
+      <c r="G1909" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1909" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1909" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1909" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1909" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1909" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1910">
+      <c r="A1910" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1910" t="inlineStr">
+        <is>
+          <t>Barrow vs Scunthorpe United</t>
+        </is>
+      </c>
+      <c r="C1910" t="inlineStr">
+        <is>
+          <t>Barrow</t>
+        </is>
+      </c>
+      <c r="D1910" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1910" t="inlineStr"/>
+      <c r="F1910" t="inlineStr"/>
+      <c r="G1910" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1910" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1910" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1910" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1910" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1910" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1911">
+      <c r="A1911" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1911" t="inlineStr">
+        <is>
+          <t>FC Halifax Town vs Boston United</t>
+        </is>
+      </c>
+      <c r="C1911" t="inlineStr">
+        <is>
+          <t>FC Halifax Town</t>
+        </is>
+      </c>
+      <c r="D1911" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1911" t="inlineStr"/>
+      <c r="F1911" t="inlineStr"/>
+      <c r="G1911" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1911" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1911" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1911" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1911" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1911" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1912">
+      <c r="A1912" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1912" t="inlineStr">
+        <is>
+          <t>Forest Green Rovers vs Wealdstone</t>
+        </is>
+      </c>
+      <c r="C1912" t="inlineStr">
+        <is>
+          <t>Forest Green Rovers</t>
+        </is>
+      </c>
+      <c r="D1912" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1912" t="inlineStr"/>
+      <c r="F1912" t="inlineStr"/>
+      <c r="G1912" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1912" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1912" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1912" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1912" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1912" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1913">
+      <c r="A1913" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1913" t="inlineStr">
+        <is>
+          <t>Gateshead vs Altrincham</t>
+        </is>
+      </c>
+      <c r="C1913" t="inlineStr">
+        <is>
+          <t>Altrincham</t>
+        </is>
+      </c>
+      <c r="D1913" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1913" t="inlineStr"/>
+      <c r="F1913" t="inlineStr"/>
+      <c r="G1913" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1913" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1913" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1913" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1913" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1913" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1914">
+      <c r="A1914" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1914" t="inlineStr">
+        <is>
+          <t>Hartlepool United vs Harrogate Town</t>
+        </is>
+      </c>
+      <c r="C1914" t="inlineStr">
+        <is>
+          <t>Harrogate Town</t>
+        </is>
+      </c>
+      <c r="D1914" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1914" t="inlineStr"/>
+      <c r="F1914" t="inlineStr"/>
+      <c r="G1914" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1914" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1914" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1914" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1914" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1914" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1915">
+      <c r="A1915" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1915" t="inlineStr">
+        <is>
+          <t>AFC Hornchurch vs Aldershot Town</t>
+        </is>
+      </c>
+      <c r="C1915" t="inlineStr">
+        <is>
+          <t>AFC Hornchurch</t>
+        </is>
+      </c>
+      <c r="D1915" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1915" t="inlineStr"/>
+      <c r="F1915" t="inlineStr"/>
+      <c r="G1915" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1915" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1915" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1915" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1915" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1915" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1916">
+      <c r="A1916" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1916" t="inlineStr">
+        <is>
+          <t>Woking vs Solihull Moors</t>
+        </is>
+      </c>
+      <c r="C1916" t="inlineStr">
+        <is>
+          <t>Woking</t>
+        </is>
+      </c>
+      <c r="D1916" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1916" t="inlineStr"/>
+      <c r="F1916" t="inlineStr"/>
+      <c r="G1916" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1916" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1916" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1916" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1916" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1916" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1917">
+      <c r="A1917" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1917" t="inlineStr">
+        <is>
+          <t>Yeovil Town vs Worthing</t>
+        </is>
+      </c>
+      <c r="C1917" t="inlineStr">
+        <is>
+          <t>Yeovil Town</t>
+        </is>
+      </c>
+      <c r="D1917" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1917" t="inlineStr"/>
+      <c r="F1917" t="inlineStr"/>
+      <c r="G1917" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1917" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1917" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1917" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1917" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1917" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1918">
+      <c r="A1918" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1918" t="inlineStr">
+        <is>
+          <t>Forfar Athletic vs Formartine United</t>
+        </is>
+      </c>
+      <c r="C1918" t="inlineStr">
+        <is>
+          <t>Forfar Athletic</t>
+        </is>
+      </c>
+      <c r="D1918" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1918" t="inlineStr"/>
+      <c r="F1918" t="inlineStr"/>
+      <c r="G1918" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1918" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1918" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1918" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1918" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1918" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1919">
+      <c r="A1919" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1919" t="inlineStr">
+        <is>
+          <t>Congo vs Cameroon</t>
+        </is>
+      </c>
+      <c r="C1919" t="inlineStr">
+        <is>
+          <t>Cameroon</t>
+        </is>
+      </c>
+      <c r="D1919" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1919" t="inlineStr"/>
+      <c r="F1919" t="inlineStr"/>
+      <c r="G1919" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1919" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1919" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1919" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1919" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1919" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1920">
+      <c r="A1920" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1920" t="inlineStr">
+        <is>
+          <t>Deportivo Pereira vs Independiente Santa Fe</t>
+        </is>
+      </c>
+      <c r="C1920" t="inlineStr">
+        <is>
+          <t>Independiente Santa Fe</t>
+        </is>
+      </c>
+      <c r="D1920" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1920" t="inlineStr"/>
+      <c r="F1920" t="inlineStr"/>
+      <c r="G1920" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1920" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1920" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1920" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1920" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1920" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1921">
+      <c r="A1921" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1921" t="inlineStr">
+        <is>
+          <t>Botafogo-SP vs Ponte Preta</t>
+        </is>
+      </c>
+      <c r="C1921" t="inlineStr">
+        <is>
+          <t>Botafogo-SP</t>
+        </is>
+      </c>
+      <c r="D1921" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1921" t="inlineStr"/>
+      <c r="F1921" t="inlineStr"/>
+      <c r="G1921" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1921" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1921" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1921" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1921" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1921" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -87673,7 +88865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -88253,6 +89445,25 @@
       </c>
       <c r="E31" t="n">
         <v>53</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>27</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>100</v>
+      </c>
+      <c r="E32" t="n">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-30
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1921"/>
+  <dimension ref="A1:L1928"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -87579,8 +87579,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1895" t="inlineStr"/>
-      <c r="F1895" t="inlineStr"/>
       <c r="G1895" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -87627,8 +87625,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1896" t="inlineStr"/>
-      <c r="F1896" t="inlineStr"/>
       <c r="G1896" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -87675,8 +87671,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1897" t="inlineStr"/>
-      <c r="F1897" t="inlineStr"/>
       <c r="G1897" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -87723,8 +87717,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1898" t="inlineStr"/>
-      <c r="F1898" t="inlineStr"/>
       <c r="G1898" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -87771,8 +87763,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1899" t="inlineStr"/>
-      <c r="F1899" t="inlineStr"/>
       <c r="G1899" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -87819,8 +87809,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1900" t="inlineStr"/>
-      <c r="F1900" t="inlineStr"/>
       <c r="G1900" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -87867,8 +87855,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1901" t="inlineStr"/>
-      <c r="F1901" t="inlineStr"/>
       <c r="G1901" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -87915,8 +87901,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1902" t="inlineStr"/>
-      <c r="F1902" t="inlineStr"/>
       <c r="G1902" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -87963,8 +87947,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1903" t="inlineStr"/>
-      <c r="F1903" t="inlineStr"/>
       <c r="G1903" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88011,8 +87993,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1904" t="inlineStr"/>
-      <c r="F1904" t="inlineStr"/>
       <c r="G1904" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88059,8 +88039,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1905" t="inlineStr"/>
-      <c r="F1905" t="inlineStr"/>
       <c r="G1905" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88107,8 +88085,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1906" t="inlineStr"/>
-      <c r="F1906" t="inlineStr"/>
       <c r="G1906" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88155,8 +88131,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1907" t="inlineStr"/>
-      <c r="F1907" t="inlineStr"/>
       <c r="G1907" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88203,8 +88177,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1908" t="inlineStr"/>
-      <c r="F1908" t="inlineStr"/>
       <c r="G1908" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88251,8 +88223,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1909" t="inlineStr"/>
-      <c r="F1909" t="inlineStr"/>
       <c r="G1909" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88299,8 +88269,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1910" t="inlineStr"/>
-      <c r="F1910" t="inlineStr"/>
       <c r="G1910" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88347,8 +88315,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1911" t="inlineStr"/>
-      <c r="F1911" t="inlineStr"/>
       <c r="G1911" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88395,8 +88361,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1912" t="inlineStr"/>
-      <c r="F1912" t="inlineStr"/>
       <c r="G1912" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88443,8 +88407,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1913" t="inlineStr"/>
-      <c r="F1913" t="inlineStr"/>
       <c r="G1913" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88491,8 +88453,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1914" t="inlineStr"/>
-      <c r="F1914" t="inlineStr"/>
       <c r="G1914" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88539,8 +88499,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1915" t="inlineStr"/>
-      <c r="F1915" t="inlineStr"/>
       <c r="G1915" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88587,8 +88545,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1916" t="inlineStr"/>
-      <c r="F1916" t="inlineStr"/>
       <c r="G1916" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88635,8 +88591,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1917" t="inlineStr"/>
-      <c r="F1917" t="inlineStr"/>
       <c r="G1917" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88683,8 +88637,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1918" t="inlineStr"/>
-      <c r="F1918" t="inlineStr"/>
       <c r="G1918" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -88731,8 +88683,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1919" t="inlineStr"/>
-      <c r="F1919" t="inlineStr"/>
       <c r="G1919" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88779,8 +88729,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1920" t="inlineStr"/>
-      <c r="F1920" t="inlineStr"/>
       <c r="G1920" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88827,8 +88775,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1921" t="inlineStr"/>
-      <c r="F1921" t="inlineStr"/>
       <c r="G1921" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -88849,6 +88795,342 @@
         <v>0</v>
       </c>
       <c r="L1921" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1922">
+      <c r="A1922" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1922" t="inlineStr">
+        <is>
+          <t>Eastleigh vs Southend United</t>
+        </is>
+      </c>
+      <c r="C1922" t="inlineStr">
+        <is>
+          <t>Southend United</t>
+        </is>
+      </c>
+      <c r="D1922" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1922" t="inlineStr"/>
+      <c r="F1922" t="inlineStr"/>
+      <c r="G1922" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1922" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1922" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1922" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1922" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1922" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1923">
+      <c r="A1923" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1923" t="inlineStr">
+        <is>
+          <t>Tamworth vs Sutton United</t>
+        </is>
+      </c>
+      <c r="C1923" t="inlineStr">
+        <is>
+          <t>Tamworth</t>
+        </is>
+      </c>
+      <c r="D1923" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1923" t="inlineStr"/>
+      <c r="F1923" t="inlineStr"/>
+      <c r="G1923" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1923" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1923" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1923" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1923" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1923" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1924">
+      <c r="A1924" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1924" t="inlineStr">
+        <is>
+          <t>Cienciano del Cusco vs Los Chankas</t>
+        </is>
+      </c>
+      <c r="C1924" t="inlineStr">
+        <is>
+          <t>Cienciano del Cusco</t>
+        </is>
+      </c>
+      <c r="D1924" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1924" t="inlineStr"/>
+      <c r="F1924" t="inlineStr"/>
+      <c r="G1924" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1924" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1924" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1924" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1924" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1924" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1925">
+      <c r="A1925" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1925" t="inlineStr">
+        <is>
+          <t>Brooklyn FC vs Detroit City FC</t>
+        </is>
+      </c>
+      <c r="C1925" t="inlineStr">
+        <is>
+          <t>Detroit City FC</t>
+        </is>
+      </c>
+      <c r="D1925" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1925" t="inlineStr"/>
+      <c r="F1925" t="inlineStr"/>
+      <c r="G1925" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1925" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1925" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1925" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1925" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1925" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1926">
+      <c r="A1926" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1926" t="inlineStr">
+        <is>
+          <t>Miami FC vs Sporting JAX</t>
+        </is>
+      </c>
+      <c r="C1926" t="inlineStr">
+        <is>
+          <t>Miami FC</t>
+        </is>
+      </c>
+      <c r="D1926" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1926" t="inlineStr"/>
+      <c r="F1926" t="inlineStr"/>
+      <c r="G1926" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1926" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1926" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1926" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1926" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1926" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1927">
+      <c r="A1927" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1927" t="inlineStr">
+        <is>
+          <t>Rhode Island FC vs Indy Eleven</t>
+        </is>
+      </c>
+      <c r="C1927" t="inlineStr">
+        <is>
+          <t>Rhode Island FC</t>
+        </is>
+      </c>
+      <c r="D1927" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1927" t="inlineStr"/>
+      <c r="F1927" t="inlineStr"/>
+      <c r="G1927" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1927" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1927" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1927" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1927" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1927" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1928">
+      <c r="A1928" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1928" t="inlineStr">
+        <is>
+          <t>D.C. United vs SC Paderborn 07</t>
+        </is>
+      </c>
+      <c r="C1928" t="inlineStr">
+        <is>
+          <t>SC Paderborn 07</t>
+        </is>
+      </c>
+      <c r="D1928" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1928" t="inlineStr"/>
+      <c r="F1928" t="inlineStr"/>
+      <c r="G1928" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H1928" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I1928" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1928" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1928" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1928" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -88865,7 +89147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -89464,6 +89746,22 @@
       </c>
       <c r="E32" t="n">
         <v>101</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>7</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 1: seleccion de partidos 2026-10-01
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1928"/>
+  <dimension ref="A1:L1952"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -88808,12 +88808,12 @@
       </c>
       <c r="B1922" t="inlineStr">
         <is>
-          <t>Eastleigh vs Southend United</t>
+          <t>Papua New Guinea vs Solomon Islands</t>
         </is>
       </c>
       <c r="C1922" t="inlineStr">
         <is>
-          <t>Southend United</t>
+          <t>Solomon Islands</t>
         </is>
       </c>
       <c r="D1922" t="inlineStr">
@@ -88825,12 +88825,12 @@
       <c r="F1922" t="inlineStr"/>
       <c r="G1922" t="inlineStr">
         <is>
-          <t>sin resolver</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="H1922" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="I1922" t="n">
@@ -88856,12 +88856,12 @@
       </c>
       <c r="B1923" t="inlineStr">
         <is>
-          <t>Tamworth vs Sutton United</t>
+          <t>Fiji vs New Caledonia</t>
         </is>
       </c>
       <c r="C1923" t="inlineStr">
         <is>
-          <t>Tamworth</t>
+          <t>Fiji</t>
         </is>
       </c>
       <c r="D1923" t="inlineStr">
@@ -88873,12 +88873,12 @@
       <c r="F1923" t="inlineStr"/>
       <c r="G1923" t="inlineStr">
         <is>
-          <t>sin resolver</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="H1923" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="I1923" t="n">
@@ -88904,29 +88904,29 @@
       </c>
       <c r="B1924" t="inlineStr">
         <is>
-          <t>Cienciano del Cusco vs Los Chankas</t>
+          <t>Seychelles vs Sri Lanka</t>
         </is>
       </c>
       <c r="C1924" t="inlineStr">
         <is>
-          <t>Cienciano del Cusco</t>
+          <t>Sri Lanka</t>
         </is>
       </c>
       <c r="D1924" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Visitante</t>
         </is>
       </c>
       <c r="E1924" t="inlineStr"/>
       <c r="F1924" t="inlineStr"/>
       <c r="G1924" t="inlineStr">
         <is>
-          <t>sin resolver</t>
+          <t>0-2</t>
         </is>
       </c>
       <c r="H1924" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="I1924" t="n">
@@ -88952,12 +88952,12 @@
       </c>
       <c r="B1925" t="inlineStr">
         <is>
-          <t>Brooklyn FC vs Detroit City FC</t>
+          <t>Eritrea vs South Africa</t>
         </is>
       </c>
       <c r="C1925" t="inlineStr">
         <is>
-          <t>Detroit City FC</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="D1925" t="inlineStr">
@@ -88969,12 +88969,12 @@
       <c r="F1925" t="inlineStr"/>
       <c r="G1925" t="inlineStr">
         <is>
-          <t>sin resolver</t>
+          <t>0-5</t>
         </is>
       </c>
       <c r="H1925" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="I1925" t="n">
@@ -89000,12 +89000,12 @@
       </c>
       <c r="B1926" t="inlineStr">
         <is>
-          <t>Miami FC vs Sporting JAX</t>
+          <t>Lithuania vs Andorra</t>
         </is>
       </c>
       <c r="C1926" t="inlineStr">
         <is>
-          <t>Miami FC</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="D1926" t="inlineStr">
@@ -89017,12 +89017,12 @@
       <c r="F1926" t="inlineStr"/>
       <c r="G1926" t="inlineStr">
         <is>
-          <t>sin resolver</t>
+          <t>3-0</t>
         </is>
       </c>
       <c r="H1926" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="I1926" t="n">
@@ -89048,29 +89048,29 @@
       </c>
       <c r="B1927" t="inlineStr">
         <is>
-          <t>Rhode Island FC vs Indy Eleven</t>
+          <t>SC Kalsdorf vs Grazer AK</t>
         </is>
       </c>
       <c r="C1927" t="inlineStr">
         <is>
-          <t>Rhode Island FC</t>
+          <t>Grazer AK</t>
         </is>
       </c>
       <c r="D1927" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Visitante</t>
         </is>
       </c>
       <c r="E1927" t="inlineStr"/>
       <c r="F1927" t="inlineStr"/>
       <c r="G1927" t="inlineStr">
         <is>
-          <t>sin resolver</t>
+          <t>1-5</t>
         </is>
       </c>
       <c r="H1927" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="I1927" t="n">
@@ -89096,41 +89096,1193 @@
       </c>
       <c r="B1928" t="inlineStr">
         <is>
-          <t>D.C. United vs SC Paderborn 07</t>
+          <t>Faroe Islands U21 vs Luxembourg U21</t>
         </is>
       </c>
       <c r="C1928" t="inlineStr">
         <is>
-          <t>SC Paderborn 07</t>
+          <t>Faroe Islands U21</t>
         </is>
       </c>
       <c r="D1928" t="inlineStr">
         <is>
-          <t>Visitante</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="E1928" t="inlineStr"/>
       <c r="F1928" t="inlineStr"/>
       <c r="G1928" t="inlineStr">
         <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1928" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1928" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1928" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1928" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1928" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1929">
+      <c r="A1929" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1929" t="inlineStr">
+        <is>
+          <t>Romania U21 vs Finland U21</t>
+        </is>
+      </c>
+      <c r="C1929" t="inlineStr">
+        <is>
+          <t>Romania U21</t>
+        </is>
+      </c>
+      <c r="D1929" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1929" t="inlineStr"/>
+      <c r="F1929" t="inlineStr"/>
+      <c r="G1929" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1929" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1929" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1929" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1929" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1929" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1930">
+      <c r="A1930" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1930" t="inlineStr">
+        <is>
+          <t>Poland U21 vs Sweden U21</t>
+        </is>
+      </c>
+      <c r="C1930" t="inlineStr">
+        <is>
+          <t>Poland U21</t>
+        </is>
+      </c>
+      <c r="D1930" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1930" t="inlineStr"/>
+      <c r="F1930" t="inlineStr"/>
+      <c r="G1930" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1930" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1930" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1930" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1930" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1930" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1931">
+      <c r="A1931" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1931" t="inlineStr">
+        <is>
+          <t>Malta U21 vs Germany U21</t>
+        </is>
+      </c>
+      <c r="C1931" t="inlineStr">
+        <is>
+          <t>Germany U21</t>
+        </is>
+      </c>
+      <c r="D1931" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1931" t="inlineStr"/>
+      <c r="F1931" t="inlineStr"/>
+      <c r="G1931" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H1931" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1931" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1931" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1931" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1931" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1932">
+      <c r="A1932" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1932" t="inlineStr">
+        <is>
+          <t>Kosovo U21 vs Cyprus U21</t>
+        </is>
+      </c>
+      <c r="C1932" t="inlineStr">
+        <is>
+          <t>Kosovo U21</t>
+        </is>
+      </c>
+      <c r="D1932" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1932" t="inlineStr"/>
+      <c r="F1932" t="inlineStr"/>
+      <c r="G1932" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1932" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1932" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1932" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1932" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1932" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1933">
+      <c r="A1933" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1933" t="inlineStr">
+        <is>
+          <t>United Arab Emirates vs Qatar</t>
+        </is>
+      </c>
+      <c r="C1933" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="D1933" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1933" t="inlineStr"/>
+      <c r="F1933" t="inlineStr"/>
+      <c r="G1933" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1933" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1933" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1933" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1933" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1933" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1934">
+      <c r="A1934" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1934" t="inlineStr">
+        <is>
+          <t>Bahrain vs Yemen</t>
+        </is>
+      </c>
+      <c r="C1934" t="inlineStr">
+        <is>
+          <t>Bahrain</t>
+        </is>
+      </c>
+      <c r="D1934" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1934" t="inlineStr"/>
+      <c r="F1934" t="inlineStr"/>
+      <c r="G1934" t="inlineStr">
+        <is>
+          <t>2-5</t>
+        </is>
+      </c>
+      <c r="H1934" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1934" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1934" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1934" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1934" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1935">
+      <c r="A1935" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1935" t="inlineStr">
+        <is>
+          <t>Scotland U21 vs Azerbaijan U21</t>
+        </is>
+      </c>
+      <c r="C1935" t="inlineStr">
+        <is>
+          <t>Scotland U21</t>
+        </is>
+      </c>
+      <c r="D1935" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1935" t="inlineStr"/>
+      <c r="F1935" t="inlineStr"/>
+      <c r="G1935" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H1935" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1935" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1935" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1935" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1935" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1936">
+      <c r="A1936" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1936" t="inlineStr">
+        <is>
+          <t>Eastleigh vs Southend United</t>
+        </is>
+      </c>
+      <c r="C1936" t="inlineStr">
+        <is>
+          <t>Southend United</t>
+        </is>
+      </c>
+      <c r="D1936" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1936" t="inlineStr"/>
+      <c r="F1936" t="inlineStr"/>
+      <c r="G1936" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1936" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1936" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1936" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1936" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1936" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1937">
+      <c r="A1937" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1937" t="inlineStr">
+        <is>
+          <t>Tamworth vs Sutton United</t>
+        </is>
+      </c>
+      <c r="C1937" t="inlineStr">
+        <is>
+          <t>Tamworth</t>
+        </is>
+      </c>
+      <c r="D1937" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1937" t="inlineStr"/>
+      <c r="F1937" t="inlineStr"/>
+      <c r="G1937" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1937" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1937" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1937" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1937" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1937" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1938">
+      <c r="A1938" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1938" t="inlineStr">
+        <is>
+          <t>Portugal U21 vs Gibraltar U21</t>
+        </is>
+      </c>
+      <c r="C1938" t="inlineStr">
+        <is>
+          <t>Portugal U21</t>
+        </is>
+      </c>
+      <c r="D1938" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1938" t="inlineStr"/>
+      <c r="F1938" t="inlineStr"/>
+      <c r="G1938" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H1938" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1938" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1938" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1938" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1938" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1939">
+      <c r="A1939" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1939" t="inlineStr">
+        <is>
+          <t>Cienciano del Cusco vs Los Chankas</t>
+        </is>
+      </c>
+      <c r="C1939" t="inlineStr">
+        <is>
+          <t>Cienciano del Cusco</t>
+        </is>
+      </c>
+      <c r="D1939" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1939" t="inlineStr"/>
+      <c r="F1939" t="inlineStr"/>
+      <c r="G1939" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1939" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1939" t="n">
+        <v>6</v>
+      </c>
+      <c r="J1939" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1939" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1939" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1940">
+      <c r="A1940" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1940" t="inlineStr">
+        <is>
+          <t>Águila vs Internacional Santa Tecla</t>
+        </is>
+      </c>
+      <c r="C1940" t="inlineStr">
+        <is>
+          <t>Águila</t>
+        </is>
+      </c>
+      <c r="D1940" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1940" t="inlineStr"/>
+      <c r="F1940" t="inlineStr"/>
+      <c r="G1940" t="inlineStr">
+        <is>
           <t>sin resolver</t>
         </is>
       </c>
-      <c r="H1928" t="inlineStr">
+      <c r="H1940" t="inlineStr">
         <is>
           <t>?</t>
         </is>
       </c>
-      <c r="I1928" t="n">
-        <v>0</v>
-      </c>
-      <c r="J1928" t="n">
-        <v>0</v>
-      </c>
-      <c r="K1928" t="n">
-        <v>0</v>
-      </c>
-      <c r="L1928" t="inlineStr">
+      <c r="I1940" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1940" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1940" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1940" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1941">
+      <c r="A1941" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1941" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Nacional Potosí</t>
+        </is>
+      </c>
+      <c r="C1941" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="D1941" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1941" t="inlineStr"/>
+      <c r="F1941" t="inlineStr"/>
+      <c r="G1941" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1941" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1941" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1941" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1941" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1941" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1942">
+      <c r="A1942" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1942" t="inlineStr">
+        <is>
+          <t>Brooklyn FC vs Detroit City FC</t>
+        </is>
+      </c>
+      <c r="C1942" t="inlineStr">
+        <is>
+          <t>Detroit City FC</t>
+        </is>
+      </c>
+      <c r="D1942" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1942" t="inlineStr"/>
+      <c r="F1942" t="inlineStr"/>
+      <c r="G1942" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H1942" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1942" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1942" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1942" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1942" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1943">
+      <c r="A1943" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1943" t="inlineStr">
+        <is>
+          <t>Miami FC vs Sporting JAX</t>
+        </is>
+      </c>
+      <c r="C1943" t="inlineStr">
+        <is>
+          <t>Miami FC</t>
+        </is>
+      </c>
+      <c r="D1943" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1943" t="inlineStr"/>
+      <c r="F1943" t="inlineStr"/>
+      <c r="G1943" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H1943" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1943" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1943" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1943" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1943" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1944">
+      <c r="A1944" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1944" t="inlineStr">
+        <is>
+          <t>Rhode Island FC vs Indy Eleven</t>
+        </is>
+      </c>
+      <c r="C1944" t="inlineStr">
+        <is>
+          <t>Rhode Island FC</t>
+        </is>
+      </c>
+      <c r="D1944" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1944" t="inlineStr"/>
+      <c r="F1944" t="inlineStr"/>
+      <c r="G1944" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1944" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1944" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1944" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1944" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1944" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1945">
+      <c r="A1945" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1945" t="inlineStr">
+        <is>
+          <t>D.C. United vs SC Paderborn 07</t>
+        </is>
+      </c>
+      <c r="C1945" t="inlineStr">
+        <is>
+          <t>SC Paderborn 07</t>
+        </is>
+      </c>
+      <c r="D1945" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1945" t="inlineStr"/>
+      <c r="F1945" t="inlineStr"/>
+      <c r="G1945" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1945" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1945" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1945" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1945" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1945" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1946">
+      <c r="A1946" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1946" t="inlineStr">
+        <is>
+          <t>Alianza FC vs C.D. Platense</t>
+        </is>
+      </c>
+      <c r="C1946" t="inlineStr">
+        <is>
+          <t>Alianza FC</t>
+        </is>
+      </c>
+      <c r="D1946" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1946" t="inlineStr"/>
+      <c r="F1946" t="inlineStr"/>
+      <c r="G1946" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1946" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1946" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1946" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1946" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1946" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1947">
+      <c r="A1947" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1947" t="inlineStr">
+        <is>
+          <t>FC Tulsa vs New Mexico United</t>
+        </is>
+      </c>
+      <c r="C1947" t="inlineStr">
+        <is>
+          <t>FC Tulsa</t>
+        </is>
+      </c>
+      <c r="D1947" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1947" t="inlineStr"/>
+      <c r="F1947" t="inlineStr"/>
+      <c r="G1947" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1947" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1947" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1947" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1947" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1947" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1948">
+      <c r="A1948" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1948" t="inlineStr">
+        <is>
+          <t>Argentina vs Bolivia</t>
+        </is>
+      </c>
+      <c r="C1948" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="D1948" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1948" t="inlineStr"/>
+      <c r="F1948" t="inlineStr"/>
+      <c r="G1948" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H1948" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1948" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1948" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1948" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1948" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1949">
+      <c r="A1949" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1949" t="inlineStr">
+        <is>
+          <t>Oriente Petrolero vs The Strongest</t>
+        </is>
+      </c>
+      <c r="C1949" t="inlineStr">
+        <is>
+          <t>Oriente Petrolero</t>
+        </is>
+      </c>
+      <c r="D1949" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1949" t="inlineStr"/>
+      <c r="F1949" t="inlineStr"/>
+      <c r="G1949" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1949" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1949" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1949" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1949" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1949" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1950">
+      <c r="A1950" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1950" t="inlineStr">
+        <is>
+          <t>Atlético Nacional vs Atlético Junior</t>
+        </is>
+      </c>
+      <c r="C1950" t="inlineStr">
+        <is>
+          <t>Atlético Nacional</t>
+        </is>
+      </c>
+      <c r="D1950" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1950" t="inlineStr"/>
+      <c r="F1950" t="inlineStr"/>
+      <c r="G1950" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1950" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1950" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1950" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1950" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1950" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1951">
+      <c r="A1951" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1951" t="inlineStr">
+        <is>
+          <t>CD FAS vs Isidro Metapán</t>
+        </is>
+      </c>
+      <c r="C1951" t="inlineStr">
+        <is>
+          <t>CD FAS</t>
+        </is>
+      </c>
+      <c r="D1951" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1951" t="inlineStr"/>
+      <c r="F1951" t="inlineStr"/>
+      <c r="G1951" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1951" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1951" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1951" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1951" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1951" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1952">
+      <c r="A1952" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1952" t="inlineStr">
+        <is>
+          <t>Sacramento Republic FC vs Las Vegas Lights FC</t>
+        </is>
+      </c>
+      <c r="C1952" t="inlineStr">
+        <is>
+          <t>Sacramento Republic FC</t>
+        </is>
+      </c>
+      <c r="D1952" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1952" t="inlineStr"/>
+      <c r="F1952" t="inlineStr"/>
+      <c r="G1952" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1952" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1952" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1952" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1952" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1952" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -89755,13 +90907,16 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>25</v>
+      </c>
+      <c r="D33" t="n">
+        <v>83.3</v>
       </c>
       <c r="E33" t="n">
-        <v>74</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -89775,7 +90930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G174"/>
+  <dimension ref="A1:G179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -93783,6 +94938,141 @@
         <v>0</v>
       </c>
     </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>fav_domina_no_gana</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>1</v>
+      </c>
+      <c r="D175" t="n">
+        <v>1</v>
+      </c>
+      <c r="E175" t="n">
+        <v>100</v>
+      </c>
+      <c r="F175" t="n">
+        <v>0</v>
+      </c>
+      <c r="G175" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>siguen_empatados_22</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>1</v>
+      </c>
+      <c r="D176" t="n">
+        <v>1</v>
+      </c>
+      <c r="E176" t="n">
+        <v>100</v>
+      </c>
+      <c r="F176" t="n">
+        <v>0</v>
+      </c>
+      <c r="G176" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>1</v>
+      </c>
+      <c r="D177" t="n">
+        <v>1</v>
+      </c>
+      <c r="E177" t="n">
+        <v>100</v>
+      </c>
+      <c r="F177" t="n">
+        <v>0</v>
+      </c>
+      <c r="G177" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>1</v>
+      </c>
+      <c r="D178" t="n">
+        <v>0</v>
+      </c>
+      <c r="E178" t="n">
+        <v>0</v>
+      </c>
+      <c r="F178" t="n">
+        <v>1</v>
+      </c>
+      <c r="G178" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>siguen_empatados_70</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>1</v>
+      </c>
+      <c r="D179" t="n">
+        <v>0</v>
+      </c>
+      <c r="E179" t="n">
+        <v>0</v>
+      </c>
+      <c r="F179" t="n">
+        <v>1</v>
+      </c>
+      <c r="G179" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 1 embebida: seleccion 2026-10-02T05:05
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1952"/>
+  <dimension ref="A1:L1970"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -88821,8 +88821,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1922" t="inlineStr"/>
-      <c r="F1922" t="inlineStr"/>
       <c r="G1922" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -88869,8 +88867,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1923" t="inlineStr"/>
-      <c r="F1923" t="inlineStr"/>
       <c r="G1923" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -88917,8 +88913,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1924" t="inlineStr"/>
-      <c r="F1924" t="inlineStr"/>
       <c r="G1924" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -88965,8 +88959,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1925" t="inlineStr"/>
-      <c r="F1925" t="inlineStr"/>
       <c r="G1925" t="inlineStr">
         <is>
           <t>0-5</t>
@@ -89013,8 +89005,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1926" t="inlineStr"/>
-      <c r="F1926" t="inlineStr"/>
       <c r="G1926" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -89061,8 +89051,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1927" t="inlineStr"/>
-      <c r="F1927" t="inlineStr"/>
       <c r="G1927" t="inlineStr">
         <is>
           <t>1-5</t>
@@ -89109,8 +89097,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1928" t="inlineStr"/>
-      <c r="F1928" t="inlineStr"/>
       <c r="G1928" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -89157,8 +89143,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1929" t="inlineStr"/>
-      <c r="F1929" t="inlineStr"/>
       <c r="G1929" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -89205,8 +89189,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1930" t="inlineStr"/>
-      <c r="F1930" t="inlineStr"/>
       <c r="G1930" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -89253,8 +89235,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1931" t="inlineStr"/>
-      <c r="F1931" t="inlineStr"/>
       <c r="G1931" t="inlineStr">
         <is>
           <t>1-4</t>
@@ -89301,8 +89281,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1932" t="inlineStr"/>
-      <c r="F1932" t="inlineStr"/>
       <c r="G1932" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -89349,8 +89327,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1933" t="inlineStr"/>
-      <c r="F1933" t="inlineStr"/>
       <c r="G1933" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -89397,8 +89373,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1934" t="inlineStr"/>
-      <c r="F1934" t="inlineStr"/>
       <c r="G1934" t="inlineStr">
         <is>
           <t>2-5</t>
@@ -89445,8 +89419,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1935" t="inlineStr"/>
-      <c r="F1935" t="inlineStr"/>
       <c r="G1935" t="inlineStr">
         <is>
           <t>5-2</t>
@@ -89493,8 +89465,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1936" t="inlineStr"/>
-      <c r="F1936" t="inlineStr"/>
       <c r="G1936" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -89541,8 +89511,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1937" t="inlineStr"/>
-      <c r="F1937" t="inlineStr"/>
       <c r="G1937" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -89589,8 +89557,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1938" t="inlineStr"/>
-      <c r="F1938" t="inlineStr"/>
       <c r="G1938" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -89637,8 +89603,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1939" t="inlineStr"/>
-      <c r="F1939" t="inlineStr"/>
       <c r="G1939" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -89685,8 +89649,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1940" t="inlineStr"/>
-      <c r="F1940" t="inlineStr"/>
       <c r="G1940" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -89733,8 +89695,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1941" t="inlineStr"/>
-      <c r="F1941" t="inlineStr"/>
       <c r="G1941" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -89781,8 +89741,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1942" t="inlineStr"/>
-      <c r="F1942" t="inlineStr"/>
       <c r="G1942" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -89829,8 +89787,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1943" t="inlineStr"/>
-      <c r="F1943" t="inlineStr"/>
       <c r="G1943" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -89877,8 +89833,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1944" t="inlineStr"/>
-      <c r="F1944" t="inlineStr"/>
       <c r="G1944" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -89925,8 +89879,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1945" t="inlineStr"/>
-      <c r="F1945" t="inlineStr"/>
       <c r="G1945" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -89973,8 +89925,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1946" t="inlineStr"/>
-      <c r="F1946" t="inlineStr"/>
       <c r="G1946" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -90021,8 +89971,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1947" t="inlineStr"/>
-      <c r="F1947" t="inlineStr"/>
       <c r="G1947" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -90069,8 +90017,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1948" t="inlineStr"/>
-      <c r="F1948" t="inlineStr"/>
       <c r="G1948" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -90117,8 +90063,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1949" t="inlineStr"/>
-      <c r="F1949" t="inlineStr"/>
       <c r="G1949" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -90165,8 +90109,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1950" t="inlineStr"/>
-      <c r="F1950" t="inlineStr"/>
       <c r="G1950" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -90213,8 +90155,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1951" t="inlineStr"/>
-      <c r="F1951" t="inlineStr"/>
       <c r="G1951" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -90261,8 +90201,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1952" t="inlineStr"/>
-      <c r="F1952" t="inlineStr"/>
       <c r="G1952" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -90283,6 +90221,870 @@
         <v>0</v>
       </c>
       <c r="L1952" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1953">
+      <c r="A1953" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1953" t="inlineStr">
+        <is>
+          <t>SSV Jahn Regensburg vs WSG Swarovski Tirol</t>
+        </is>
+      </c>
+      <c r="C1953" t="inlineStr">
+        <is>
+          <t>SSV Jahn Regensburg</t>
+        </is>
+      </c>
+      <c r="D1953" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1953" t="inlineStr"/>
+      <c r="F1953" t="inlineStr"/>
+      <c r="G1953" t="inlineStr">
+        <is>
+          <t>0-6</t>
+        </is>
+      </c>
+      <c r="H1953" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1953" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1953" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1953" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1953" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1954">
+      <c r="A1954" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1954" t="inlineStr">
+        <is>
+          <t>Greece U21 vs Latvia U21</t>
+        </is>
+      </c>
+      <c r="C1954" t="inlineStr">
+        <is>
+          <t>Greece U21</t>
+        </is>
+      </c>
+      <c r="D1954" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1954" t="inlineStr"/>
+      <c r="F1954" t="inlineStr"/>
+      <c r="G1954" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H1954" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1954" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1954" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1954" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1954" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1955">
+      <c r="A1955" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1955" t="inlineStr">
+        <is>
+          <t>VfB Stuttgart vs SpVgg Greuther Fürth</t>
+        </is>
+      </c>
+      <c r="C1955" t="inlineStr">
+        <is>
+          <t>VfB Stuttgart</t>
+        </is>
+      </c>
+      <c r="D1955" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1955" t="inlineStr"/>
+      <c r="F1955" t="inlineStr"/>
+      <c r="G1955" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H1955" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1955" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1955" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1955" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1955" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1956">
+      <c r="A1956" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1956" t="inlineStr">
+        <is>
+          <t>Azerbaijan vs Liechtenstein</t>
+        </is>
+      </c>
+      <c r="C1956" t="inlineStr">
+        <is>
+          <t>Azerbaijan</t>
+        </is>
+      </c>
+      <c r="D1956" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1956" t="inlineStr"/>
+      <c r="F1956" t="inlineStr"/>
+      <c r="G1956" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1956" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1956" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1956" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1956" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1956" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1957">
+      <c r="A1957" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1957" t="inlineStr">
+        <is>
+          <t>Guinea vs Kenya</t>
+        </is>
+      </c>
+      <c r="C1957" t="inlineStr">
+        <is>
+          <t>Guinea</t>
+        </is>
+      </c>
+      <c r="D1957" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1957" t="inlineStr"/>
+      <c r="F1957" t="inlineStr"/>
+      <c r="G1957" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1957" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1957" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1957" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1957" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1957" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1958">
+      <c r="A1958" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1958" t="inlineStr">
+        <is>
+          <t>North Macedonia U21 vs Montenegro U21</t>
+        </is>
+      </c>
+      <c r="C1958" t="inlineStr">
+        <is>
+          <t>North Macedonia U21</t>
+        </is>
+      </c>
+      <c r="D1958" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1958" t="inlineStr"/>
+      <c r="F1958" t="inlineStr"/>
+      <c r="G1958" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1958" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1958" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1958" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1958" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1958" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1959">
+      <c r="A1959" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1959" t="inlineStr">
+        <is>
+          <t>Germany vs Serbia</t>
+        </is>
+      </c>
+      <c r="C1959" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D1959" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1959" t="inlineStr"/>
+      <c r="F1959" t="inlineStr"/>
+      <c r="G1959" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1959" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1959" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1959" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1959" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1959" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1960">
+      <c r="A1960" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1960" t="inlineStr">
+        <is>
+          <t>Greece vs Netherlands</t>
+        </is>
+      </c>
+      <c r="C1960" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="D1960" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1960" t="inlineStr"/>
+      <c r="F1960" t="inlineStr"/>
+      <c r="G1960" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H1960" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1960" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1960" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1960" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1960" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1961">
+      <c r="A1961" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1961" t="inlineStr">
+        <is>
+          <t>Denmark vs Portugal</t>
+        </is>
+      </c>
+      <c r="C1961" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D1961" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1961" t="inlineStr"/>
+      <c r="F1961" t="inlineStr"/>
+      <c r="G1961" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H1961" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1961" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1961" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1961" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1961" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1962">
+      <c r="A1962" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1962" t="inlineStr">
+        <is>
+          <t>Wales vs Norway</t>
+        </is>
+      </c>
+      <c r="C1962" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="D1962" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1962" t="inlineStr"/>
+      <c r="F1962" t="inlineStr"/>
+      <c r="G1962" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1962" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1962" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1962" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1962" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1962" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1963">
+      <c r="A1963" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1963" t="inlineStr">
+        <is>
+          <t>Republic of Ireland vs Austria</t>
+        </is>
+      </c>
+      <c r="C1963" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="D1963" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1963" t="inlineStr"/>
+      <c r="F1963" t="inlineStr"/>
+      <c r="G1963" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H1963" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1963" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1963" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1963" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1963" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1964">
+      <c r="A1964" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1964" t="inlineStr">
+        <is>
+          <t>Israel vs Kosovo</t>
+        </is>
+      </c>
+      <c r="C1964" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+      <c r="D1964" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1964" t="inlineStr"/>
+      <c r="F1964" t="inlineStr"/>
+      <c r="G1964" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1964" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1964" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1964" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1964" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1964" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1965">
+      <c r="A1965" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1965" t="inlineStr">
+        <is>
+          <t>Malta vs Gibraltar</t>
+        </is>
+      </c>
+      <c r="C1965" t="inlineStr">
+        <is>
+          <t>Malta</t>
+        </is>
+      </c>
+      <c r="D1965" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1965" t="inlineStr"/>
+      <c r="F1965" t="inlineStr"/>
+      <c r="G1965" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1965" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1965" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1965" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1965" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1965" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1966">
+      <c r="A1966" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1966" t="inlineStr">
+        <is>
+          <t>British Virgin Islands vs Montserrat</t>
+        </is>
+      </c>
+      <c r="C1966" t="inlineStr">
+        <is>
+          <t>Montserrat</t>
+        </is>
+      </c>
+      <c r="D1966" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1966" t="inlineStr"/>
+      <c r="F1966" t="inlineStr"/>
+      <c r="G1966" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H1966" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1966" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1966" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1966" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1966" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1967">
+      <c r="A1967" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1967" t="inlineStr">
+        <is>
+          <t>US Virgin Islands vs St. Martin</t>
+        </is>
+      </c>
+      <c r="C1967" t="inlineStr">
+        <is>
+          <t>St. Martin</t>
+        </is>
+      </c>
+      <c r="D1967" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1967" t="inlineStr"/>
+      <c r="F1967" t="inlineStr"/>
+      <c r="G1967" t="inlineStr">
+        <is>
+          <t>0-5</t>
+        </is>
+      </c>
+      <c r="H1967" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1967" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1967" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1967" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1967" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1968">
+      <c r="A1968" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1968" t="inlineStr">
+        <is>
+          <t>Dominica vs Guyana</t>
+        </is>
+      </c>
+      <c r="C1968" t="inlineStr">
+        <is>
+          <t>Guyana</t>
+        </is>
+      </c>
+      <c r="D1968" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1968" t="inlineStr"/>
+      <c r="F1968" t="inlineStr"/>
+      <c r="G1968" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
+      <c r="H1968" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1968" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1968" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1968" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1968" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1969">
+      <c r="A1969" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1969" t="inlineStr">
+        <is>
+          <t>Fuerte San Francisco vs Luis Ángel Firpo</t>
+        </is>
+      </c>
+      <c r="C1969" t="inlineStr">
+        <is>
+          <t>Luis Ángel Firpo</t>
+        </is>
+      </c>
+      <c r="D1969" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1969" t="inlineStr"/>
+      <c r="F1969" t="inlineStr"/>
+      <c r="G1969" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H1969" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1969" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1969" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1969" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1969" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1970">
+      <c r="A1970" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1970" t="inlineStr">
+        <is>
+          <t>Curaçao vs Trinidad and Tobago</t>
+        </is>
+      </c>
+      <c r="C1970" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+      <c r="D1970" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1970" t="inlineStr"/>
+      <c r="F1970" t="inlineStr"/>
+      <c r="G1970" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1970" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1970" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1970" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1970" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1970" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -90299,7 +91101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -90917,6 +91719,25 @@
       </c>
       <c r="E33" t="n">
         <v>97</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>18</v>
+      </c>
+      <c r="C34" t="n">
+        <v>14</v>
+      </c>
+      <c r="D34" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="E34" t="n">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 1: seleccion de partidos 2026-10-05
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1970"/>
+  <dimension ref="A1:L2053"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -90247,8 +90247,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1953" t="inlineStr"/>
-      <c r="F1953" t="inlineStr"/>
       <c r="G1953" t="inlineStr">
         <is>
           <t>0-6</t>
@@ -90295,8 +90293,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1954" t="inlineStr"/>
-      <c r="F1954" t="inlineStr"/>
       <c r="G1954" t="inlineStr">
         <is>
           <t>4-2</t>
@@ -90343,8 +90339,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1955" t="inlineStr"/>
-      <c r="F1955" t="inlineStr"/>
       <c r="G1955" t="inlineStr">
         <is>
           <t>5-0</t>
@@ -90391,8 +90385,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1956" t="inlineStr"/>
-      <c r="F1956" t="inlineStr"/>
       <c r="G1956" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -90439,8 +90431,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1957" t="inlineStr"/>
-      <c r="F1957" t="inlineStr"/>
       <c r="G1957" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -90487,8 +90477,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1958" t="inlineStr"/>
-      <c r="F1958" t="inlineStr"/>
       <c r="G1958" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -90535,8 +90523,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1959" t="inlineStr"/>
-      <c r="F1959" t="inlineStr"/>
       <c r="G1959" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -90583,8 +90569,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1960" t="inlineStr"/>
-      <c r="F1960" t="inlineStr"/>
       <c r="G1960" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -90631,8 +90615,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1961" t="inlineStr"/>
-      <c r="F1961" t="inlineStr"/>
       <c r="G1961" t="inlineStr">
         <is>
           <t>2-4</t>
@@ -90679,8 +90661,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1962" t="inlineStr"/>
-      <c r="F1962" t="inlineStr"/>
       <c r="G1962" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -90727,8 +90707,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1963" t="inlineStr"/>
-      <c r="F1963" t="inlineStr"/>
       <c r="G1963" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -90775,8 +90753,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1964" t="inlineStr"/>
-      <c r="F1964" t="inlineStr"/>
       <c r="G1964" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -90823,8 +90799,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1965" t="inlineStr"/>
-      <c r="F1965" t="inlineStr"/>
       <c r="G1965" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -90871,8 +90845,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1966" t="inlineStr"/>
-      <c r="F1966" t="inlineStr"/>
       <c r="G1966" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -90919,8 +90891,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1967" t="inlineStr"/>
-      <c r="F1967" t="inlineStr"/>
       <c r="G1967" t="inlineStr">
         <is>
           <t>0-5</t>
@@ -90967,8 +90937,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1968" t="inlineStr"/>
-      <c r="F1968" t="inlineStr"/>
       <c r="G1968" t="inlineStr">
         <is>
           <t>1-5</t>
@@ -91015,8 +90983,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1969" t="inlineStr"/>
-      <c r="F1969" t="inlineStr"/>
       <c r="G1969" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -91063,8 +91029,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1970" t="inlineStr"/>
-      <c r="F1970" t="inlineStr"/>
       <c r="G1970" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -91085,6 +91049,3990 @@
         <v>0</v>
       </c>
       <c r="L1970" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1971">
+      <c r="A1971" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1971" t="inlineStr">
+        <is>
+          <t>CSM Slatina vs CSU Craiova</t>
+        </is>
+      </c>
+      <c r="C1971" t="inlineStr">
+        <is>
+          <t>CSM Slatina</t>
+        </is>
+      </c>
+      <c r="D1971" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1971" t="inlineStr"/>
+      <c r="F1971" t="inlineStr"/>
+      <c r="G1971" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H1971" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1971" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1971" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1971" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1971" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1972">
+      <c r="A1972" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1972" t="inlineStr">
+        <is>
+          <t>Dinamo Minsk vs FK Uni Iks Labs Minsk</t>
+        </is>
+      </c>
+      <c r="C1972" t="inlineStr">
+        <is>
+          <t>Dinamo Minsk</t>
+        </is>
+      </c>
+      <c r="D1972" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1972" t="inlineStr"/>
+      <c r="F1972" t="inlineStr"/>
+      <c r="G1972" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1972" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1972" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1972" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1972" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1972" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1973">
+      <c r="A1973" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1973" t="inlineStr">
+        <is>
+          <t>Dinamo Moscow vs Rodina Moscow</t>
+        </is>
+      </c>
+      <c r="C1973" t="inlineStr">
+        <is>
+          <t>Dinamo Moscow</t>
+        </is>
+      </c>
+      <c r="D1973" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1973" t="inlineStr"/>
+      <c r="F1973" t="inlineStr"/>
+      <c r="G1973" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H1973" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1973" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1973" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1973" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1973" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1974">
+      <c r="A1974" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1974" t="inlineStr">
+        <is>
+          <t>FC Kolos Kovalivka vs FC Zorya Luhansk</t>
+        </is>
+      </c>
+      <c r="C1974" t="inlineStr">
+        <is>
+          <t>FC Kolos Kovalivka</t>
+        </is>
+      </c>
+      <c r="D1974" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1974" t="inlineStr"/>
+      <c r="F1974" t="inlineStr"/>
+      <c r="G1974" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H1974" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1974" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1974" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1974" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1974" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1975">
+      <c r="A1975" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1975" t="inlineStr">
+        <is>
+          <t>Granada vs Eibar</t>
+        </is>
+      </c>
+      <c r="C1975" t="inlineStr">
+        <is>
+          <t>Eibar</t>
+        </is>
+      </c>
+      <c r="D1975" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1975" t="inlineStr"/>
+      <c r="F1975" t="inlineStr"/>
+      <c r="G1975" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1975" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1975" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1975" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1975" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1975" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1976">
+      <c r="A1976" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1976" t="inlineStr">
+        <is>
+          <t>FC Twente vs FC Utrecht</t>
+        </is>
+      </c>
+      <c r="C1976" t="inlineStr">
+        <is>
+          <t>FC Twente</t>
+        </is>
+      </c>
+      <c r="D1976" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1976" t="inlineStr"/>
+      <c r="F1976" t="inlineStr"/>
+      <c r="G1976" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1976" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1976" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1976" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1976" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1976" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1977">
+      <c r="A1977" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1977" t="inlineStr">
+        <is>
+          <t>Atlético Unión Güímar vs Sporting Hortaleza</t>
+        </is>
+      </c>
+      <c r="C1977" t="inlineStr">
+        <is>
+          <t>Sporting Hortaleza</t>
+        </is>
+      </c>
+      <c r="D1977" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1977" t="inlineStr"/>
+      <c r="F1977" t="inlineStr"/>
+      <c r="G1977" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1977" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1977" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1977" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1977" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1977" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1978">
+      <c r="A1978" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1978" t="inlineStr">
+        <is>
+          <t>CSKA Moscow vs FC Arsenal Tula</t>
+        </is>
+      </c>
+      <c r="C1978" t="inlineStr">
+        <is>
+          <t>FC Arsenal Tula</t>
+        </is>
+      </c>
+      <c r="D1978" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1978" t="inlineStr"/>
+      <c r="F1978" t="inlineStr"/>
+      <c r="G1978" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1978" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1978" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1978" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1978" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1978" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1979">
+      <c r="A1979" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1979" t="inlineStr">
+        <is>
+          <t>Real Sociedad II vs Granada</t>
+        </is>
+      </c>
+      <c r="C1979" t="inlineStr">
+        <is>
+          <t>Real Sociedad II</t>
+        </is>
+      </c>
+      <c r="D1979" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1979" t="inlineStr"/>
+      <c r="F1979" t="inlineStr"/>
+      <c r="G1979" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H1979" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1979" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1979" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1979" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1979" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1980">
+      <c r="A1980" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1980" t="inlineStr">
+        <is>
+          <t>Comoros vs Senegal</t>
+        </is>
+      </c>
+      <c r="C1980" t="inlineStr">
+        <is>
+          <t>Comoros</t>
+        </is>
+      </c>
+      <c r="D1980" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1980" t="inlineStr"/>
+      <c r="F1980" t="inlineStr"/>
+      <c r="G1980" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1980" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1980" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1980" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1980" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1980" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1981">
+      <c r="A1981" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1981" t="inlineStr">
+        <is>
+          <t>Aston Villa vs Crystal Palace</t>
+        </is>
+      </c>
+      <c r="C1981" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="D1981" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1981" t="inlineStr"/>
+      <c r="F1981" t="inlineStr"/>
+      <c r="G1981" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1981" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1981" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1981" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1981" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1981" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1982">
+      <c r="A1982" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1982" t="inlineStr">
+        <is>
+          <t>Brighton &amp; Hove Albion vs Charlton Athletic</t>
+        </is>
+      </c>
+      <c r="C1982" t="inlineStr">
+        <is>
+          <t>Brighton &amp; Hove Albion</t>
+        </is>
+      </c>
+      <c r="D1982" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1982" t="inlineStr"/>
+      <c r="F1982" t="inlineStr"/>
+      <c r="G1982" t="inlineStr">
+        <is>
+          <t>5-1</t>
+        </is>
+      </c>
+      <c r="H1982" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1982" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1982" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1982" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1982" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1983">
+      <c r="A1983" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1983" t="inlineStr">
+        <is>
+          <t>Everton vs Birmingham City</t>
+        </is>
+      </c>
+      <c r="C1983" t="inlineStr">
+        <is>
+          <t>Everton</t>
+        </is>
+      </c>
+      <c r="D1983" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1983" t="inlineStr"/>
+      <c r="F1983" t="inlineStr"/>
+      <c r="G1983" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H1983" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1983" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1983" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1983" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1983" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1984">
+      <c r="A1984" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1984" t="inlineStr">
+        <is>
+          <t>Tottenham Hotspur vs London City Lionesses</t>
+        </is>
+      </c>
+      <c r="C1984" t="inlineStr">
+        <is>
+          <t>Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="D1984" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1984" t="inlineStr"/>
+      <c r="F1984" t="inlineStr"/>
+      <c r="G1984" t="inlineStr">
+        <is>
+          <t>1-6</t>
+        </is>
+      </c>
+      <c r="H1984" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1984" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1984" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1984" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1984" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1985">
+      <c r="A1985" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1985" t="inlineStr">
+        <is>
+          <t>West Ham United vs Chelsea</t>
+        </is>
+      </c>
+      <c r="C1985" t="inlineStr">
+        <is>
+          <t>Chelsea</t>
+        </is>
+      </c>
+      <c r="D1985" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1985" t="inlineStr"/>
+      <c r="F1985" t="inlineStr"/>
+      <c r="G1985" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H1985" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1985" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1985" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1985" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1985" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1986">
+      <c r="A1986" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1986" t="inlineStr">
+        <is>
+          <t>FC Fleury 91 vs Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="C1986" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="D1986" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1986" t="inlineStr"/>
+      <c r="F1986" t="inlineStr"/>
+      <c r="G1986" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H1986" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1986" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1986" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1986" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1986" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1987">
+      <c r="A1987" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1987" t="inlineStr">
+        <is>
+          <t>Hamburg SV vs F.C. København</t>
+        </is>
+      </c>
+      <c r="C1987" t="inlineStr">
+        <is>
+          <t>F.C. København</t>
+        </is>
+      </c>
+      <c r="D1987" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1987" t="inlineStr"/>
+      <c r="F1987" t="inlineStr"/>
+      <c r="G1987" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H1987" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1987" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1987" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1987" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1987" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1988">
+      <c r="A1988" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1988" t="inlineStr">
+        <is>
+          <t>Kyrgyz Republic vs Lebanon</t>
+        </is>
+      </c>
+      <c r="C1988" t="inlineStr">
+        <is>
+          <t>Kyrgyz Republic</t>
+        </is>
+      </c>
+      <c r="D1988" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1988" t="inlineStr"/>
+      <c r="F1988" t="inlineStr"/>
+      <c r="G1988" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H1988" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1988" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1988" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1988" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1988" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1989">
+      <c r="A1989" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1989" t="inlineStr">
+        <is>
+          <t>AE Prat vs CF San Rafael</t>
+        </is>
+      </c>
+      <c r="C1989" t="inlineStr">
+        <is>
+          <t>AE Prat</t>
+        </is>
+      </c>
+      <c r="D1989" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1989" t="inlineStr"/>
+      <c r="F1989" t="inlineStr"/>
+      <c r="G1989" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H1989" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1989" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1989" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1989" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1989" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1990">
+      <c r="A1990" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1990" t="inlineStr">
+        <is>
+          <t>CD San José vs Auriense Cented Academy</t>
+        </is>
+      </c>
+      <c r="C1990" t="inlineStr">
+        <is>
+          <t>Auriense Cented Academy</t>
+        </is>
+      </c>
+      <c r="D1990" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1990" t="inlineStr"/>
+      <c r="F1990" t="inlineStr"/>
+      <c r="G1990" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1990" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1990" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1990" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1990" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1990" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1991">
+      <c r="A1991" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1991" t="inlineStr">
+        <is>
+          <t>SD Noja vs Ribadesella</t>
+        </is>
+      </c>
+      <c r="C1991" t="inlineStr">
+        <is>
+          <t>Ribadesella</t>
+        </is>
+      </c>
+      <c r="D1991" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1991" t="inlineStr"/>
+      <c r="F1991" t="inlineStr"/>
+      <c r="G1991" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H1991" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1991" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1991" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1991" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1991" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1992">
+      <c r="A1992" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1992" t="inlineStr">
+        <is>
+          <t>Enosis Neon Paralimni vs Anorthosis</t>
+        </is>
+      </c>
+      <c r="C1992" t="inlineStr">
+        <is>
+          <t>Enosis Neon Paralimni</t>
+        </is>
+      </c>
+      <c r="D1992" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1992" t="inlineStr"/>
+      <c r="F1992" t="inlineStr"/>
+      <c r="G1992" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H1992" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1992" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1992" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1992" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1992" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1993">
+      <c r="A1993" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1993" t="inlineStr">
+        <is>
+          <t>Gjilani vs KF Bashkimi 1947</t>
+        </is>
+      </c>
+      <c r="C1993" t="inlineStr">
+        <is>
+          <t>Gjilani</t>
+        </is>
+      </c>
+      <c r="D1993" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1993" t="inlineStr"/>
+      <c r="F1993" t="inlineStr"/>
+      <c r="G1993" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1993" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1993" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1993" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1993" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1993" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1994">
+      <c r="A1994" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1994" t="inlineStr">
+        <is>
+          <t>ADO Den Haag vs PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="C1994" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="D1994" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1994" t="inlineStr"/>
+      <c r="F1994" t="inlineStr"/>
+      <c r="G1994" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H1994" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1994" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1994" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1994" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1994" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1995">
+      <c r="A1995" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1995" t="inlineStr">
+        <is>
+          <t>De Graafschap vs AZ Alkmaar</t>
+        </is>
+      </c>
+      <c r="C1995" t="inlineStr">
+        <is>
+          <t>AZ Alkmaar</t>
+        </is>
+      </c>
+      <c r="D1995" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1995" t="inlineStr"/>
+      <c r="F1995" t="inlineStr"/>
+      <c r="G1995" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1995" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I1995" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1995" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1995" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1995" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1996">
+      <c r="A1996" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1996" t="inlineStr">
+        <is>
+          <t>Feyenoord Rotterdam vs Ajax Amsterdam</t>
+        </is>
+      </c>
+      <c r="C1996" t="inlineStr">
+        <is>
+          <t>Ajax Amsterdam</t>
+        </is>
+      </c>
+      <c r="D1996" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E1996" t="inlineStr"/>
+      <c r="F1996" t="inlineStr"/>
+      <c r="G1996" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H1996" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1996" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1996" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1996" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1996" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1997">
+      <c r="A1997" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1997" t="inlineStr">
+        <is>
+          <t>Sporting de Alcázar vs CP Talayuela</t>
+        </is>
+      </c>
+      <c r="C1997" t="inlineStr">
+        <is>
+          <t>Sporting de Alcázar</t>
+        </is>
+      </c>
+      <c r="D1997" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1997" t="inlineStr"/>
+      <c r="F1997" t="inlineStr"/>
+      <c r="G1997" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H1997" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1997" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1997" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1997" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1997" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1998">
+      <c r="A1998" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1998" t="inlineStr">
+        <is>
+          <t>Molde vs Kristiansund BK</t>
+        </is>
+      </c>
+      <c r="C1998" t="inlineStr">
+        <is>
+          <t>Molde</t>
+        </is>
+      </c>
+      <c r="D1998" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1998" t="inlineStr"/>
+      <c r="F1998" t="inlineStr"/>
+      <c r="G1998" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H1998" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1998" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1998" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1998" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1998" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1999">
+      <c r="A1999" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B1999" t="inlineStr">
+        <is>
+          <t>Manchester City vs Arsenal</t>
+        </is>
+      </c>
+      <c r="C1999" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="D1999" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E1999" t="inlineStr"/>
+      <c r="F1999" t="inlineStr"/>
+      <c r="G1999" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H1999" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I1999" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1999" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1999" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1999" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2000">
+      <c r="A2000" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2000" t="inlineStr">
+        <is>
+          <t>Tavernes de la Valldigna vs Maracena</t>
+        </is>
+      </c>
+      <c r="C2000" t="inlineStr">
+        <is>
+          <t>Tavernes de la Valldigna</t>
+        </is>
+      </c>
+      <c r="D2000" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2000" t="inlineStr"/>
+      <c r="F2000" t="inlineStr"/>
+      <c r="G2000" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2000" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2000" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2000" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2000" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2000" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2001">
+      <c r="A2001" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2001" t="inlineStr">
+        <is>
+          <t>Zenit St Petersburg vs BATE Borisov</t>
+        </is>
+      </c>
+      <c r="C2001" t="inlineStr">
+        <is>
+          <t>Zenit St Petersburg</t>
+        </is>
+      </c>
+      <c r="D2001" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2001" t="inlineStr"/>
+      <c r="F2001" t="inlineStr"/>
+      <c r="G2001" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H2001" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2001" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2001" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2001" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2001" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2002">
+      <c r="A2002" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2002" t="inlineStr">
+        <is>
+          <t>Kosovo vs Austria</t>
+        </is>
+      </c>
+      <c r="C2002" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+      <c r="D2002" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2002" t="inlineStr"/>
+      <c r="F2002" t="inlineStr"/>
+      <c r="G2002" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2002" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2002" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2002" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2002" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2002" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2003">
+      <c r="A2003" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2003" t="inlineStr">
+        <is>
+          <t>Malta vs Andorra</t>
+        </is>
+      </c>
+      <c r="C2003" t="inlineStr">
+        <is>
+          <t>Malta</t>
+        </is>
+      </c>
+      <c r="D2003" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2003" t="inlineStr"/>
+      <c r="F2003" t="inlineStr"/>
+      <c r="G2003" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H2003" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2003" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2003" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2003" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2003" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2004">
+      <c r="A2004" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2004" t="inlineStr">
+        <is>
+          <t>Boston River vs Juventud</t>
+        </is>
+      </c>
+      <c r="C2004" t="inlineStr">
+        <is>
+          <t>Juventud</t>
+        </is>
+      </c>
+      <c r="D2004" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2004" t="inlineStr"/>
+      <c r="F2004" t="inlineStr"/>
+      <c r="G2004" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2004" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2004" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2004" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2004" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2004" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2005">
+      <c r="A2005" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2005" t="inlineStr">
+        <is>
+          <t>Castellón vs Ceuta</t>
+        </is>
+      </c>
+      <c r="C2005" t="inlineStr">
+        <is>
+          <t>Castellón</t>
+        </is>
+      </c>
+      <c r="D2005" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2005" t="inlineStr"/>
+      <c r="F2005" t="inlineStr"/>
+      <c r="G2005" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2005" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2005" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2005" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2005" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2005" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2006">
+      <c r="A2006" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2006" t="inlineStr">
+        <is>
+          <t>Las Palmas vs Real Valladolid</t>
+        </is>
+      </c>
+      <c r="C2006" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="D2006" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2006" t="inlineStr"/>
+      <c r="F2006" t="inlineStr"/>
+      <c r="G2006" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H2006" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2006" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2006" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2006" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2006" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2007">
+      <c r="A2007" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2007" t="inlineStr">
+        <is>
+          <t>Gotham FC vs Angel City FC</t>
+        </is>
+      </c>
+      <c r="C2007" t="inlineStr">
+        <is>
+          <t>Gotham FC</t>
+        </is>
+      </c>
+      <c r="D2007" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2007" t="inlineStr"/>
+      <c r="F2007" t="inlineStr"/>
+      <c r="G2007" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2007" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2007" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2007" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2007" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2007" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2008">
+      <c r="A2008" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2008" t="inlineStr">
+        <is>
+          <t>Barcelona vs Real Madrid</t>
+        </is>
+      </c>
+      <c r="C2008" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D2008" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2008" t="inlineStr"/>
+      <c r="F2008" t="inlineStr"/>
+      <c r="G2008" t="inlineStr">
+        <is>
+          <t>7-0</t>
+        </is>
+      </c>
+      <c r="H2008" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2008" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2008" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2008" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2008" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2009">
+      <c r="A2009" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2009" t="inlineStr">
+        <is>
+          <t>AFC Toronto vs Vancouver Rise FC</t>
+        </is>
+      </c>
+      <c r="C2009" t="inlineStr">
+        <is>
+          <t>AFC Toronto</t>
+        </is>
+      </c>
+      <c r="D2009" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2009" t="inlineStr"/>
+      <c r="F2009" t="inlineStr"/>
+      <c r="G2009" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H2009" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2009" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2009" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2009" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2009" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2010">
+      <c r="A2010" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2010" t="inlineStr">
+        <is>
+          <t>Valencia vs Real Sociedad</t>
+        </is>
+      </c>
+      <c r="C2010" t="inlineStr">
+        <is>
+          <t>Real Sociedad</t>
+        </is>
+      </c>
+      <c r="D2010" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2010" t="inlineStr"/>
+      <c r="F2010" t="inlineStr"/>
+      <c r="G2010" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H2010" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2010" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2010" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2010" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2010" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2011">
+      <c r="A2011" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2011" t="inlineStr">
+        <is>
+          <t>Huracán vs Aldosivi</t>
+        </is>
+      </c>
+      <c r="C2011" t="inlineStr">
+        <is>
+          <t>Huracán</t>
+        </is>
+      </c>
+      <c r="D2011" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2011" t="inlineStr"/>
+      <c r="F2011" t="inlineStr"/>
+      <c r="G2011" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H2011" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2011" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2011" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2011" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2011" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2012">
+      <c r="A2012" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2012" t="inlineStr">
+        <is>
+          <t>Egypt vs South Africa</t>
+        </is>
+      </c>
+      <c r="C2012" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="D2012" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2012" t="inlineStr"/>
+      <c r="F2012" t="inlineStr"/>
+      <c r="G2012" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H2012" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2012" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2012" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2012" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2012" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2013">
+      <c r="A2013" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2013" t="inlineStr">
+        <is>
+          <t>Morocco vs Mali</t>
+        </is>
+      </c>
+      <c r="C2013" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="D2013" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2013" t="inlineStr"/>
+      <c r="F2013" t="inlineStr"/>
+      <c r="G2013" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2013" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2013" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2013" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2013" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2013" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2014">
+      <c r="A2014" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2014" t="inlineStr">
+        <is>
+          <t>Leones Negros vs Dorados de Sinaloa</t>
+        </is>
+      </c>
+      <c r="C2014" t="inlineStr">
+        <is>
+          <t>Leones Negros</t>
+        </is>
+      </c>
+      <c r="D2014" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2014" t="inlineStr"/>
+      <c r="F2014" t="inlineStr"/>
+      <c r="G2014" t="inlineStr">
+        <is>
+          <t>6-3</t>
+        </is>
+      </c>
+      <c r="H2014" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2014" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2014" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2014" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2014" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2015">
+      <c r="A2015" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2015" t="inlineStr">
+        <is>
+          <t>Agropecuario vs Midland</t>
+        </is>
+      </c>
+      <c r="C2015" t="inlineStr">
+        <is>
+          <t>Agropecuario</t>
+        </is>
+      </c>
+      <c r="D2015" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2015" t="inlineStr"/>
+      <c r="F2015" t="inlineStr"/>
+      <c r="G2015" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2015" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2015" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2015" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2015" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2015" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2016">
+      <c r="A2016" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2016" t="inlineStr">
+        <is>
+          <t>Comunicaciones vs Flandria</t>
+        </is>
+      </c>
+      <c r="C2016" t="inlineStr">
+        <is>
+          <t>Comunicaciones</t>
+        </is>
+      </c>
+      <c r="D2016" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2016" t="inlineStr"/>
+      <c r="F2016" t="inlineStr"/>
+      <c r="G2016" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2016" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2016" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2016" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2016" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2016" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2017">
+      <c r="A2017" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2017" t="inlineStr">
+        <is>
+          <t>Chacarita Juniors vs Patronato</t>
+        </is>
+      </c>
+      <c r="C2017" t="inlineStr">
+        <is>
+          <t>Patronato</t>
+        </is>
+      </c>
+      <c r="D2017" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2017" t="inlineStr"/>
+      <c r="F2017" t="inlineStr"/>
+      <c r="G2017" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H2017" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2017" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2017" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2017" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2017" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2018">
+      <c r="A2018" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2018" t="inlineStr">
+        <is>
+          <t>San Telmo vs Almirante Brown</t>
+        </is>
+      </c>
+      <c r="C2018" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="D2018" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2018" t="inlineStr"/>
+      <c r="F2018" t="inlineStr"/>
+      <c r="G2018" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H2018" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2018" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2018" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2018" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2018" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2019">
+      <c r="A2019" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2019" t="inlineStr">
+        <is>
+          <t>O'Higgins vs Deportes Concepcion</t>
+        </is>
+      </c>
+      <c r="C2019" t="inlineStr">
+        <is>
+          <t>O'Higgins</t>
+        </is>
+      </c>
+      <c r="D2019" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2019" t="inlineStr"/>
+      <c r="F2019" t="inlineStr"/>
+      <c r="G2019" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H2019" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2019" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2019" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2019" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2019" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2020">
+      <c r="A2020" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2020" t="inlineStr">
+        <is>
+          <t>Greece vs Germany</t>
+        </is>
+      </c>
+      <c r="C2020" t="inlineStr">
+        <is>
+          <t>Greece</t>
+        </is>
+      </c>
+      <c r="D2020" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2020" t="inlineStr"/>
+      <c r="F2020" t="inlineStr"/>
+      <c r="G2020" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2020" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2020" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2020" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2020" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2020" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2021">
+      <c r="A2021" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2021" t="inlineStr">
+        <is>
+          <t>Netherlands vs Serbia</t>
+        </is>
+      </c>
+      <c r="C2021" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="D2021" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2021" t="inlineStr"/>
+      <c r="F2021" t="inlineStr"/>
+      <c r="G2021" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H2021" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2021" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2021" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2021" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2021" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2022">
+      <c r="A2022" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2022" t="inlineStr">
+        <is>
+          <t>Portugal vs Norway</t>
+        </is>
+      </c>
+      <c r="C2022" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D2022" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2022" t="inlineStr"/>
+      <c r="F2022" t="inlineStr"/>
+      <c r="G2022" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H2022" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2022" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2022" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2022" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2022" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2023">
+      <c r="A2023" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2023" t="inlineStr">
+        <is>
+          <t>Republic of Ireland vs Israel</t>
+        </is>
+      </c>
+      <c r="C2023" t="inlineStr">
+        <is>
+          <t>Republic of Ireland</t>
+        </is>
+      </c>
+      <c r="D2023" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2023" t="inlineStr"/>
+      <c r="F2023" t="inlineStr"/>
+      <c r="G2023" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2023" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2023" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2023" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2023" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2023" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2024">
+      <c r="A2024" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2024" t="inlineStr">
+        <is>
+          <t>Wales vs Denmark</t>
+        </is>
+      </c>
+      <c r="C2024" t="inlineStr">
+        <is>
+          <t>Wales</t>
+        </is>
+      </c>
+      <c r="D2024" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2024" t="inlineStr"/>
+      <c r="F2024" t="inlineStr"/>
+      <c r="G2024" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H2024" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2024" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2024" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2024" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2024" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2025">
+      <c r="A2025" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2025" t="inlineStr">
+        <is>
+          <t>Guyana vs Dominica</t>
+        </is>
+      </c>
+      <c r="C2025" t="inlineStr">
+        <is>
+          <t>Guyana</t>
+        </is>
+      </c>
+      <c r="D2025" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2025" t="inlineStr"/>
+      <c r="F2025" t="inlineStr"/>
+      <c r="G2025" t="inlineStr">
+        <is>
+          <t>8-1</t>
+        </is>
+      </c>
+      <c r="H2025" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2025" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2025" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2025" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2025" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2026">
+      <c r="A2026" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2026" t="inlineStr">
+        <is>
+          <t>Hartford Athletic vs Louisville City FC</t>
+        </is>
+      </c>
+      <c r="C2026" t="inlineStr">
+        <is>
+          <t>Hartford Athletic</t>
+        </is>
+      </c>
+      <c r="D2026" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2026" t="inlineStr"/>
+      <c r="F2026" t="inlineStr"/>
+      <c r="G2026" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H2026" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2026" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2026" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2026" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2026" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2027">
+      <c r="A2027" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2027" t="inlineStr">
+        <is>
+          <t>CD Sabadell vs FC Andorra</t>
+        </is>
+      </c>
+      <c r="C2027" t="inlineStr">
+        <is>
+          <t>CD Sabadell</t>
+        </is>
+      </c>
+      <c r="D2027" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2027" t="inlineStr"/>
+      <c r="F2027" t="inlineStr"/>
+      <c r="G2027" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2027" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2027" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2027" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2027" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2027" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2028">
+      <c r="A2028" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2028" t="inlineStr">
+        <is>
+          <t>Girona vs Mallorca</t>
+        </is>
+      </c>
+      <c r="C2028" t="inlineStr">
+        <is>
+          <t>Girona</t>
+        </is>
+      </c>
+      <c r="D2028" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2028" t="inlineStr"/>
+      <c r="F2028" t="inlineStr"/>
+      <c r="G2028" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2028" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2028" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2028" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2028" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2028" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2029">
+      <c r="A2029" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2029" t="inlineStr">
+        <is>
+          <t>Cerro vs Montevideo Wanderers</t>
+        </is>
+      </c>
+      <c r="C2029" t="inlineStr">
+        <is>
+          <t>Cerro</t>
+        </is>
+      </c>
+      <c r="D2029" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2029" t="inlineStr"/>
+      <c r="F2029" t="inlineStr"/>
+      <c r="G2029" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H2029" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2029" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2029" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2029" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2029" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2030">
+      <c r="A2030" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2030" t="inlineStr">
+        <is>
+          <t>Deportivo Pasto vs Fortaleza CEIF</t>
+        </is>
+      </c>
+      <c r="C2030" t="inlineStr">
+        <is>
+          <t>Deportivo Pasto</t>
+        </is>
+      </c>
+      <c r="D2030" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2030" t="inlineStr"/>
+      <c r="F2030" t="inlineStr"/>
+      <c r="G2030" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2030" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2030" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2030" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2030" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2030" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2031">
+      <c r="A2031" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2031" t="inlineStr">
+        <is>
+          <t>GV San José vs Blooming</t>
+        </is>
+      </c>
+      <c r="C2031" t="inlineStr">
+        <is>
+          <t>GV San José</t>
+        </is>
+      </c>
+      <c r="D2031" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2031" t="inlineStr"/>
+      <c r="F2031" t="inlineStr"/>
+      <c r="G2031" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H2031" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2031" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2031" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2031" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2031" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2032">
+      <c r="A2032" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2032" t="inlineStr">
+        <is>
+          <t>Central Norte vs Racing (Córdoba)</t>
+        </is>
+      </c>
+      <c r="C2032" t="inlineStr">
+        <is>
+          <t>Central Norte</t>
+        </is>
+      </c>
+      <c r="D2032" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2032" t="inlineStr"/>
+      <c r="F2032" t="inlineStr"/>
+      <c r="G2032" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2032" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2032" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2032" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2032" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2032" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2033">
+      <c r="A2033" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2033" t="inlineStr">
+        <is>
+          <t>Turks and Caicos Islands vs British Virgin Islands</t>
+        </is>
+      </c>
+      <c r="C2033" t="inlineStr">
+        <is>
+          <t>Turks and Caicos Islands</t>
+        </is>
+      </c>
+      <c r="D2033" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2033" t="inlineStr"/>
+      <c r="F2033" t="inlineStr"/>
+      <c r="G2033" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H2033" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2033" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2033" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2033" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2033" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2034">
+      <c r="A2034" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2034" t="inlineStr">
+        <is>
+          <t>Güemes vs Colegiales</t>
+        </is>
+      </c>
+      <c r="C2034" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="D2034" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2034" t="inlineStr"/>
+      <c r="F2034" t="inlineStr"/>
+      <c r="G2034" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H2034" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2034" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2034" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2034" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2034" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2035">
+      <c r="A2035" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2035" t="inlineStr">
+        <is>
+          <t>San Martín (San Juan) vs Almagro</t>
+        </is>
+      </c>
+      <c r="C2035" t="inlineStr">
+        <is>
+          <t>San Martín (San Juan)</t>
+        </is>
+      </c>
+      <c r="D2035" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2035" t="inlineStr"/>
+      <c r="F2035" t="inlineStr"/>
+      <c r="G2035" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H2035" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2035" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2035" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2035" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2035" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2036">
+      <c r="A2036" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2036" t="inlineStr">
+        <is>
+          <t>Chaco For Ever vs Defensores de Belgrano</t>
+        </is>
+      </c>
+      <c r="C2036" t="inlineStr">
+        <is>
+          <t>Chaco For Ever</t>
+        </is>
+      </c>
+      <c r="D2036" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2036" t="inlineStr"/>
+      <c r="F2036" t="inlineStr"/>
+      <c r="G2036" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H2036" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2036" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2036" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2036" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2036" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2037">
+      <c r="A2037" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2037" t="inlineStr">
+        <is>
+          <t>Atletico Rafaela vs Atlanta</t>
+        </is>
+      </c>
+      <c r="C2037" t="inlineStr">
+        <is>
+          <t>Atletico Rafaela</t>
+        </is>
+      </c>
+      <c r="D2037" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2037" t="inlineStr"/>
+      <c r="F2037" t="inlineStr"/>
+      <c r="G2037" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H2037" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2037" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2037" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2037" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2037" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2038">
+      <c r="A2038" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2038" t="inlineStr">
+        <is>
+          <t>Tampa Bay Sun FC vs Lexington SC</t>
+        </is>
+      </c>
+      <c r="C2038" t="inlineStr">
+        <is>
+          <t>Tampa Bay Sun FC</t>
+        </is>
+      </c>
+      <c r="D2038" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2038" t="inlineStr"/>
+      <c r="F2038" t="inlineStr"/>
+      <c r="G2038" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2038" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2038" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2038" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2038" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2038" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2039">
+      <c r="A2039" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2039" t="inlineStr">
+        <is>
+          <t>Godoy Cruz Antonio Tomba vs Los Andes</t>
+        </is>
+      </c>
+      <c r="C2039" t="inlineStr">
+        <is>
+          <t>Godoy Cruz Antonio Tomba</t>
+        </is>
+      </c>
+      <c r="D2039" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2039" t="inlineStr"/>
+      <c r="F2039" t="inlineStr"/>
+      <c r="G2039" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H2039" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2039" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2039" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2039" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2039" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2040">
+      <c r="A2040" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2040" t="inlineStr">
+        <is>
+          <t>Cúcuta Deportivo vs Deportivo Pereira</t>
+        </is>
+      </c>
+      <c r="C2040" t="inlineStr">
+        <is>
+          <t>Cúcuta Deportivo</t>
+        </is>
+      </c>
+      <c r="D2040" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2040" t="inlineStr"/>
+      <c r="F2040" t="inlineStr"/>
+      <c r="G2040" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H2040" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2040" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2040" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2040" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2040" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2041">
+      <c r="A2041" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2041" t="inlineStr">
+        <is>
+          <t>Internacional de Bogotá vs Once Caldas</t>
+        </is>
+      </c>
+      <c r="C2041" t="inlineStr">
+        <is>
+          <t>Internacional de Bogotá</t>
+        </is>
+      </c>
+      <c r="D2041" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2041" t="inlineStr"/>
+      <c r="F2041" t="inlineStr"/>
+      <c r="G2041" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2041" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2041" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2041" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2041" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2041" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2042">
+      <c r="A2042" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2042" t="inlineStr">
+        <is>
+          <t>Puerto Rico vs Cayman Islands</t>
+        </is>
+      </c>
+      <c r="C2042" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+      <c r="D2042" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2042" t="inlineStr"/>
+      <c r="F2042" t="inlineStr"/>
+      <c r="G2042" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H2042" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2042" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2042" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2042" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2042" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2043">
+      <c r="A2043" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2043" t="inlineStr">
+        <is>
+          <t>Trinidad and Tobago vs Curaçao</t>
+        </is>
+      </c>
+      <c r="C2043" t="inlineStr">
+        <is>
+          <t>Trinidad and Tobago</t>
+        </is>
+      </c>
+      <c r="D2043" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2043" t="inlineStr"/>
+      <c r="F2043" t="inlineStr"/>
+      <c r="G2043" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2043" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2043" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2043" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2043" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2043" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2044">
+      <c r="A2044" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2044" t="inlineStr">
+        <is>
+          <t>Argentinos Juniors vs Tigre</t>
+        </is>
+      </c>
+      <c r="C2044" t="inlineStr">
+        <is>
+          <t>Argentinos Juniors</t>
+        </is>
+      </c>
+      <c r="D2044" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2044" t="inlineStr"/>
+      <c r="F2044" t="inlineStr"/>
+      <c r="G2044" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H2044" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2044" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2044" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2044" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2044" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2045">
+      <c r="A2045" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2045" t="inlineStr">
+        <is>
+          <t>Racing (Montevideo) vs Peñarol</t>
+        </is>
+      </c>
+      <c r="C2045" t="inlineStr">
+        <is>
+          <t>Peñarol</t>
+        </is>
+      </c>
+      <c r="D2045" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2045" t="inlineStr"/>
+      <c r="F2045" t="inlineStr"/>
+      <c r="G2045" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H2045" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2045" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2045" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2045" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2045" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2046">
+      <c r="A2046" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2046" t="inlineStr">
+        <is>
+          <t>Bolivia vs Gambia</t>
+        </is>
+      </c>
+      <c r="C2046" t="inlineStr">
+        <is>
+          <t>Bolivia</t>
+        </is>
+      </c>
+      <c r="D2046" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2046" t="inlineStr"/>
+      <c r="F2046" t="inlineStr"/>
+      <c r="G2046" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2046" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2046" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2046" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2046" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2046" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2047">
+      <c r="A2047" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2047" t="inlineStr">
+        <is>
+          <t>Houston Dash vs Washington Spirit</t>
+        </is>
+      </c>
+      <c r="C2047" t="inlineStr">
+        <is>
+          <t>Houston Dash</t>
+        </is>
+      </c>
+      <c r="D2047" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2047" t="inlineStr"/>
+      <c r="F2047" t="inlineStr"/>
+      <c r="G2047" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H2047" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2047" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2047" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2047" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2047" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2048">
+      <c r="A2048" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2048" t="inlineStr">
+        <is>
+          <t>Aruba vs Anguilla</t>
+        </is>
+      </c>
+      <c r="C2048" t="inlineStr">
+        <is>
+          <t>Aruba</t>
+        </is>
+      </c>
+      <c r="D2048" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2048" t="inlineStr"/>
+      <c r="F2048" t="inlineStr"/>
+      <c r="G2048" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H2048" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2048" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2048" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2048" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2048" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2049">
+      <c r="A2049" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2049" t="inlineStr">
+        <is>
+          <t>Guadalajara vs FC Juárez</t>
+        </is>
+      </c>
+      <c r="C2049" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="D2049" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2049" t="inlineStr"/>
+      <c r="F2049" t="inlineStr"/>
+      <c r="G2049" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H2049" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2049" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2049" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2049" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2049" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2050">
+      <c r="A2050" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2050" t="inlineStr">
+        <is>
+          <t>Atlético Bucaramanga vs Atlético Junior</t>
+        </is>
+      </c>
+      <c r="C2050" t="inlineStr">
+        <is>
+          <t>Atlético Bucaramanga</t>
+        </is>
+      </c>
+      <c r="D2050" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2050" t="inlineStr"/>
+      <c r="F2050" t="inlineStr"/>
+      <c r="G2050" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H2050" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2050" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2050" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2050" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2050" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2051">
+      <c r="A2051" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2051" t="inlineStr">
+        <is>
+          <t>Guadalajara vs América</t>
+        </is>
+      </c>
+      <c r="C2051" t="inlineStr">
+        <is>
+          <t>América</t>
+        </is>
+      </c>
+      <c r="D2051" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2051" t="inlineStr"/>
+      <c r="F2051" t="inlineStr"/>
+      <c r="G2051" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H2051" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2051" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2051" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2051" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2051" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2052">
+      <c r="A2052" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2052" t="inlineStr">
+        <is>
+          <t>Pachuca vs Toluca</t>
+        </is>
+      </c>
+      <c r="C2052" t="inlineStr">
+        <is>
+          <t>Toluca</t>
+        </is>
+      </c>
+      <c r="D2052" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2052" t="inlineStr"/>
+      <c r="F2052" t="inlineStr"/>
+      <c r="G2052" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H2052" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2052" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2052" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2052" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2052" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2053">
+      <c r="A2053" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B2053" t="inlineStr">
+        <is>
+          <t>Llaneros FC vs América de Cali</t>
+        </is>
+      </c>
+      <c r="C2053" t="inlineStr">
+        <is>
+          <t>América de Cali</t>
+        </is>
+      </c>
+      <c r="D2053" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2053" t="inlineStr"/>
+      <c r="F2053" t="inlineStr"/>
+      <c r="G2053" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H2053" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2053" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2053" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2053" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2053" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -91101,7 +95049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -91738,6 +95686,25 @@
       </c>
       <c r="E34" t="n">
         <v>85</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>83</v>
+      </c>
+      <c r="C35" t="n">
+        <v>52</v>
+      </c>
+      <c r="D35" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="E35" t="n">
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 1: seleccion de partidos 2026-10-06
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2053"/>
+  <dimension ref="A1:L2086"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -91075,8 +91075,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1971" t="inlineStr"/>
-      <c r="F1971" t="inlineStr"/>
       <c r="G1971" t="inlineStr">
         <is>
           <t>0-4</t>
@@ -91123,8 +91121,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1972" t="inlineStr"/>
-      <c r="F1972" t="inlineStr"/>
       <c r="G1972" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -91171,8 +91167,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1973" t="inlineStr"/>
-      <c r="F1973" t="inlineStr"/>
       <c r="G1973" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -91219,8 +91213,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1974" t="inlineStr"/>
-      <c r="F1974" t="inlineStr"/>
       <c r="G1974" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -91267,8 +91259,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1975" t="inlineStr"/>
-      <c r="F1975" t="inlineStr"/>
       <c r="G1975" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -91315,8 +91305,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1976" t="inlineStr"/>
-      <c r="F1976" t="inlineStr"/>
       <c r="G1976" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -91363,8 +91351,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1977" t="inlineStr"/>
-      <c r="F1977" t="inlineStr"/>
       <c r="G1977" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -91411,8 +91397,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1978" t="inlineStr"/>
-      <c r="F1978" t="inlineStr"/>
       <c r="G1978" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -91459,8 +91443,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1979" t="inlineStr"/>
-      <c r="F1979" t="inlineStr"/>
       <c r="G1979" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -91507,8 +91489,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1980" t="inlineStr"/>
-      <c r="F1980" t="inlineStr"/>
       <c r="G1980" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -91555,8 +91535,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1981" t="inlineStr"/>
-      <c r="F1981" t="inlineStr"/>
       <c r="G1981" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -91603,8 +91581,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1982" t="inlineStr"/>
-      <c r="F1982" t="inlineStr"/>
       <c r="G1982" t="inlineStr">
         <is>
           <t>5-1</t>
@@ -91651,8 +91627,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1983" t="inlineStr"/>
-      <c r="F1983" t="inlineStr"/>
       <c r="G1983" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -91699,8 +91673,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1984" t="inlineStr"/>
-      <c r="F1984" t="inlineStr"/>
       <c r="G1984" t="inlineStr">
         <is>
           <t>1-6</t>
@@ -91747,8 +91719,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1985" t="inlineStr"/>
-      <c r="F1985" t="inlineStr"/>
       <c r="G1985" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -91795,8 +91765,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1986" t="inlineStr"/>
-      <c r="F1986" t="inlineStr"/>
       <c r="G1986" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -91843,8 +91811,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1987" t="inlineStr"/>
-      <c r="F1987" t="inlineStr"/>
       <c r="G1987" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -91891,8 +91857,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1988" t="inlineStr"/>
-      <c r="F1988" t="inlineStr"/>
       <c r="G1988" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -91939,8 +91903,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1989" t="inlineStr"/>
-      <c r="F1989" t="inlineStr"/>
       <c r="G1989" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -91987,8 +91949,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1990" t="inlineStr"/>
-      <c r="F1990" t="inlineStr"/>
       <c r="G1990" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -92035,8 +91995,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1991" t="inlineStr"/>
-      <c r="F1991" t="inlineStr"/>
       <c r="G1991" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -92083,8 +92041,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1992" t="inlineStr"/>
-      <c r="F1992" t="inlineStr"/>
       <c r="G1992" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -92131,8 +92087,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1993" t="inlineStr"/>
-      <c r="F1993" t="inlineStr"/>
       <c r="G1993" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -92179,8 +92133,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1994" t="inlineStr"/>
-      <c r="F1994" t="inlineStr"/>
       <c r="G1994" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -92227,8 +92179,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1995" t="inlineStr"/>
-      <c r="F1995" t="inlineStr"/>
       <c r="G1995" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -92275,8 +92225,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E1996" t="inlineStr"/>
-      <c r="F1996" t="inlineStr"/>
       <c r="G1996" t="inlineStr">
         <is>
           <t>1-4</t>
@@ -92323,8 +92271,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1997" t="inlineStr"/>
-      <c r="F1997" t="inlineStr"/>
       <c r="G1997" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -92371,8 +92317,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1998" t="inlineStr"/>
-      <c r="F1998" t="inlineStr"/>
       <c r="G1998" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -92419,8 +92363,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E1999" t="inlineStr"/>
-      <c r="F1999" t="inlineStr"/>
       <c r="G1999" t="inlineStr">
         <is>
           <t>4-2</t>
@@ -92467,8 +92409,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2000" t="inlineStr"/>
-      <c r="F2000" t="inlineStr"/>
       <c r="G2000" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -92515,8 +92455,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2001" t="inlineStr"/>
-      <c r="F2001" t="inlineStr"/>
       <c r="G2001" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -92563,8 +92501,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2002" t="inlineStr"/>
-      <c r="F2002" t="inlineStr"/>
       <c r="G2002" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -92611,8 +92547,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2003" t="inlineStr"/>
-      <c r="F2003" t="inlineStr"/>
       <c r="G2003" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -92659,8 +92593,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2004" t="inlineStr"/>
-      <c r="F2004" t="inlineStr"/>
       <c r="G2004" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -92707,8 +92639,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2005" t="inlineStr"/>
-      <c r="F2005" t="inlineStr"/>
       <c r="G2005" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -92755,8 +92685,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2006" t="inlineStr"/>
-      <c r="F2006" t="inlineStr"/>
       <c r="G2006" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -92803,8 +92731,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2007" t="inlineStr"/>
-      <c r="F2007" t="inlineStr"/>
       <c r="G2007" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -92851,8 +92777,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2008" t="inlineStr"/>
-      <c r="F2008" t="inlineStr"/>
       <c r="G2008" t="inlineStr">
         <is>
           <t>7-0</t>
@@ -92899,8 +92823,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2009" t="inlineStr"/>
-      <c r="F2009" t="inlineStr"/>
       <c r="G2009" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -92947,8 +92869,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2010" t="inlineStr"/>
-      <c r="F2010" t="inlineStr"/>
       <c r="G2010" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -92995,8 +92915,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2011" t="inlineStr"/>
-      <c r="F2011" t="inlineStr"/>
       <c r="G2011" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -93043,8 +92961,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2012" t="inlineStr"/>
-      <c r="F2012" t="inlineStr"/>
       <c r="G2012" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -93091,8 +93007,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2013" t="inlineStr"/>
-      <c r="F2013" t="inlineStr"/>
       <c r="G2013" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -93139,8 +93053,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2014" t="inlineStr"/>
-      <c r="F2014" t="inlineStr"/>
       <c r="G2014" t="inlineStr">
         <is>
           <t>6-3</t>
@@ -93187,8 +93099,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2015" t="inlineStr"/>
-      <c r="F2015" t="inlineStr"/>
       <c r="G2015" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -93235,8 +93145,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2016" t="inlineStr"/>
-      <c r="F2016" t="inlineStr"/>
       <c r="G2016" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -93283,8 +93191,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2017" t="inlineStr"/>
-      <c r="F2017" t="inlineStr"/>
       <c r="G2017" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -93331,8 +93237,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2018" t="inlineStr"/>
-      <c r="F2018" t="inlineStr"/>
       <c r="G2018" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -93379,8 +93283,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2019" t="inlineStr"/>
-      <c r="F2019" t="inlineStr"/>
       <c r="G2019" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -93427,8 +93329,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2020" t="inlineStr"/>
-      <c r="F2020" t="inlineStr"/>
       <c r="G2020" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -93475,8 +93375,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2021" t="inlineStr"/>
-      <c r="F2021" t="inlineStr"/>
       <c r="G2021" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -93523,8 +93421,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2022" t="inlineStr"/>
-      <c r="F2022" t="inlineStr"/>
       <c r="G2022" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -93571,8 +93467,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2023" t="inlineStr"/>
-      <c r="F2023" t="inlineStr"/>
       <c r="G2023" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -93619,8 +93513,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2024" t="inlineStr"/>
-      <c r="F2024" t="inlineStr"/>
       <c r="G2024" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -93667,8 +93559,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2025" t="inlineStr"/>
-      <c r="F2025" t="inlineStr"/>
       <c r="G2025" t="inlineStr">
         <is>
           <t>8-1</t>
@@ -93715,8 +93605,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2026" t="inlineStr"/>
-      <c r="F2026" t="inlineStr"/>
       <c r="G2026" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -93763,8 +93651,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2027" t="inlineStr"/>
-      <c r="F2027" t="inlineStr"/>
       <c r="G2027" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -93811,8 +93697,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2028" t="inlineStr"/>
-      <c r="F2028" t="inlineStr"/>
       <c r="G2028" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -93859,8 +93743,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2029" t="inlineStr"/>
-      <c r="F2029" t="inlineStr"/>
       <c r="G2029" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -93907,8 +93789,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2030" t="inlineStr"/>
-      <c r="F2030" t="inlineStr"/>
       <c r="G2030" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -93955,8 +93835,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2031" t="inlineStr"/>
-      <c r="F2031" t="inlineStr"/>
       <c r="G2031" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -94003,8 +93881,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2032" t="inlineStr"/>
-      <c r="F2032" t="inlineStr"/>
       <c r="G2032" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -94051,8 +93927,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2033" t="inlineStr"/>
-      <c r="F2033" t="inlineStr"/>
       <c r="G2033" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -94099,8 +93973,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2034" t="inlineStr"/>
-      <c r="F2034" t="inlineStr"/>
       <c r="G2034" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -94147,8 +94019,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2035" t="inlineStr"/>
-      <c r="F2035" t="inlineStr"/>
       <c r="G2035" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -94195,8 +94065,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2036" t="inlineStr"/>
-      <c r="F2036" t="inlineStr"/>
       <c r="G2036" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -94243,8 +94111,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2037" t="inlineStr"/>
-      <c r="F2037" t="inlineStr"/>
       <c r="G2037" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -94291,8 +94157,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2038" t="inlineStr"/>
-      <c r="F2038" t="inlineStr"/>
       <c r="G2038" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -94339,8 +94203,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2039" t="inlineStr"/>
-      <c r="F2039" t="inlineStr"/>
       <c r="G2039" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -94387,8 +94249,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2040" t="inlineStr"/>
-      <c r="F2040" t="inlineStr"/>
       <c r="G2040" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -94435,8 +94295,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2041" t="inlineStr"/>
-      <c r="F2041" t="inlineStr"/>
       <c r="G2041" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -94483,8 +94341,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2042" t="inlineStr"/>
-      <c r="F2042" t="inlineStr"/>
       <c r="G2042" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -94531,8 +94387,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2043" t="inlineStr"/>
-      <c r="F2043" t="inlineStr"/>
       <c r="G2043" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -94579,8 +94433,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2044" t="inlineStr"/>
-      <c r="F2044" t="inlineStr"/>
       <c r="G2044" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -94627,8 +94479,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2045" t="inlineStr"/>
-      <c r="F2045" t="inlineStr"/>
       <c r="G2045" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -94675,8 +94525,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2046" t="inlineStr"/>
-      <c r="F2046" t="inlineStr"/>
       <c r="G2046" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -94723,8 +94571,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2047" t="inlineStr"/>
-      <c r="F2047" t="inlineStr"/>
       <c r="G2047" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -94771,8 +94617,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2048" t="inlineStr"/>
-      <c r="F2048" t="inlineStr"/>
       <c r="G2048" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -94819,8 +94663,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2049" t="inlineStr"/>
-      <c r="F2049" t="inlineStr"/>
       <c r="G2049" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -94867,8 +94709,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2050" t="inlineStr"/>
-      <c r="F2050" t="inlineStr"/>
       <c r="G2050" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -94915,8 +94755,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2051" t="inlineStr"/>
-      <c r="F2051" t="inlineStr"/>
       <c r="G2051" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -94963,8 +94801,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2052" t="inlineStr"/>
-      <c r="F2052" t="inlineStr"/>
       <c r="G2052" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -95011,8 +94847,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2053" t="inlineStr"/>
-      <c r="F2053" t="inlineStr"/>
       <c r="G2053" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -95033,6 +94867,1590 @@
         <v>0</v>
       </c>
       <c r="L2053" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2054">
+      <c r="A2054" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2054" t="inlineStr">
+        <is>
+          <t>Uganda vs Congo DR</t>
+        </is>
+      </c>
+      <c r="C2054" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="D2054" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2054" t="inlineStr"/>
+      <c r="F2054" t="inlineStr"/>
+      <c r="G2054" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2054" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2054" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2054" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2054" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2054" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2055">
+      <c r="A2055" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2055" t="inlineStr">
+        <is>
+          <t>Ukraine U21 vs Albania U21</t>
+        </is>
+      </c>
+      <c r="C2055" t="inlineStr">
+        <is>
+          <t>Ukraine U21</t>
+        </is>
+      </c>
+      <c r="D2055" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2055" t="inlineStr"/>
+      <c r="F2055" t="inlineStr"/>
+      <c r="G2055" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H2055" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2055" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2055" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2055" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2055" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2056">
+      <c r="A2056" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2056" t="inlineStr">
+        <is>
+          <t>Montenegro U21 vs Armenia U21</t>
+        </is>
+      </c>
+      <c r="C2056" t="inlineStr">
+        <is>
+          <t>Montenegro U21</t>
+        </is>
+      </c>
+      <c r="D2056" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2056" t="inlineStr"/>
+      <c r="F2056" t="inlineStr"/>
+      <c r="G2056" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2056" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2056" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2056" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2056" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2056" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2057">
+      <c r="A2057" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2057" t="inlineStr">
+        <is>
+          <t>Mauritius vs Sri Lanka</t>
+        </is>
+      </c>
+      <c r="C2057" t="inlineStr">
+        <is>
+          <t>Mauritius</t>
+        </is>
+      </c>
+      <c r="D2057" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2057" t="inlineStr"/>
+      <c r="F2057" t="inlineStr"/>
+      <c r="G2057" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H2057" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2057" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2057" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2057" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2057" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2058">
+      <c r="A2058" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2058" t="inlineStr">
+        <is>
+          <t>Cyprus vs Latvia</t>
+        </is>
+      </c>
+      <c r="C2058" t="inlineStr">
+        <is>
+          <t>Cyprus</t>
+        </is>
+      </c>
+      <c r="D2058" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2058" t="inlineStr"/>
+      <c r="F2058" t="inlineStr"/>
+      <c r="G2058" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H2058" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2058" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2058" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2058" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2058" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2059">
+      <c r="A2059" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2059" t="inlineStr">
+        <is>
+          <t>Rwanda vs Kenya</t>
+        </is>
+      </c>
+      <c r="C2059" t="inlineStr">
+        <is>
+          <t>Rwanda</t>
+        </is>
+      </c>
+      <c r="D2059" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2059" t="inlineStr"/>
+      <c r="F2059" t="inlineStr"/>
+      <c r="G2059" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2059" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2059" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2059" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2059" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2059" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2060">
+      <c r="A2060" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2060" t="inlineStr">
+        <is>
+          <t>Serbia U21 vs Russia U21</t>
+        </is>
+      </c>
+      <c r="C2060" t="inlineStr">
+        <is>
+          <t>Russia U21</t>
+        </is>
+      </c>
+      <c r="D2060" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2060" t="inlineStr"/>
+      <c r="F2060" t="inlineStr"/>
+      <c r="G2060" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H2060" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2060" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2060" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2060" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2060" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2061">
+      <c r="A2061" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2061" t="inlineStr">
+        <is>
+          <t>Italy U21 vs Poland U21</t>
+        </is>
+      </c>
+      <c r="C2061" t="inlineStr">
+        <is>
+          <t>Italy U21</t>
+        </is>
+      </c>
+      <c r="D2061" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2061" t="inlineStr"/>
+      <c r="F2061" t="inlineStr"/>
+      <c r="G2061" t="inlineStr">
+        <is>
+          <t>6-2</t>
+        </is>
+      </c>
+      <c r="H2061" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2061" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2061" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2061" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2061" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2062">
+      <c r="A2062" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2062" t="inlineStr">
+        <is>
+          <t>Sweden U21 vs North Macedonia U21</t>
+        </is>
+      </c>
+      <c r="C2062" t="inlineStr">
+        <is>
+          <t>Sweden U21</t>
+        </is>
+      </c>
+      <c r="D2062" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2062" t="inlineStr"/>
+      <c r="F2062" t="inlineStr"/>
+      <c r="G2062" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H2062" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2062" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2062" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2062" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2062" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2063">
+      <c r="A2063" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2063" t="inlineStr">
+        <is>
+          <t>UAI Urquiza vs Ituzaingó</t>
+        </is>
+      </c>
+      <c r="C2063" t="inlineStr">
+        <is>
+          <t>UAI Urquiza</t>
+        </is>
+      </c>
+      <c r="D2063" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2063" t="inlineStr"/>
+      <c r="F2063" t="inlineStr"/>
+      <c r="G2063" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H2063" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2063" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2063" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2063" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2063" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2064">
+      <c r="A2064" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2064" t="inlineStr">
+        <is>
+          <t>Córdoba vs Tenerife</t>
+        </is>
+      </c>
+      <c r="C2064" t="inlineStr">
+        <is>
+          <t>Tenerife</t>
+        </is>
+      </c>
+      <c r="D2064" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2064" t="inlineStr"/>
+      <c r="F2064" t="inlineStr"/>
+      <c r="G2064" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H2064" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2064" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2064" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2064" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2064" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2065">
+      <c r="A2065" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2065" t="inlineStr">
+        <is>
+          <t>Bosnia-Herzegovina vs Poland</t>
+        </is>
+      </c>
+      <c r="C2065" t="inlineStr">
+        <is>
+          <t>Bosnia-Herzegovina</t>
+        </is>
+      </c>
+      <c r="D2065" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2065" t="inlineStr"/>
+      <c r="F2065" t="inlineStr"/>
+      <c r="G2065" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H2065" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2065" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2065" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2065" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2065" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2066">
+      <c r="A2066" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2066" t="inlineStr">
+        <is>
+          <t>France vs Belgium</t>
+        </is>
+      </c>
+      <c r="C2066" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D2066" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2066" t="inlineStr"/>
+      <c r="F2066" t="inlineStr"/>
+      <c r="G2066" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H2066" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2066" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2066" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2066" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2066" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2067">
+      <c r="A2067" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2067" t="inlineStr">
+        <is>
+          <t>Italy vs Türkiye</t>
+        </is>
+      </c>
+      <c r="C2067" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="D2067" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2067" t="inlineStr"/>
+      <c r="F2067" t="inlineStr"/>
+      <c r="G2067" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H2067" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2067" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2067" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2067" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2067" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2068">
+      <c r="A2068" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2068" t="inlineStr">
+        <is>
+          <t>Montenegro vs Armenia</t>
+        </is>
+      </c>
+      <c r="C2068" t="inlineStr">
+        <is>
+          <t>Montenegro</t>
+        </is>
+      </c>
+      <c r="D2068" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2068" t="inlineStr"/>
+      <c r="F2068" t="inlineStr"/>
+      <c r="G2068" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2068" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2068" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2068" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2068" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2068" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2069">
+      <c r="A2069" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2069" t="inlineStr">
+        <is>
+          <t>Northern Ireland vs Georgia</t>
+        </is>
+      </c>
+      <c r="C2069" t="inlineStr">
+        <is>
+          <t>Northern Ireland</t>
+        </is>
+      </c>
+      <c r="D2069" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2069" t="inlineStr"/>
+      <c r="F2069" t="inlineStr"/>
+      <c r="G2069" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2069" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2069" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2069" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2069" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2069" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2070">
+      <c r="A2070" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2070" t="inlineStr">
+        <is>
+          <t>Romania vs Sweden</t>
+        </is>
+      </c>
+      <c r="C2070" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="D2070" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2070" t="inlineStr"/>
+      <c r="F2070" t="inlineStr"/>
+      <c r="G2070" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H2070" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2070" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2070" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2070" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2070" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2071">
+      <c r="A2071" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2071" t="inlineStr">
+        <is>
+          <t>Ukraine vs Hungary</t>
+        </is>
+      </c>
+      <c r="C2071" t="inlineStr">
+        <is>
+          <t>Ukraine</t>
+        </is>
+      </c>
+      <c r="D2071" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2071" t="inlineStr"/>
+      <c r="F2071" t="inlineStr"/>
+      <c r="G2071" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H2071" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2071" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2071" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2071" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2071" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2072">
+      <c r="A2072" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2072" t="inlineStr">
+        <is>
+          <t>Guadeloupe vs St. Lucia</t>
+        </is>
+      </c>
+      <c r="C2072" t="inlineStr">
+        <is>
+          <t>Guadeloupe</t>
+        </is>
+      </c>
+      <c r="D2072" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2072" t="inlineStr"/>
+      <c r="F2072" t="inlineStr"/>
+      <c r="G2072" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H2072" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2072" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2072" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2072" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2072" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2073">
+      <c r="A2073" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2073" t="inlineStr">
+        <is>
+          <t>Deportivo Riestra vs Central Córdoba (Santiago del Estero)</t>
+        </is>
+      </c>
+      <c r="C2073" t="inlineStr">
+        <is>
+          <t>Deportivo Riestra</t>
+        </is>
+      </c>
+      <c r="D2073" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2073" t="inlineStr"/>
+      <c r="F2073" t="inlineStr"/>
+      <c r="G2073" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2073" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2073" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2073" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2073" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2073" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2074">
+      <c r="A2074" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2074" t="inlineStr">
+        <is>
+          <t>Nueva Chicago vs Deportivo Maipú</t>
+        </is>
+      </c>
+      <c r="C2074" t="inlineStr">
+        <is>
+          <t>Deportivo Maipú</t>
+        </is>
+      </c>
+      <c r="D2074" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2074" t="inlineStr"/>
+      <c r="F2074" t="inlineStr"/>
+      <c r="G2074" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H2074" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2074" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2074" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2074" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2074" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2075">
+      <c r="A2075" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2075" t="inlineStr">
+        <is>
+          <t>Cuba vs St. Kitts and Nevis</t>
+        </is>
+      </c>
+      <c r="C2075" t="inlineStr">
+        <is>
+          <t>Cuba</t>
+        </is>
+      </c>
+      <c r="D2075" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2075" t="inlineStr"/>
+      <c r="F2075" t="inlineStr"/>
+      <c r="G2075" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H2075" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2075" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2075" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2075" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2075" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2076">
+      <c r="A2076" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2076" t="inlineStr">
+        <is>
+          <t>Martinique vs El Salvador</t>
+        </is>
+      </c>
+      <c r="C2076" t="inlineStr">
+        <is>
+          <t>Martinique</t>
+        </is>
+      </c>
+      <c r="D2076" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2076" t="inlineStr"/>
+      <c r="F2076" t="inlineStr"/>
+      <c r="G2076" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2076" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2076" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2076" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2076" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2076" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2077">
+      <c r="A2077" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2077" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata vs Gimnasia (Mendoza)</t>
+        </is>
+      </c>
+      <c r="C2077" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="D2077" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2077" t="inlineStr"/>
+      <c r="F2077" t="inlineStr"/>
+      <c r="G2077" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H2077" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2077" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2077" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2077" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2077" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2078">
+      <c r="A2078" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2078" t="inlineStr">
+        <is>
+          <t>Vélez Sarsfield vs Platense</t>
+        </is>
+      </c>
+      <c r="C2078" t="inlineStr">
+        <is>
+          <t>Vélez Sarsfield</t>
+        </is>
+      </c>
+      <c r="D2078" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2078" t="inlineStr"/>
+      <c r="F2078" t="inlineStr"/>
+      <c r="G2078" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H2078" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2078" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2078" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2078" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2078" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2079">
+      <c r="A2079" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2079" t="inlineStr">
+        <is>
+          <t>Cerro Porteño vs 2 de Mayo</t>
+        </is>
+      </c>
+      <c r="C2079" t="inlineStr">
+        <is>
+          <t>2 de Mayo</t>
+        </is>
+      </c>
+      <c r="D2079" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2079" t="inlineStr"/>
+      <c r="F2079" t="inlineStr"/>
+      <c r="G2079" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H2079" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2079" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2079" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2079" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2079" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2080">
+      <c r="A2080" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2080" t="inlineStr">
+        <is>
+          <t>Nacional vs Montevideo City Torque</t>
+        </is>
+      </c>
+      <c r="C2080" t="inlineStr">
+        <is>
+          <t>Montevideo City Torque</t>
+        </is>
+      </c>
+      <c r="D2080" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2080" t="inlineStr"/>
+      <c r="F2080" t="inlineStr"/>
+      <c r="G2080" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H2080" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2080" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2080" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2080" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2080" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2081">
+      <c r="A2081" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2081" t="inlineStr">
+        <is>
+          <t>Bermuda vs Barbados</t>
+        </is>
+      </c>
+      <c r="C2081" t="inlineStr">
+        <is>
+          <t>Bermuda</t>
+        </is>
+      </c>
+      <c r="D2081" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2081" t="inlineStr"/>
+      <c r="F2081" t="inlineStr"/>
+      <c r="G2081" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H2081" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2081" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2081" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2081" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2081" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2082">
+      <c r="A2082" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2082" t="inlineStr">
+        <is>
+          <t>Grenada vs Bonaire</t>
+        </is>
+      </c>
+      <c r="C2082" t="inlineStr">
+        <is>
+          <t>Grenada</t>
+        </is>
+      </c>
+      <c r="D2082" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2082" t="inlineStr"/>
+      <c r="F2082" t="inlineStr"/>
+      <c r="G2082" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H2082" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2082" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2082" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2082" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2082" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2083">
+      <c r="A2083" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2083" t="inlineStr">
+        <is>
+          <t>Guatemala vs Suriname</t>
+        </is>
+      </c>
+      <c r="C2083" t="inlineStr">
+        <is>
+          <t>Guatemala</t>
+        </is>
+      </c>
+      <c r="D2083" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2083" t="inlineStr"/>
+      <c r="F2083" t="inlineStr"/>
+      <c r="G2083" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H2083" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2083" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2083" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2083" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2083" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2084">
+      <c r="A2084" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2084" t="inlineStr">
+        <is>
+          <t>Banfield vs Rosario Central</t>
+        </is>
+      </c>
+      <c r="C2084" t="inlineStr">
+        <is>
+          <t>Rosario Central</t>
+        </is>
+      </c>
+      <c r="D2084" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2084" t="inlineStr"/>
+      <c r="F2084" t="inlineStr"/>
+      <c r="G2084" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2084" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2084" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2084" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2084" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2084" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2085">
+      <c r="A2085" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2085" t="inlineStr">
+        <is>
+          <t>Honduras vs Jamaica</t>
+        </is>
+      </c>
+      <c r="C2085" t="inlineStr">
+        <is>
+          <t>Honduras</t>
+        </is>
+      </c>
+      <c r="D2085" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2085" t="inlineStr"/>
+      <c r="F2085" t="inlineStr"/>
+      <c r="G2085" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2085" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2085" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2085" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2085" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2085" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2086">
+      <c r="A2086" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B2086" t="inlineStr">
+        <is>
+          <t>Austria U21 vs South Korea U21</t>
+        </is>
+      </c>
+      <c r="C2086" t="inlineStr">
+        <is>
+          <t>Austria U21</t>
+        </is>
+      </c>
+      <c r="D2086" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2086" t="inlineStr"/>
+      <c r="F2086" t="inlineStr"/>
+      <c r="G2086" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2086" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2086" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2086" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2086" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2086" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -95049,7 +96467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -95705,6 +97123,25 @@
       </c>
       <c r="E35" t="n">
         <v>150</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>33</v>
+      </c>
+      <c r="C36" t="n">
+        <v>17</v>
+      </c>
+      <c r="D36" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="E36" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -95718,7 +97155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G179"/>
+  <dimension ref="A1:G185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -99861,6 +101298,168 @@
         <v>0</v>
       </c>
     </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>2</v>
+      </c>
+      <c r="D180" t="n">
+        <v>2</v>
+      </c>
+      <c r="E180" t="n">
+        <v>100</v>
+      </c>
+      <c r="F180" t="n">
+        <v>0</v>
+      </c>
+      <c r="G180" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>2</v>
+      </c>
+      <c r="D181" t="n">
+        <v>1</v>
+      </c>
+      <c r="E181" t="n">
+        <v>50</v>
+      </c>
+      <c r="F181" t="n">
+        <v>1</v>
+      </c>
+      <c r="G181" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>posible_descuento</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>1</v>
+      </c>
+      <c r="D182" t="n">
+        <v>1</v>
+      </c>
+      <c r="E182" t="n">
+        <v>100</v>
+      </c>
+      <c r="F182" t="n">
+        <v>0</v>
+      </c>
+      <c r="G182" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>siguen_empatados_70</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>1</v>
+      </c>
+      <c r="D183" t="n">
+        <v>0</v>
+      </c>
+      <c r="E183" t="n">
+        <v>0</v>
+      </c>
+      <c r="F183" t="n">
+        <v>1</v>
+      </c>
+      <c r="G183" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>siguen_empatados_22</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>2</v>
+      </c>
+      <c r="D184" t="n">
+        <v>1</v>
+      </c>
+      <c r="E184" t="n">
+        <v>50</v>
+      </c>
+      <c r="F184" t="n">
+        <v>1</v>
+      </c>
+      <c r="G184" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>1</v>
+      </c>
+      <c r="D185" t="n">
+        <v>0</v>
+      </c>
+      <c r="E185" t="n">
+        <v>0</v>
+      </c>
+      <c r="F185" t="n">
+        <v>1</v>
+      </c>
+      <c r="G185" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 1 embebida: seleccion 2026-10-07T05:03
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2086"/>
+  <dimension ref="A1:L2169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -94893,8 +94893,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2054" t="inlineStr"/>
-      <c r="F2054" t="inlineStr"/>
       <c r="G2054" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -94941,8 +94939,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2055" t="inlineStr"/>
-      <c r="F2055" t="inlineStr"/>
       <c r="G2055" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -94989,8 +94985,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2056" t="inlineStr"/>
-      <c r="F2056" t="inlineStr"/>
       <c r="G2056" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -95037,8 +95031,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2057" t="inlineStr"/>
-      <c r="F2057" t="inlineStr"/>
       <c r="G2057" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -95085,8 +95077,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2058" t="inlineStr"/>
-      <c r="F2058" t="inlineStr"/>
       <c r="G2058" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -95133,8 +95123,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2059" t="inlineStr"/>
-      <c r="F2059" t="inlineStr"/>
       <c r="G2059" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -95181,8 +95169,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2060" t="inlineStr"/>
-      <c r="F2060" t="inlineStr"/>
       <c r="G2060" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -95229,8 +95215,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2061" t="inlineStr"/>
-      <c r="F2061" t="inlineStr"/>
       <c r="G2061" t="inlineStr">
         <is>
           <t>6-2</t>
@@ -95277,8 +95261,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2062" t="inlineStr"/>
-      <c r="F2062" t="inlineStr"/>
       <c r="G2062" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -95325,8 +95307,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2063" t="inlineStr"/>
-      <c r="F2063" t="inlineStr"/>
       <c r="G2063" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -95373,8 +95353,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2064" t="inlineStr"/>
-      <c r="F2064" t="inlineStr"/>
       <c r="G2064" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -95421,8 +95399,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2065" t="inlineStr"/>
-      <c r="F2065" t="inlineStr"/>
       <c r="G2065" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -95469,8 +95445,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2066" t="inlineStr"/>
-      <c r="F2066" t="inlineStr"/>
       <c r="G2066" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -95517,8 +95491,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2067" t="inlineStr"/>
-      <c r="F2067" t="inlineStr"/>
       <c r="G2067" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -95565,8 +95537,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2068" t="inlineStr"/>
-      <c r="F2068" t="inlineStr"/>
       <c r="G2068" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -95613,8 +95583,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2069" t="inlineStr"/>
-      <c r="F2069" t="inlineStr"/>
       <c r="G2069" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -95661,8 +95629,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2070" t="inlineStr"/>
-      <c r="F2070" t="inlineStr"/>
       <c r="G2070" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -95709,8 +95675,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2071" t="inlineStr"/>
-      <c r="F2071" t="inlineStr"/>
       <c r="G2071" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -95757,8 +95721,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2072" t="inlineStr"/>
-      <c r="F2072" t="inlineStr"/>
       <c r="G2072" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -95805,8 +95767,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2073" t="inlineStr"/>
-      <c r="F2073" t="inlineStr"/>
       <c r="G2073" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -95853,8 +95813,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2074" t="inlineStr"/>
-      <c r="F2074" t="inlineStr"/>
       <c r="G2074" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -95901,8 +95859,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2075" t="inlineStr"/>
-      <c r="F2075" t="inlineStr"/>
       <c r="G2075" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -95949,8 +95905,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2076" t="inlineStr"/>
-      <c r="F2076" t="inlineStr"/>
       <c r="G2076" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -95997,8 +95951,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2077" t="inlineStr"/>
-      <c r="F2077" t="inlineStr"/>
       <c r="G2077" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -96045,8 +95997,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2078" t="inlineStr"/>
-      <c r="F2078" t="inlineStr"/>
       <c r="G2078" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -96093,8 +96043,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2079" t="inlineStr"/>
-      <c r="F2079" t="inlineStr"/>
       <c r="G2079" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -96141,8 +96089,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2080" t="inlineStr"/>
-      <c r="F2080" t="inlineStr"/>
       <c r="G2080" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -96189,8 +96135,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2081" t="inlineStr"/>
-      <c r="F2081" t="inlineStr"/>
       <c r="G2081" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -96237,8 +96181,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2082" t="inlineStr"/>
-      <c r="F2082" t="inlineStr"/>
       <c r="G2082" t="inlineStr">
         <is>
           <t>1-4</t>
@@ -96285,8 +96227,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2083" t="inlineStr"/>
-      <c r="F2083" t="inlineStr"/>
       <c r="G2083" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -96333,8 +96273,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2084" t="inlineStr"/>
-      <c r="F2084" t="inlineStr"/>
       <c r="G2084" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -96381,8 +96319,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2085" t="inlineStr"/>
-      <c r="F2085" t="inlineStr"/>
       <c r="G2085" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -96429,8 +96365,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E2086" t="inlineStr"/>
-      <c r="F2086" t="inlineStr"/>
       <c r="G2086" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -96451,6 +96385,3990 @@
         <v>0</v>
       </c>
       <c r="L2086" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2087">
+      <c r="A2087" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2087" t="inlineStr">
+        <is>
+          <t>IFK Norrköping vs Kalmar FF</t>
+        </is>
+      </c>
+      <c r="C2087" t="inlineStr">
+        <is>
+          <t>IFK Norrköping</t>
+        </is>
+      </c>
+      <c r="D2087" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2087" t="inlineStr"/>
+      <c r="F2087" t="inlineStr"/>
+      <c r="G2087" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2087" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2087" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2087" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2087" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2087" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2088">
+      <c r="A2088" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2088" t="inlineStr">
+        <is>
+          <t>China vs Tajikistan</t>
+        </is>
+      </c>
+      <c r="C2088" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="D2088" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2088" t="inlineStr"/>
+      <c r="F2088" t="inlineStr"/>
+      <c r="G2088" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H2088" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2088" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2088" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2088" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2088" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2089">
+      <c r="A2089" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2089" t="inlineStr">
+        <is>
+          <t>Azerbaijan U21 vs Gibraltar U21</t>
+        </is>
+      </c>
+      <c r="C2089" t="inlineStr">
+        <is>
+          <t>Azerbaijan U21</t>
+        </is>
+      </c>
+      <c r="D2089" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2089" t="inlineStr"/>
+      <c r="F2089" t="inlineStr"/>
+      <c r="G2089" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H2089" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2089" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2089" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2089" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2089" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2090">
+      <c r="A2090" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2090" t="inlineStr">
+        <is>
+          <t>Kazakhstan vs Faroe Islands</t>
+        </is>
+      </c>
+      <c r="C2090" t="inlineStr">
+        <is>
+          <t>Faroe Islands</t>
+        </is>
+      </c>
+      <c r="D2090" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2090" t="inlineStr"/>
+      <c r="F2090" t="inlineStr"/>
+      <c r="G2090" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H2090" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2090" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2090" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2090" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2090" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2091">
+      <c r="A2091" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2091" t="inlineStr">
+        <is>
+          <t>India vs Uruguay</t>
+        </is>
+      </c>
+      <c r="C2091" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D2091" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2091" t="inlineStr"/>
+      <c r="F2091" t="inlineStr"/>
+      <c r="G2091" t="inlineStr">
+        <is>
+          <t>1-6</t>
+        </is>
+      </c>
+      <c r="H2091" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2091" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2091" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2091" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2091" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2092">
+      <c r="A2092" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2092" t="inlineStr">
+        <is>
+          <t>Moldova U21 vs Kazakhstan U21</t>
+        </is>
+      </c>
+      <c r="C2092" t="inlineStr">
+        <is>
+          <t>Moldova U21</t>
+        </is>
+      </c>
+      <c r="D2092" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2092" t="inlineStr"/>
+      <c r="F2092" t="inlineStr"/>
+      <c r="G2092" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H2092" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2092" t="n">
+        <v>3</v>
+      </c>
+      <c r="J2092" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2092" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2092" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2093">
+      <c r="A2093" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2093" t="inlineStr">
+        <is>
+          <t>Russia vs Nigeria</t>
+        </is>
+      </c>
+      <c r="C2093" t="inlineStr">
+        <is>
+          <t>Russia</t>
+        </is>
+      </c>
+      <c r="D2093" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2093" t="inlineStr"/>
+      <c r="F2093" t="inlineStr"/>
+      <c r="G2093" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H2093" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2093" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2093" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2093" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2093" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2094">
+      <c r="A2094" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2094" t="inlineStr">
+        <is>
+          <t>Germany U21 vs Georgia U21</t>
+        </is>
+      </c>
+      <c r="C2094" t="inlineStr">
+        <is>
+          <t>Germany U21</t>
+        </is>
+      </c>
+      <c r="D2094" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2094" t="inlineStr"/>
+      <c r="F2094" t="inlineStr"/>
+      <c r="G2094" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H2094" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2094" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2094" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2094" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2094" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2095">
+      <c r="A2095" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2095" t="inlineStr">
+        <is>
+          <t>Latvia U21 vs Malta U21</t>
+        </is>
+      </c>
+      <c r="C2095" t="inlineStr">
+        <is>
+          <t>Malta U21</t>
+        </is>
+      </c>
+      <c r="D2095" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2095" t="inlineStr"/>
+      <c r="F2095" t="inlineStr"/>
+      <c r="G2095" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H2095" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2095" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2095" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2095" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2095" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2096">
+      <c r="A2096" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2096" t="inlineStr">
+        <is>
+          <t>Bulgaria U21 vs Scotland U21</t>
+        </is>
+      </c>
+      <c r="C2096" t="inlineStr">
+        <is>
+          <t>Scotland U21</t>
+        </is>
+      </c>
+      <c r="D2096" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2096" t="inlineStr"/>
+      <c r="F2096" t="inlineStr"/>
+      <c r="G2096" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H2096" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2096" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2096" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2096" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2096" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2097">
+      <c r="A2097" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2097" t="inlineStr">
+        <is>
+          <t>Denmark U21 vs Belgium U21</t>
+        </is>
+      </c>
+      <c r="C2097" t="inlineStr">
+        <is>
+          <t>Denmark U21</t>
+        </is>
+      </c>
+      <c r="D2097" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2097" t="inlineStr"/>
+      <c r="F2097" t="inlineStr"/>
+      <c r="G2097" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2097" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2097" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2097" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2097" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2097" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2098">
+      <c r="A2098" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2098" t="inlineStr">
+        <is>
+          <t>Portugal U21 vs Czechia U21</t>
+        </is>
+      </c>
+      <c r="C2098" t="inlineStr">
+        <is>
+          <t>Portugal U21</t>
+        </is>
+      </c>
+      <c r="D2098" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2098" t="inlineStr"/>
+      <c r="F2098" t="inlineStr"/>
+      <c r="G2098" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H2098" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2098" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2098" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2098" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2098" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2099">
+      <c r="A2099" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2099" t="inlineStr">
+        <is>
+          <t>Wales U21 vs Austria U21</t>
+        </is>
+      </c>
+      <c r="C2099" t="inlineStr">
+        <is>
+          <t>Austria U21</t>
+        </is>
+      </c>
+      <c r="D2099" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2099" t="inlineStr"/>
+      <c r="F2099" t="inlineStr"/>
+      <c r="G2099" t="inlineStr">
+        <is>
+          <t>1-7</t>
+        </is>
+      </c>
+      <c r="H2099" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2099" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2099" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2099" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2099" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2100">
+      <c r="A2100" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2100" t="inlineStr">
+        <is>
+          <t>Netherlands U21 vs Bosnia-Herzegovina U21</t>
+        </is>
+      </c>
+      <c r="C2100" t="inlineStr">
+        <is>
+          <t>Netherlands U21</t>
+        </is>
+      </c>
+      <c r="D2100" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2100" t="inlineStr"/>
+      <c r="F2100" t="inlineStr"/>
+      <c r="G2100" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H2100" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2100" t="n">
+        <v>4</v>
+      </c>
+      <c r="J2100" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2100" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2100" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2101">
+      <c r="A2101" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2101" t="inlineStr">
+        <is>
+          <t>Norway U21 vs Israel U21</t>
+        </is>
+      </c>
+      <c r="C2101" t="inlineStr">
+        <is>
+          <t>Norway U21</t>
+        </is>
+      </c>
+      <c r="D2101" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2101" t="inlineStr"/>
+      <c r="F2101" t="inlineStr"/>
+      <c r="G2101" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2101" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2101" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2101" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2101" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2101" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2102">
+      <c r="A2102" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2102" t="inlineStr">
+        <is>
+          <t>Algeria vs Niger</t>
+        </is>
+      </c>
+      <c r="C2102" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="D2102" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2102" t="inlineStr"/>
+      <c r="F2102" t="inlineStr"/>
+      <c r="G2102" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H2102" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2102" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2102" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2102" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2102" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2103">
+      <c r="A2103" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2103" t="inlineStr">
+        <is>
+          <t>Jordan vs Venezuela</t>
+        </is>
+      </c>
+      <c r="C2103" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="D2103" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2103" t="inlineStr"/>
+      <c r="F2103" t="inlineStr"/>
+      <c r="G2103" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2103" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2103" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2103" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2103" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2103" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2104">
+      <c r="A2104" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2104" t="inlineStr">
+        <is>
+          <t>Andorra U21 vs Slovakia U21</t>
+        </is>
+      </c>
+      <c r="C2104" t="inlineStr">
+        <is>
+          <t>Slovakia U21</t>
+        </is>
+      </c>
+      <c r="D2104" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2104" t="inlineStr"/>
+      <c r="F2104" t="inlineStr"/>
+      <c r="G2104" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H2104" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2104" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2104" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2104" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2104" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2105">
+      <c r="A2105" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2105" t="inlineStr">
+        <is>
+          <t>Cyprus U21 vs San Marino U21</t>
+        </is>
+      </c>
+      <c r="C2105" t="inlineStr">
+        <is>
+          <t>Cyprus U21</t>
+        </is>
+      </c>
+      <c r="D2105" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2105" t="inlineStr"/>
+      <c r="F2105" t="inlineStr"/>
+      <c r="G2105" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H2105" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2105" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2105" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2105" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2105" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2106">
+      <c r="A2106" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2106" t="inlineStr">
+        <is>
+          <t>Faroe Islands U21 vs Iceland U21</t>
+        </is>
+      </c>
+      <c r="C2106" t="inlineStr">
+        <is>
+          <t>Iceland U21</t>
+        </is>
+      </c>
+      <c r="D2106" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2106" t="inlineStr"/>
+      <c r="F2106" t="inlineStr"/>
+      <c r="G2106" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H2106" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2106" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2106" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2106" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2106" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2107">
+      <c r="A2107" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2107" t="inlineStr">
+        <is>
+          <t>France U21 vs Switzerland U21</t>
+        </is>
+      </c>
+      <c r="C2107" t="inlineStr">
+        <is>
+          <t>France U21</t>
+        </is>
+      </c>
+      <c r="D2107" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2107" t="inlineStr"/>
+      <c r="F2107" t="inlineStr"/>
+      <c r="G2107" t="inlineStr">
+        <is>
+          <t>7-1</t>
+        </is>
+      </c>
+      <c r="H2107" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2107" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2107" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2107" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2107" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2108">
+      <c r="A2108" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2108" t="inlineStr">
+        <is>
+          <t>Kosovo U21 vs Finland U21</t>
+        </is>
+      </c>
+      <c r="C2108" t="inlineStr">
+        <is>
+          <t>Kosovo U21</t>
+        </is>
+      </c>
+      <c r="D2108" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2108" t="inlineStr"/>
+      <c r="F2108" t="inlineStr"/>
+      <c r="G2108" t="inlineStr">
+        <is>
+          <t>4-4</t>
+        </is>
+      </c>
+      <c r="H2108" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2108" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2108" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2108" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2108" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2109">
+      <c r="A2109" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2109" t="inlineStr">
+        <is>
+          <t>Lithuania U21 vs Croatia U21</t>
+        </is>
+      </c>
+      <c r="C2109" t="inlineStr">
+        <is>
+          <t>Croatia U21</t>
+        </is>
+      </c>
+      <c r="D2109" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2109" t="inlineStr"/>
+      <c r="F2109" t="inlineStr"/>
+      <c r="G2109" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H2109" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2109" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2109" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2109" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2109" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2110">
+      <c r="A2110" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2110" t="inlineStr">
+        <is>
+          <t>Luxembourg U21 vs Estonia U21</t>
+        </is>
+      </c>
+      <c r="C2110" t="inlineStr">
+        <is>
+          <t>Luxembourg U21</t>
+        </is>
+      </c>
+      <c r="D2110" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2110" t="inlineStr"/>
+      <c r="F2110" t="inlineStr"/>
+      <c r="G2110" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H2110" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2110" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2110" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2110" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2110" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2111">
+      <c r="A2111" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2111" t="inlineStr">
+        <is>
+          <t>Republic of Ireland U21 vs England U21</t>
+        </is>
+      </c>
+      <c r="C2111" t="inlineStr">
+        <is>
+          <t>Republic of Ireland U21</t>
+        </is>
+      </c>
+      <c r="D2111" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2111" t="inlineStr"/>
+      <c r="F2111" t="inlineStr"/>
+      <c r="G2111" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H2111" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2111" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2111" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2111" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2111" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2112">
+      <c r="A2112" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2112" t="inlineStr">
+        <is>
+          <t>Spain U21 vs Romania U21</t>
+        </is>
+      </c>
+      <c r="C2112" t="inlineStr">
+        <is>
+          <t>Spain U21</t>
+        </is>
+      </c>
+      <c r="D2112" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2112" t="inlineStr"/>
+      <c r="F2112" t="inlineStr"/>
+      <c r="G2112" t="inlineStr">
+        <is>
+          <t>7-1</t>
+        </is>
+      </c>
+      <c r="H2112" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2112" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2112" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2112" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2112" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2113">
+      <c r="A2113" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2113" t="inlineStr">
+        <is>
+          <t>Türkiye U21 vs Hungary U21</t>
+        </is>
+      </c>
+      <c r="C2113" t="inlineStr">
+        <is>
+          <t>Türkiye U21</t>
+        </is>
+      </c>
+      <c r="D2113" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2113" t="inlineStr"/>
+      <c r="F2113" t="inlineStr"/>
+      <c r="G2113" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2113" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2113" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2113" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2113" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2113" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2114">
+      <c r="A2114" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2114" t="inlineStr">
+        <is>
+          <t>AFC Wimbledon vs Barnet</t>
+        </is>
+      </c>
+      <c r="C2114" t="inlineStr">
+        <is>
+          <t>AFC Wimbledon</t>
+        </is>
+      </c>
+      <c r="D2114" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2114" t="inlineStr"/>
+      <c r="F2114" t="inlineStr"/>
+      <c r="G2114" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2114" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2114" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2114" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2114" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2114" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2115">
+      <c r="A2115" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2115" t="inlineStr">
+        <is>
+          <t>Cambridge United vs Northampton Town</t>
+        </is>
+      </c>
+      <c r="C2115" t="inlineStr">
+        <is>
+          <t>Cambridge United</t>
+        </is>
+      </c>
+      <c r="D2115" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2115" t="inlineStr"/>
+      <c r="F2115" t="inlineStr"/>
+      <c r="G2115" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H2115" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2115" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2115" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2115" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2115" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2116">
+      <c r="A2116" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2116" t="inlineStr">
+        <is>
+          <t>Exeter City vs Oxford United</t>
+        </is>
+      </c>
+      <c r="C2116" t="inlineStr">
+        <is>
+          <t>Oxford United</t>
+        </is>
+      </c>
+      <c r="D2116" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2116" t="inlineStr"/>
+      <c r="F2116" t="inlineStr"/>
+      <c r="G2116" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H2116" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2116" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2116" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2116" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2116" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2117">
+      <c r="A2117" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2117" t="inlineStr">
+        <is>
+          <t>Huddersfield Town vs Rochdale</t>
+        </is>
+      </c>
+      <c r="C2117" t="inlineStr">
+        <is>
+          <t>Huddersfield Town</t>
+        </is>
+      </c>
+      <c r="D2117" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2117" t="inlineStr"/>
+      <c r="F2117" t="inlineStr"/>
+      <c r="G2117" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H2117" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2117" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2117" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2117" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2117" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2118">
+      <c r="A2118" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2118" t="inlineStr">
+        <is>
+          <t>Milton Keynes Dons vs Brentford U21</t>
+        </is>
+      </c>
+      <c r="C2118" t="inlineStr">
+        <is>
+          <t>Brentford U21</t>
+        </is>
+      </c>
+      <c r="D2118" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2118" t="inlineStr"/>
+      <c r="F2118" t="inlineStr"/>
+      <c r="G2118" t="inlineStr">
+        <is>
+          <t>7-1</t>
+        </is>
+      </c>
+      <c r="H2118" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2118" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2118" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2118" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2118" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2119">
+      <c r="A2119" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2119" t="inlineStr">
+        <is>
+          <t>Newport County vs Plymouth Argyle</t>
+        </is>
+      </c>
+      <c r="C2119" t="inlineStr">
+        <is>
+          <t>Plymouth Argyle</t>
+        </is>
+      </c>
+      <c r="D2119" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2119" t="inlineStr"/>
+      <c r="F2119" t="inlineStr"/>
+      <c r="G2119" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H2119" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2119" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2119" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2119" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2119" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2120">
+      <c r="A2120" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2120" t="inlineStr">
+        <is>
+          <t>Peterborough United vs Ipswich Town U21</t>
+        </is>
+      </c>
+      <c r="C2120" t="inlineStr">
+        <is>
+          <t>Peterborough United</t>
+        </is>
+      </c>
+      <c r="D2120" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2120" t="inlineStr"/>
+      <c r="F2120" t="inlineStr"/>
+      <c r="G2120" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H2120" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2120" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2120" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2120" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2120" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2121">
+      <c r="A2121" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2121" t="inlineStr">
+        <is>
+          <t>Rotherham United vs Bradford City</t>
+        </is>
+      </c>
+      <c r="C2121" t="inlineStr">
+        <is>
+          <t>Bradford City</t>
+        </is>
+      </c>
+      <c r="D2121" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2121" t="inlineStr"/>
+      <c r="F2121" t="inlineStr"/>
+      <c r="G2121" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H2121" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2121" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2121" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2121" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2121" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2122">
+      <c r="A2122" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2122" t="inlineStr">
+        <is>
+          <t>Sheffield Wednesday vs Sunderland U21</t>
+        </is>
+      </c>
+      <c r="C2122" t="inlineStr">
+        <is>
+          <t>Sheffield Wednesday</t>
+        </is>
+      </c>
+      <c r="D2122" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2122" t="inlineStr"/>
+      <c r="F2122" t="inlineStr"/>
+      <c r="G2122" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H2122" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2122" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2122" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2122" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2122" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2123">
+      <c r="A2123" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2123" t="inlineStr">
+        <is>
+          <t>Shrewsbury Town vs Stockport County</t>
+        </is>
+      </c>
+      <c r="C2123" t="inlineStr">
+        <is>
+          <t>Stockport County</t>
+        </is>
+      </c>
+      <c r="D2123" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2123" t="inlineStr"/>
+      <c r="F2123" t="inlineStr"/>
+      <c r="G2123" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H2123" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2123" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2123" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2123" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2123" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2124">
+      <c r="A2124" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2124" t="inlineStr">
+        <is>
+          <t>Stevenage vs Leicester City</t>
+        </is>
+      </c>
+      <c r="C2124" t="inlineStr">
+        <is>
+          <t>Stevenage</t>
+        </is>
+      </c>
+      <c r="D2124" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2124" t="inlineStr"/>
+      <c r="F2124" t="inlineStr"/>
+      <c r="G2124" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H2124" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2124" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2124" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2124" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2124" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2125">
+      <c r="A2125" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2125" t="inlineStr">
+        <is>
+          <t>Wycombe Wanderers vs Bristol Rovers</t>
+        </is>
+      </c>
+      <c r="C2125" t="inlineStr">
+        <is>
+          <t>Wycombe Wanderers</t>
+        </is>
+      </c>
+      <c r="D2125" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2125" t="inlineStr"/>
+      <c r="F2125" t="inlineStr"/>
+      <c r="G2125" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H2125" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2125" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2125" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2125" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2125" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2126">
+      <c r="A2126" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2126" t="inlineStr">
+        <is>
+          <t>Atherton Collieries vs Trafford</t>
+        </is>
+      </c>
+      <c r="C2126" t="inlineStr">
+        <is>
+          <t>Atherton Collieries</t>
+        </is>
+      </c>
+      <c r="D2126" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2126" t="inlineStr"/>
+      <c r="F2126" t="inlineStr"/>
+      <c r="G2126" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H2126" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2126" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2126" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2126" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2126" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2127">
+      <c r="A2127" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2127" t="inlineStr">
+        <is>
+          <t>Halesown Town FC vs Stafford Rangers</t>
+        </is>
+      </c>
+      <c r="C2127" t="inlineStr">
+        <is>
+          <t>Halesown Town FC</t>
+        </is>
+      </c>
+      <c r="D2127" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2127" t="inlineStr"/>
+      <c r="F2127" t="inlineStr"/>
+      <c r="G2127" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H2127" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2127" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2127" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2127" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2127" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2128">
+      <c r="A2128" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2128" t="inlineStr">
+        <is>
+          <t>Scarborough Athletic vs Macclesfield FC</t>
+        </is>
+      </c>
+      <c r="C2128" t="inlineStr">
+        <is>
+          <t>Scarborough Athletic</t>
+        </is>
+      </c>
+      <c r="D2128" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2128" t="inlineStr"/>
+      <c r="F2128" t="inlineStr"/>
+      <c r="G2128" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H2128" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2128" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2128" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2128" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2128" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2129">
+      <c r="A2129" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2129" t="inlineStr">
+        <is>
+          <t>Spalding United vs Bury Town U21</t>
+        </is>
+      </c>
+      <c r="C2129" t="inlineStr">
+        <is>
+          <t>Spalding United</t>
+        </is>
+      </c>
+      <c r="D2129" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2129" t="inlineStr"/>
+      <c r="F2129" t="inlineStr"/>
+      <c r="G2129" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H2129" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2129" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2129" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2129" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2129" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2130">
+      <c r="A2130" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2130" t="inlineStr">
+        <is>
+          <t>Wingate &amp; Finchley vs Bedford Town</t>
+        </is>
+      </c>
+      <c r="C2130" t="inlineStr">
+        <is>
+          <t>Wingate &amp; Finchley</t>
+        </is>
+      </c>
+      <c r="D2130" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2130" t="inlineStr"/>
+      <c r="F2130" t="inlineStr"/>
+      <c r="G2130" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H2130" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2130" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2130" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2130" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2130" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2131">
+      <c r="A2131" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2131" t="inlineStr">
+        <is>
+          <t>Albania vs San Marino</t>
+        </is>
+      </c>
+      <c r="C2131" t="inlineStr">
+        <is>
+          <t>Albania</t>
+        </is>
+      </c>
+      <c r="D2131" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2131" t="inlineStr"/>
+      <c r="F2131" t="inlineStr"/>
+      <c r="G2131" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H2131" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2131" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2131" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2131" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2131" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2132">
+      <c r="A2132" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2132" t="inlineStr">
+        <is>
+          <t>Belarus vs Finland</t>
+        </is>
+      </c>
+      <c r="C2132" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D2132" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2132" t="inlineStr"/>
+      <c r="F2132" t="inlineStr"/>
+      <c r="G2132" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H2132" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2132" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2132" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2132" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2132" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2133">
+      <c r="A2133" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2133" t="inlineStr">
+        <is>
+          <t>Croatia vs Spain</t>
+        </is>
+      </c>
+      <c r="C2133" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D2133" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2133" t="inlineStr"/>
+      <c r="F2133" t="inlineStr"/>
+      <c r="G2133" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H2133" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2133" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2133" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2133" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2133" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2134">
+      <c r="A2134" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2134" t="inlineStr">
+        <is>
+          <t>England vs Czechia</t>
+        </is>
+      </c>
+      <c r="C2134" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D2134" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2134" t="inlineStr"/>
+      <c r="F2134" t="inlineStr"/>
+      <c r="G2134" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H2134" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2134" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2134" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2134" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2134" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2135">
+      <c r="A2135" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2135" t="inlineStr">
+        <is>
+          <t>Estonia vs Iceland</t>
+        </is>
+      </c>
+      <c r="C2135" t="inlineStr">
+        <is>
+          <t>Iceland</t>
+        </is>
+      </c>
+      <c r="D2135" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2135" t="inlineStr"/>
+      <c r="F2135" t="inlineStr"/>
+      <c r="G2135" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2135" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2135" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2135" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2135" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2135" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2136">
+      <c r="A2136" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2136" t="inlineStr">
+        <is>
+          <t>Moldova vs Slovakia</t>
+        </is>
+      </c>
+      <c r="C2136" t="inlineStr">
+        <is>
+          <t>Slovakia</t>
+        </is>
+      </c>
+      <c r="D2136" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2136" t="inlineStr"/>
+      <c r="F2136" t="inlineStr"/>
+      <c r="G2136" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H2136" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2136" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2136" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2136" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2136" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2137">
+      <c r="A2137" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2137" t="inlineStr">
+        <is>
+          <t>Scotland vs Slovenia</t>
+        </is>
+      </c>
+      <c r="C2137" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="D2137" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2137" t="inlineStr"/>
+      <c r="F2137" t="inlineStr"/>
+      <c r="G2137" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H2137" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2137" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2137" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2137" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2137" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2138">
+      <c r="A2138" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2138" t="inlineStr">
+        <is>
+          <t>Switzerland vs North Macedonia</t>
+        </is>
+      </c>
+      <c r="C2138" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D2138" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2138" t="inlineStr"/>
+      <c r="F2138" t="inlineStr"/>
+      <c r="G2138" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H2138" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2138" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2138" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2138" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2138" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2139">
+      <c r="A2139" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2139" t="inlineStr">
+        <is>
+          <t>Crawley Town vs Bromley</t>
+        </is>
+      </c>
+      <c r="C2139" t="inlineStr">
+        <is>
+          <t>Bromley</t>
+        </is>
+      </c>
+      <c r="D2139" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2139" t="inlineStr"/>
+      <c r="F2139" t="inlineStr"/>
+      <c r="G2139" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H2139" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2139" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2139" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2139" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2139" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2140">
+      <c r="A2140" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2140" t="inlineStr">
+        <is>
+          <t>Angola vs Malawi</t>
+        </is>
+      </c>
+      <c r="C2140" t="inlineStr">
+        <is>
+          <t>Angola</t>
+        </is>
+      </c>
+      <c r="D2140" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2140" t="inlineStr"/>
+      <c r="F2140" t="inlineStr"/>
+      <c r="G2140" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H2140" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2140" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2140" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2140" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2140" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2141">
+      <c r="A2141" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2141" t="inlineStr">
+        <is>
+          <t>Real Oruro vs Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="C2141" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="D2141" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2141" t="inlineStr"/>
+      <c r="F2141" t="inlineStr"/>
+      <c r="G2141" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H2141" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2141" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2141" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2141" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2141" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2142">
+      <c r="A2142" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2142" t="inlineStr">
+        <is>
+          <t>Villanova Wildcats vs New Haven Chargers</t>
+        </is>
+      </c>
+      <c r="C2142" t="inlineStr">
+        <is>
+          <t>Villanova Wildcats</t>
+        </is>
+      </c>
+      <c r="D2142" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2142" t="inlineStr"/>
+      <c r="F2142" t="inlineStr"/>
+      <c r="G2142" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H2142" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2142" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2142" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2142" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2142" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2143">
+      <c r="A2143" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2143" t="inlineStr">
+        <is>
+          <t>Montserrat vs Turks and Caicos Islands</t>
+        </is>
+      </c>
+      <c r="C2143" t="inlineStr">
+        <is>
+          <t>Montserrat</t>
+        </is>
+      </c>
+      <c r="D2143" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2143" t="inlineStr"/>
+      <c r="F2143" t="inlineStr"/>
+      <c r="G2143" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H2143" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2143" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2143" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2143" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2143" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2144">
+      <c r="A2144" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2144" t="inlineStr">
+        <is>
+          <t>St. Martin vs Bahamas</t>
+        </is>
+      </c>
+      <c r="C2144" t="inlineStr">
+        <is>
+          <t>St. Martin</t>
+        </is>
+      </c>
+      <c r="D2144" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2144" t="inlineStr"/>
+      <c r="F2144" t="inlineStr"/>
+      <c r="G2144" t="inlineStr">
+        <is>
+          <t>6-0</t>
+        </is>
+      </c>
+      <c r="H2144" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2144" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2144" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2144" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2144" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2145">
+      <c r="A2145" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2145" t="inlineStr">
+        <is>
+          <t>Sportivo Ameliano vs Rubio Ñú</t>
+        </is>
+      </c>
+      <c r="C2145" t="inlineStr">
+        <is>
+          <t>Sportivo Ameliano</t>
+        </is>
+      </c>
+      <c r="D2145" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2145" t="inlineStr"/>
+      <c r="F2145" t="inlineStr"/>
+      <c r="G2145" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H2145" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2145" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2145" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2145" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2145" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2146">
+      <c r="A2146" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2146" t="inlineStr">
+        <is>
+          <t>St. Vincent and the Grenadines vs Sint Maarten</t>
+        </is>
+      </c>
+      <c r="C2146" t="inlineStr">
+        <is>
+          <t>St. Vincent and the Grenadines</t>
+        </is>
+      </c>
+      <c r="D2146" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2146" t="inlineStr"/>
+      <c r="F2146" t="inlineStr"/>
+      <c r="G2146" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H2146" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2146" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2146" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2146" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2146" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2147">
+      <c r="A2147" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2147" t="inlineStr">
+        <is>
+          <t>Real Potosí vs San Antonio Bulo Bulo</t>
+        </is>
+      </c>
+      <c r="C2147" t="inlineStr">
+        <is>
+          <t>Real Potosí</t>
+        </is>
+      </c>
+      <c r="D2147" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2147" t="inlineStr"/>
+      <c r="F2147" t="inlineStr"/>
+      <c r="G2147" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H2147" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2147" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2147" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2147" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2147" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2148">
+      <c r="A2148" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2148" t="inlineStr">
+        <is>
+          <t>Charlotte 49ers vs Mercer Bears</t>
+        </is>
+      </c>
+      <c r="C2148" t="inlineStr">
+        <is>
+          <t>Charlotte 49ers</t>
+        </is>
+      </c>
+      <c r="D2148" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2148" t="inlineStr"/>
+      <c r="F2148" t="inlineStr"/>
+      <c r="G2148" t="inlineStr">
+        <is>
+          <t>6-0</t>
+        </is>
+      </c>
+      <c r="H2148" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2148" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2148" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2148" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2148" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2149">
+      <c r="A2149" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2149" t="inlineStr">
+        <is>
+          <t>Coastal Carolina Chanticleers vs Campbell Fighting Camels</t>
+        </is>
+      </c>
+      <c r="C2149" t="inlineStr">
+        <is>
+          <t>Coastal Carolina Chanticleers</t>
+        </is>
+      </c>
+      <c r="D2149" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2149" t="inlineStr"/>
+      <c r="F2149" t="inlineStr"/>
+      <c r="G2149" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H2149" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2149" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2149" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2149" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2149" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2150">
+      <c r="A2150" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2150" t="inlineStr">
+        <is>
+          <t>Louisville Cardinals vs DePaul Blue Demons</t>
+        </is>
+      </c>
+      <c r="C2150" t="inlineStr">
+        <is>
+          <t>Louisville Cardinals</t>
+        </is>
+      </c>
+      <c r="D2150" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2150" t="inlineStr"/>
+      <c r="F2150" t="inlineStr"/>
+      <c r="G2150" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H2150" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2150" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2150" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2150" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2150" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2151">
+      <c r="A2151" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2151" t="inlineStr">
+        <is>
+          <t>Loyola Maryland Greyhounds vs Pennsylvania Quakers</t>
+        </is>
+      </c>
+      <c r="C2151" t="inlineStr">
+        <is>
+          <t>Pennsylvania Quakers</t>
+        </is>
+      </c>
+      <c r="D2151" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2151" t="inlineStr"/>
+      <c r="F2151" t="inlineStr"/>
+      <c r="G2151" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2151" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2151" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2151" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2151" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2151" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2152">
+      <c r="A2152" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2152" t="inlineStr">
+        <is>
+          <t>Northeastern Huskies vs Harvard Crimson</t>
+        </is>
+      </c>
+      <c r="C2152" t="inlineStr">
+        <is>
+          <t>Northeastern Huskies</t>
+        </is>
+      </c>
+      <c r="D2152" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2152" t="inlineStr"/>
+      <c r="F2152" t="inlineStr"/>
+      <c r="G2152" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H2152" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2152" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2152" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2152" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2152" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2153">
+      <c r="A2153" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2153" t="inlineStr">
+        <is>
+          <t>UConn Huskies vs Bryant Bulldogs</t>
+        </is>
+      </c>
+      <c r="C2153" t="inlineStr">
+        <is>
+          <t>Bryant Bulldogs</t>
+        </is>
+      </c>
+      <c r="D2153" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2153" t="inlineStr"/>
+      <c r="F2153" t="inlineStr"/>
+      <c r="G2153" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H2153" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2153" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2153" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2153" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2153" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2154">
+      <c r="A2154" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2154" t="inlineStr">
+        <is>
+          <t>Virginia Cavaliers vs Queens University Royals</t>
+        </is>
+      </c>
+      <c r="C2154" t="inlineStr">
+        <is>
+          <t>Virginia Cavaliers</t>
+        </is>
+      </c>
+      <c r="D2154" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2154" t="inlineStr"/>
+      <c r="F2154" t="inlineStr"/>
+      <c r="G2154" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H2154" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2154" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2154" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2154" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2154" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2155">
+      <c r="A2155" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2155" t="inlineStr">
+        <is>
+          <t>Wisconsin Badgers vs Lakeland</t>
+        </is>
+      </c>
+      <c r="C2155" t="inlineStr">
+        <is>
+          <t>Wisconsin Badgers</t>
+        </is>
+      </c>
+      <c r="D2155" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2155" t="inlineStr"/>
+      <c r="F2155" t="inlineStr"/>
+      <c r="G2155" t="inlineStr">
+        <is>
+          <t>8-0</t>
+        </is>
+      </c>
+      <c r="H2155" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2155" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2155" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2155" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2155" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2156">
+      <c r="A2156" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2156" t="inlineStr">
+        <is>
+          <t>Club Olimpia vs Nacional Asunción</t>
+        </is>
+      </c>
+      <c r="C2156" t="inlineStr">
+        <is>
+          <t>Club Olimpia</t>
+        </is>
+      </c>
+      <c r="D2156" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2156" t="inlineStr"/>
+      <c r="F2156" t="inlineStr"/>
+      <c r="G2156" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2156" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2156" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2156" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2156" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2156" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2157">
+      <c r="A2157" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2157" t="inlineStr">
+        <is>
+          <t>Sport vs São Bernardo</t>
+        </is>
+      </c>
+      <c r="C2157" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="D2157" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2157" t="inlineStr"/>
+      <c r="F2157" t="inlineStr"/>
+      <c r="G2157" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H2157" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2157" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2157" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2157" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2157" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2158">
+      <c r="A2158" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2158" t="inlineStr">
+        <is>
+          <t>Columbia Lions vs Brown Bears</t>
+        </is>
+      </c>
+      <c r="C2158" t="inlineStr">
+        <is>
+          <t>Columbia Lions</t>
+        </is>
+      </c>
+      <c r="D2158" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2158" t="inlineStr"/>
+      <c r="F2158" t="inlineStr"/>
+      <c r="G2158" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H2158" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2158" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2158" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2158" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2158" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2159">
+      <c r="A2159" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2159" t="inlineStr">
+        <is>
+          <t>Xavier Muskateers vs Evansville Purple Aces</t>
+        </is>
+      </c>
+      <c r="C2159" t="inlineStr">
+        <is>
+          <t>Xavier Muskateers</t>
+        </is>
+      </c>
+      <c r="D2159" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2159" t="inlineStr"/>
+      <c r="F2159" t="inlineStr"/>
+      <c r="G2159" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H2159" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2159" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2159" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2159" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2159" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2160">
+      <c r="A2160" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2160" t="inlineStr">
+        <is>
+          <t>Argentina vs Benin</t>
+        </is>
+      </c>
+      <c r="C2160" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="D2160" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2160" t="inlineStr"/>
+      <c r="F2160" t="inlineStr"/>
+      <c r="G2160" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H2160" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2160" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2160" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2160" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2160" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2161">
+      <c r="A2161" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2161" t="inlineStr">
+        <is>
+          <t>Antigua and Barbuda vs Aruba</t>
+        </is>
+      </c>
+      <c r="C2161" t="inlineStr">
+        <is>
+          <t>Aruba</t>
+        </is>
+      </c>
+      <c r="D2161" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2161" t="inlineStr"/>
+      <c r="F2161" t="inlineStr"/>
+      <c r="G2161" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H2161" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2161" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2161" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2161" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2161" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2162">
+      <c r="A2162" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2162" t="inlineStr">
+        <is>
+          <t>Goiás vs Athletic</t>
+        </is>
+      </c>
+      <c r="C2162" t="inlineStr">
+        <is>
+          <t>Goiás</t>
+        </is>
+      </c>
+      <c r="D2162" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2162" t="inlineStr"/>
+      <c r="F2162" t="inlineStr"/>
+      <c r="G2162" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H2162" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2162" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2162" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2162" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2162" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2163">
+      <c r="A2163" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2163" t="inlineStr">
+        <is>
+          <t>Colo Colo vs Puerto Montt</t>
+        </is>
+      </c>
+      <c r="C2163" t="inlineStr">
+        <is>
+          <t>Colo Colo</t>
+        </is>
+      </c>
+      <c r="D2163" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2163" t="inlineStr"/>
+      <c r="F2163" t="inlineStr"/>
+      <c r="G2163" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H2163" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2163" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2163" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2163" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2163" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2164">
+      <c r="A2164" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2164" t="inlineStr">
+        <is>
+          <t>Colombia vs Peru</t>
+        </is>
+      </c>
+      <c r="C2164" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="D2164" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2164" t="inlineStr"/>
+      <c r="F2164" t="inlineStr"/>
+      <c r="G2164" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H2164" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2164" t="n">
+        <v>3</v>
+      </c>
+      <c r="J2164" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2164" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2164" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2165">
+      <c r="A2165" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2165" t="inlineStr">
+        <is>
+          <t>Aurora vs ABB</t>
+        </is>
+      </c>
+      <c r="C2165" t="inlineStr">
+        <is>
+          <t>Aurora</t>
+        </is>
+      </c>
+      <c r="D2165" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2165" t="inlineStr"/>
+      <c r="F2165" t="inlineStr"/>
+      <c r="G2165" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H2165" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2165" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2165" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2165" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2165" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2166">
+      <c r="A2166" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2166" t="inlineStr">
+        <is>
+          <t>Chicago Fire FC vs Vancouver Whitecaps</t>
+        </is>
+      </c>
+      <c r="C2166" t="inlineStr">
+        <is>
+          <t>Chicago Fire FC</t>
+        </is>
+      </c>
+      <c r="D2166" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2166" t="inlineStr"/>
+      <c r="F2166" t="inlineStr"/>
+      <c r="G2166" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H2166" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2166" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2166" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2166" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2166" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2167">
+      <c r="A2167" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2167" t="inlineStr">
+        <is>
+          <t>Ponte Preta vs Juventude</t>
+        </is>
+      </c>
+      <c r="C2167" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="D2167" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E2167" t="inlineStr"/>
+      <c r="F2167" t="inlineStr"/>
+      <c r="G2167" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H2167" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2167" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2167" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2167" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2167" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2168">
+      <c r="A2168" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2168" t="inlineStr">
+        <is>
+          <t>French Guiana vs Belize</t>
+        </is>
+      </c>
+      <c r="C2168" t="inlineStr">
+        <is>
+          <t>French Guiana</t>
+        </is>
+      </c>
+      <c r="D2168" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2168" t="inlineStr"/>
+      <c r="F2168" t="inlineStr"/>
+      <c r="G2168" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H2168" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2168" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2168" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2168" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2168" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="2169">
+      <c r="A2169" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B2169" t="inlineStr">
+        <is>
+          <t>Mexico vs Chile</t>
+        </is>
+      </c>
+      <c r="C2169" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="D2169" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E2169" t="inlineStr"/>
+      <c r="F2169" t="inlineStr"/>
+      <c r="G2169" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H2169" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I2169" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2169" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2169" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2169" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -96467,7 +100385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -97142,6 +101060,25 @@
       </c>
       <c r="E36" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>83</v>
+      </c>
+      <c r="C37" t="n">
+        <v>63</v>
+      </c>
+      <c r="D37" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="E37" t="n">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -97155,7 +101092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G185"/>
+  <dimension ref="A1:G194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -101460,6 +105397,249 @@
         <v>0</v>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>6</v>
+      </c>
+      <c r="D186" t="n">
+        <v>4</v>
+      </c>
+      <c r="E186" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F186" t="n">
+        <v>2</v>
+      </c>
+      <c r="G186" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>posible_descuento</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>2</v>
+      </c>
+      <c r="D187" t="n">
+        <v>1</v>
+      </c>
+      <c r="E187" t="n">
+        <v>50</v>
+      </c>
+      <c r="F187" t="n">
+        <v>1</v>
+      </c>
+      <c r="G187" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>9</v>
+      </c>
+      <c r="D188" t="n">
+        <v>6</v>
+      </c>
+      <c r="E188" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F188" t="n">
+        <v>3</v>
+      </c>
+      <c r="G188" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>4</v>
+      </c>
+      <c r="D189" t="n">
+        <v>3</v>
+      </c>
+      <c r="E189" t="n">
+        <v>75</v>
+      </c>
+      <c r="F189" t="n">
+        <v>1</v>
+      </c>
+      <c r="G189" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>4</v>
+      </c>
+      <c r="D190" t="n">
+        <v>4</v>
+      </c>
+      <c r="E190" t="n">
+        <v>100</v>
+      </c>
+      <c r="F190" t="n">
+        <v>0</v>
+      </c>
+      <c r="G190" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>siguen_empatados_55</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>1</v>
+      </c>
+      <c r="D191" t="n">
+        <v>1</v>
+      </c>
+      <c r="E191" t="n">
+        <v>100</v>
+      </c>
+      <c r="F191" t="n">
+        <v>0</v>
+      </c>
+      <c r="G191" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>siguen_empatados_70</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>2</v>
+      </c>
+      <c r="D192" t="n">
+        <v>2</v>
+      </c>
+      <c r="E192" t="n">
+        <v>100</v>
+      </c>
+      <c r="F192" t="n">
+        <v>0</v>
+      </c>
+      <c r="G192" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>2</v>
+      </c>
+      <c r="D193" t="n">
+        <v>0</v>
+      </c>
+      <c r="E193" t="n">
+        <v>0</v>
+      </c>
+      <c r="F193" t="n">
+        <v>2</v>
+      </c>
+      <c r="G193" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>siguen_empatados_22</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>3</v>
+      </c>
+      <c r="D194" t="n">
+        <v>3</v>
+      </c>
+      <c r="E194" t="n">
+        <v>100</v>
+      </c>
+      <c r="F194" t="n">
+        <v>0</v>
+      </c>
+      <c r="G194" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>